<commit_message>
Add commander progression system + make morale a real combat stat
- governor.gd: add morale int (0-100, default 50)
- army.gd: apply morale multiplier to armyPunch/armyDefence in surveySelf()
  (morale 50 = +12.5%, morale 100 = +25%, morale 0 = no bonus)
- world.gd: fix _apply_morale_boost() to actually modify governor.morale;
  add promote_commander outcome (increments governorLevel 1→2→3, sets
  questComplete at level 3); add _commander_turns dict, _tick_commander_turns(),
  _check_cmd_merit/recognition/thanks() firing at 5/20/50 turns served
- events.csv: replace CMD_OBJECTIVE_1 + CMD_REUNION with CMD_MERIT,
  CMD_RECOGNITION, CMD_THANKS (3-stage chain keyed to governorLevel)
- event_buttons.csv: replace old CMD buttons with promote_commander +
  morale_boost buttons; CMD_THANKS BTN2 is explicit gated
- event_masterdoc.xlsx + build script updated (117 events total)

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -987,7 +987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N132"/>
+  <dimension ref="A1:N133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5599,12 +5599,12 @@
       </c>
       <c r="C74" s="30" t="inlineStr">
         <is>
-          <t>CMD_OBJECTIVE_1</t>
+          <t>CMD_MERIT</t>
         </is>
       </c>
       <c r="D74" s="31" t="inlineStr">
         <is>
-          <t>A COMMANDER COMPLETES THEIR FIRST TASK</t>
+          <t>FIELD PROMOTION: [COMMANDER_NAME] DISTINGUISHED IN EARLY OPERATIONS</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="G74" s="31" t="inlineStr">
         <is>
-          <t>→ CMD_REUNION (arc conclusion)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr">
@@ -5627,11 +5627,7 @@
           <t>FIRST PASS</t>
         </is>
       </c>
-      <c r="I74" s="30" t="inlineStr">
-        <is>
-          <t>commander_obj1</t>
-        </is>
-      </c>
+      <c r="I74" s="30" t="inlineStr"/>
       <c r="J74" s="7" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -5650,7 +5646,7 @@
       </c>
       <c r="N74" s="31" t="inlineStr">
         <is>
-          <t>commander_objective type; non-repeatable; [COMMANDER_NAME] substitution</t>
+          <t>Fires at governorLevel==1 after 5 turns stationed; promote_commander BTN1; morale_boost BTN2</t>
         </is>
       </c>
     </row>
@@ -5667,148 +5663,140 @@
       </c>
       <c r="C75" s="30" t="inlineStr">
         <is>
-          <t>CMD_REUNION</t>
+          <t>CMD_RECOGNITION</t>
         </is>
       </c>
       <c r="D75" s="31" t="inlineStr">
         <is>
-          <t>THE REUNION</t>
-        </is>
-      </c>
-      <c r="E75" s="22" t="inlineStr">
+          <t>CITATION FOR EXCEPTIONAL SERVICE: [COMMANDER_NAME] AT [TILE_NAME]</t>
+        </is>
+      </c>
+      <c r="E75" s="28" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="F75" s="31" t="inlineStr">
+        <is>
+          <t>CMD_MERIT</t>
+        </is>
+      </c>
+      <c r="G75" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I75" s="30" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K75" s="32" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L75" s="30" t="inlineStr"/>
+      <c r="M75" s="32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N75" s="31" t="inlineStr">
+        <is>
+          <t>Fires at governorLevel==2 after 20 turns stationed; promote_commander BTN1; claim_change BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>Commander</t>
+        </is>
+      </c>
+      <c r="B76" s="29" t="inlineStr">
+        <is>
+          <t>Commander Arc</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>CMD_THANKS</t>
+        </is>
+      </c>
+      <c r="D76" s="31" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE DELIVERS PERSONAL THANKS TO [COMMANDER_NAME] AT [TILE_NAME]</t>
+        </is>
+      </c>
+      <c r="E76" s="22" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="F75" s="31" t="inlineStr">
-        <is>
-          <t>CMD_OBJECTIVE_1</t>
-        </is>
-      </c>
-      <c r="G75" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I75" s="30" t="inlineStr">
-        <is>
-          <t>commander_reunion</t>
-        </is>
-      </c>
-      <c r="J75" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K75" s="26" t="inlineStr">
+      <c r="F76" s="31" t="inlineStr">
+        <is>
+          <t>CMD_RECOGNITION</t>
+        </is>
+      </c>
+      <c r="G76" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I76" s="30" t="inlineStr"/>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K76" s="26" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="L75" s="30" t="inlineStr">
+      <c r="L76" s="30" t="inlineStr">
         <is>
           <t>explicit</t>
         </is>
       </c>
-      <c r="M75" s="32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N75" s="31" t="inlineStr">
-        <is>
-          <t>commander_reunion type; explicit gated; non-repeatable</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="8" customHeight="1">
-      <c r="A76" s="9" t="n"/>
-      <c r="B76" s="9" t="n"/>
-      <c r="C76" s="9" t="n"/>
-      <c r="D76" s="9" t="n"/>
-      <c r="E76" s="9" t="n"/>
-      <c r="F76" s="9" t="n"/>
-      <c r="G76" s="9" t="n"/>
-      <c r="H76" s="9" t="n"/>
-      <c r="I76" s="9" t="n"/>
-      <c r="J76" s="9" t="n"/>
-      <c r="K76" s="9" t="n"/>
-      <c r="L76" s="9" t="n"/>
-      <c r="M76" s="9" t="n"/>
-      <c r="N76" s="9" t="n"/>
-    </row>
-    <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="33" t="inlineStr">
-        <is>
-          <t>Fort Chain</t>
-        </is>
-      </c>
-      <c r="B77" s="33" t="inlineStr">
-        <is>
-          <t>Fort Disrepair</t>
-        </is>
-      </c>
-      <c r="C77" s="34" t="inlineStr">
-        <is>
-          <t>FORT_001</t>
-        </is>
-      </c>
-      <c r="D77" s="35" t="inlineStr">
-        <is>
-          <t>FORT [TILE_NAME]: STRUCTURAL CONCERNS AND A PAMPHLET PROBLEM</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F77" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G77" s="35" t="inlineStr">
-        <is>
-          <t>→ FORT_003 (BTN1) | → FORT_004 (BTN2)</t>
-        </is>
-      </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I77" s="34" t="inlineStr">
-        <is>
-          <t>fort_pamphlets</t>
-        </is>
-      </c>
-      <c r="J77" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K77" s="36" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L77" s="34" t="inlineStr"/>
-      <c r="M77" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N77" s="35" t="inlineStr">
-        <is>
-          <t>Fires at Fortress tiles; requires governor + no fortDisrepair; army station required</t>
-        </is>
-      </c>
+      <c r="M76" s="32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N76" s="31" t="inlineStr">
+        <is>
+          <t>Fires at governorLevel==3 after 50 turns stationed; BTN2 explicit morale_boost +40; non-repeatable</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="8" customHeight="1">
+      <c r="A77" s="9" t="n"/>
+      <c r="B77" s="9" t="n"/>
+      <c r="C77" s="9" t="n"/>
+      <c r="D77" s="9" t="n"/>
+      <c r="E77" s="9" t="n"/>
+      <c r="F77" s="9" t="n"/>
+      <c r="G77" s="9" t="n"/>
+      <c r="H77" s="9" t="n"/>
+      <c r="I77" s="9" t="n"/>
+      <c r="J77" s="9" t="n"/>
+      <c r="K77" s="9" t="n"/>
+      <c r="L77" s="9" t="n"/>
+      <c r="M77" s="9" t="n"/>
+      <c r="N77" s="9" t="n"/>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="33" t="inlineStr">
@@ -5823,27 +5811,27 @@
       </c>
       <c r="C78" s="34" t="inlineStr">
         <is>
-          <t>FORT_003</t>
+          <t>FORT_001</t>
         </is>
       </c>
       <c r="D78" s="35" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE FIRES [COMMANDER_NAME] IN FRONT OF GOD AND THE GARRISON</t>
-        </is>
-      </c>
-      <c r="E78" s="28" t="inlineStr">
-        <is>
-          <t>Branch</t>
+          <t>FORT [TILE_NAME]: STRUCTURAL CONCERNS AND A PAMPHLET PROBLEM</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F78" s="35" t="inlineStr">
         <is>
-          <t>FORT_001 BTN1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G78" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ FORT_003 (BTN1) | → FORT_004 (BTN2)</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr">
@@ -5853,7 +5841,7 @@
       </c>
       <c r="I78" s="34" t="inlineStr">
         <is>
-          <t>fort_confrontation</t>
+          <t>fort_pamphlets</t>
         </is>
       </c>
       <c r="J78" s="7" t="inlineStr">
@@ -5874,7 +5862,7 @@
       </c>
       <c r="N78" s="35" t="inlineStr">
         <is>
-          <t>Public confrontation path; removes governor; generates replacement</t>
+          <t>Fires at Fortress tiles; requires governor + no fortDisrepair; army station required</t>
         </is>
       </c>
     </row>
@@ -5891,12 +5879,12 @@
       </c>
       <c r="C79" s="34" t="inlineStr">
         <is>
-          <t>FORT_004</t>
+          <t>FORT_003</t>
         </is>
       </c>
       <c r="D79" s="35" t="inlineStr">
         <is>
-          <t>FORT [TILE_NAME] REPAIR ORDER SIGNED — GRIEVANCES RESOLVED</t>
+          <t>PRESIDENT CARLISLE FIRES [COMMANDER_NAME] IN FRONT OF GOD AND THE GARRISON</t>
         </is>
       </c>
       <c r="E79" s="28" t="inlineStr">
@@ -5906,12 +5894,12 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>FORT_001 BTN2</t>
+          <t>FORT_001 BTN1</t>
         </is>
       </c>
       <c r="G79" s="35" t="inlineStr">
         <is>
-          <t>→ FORT_005</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H79" s="6" t="inlineStr">
@@ -5921,7 +5909,7 @@
       </c>
       <c r="I79" s="34" t="inlineStr">
         <is>
-          <t>fort_handshake</t>
+          <t>fort_confrontation</t>
         </is>
       </c>
       <c r="J79" s="7" t="inlineStr">
@@ -5942,7 +5930,7 @@
       </c>
       <c r="N79" s="35" t="inlineStr">
         <is>
-          <t>Private resolution path; repair_fort outcome; chains to FORT_005</t>
+          <t>Public confrontation path; removes governor; generates replacement</t>
         </is>
       </c>
     </row>
@@ -5959,148 +5947,148 @@
       </c>
       <c r="C80" s="34" t="inlineStr">
         <is>
+          <t>FORT_004</t>
+        </is>
+      </c>
+      <c r="D80" s="35" t="inlineStr">
+        <is>
+          <t>FORT [TILE_NAME] REPAIR ORDER SIGNED — GRIEVANCES RESOLVED</t>
+        </is>
+      </c>
+      <c r="E80" s="28" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="F80" s="35" t="inlineStr">
+        <is>
+          <t>FORT_001 BTN2</t>
+        </is>
+      </c>
+      <c r="G80" s="35" t="inlineStr">
+        <is>
+          <t>→ FORT_005</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I80" s="34" t="inlineStr">
+        <is>
+          <t>fort_handshake</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K80" s="36" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L80" s="34" t="inlineStr"/>
+      <c r="M80" s="36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N80" s="35" t="inlineStr">
+        <is>
+          <t>Private resolution path; repair_fort outcome; chains to FORT_005</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="33" t="inlineStr">
+        <is>
+          <t>Fort Chain</t>
+        </is>
+      </c>
+      <c r="B81" s="33" t="inlineStr">
+        <is>
+          <t>Fort Disrepair</t>
+        </is>
+      </c>
+      <c r="C81" s="34" t="inlineStr">
+        <is>
           <t>FORT_005</t>
         </is>
       </c>
-      <c r="D80" s="35" t="inlineStr">
+      <c r="D81" s="35" t="inlineStr">
         <is>
           <t>CLASSIFIED DIPLOMATIC PROCEEDINGS AT [TILE_NAME]</t>
         </is>
       </c>
-      <c r="E80" s="22" t="inlineStr">
+      <c r="E81" s="22" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="F80" s="35" t="inlineStr">
+      <c r="F81" s="35" t="inlineStr">
         <is>
           <t>FORT_004</t>
         </is>
       </c>
-      <c r="G80" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I80" s="34" t="inlineStr">
+      <c r="G81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I81" s="34" t="inlineStr">
         <is>
           <t>fort_diplomatic</t>
         </is>
       </c>
-      <c r="J80" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K80" s="26" t="inlineStr">
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K81" s="26" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="L80" s="34" t="inlineStr">
+      <c r="L81" s="34" t="inlineStr">
         <is>
           <t>explicit</t>
         </is>
       </c>
-      <c r="M80" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N80" s="35" t="inlineStr">
+      <c r="M81" s="36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N81" s="35" t="inlineStr">
         <is>
           <t>Explicit reward event; BTN1 explicit morale+30 / BTN2 standard morale+10</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="8" customHeight="1">
-      <c r="A81" s="9" t="n"/>
-      <c r="B81" s="9" t="n"/>
-      <c r="C81" s="9" t="n"/>
-      <c r="D81" s="9" t="n"/>
-      <c r="E81" s="9" t="n"/>
-      <c r="F81" s="9" t="n"/>
-      <c r="G81" s="9" t="n"/>
-      <c r="H81" s="9" t="n"/>
-      <c r="I81" s="9" t="n"/>
-      <c r="J81" s="9" t="n"/>
-      <c r="K81" s="9" t="n"/>
-      <c r="L81" s="9" t="n"/>
-      <c r="M81" s="9" t="n"/>
-      <c r="N81" s="9" t="n"/>
-    </row>
-    <row r="82" ht="30" customHeight="1">
-      <c r="A82" s="37" t="inlineStr">
-        <is>
-          <t>Collapse</t>
-        </is>
-      </c>
-      <c r="B82" s="37" t="inlineStr">
-        <is>
-          <t>Republic Falls</t>
-        </is>
-      </c>
-      <c r="C82" s="38" t="inlineStr">
-        <is>
-          <t>COLLAPSE_01</t>
-        </is>
-      </c>
-      <c r="D82" s="39" t="inlineStr">
-        <is>
-          <t>THE REPUBLIC HAS FALLEN</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F82" s="39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G82" s="39" t="inlineStr">
-        <is>
-          <t>→ COLLAPSE_02</t>
-        </is>
-      </c>
-      <c r="H82" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I82" s="38" t="inlineStr">
-        <is>
-          <t>collapse_republic</t>
-        </is>
-      </c>
-      <c r="J82" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K82" s="40" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L82" s="38" t="inlineStr"/>
-      <c r="M82" s="40" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N82" s="39" t="inlineStr">
-        <is>
-          <t>trigger_collapse outcome; fires when all metros fall</t>
-        </is>
-      </c>
+    <row r="82" ht="8" customHeight="1">
+      <c r="A82" s="9" t="n"/>
+      <c r="B82" s="9" t="n"/>
+      <c r="C82" s="9" t="n"/>
+      <c r="D82" s="9" t="n"/>
+      <c r="E82" s="9" t="n"/>
+      <c r="F82" s="9" t="n"/>
+      <c r="G82" s="9" t="n"/>
+      <c r="H82" s="9" t="n"/>
+      <c r="I82" s="9" t="n"/>
+      <c r="J82" s="9" t="n"/>
+      <c r="K82" s="9" t="n"/>
+      <c r="L82" s="9" t="n"/>
+      <c r="M82" s="9" t="n"/>
+      <c r="N82" s="9" t="n"/>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="37" t="inlineStr">
@@ -6115,148 +6103,148 @@
       </c>
       <c r="C83" s="38" t="inlineStr">
         <is>
+          <t>COLLAPSE_01</t>
+        </is>
+      </c>
+      <c r="D83" s="39" t="inlineStr">
+        <is>
+          <t>THE REPUBLIC HAS FALLEN</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F83" s="39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G83" s="39" t="inlineStr">
+        <is>
+          <t>→ COLLAPSE_02</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I83" s="38" t="inlineStr">
+        <is>
+          <t>collapse_republic</t>
+        </is>
+      </c>
+      <c r="J83" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K83" s="40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L83" s="38" t="inlineStr"/>
+      <c r="M83" s="40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N83" s="39" t="inlineStr">
+        <is>
+          <t>trigger_collapse outcome; fires when all metros fall</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="37" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+      <c r="B84" s="37" t="inlineStr">
+        <is>
+          <t>Republic Falls</t>
+        </is>
+      </c>
+      <c r="C84" s="38" t="inlineStr">
+        <is>
           <t>COLLAPSE_02</t>
         </is>
       </c>
-      <c r="D83" s="39" t="inlineStr">
+      <c r="D84" s="39" t="inlineStr">
         <is>
           <t>WASHINGTON STANDS ALONE</t>
         </is>
       </c>
-      <c r="E83" s="22" t="inlineStr">
+      <c r="E84" s="22" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="F83" s="39" t="inlineStr">
+      <c r="F84" s="39" t="inlineStr">
         <is>
           <t>COLLAPSE_01</t>
         </is>
       </c>
-      <c r="G83" s="39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H83" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I83" s="38" t="inlineStr">
+      <c r="G84" s="39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I84" s="38" t="inlineStr">
         <is>
           <t>ualani_washington</t>
         </is>
       </c>
-      <c r="J83" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K83" s="26" t="inlineStr">
+      <c r="J84" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K84" s="26" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="L83" s="38" t="inlineStr">
+      <c r="L84" s="38" t="inlineStr">
         <is>
           <t>explicit option</t>
         </is>
       </c>
-      <c r="M83" s="40" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N83" s="39" t="inlineStr">
+      <c r="M84" s="40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N84" s="39" t="inlineStr">
         <is>
           <t>BTN1 explicit 'The Long Night' morale+30 / BTN2 standard 'Hold the Line' morale+10</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="8" customHeight="1">
-      <c r="A84" s="9" t="n"/>
-      <c r="B84" s="9" t="n"/>
-      <c r="C84" s="9" t="n"/>
-      <c r="D84" s="9" t="n"/>
-      <c r="E84" s="9" t="n"/>
-      <c r="F84" s="9" t="n"/>
-      <c r="G84" s="9" t="n"/>
-      <c r="H84" s="9" t="n"/>
-      <c r="I84" s="9" t="n"/>
-      <c r="J84" s="9" t="n"/>
-      <c r="K84" s="9" t="n"/>
-      <c r="L84" s="9" t="n"/>
-      <c r="M84" s="9" t="n"/>
-      <c r="N84" s="9" t="n"/>
-    </row>
-    <row r="85" ht="30" customHeight="1">
-      <c r="A85" s="41" t="inlineStr">
-        <is>
-          <t>Tile Crisis</t>
-        </is>
-      </c>
-      <c r="B85" s="41" t="inlineStr">
-        <is>
-          <t>Harvest Crisis</t>
-        </is>
-      </c>
-      <c r="C85" s="42" t="inlineStr">
-        <is>
-          <t>HARVEST_001</t>
-        </is>
-      </c>
-      <c r="D85" s="43" t="inlineStr">
-        <is>
-          <t>THE ARMY ATE THE SEED CORN</t>
-        </is>
-      </c>
-      <c r="E85" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F85" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G85" s="43" t="inlineStr">
-        <is>
-          <t>→ HARVEST_VISIT_01 (BTN1 mission)</t>
-        </is>
-      </c>
-      <c r="H85" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I85" s="42" t="inlineStr">
-        <is>
-          <t>harvest_crisis</t>
-        </is>
-      </c>
-      <c r="J85" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K85" s="44" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L85" s="42" t="inlineStr"/>
-      <c r="M85" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N85" s="43" t="inlineStr">
-        <is>
-          <t>Fires when food &lt; 50; Farm tile required; set_mission_flag BTN1</t>
-        </is>
-      </c>
+    <row r="85" ht="8" customHeight="1">
+      <c r="A85" s="9" t="n"/>
+      <c r="B85" s="9" t="n"/>
+      <c r="C85" s="9" t="n"/>
+      <c r="D85" s="9" t="n"/>
+      <c r="E85" s="9" t="n"/>
+      <c r="F85" s="9" t="n"/>
+      <c r="G85" s="9" t="n"/>
+      <c r="H85" s="9" t="n"/>
+      <c r="I85" s="9" t="n"/>
+      <c r="J85" s="9" t="n"/>
+      <c r="K85" s="9" t="n"/>
+      <c r="L85" s="9" t="n"/>
+      <c r="M85" s="9" t="n"/>
+      <c r="N85" s="9" t="n"/>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="41" t="inlineStr">
@@ -6271,27 +6259,27 @@
       </c>
       <c r="C86" s="42" t="inlineStr">
         <is>
-          <t>HARVEST_VISIT_01</t>
+          <t>HARVEST_001</t>
         </is>
       </c>
       <c r="D86" s="43" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE SAVES THE HARVEST</t>
-        </is>
-      </c>
-      <c r="E86" s="22" t="inlineStr">
-        <is>
-          <t>Followup</t>
+          <t>THE ARMY ATE THE SEED CORN</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F86" s="43" t="inlineStr">
         <is>
-          <t>HARVEST_001 BTN1 (army mission)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G86" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ HARVEST_VISIT_01 (BTN1 mission)</t>
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr">
@@ -6301,7 +6289,7 @@
       </c>
       <c r="I86" s="42" t="inlineStr">
         <is>
-          <t>harvest_complete</t>
+          <t>harvest_crisis</t>
         </is>
       </c>
       <c r="J86" s="7" t="inlineStr">
@@ -6309,16 +6297,12 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K86" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L86" s="42" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
+      <c r="K86" s="44" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L86" s="42" t="inlineStr"/>
       <c r="M86" s="44" t="inlineStr">
         <is>
           <t>0</t>
@@ -6326,7 +6310,7 @@
       </c>
       <c r="N86" s="43" t="inlineStr">
         <is>
-          <t>BTN2 explicit 'Presidential Persuasion' +food 80 vs BTN1 standard +food 60</t>
+          <t>Fires when food &lt; 50; Farm tile required; set_mission_flag BTN1</t>
         </is>
       </c>
     </row>
@@ -6338,32 +6322,32 @@
       </c>
       <c r="B87" s="41" t="inlineStr">
         <is>
-          <t>Harbor Threat</t>
+          <t>Harvest Crisis</t>
         </is>
       </c>
       <c r="C87" s="42" t="inlineStr">
         <is>
-          <t>HARBOR_001</t>
+          <t>HARVEST_VISIT_01</t>
         </is>
       </c>
       <c r="D87" s="43" t="inlineStr">
         <is>
-          <t>CROWN VESSELS SPOTTED: DOCK AT [TILE_NAME] AT RISK</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>PRESIDENT CARLISLE SAVES THE HARVEST</t>
+        </is>
+      </c>
+      <c r="E87" s="22" t="inlineStr">
+        <is>
+          <t>Followup</t>
         </is>
       </c>
       <c r="F87" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HARVEST_001 BTN1 (army mission)</t>
         </is>
       </c>
       <c r="G87" s="43" t="inlineStr">
         <is>
-          <t>→ HARBOR_ESCORT_01 (BTN1) | → HARBOR_BURN_01 (BTN2)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H87" s="6" t="inlineStr">
@@ -6373,7 +6357,7 @@
       </c>
       <c r="I87" s="42" t="inlineStr">
         <is>
-          <t>harbor_threat</t>
+          <t>harvest_complete</t>
         </is>
       </c>
       <c r="J87" s="7" t="inlineStr">
@@ -6381,12 +6365,16 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K87" s="44" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L87" s="42" t="inlineStr"/>
+      <c r="K87" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L87" s="42" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M87" s="44" t="inlineStr">
         <is>
           <t>0</t>
@@ -6394,7 +6382,7 @@
       </c>
       <c r="N87" s="43" t="inlineStr">
         <is>
-          <t>Dock tile required + UK neighbor; army station required</t>
+          <t>BTN2 explicit 'Presidential Persuasion' +food 80 vs BTN1 standard +food 60</t>
         </is>
       </c>
     </row>
@@ -6411,27 +6399,27 @@
       </c>
       <c r="C88" s="42" t="inlineStr">
         <is>
-          <t>HARBOR_ESCORT_01</t>
+          <t>HARBOR_001</t>
         </is>
       </c>
       <c r="D88" s="43" t="inlineStr">
         <is>
-          <t>HARBOR SECURED: CROWN FRIGATE RETREATS</t>
-        </is>
-      </c>
-      <c r="E88" s="28" t="inlineStr">
-        <is>
-          <t>Branch</t>
+          <t>CROWN VESSELS SPOTTED: DOCK AT [TILE_NAME] AT RISK</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F88" s="43" t="inlineStr">
         <is>
-          <t>HARBOR_001 BTN1 (army mission)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G88" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ HARBOR_ESCORT_01 (BTN1) | → HARBOR_BURN_01 (BTN2)</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
@@ -6441,7 +6429,7 @@
       </c>
       <c r="I88" s="42" t="inlineStr">
         <is>
-          <t>harbor_secure</t>
+          <t>harbor_threat</t>
         </is>
       </c>
       <c r="J88" s="7" t="inlineStr">
@@ -6462,7 +6450,7 @@
       </c>
       <c r="N88" s="43" t="inlineStr">
         <is>
-          <t>+food 30; garrison path</t>
+          <t>Dock tile required + UK neighbor; army station required</t>
         </is>
       </c>
     </row>
@@ -6479,12 +6467,12 @@
       </c>
       <c r="C89" s="42" t="inlineStr">
         <is>
-          <t>HARBOR_BURN_01</t>
+          <t>HARBOR_ESCORT_01</t>
         </is>
       </c>
       <c r="D89" s="43" t="inlineStr">
         <is>
-          <t>DOCK FACILITIES DESTROYED: ACCESS DENIED</t>
+          <t>HARBOR SECURED: CROWN FRIGATE RETREATS</t>
         </is>
       </c>
       <c r="E89" s="28" t="inlineStr">
@@ -6494,7 +6482,7 @@
       </c>
       <c r="F89" s="43" t="inlineStr">
         <is>
-          <t>HARBOR_001 BTN2 (army mission)</t>
+          <t>HARBOR_001 BTN1 (army mission)</t>
         </is>
       </c>
       <c r="G89" s="43" t="inlineStr">
@@ -6509,7 +6497,7 @@
       </c>
       <c r="I89" s="42" t="inlineStr">
         <is>
-          <t>harbor_burned</t>
+          <t>harbor_secure</t>
         </is>
       </c>
       <c r="J89" s="7" t="inlineStr">
@@ -6530,7 +6518,7 @@
       </c>
       <c r="N89" s="43" t="inlineStr">
         <is>
-          <t>disable_building Dock 8 turns; destruction path</t>
+          <t>+food 30; garrison path</t>
         </is>
       </c>
     </row>
@@ -6542,32 +6530,32 @@
       </c>
       <c r="B90" s="41" t="inlineStr">
         <is>
-          <t>Forge Threat</t>
+          <t>Harbor Threat</t>
         </is>
       </c>
       <c r="C90" s="42" t="inlineStr">
         <is>
-          <t>FORGE_001</t>
+          <t>HARBOR_BURN_01</t>
         </is>
       </c>
       <c r="D90" s="43" t="inlineStr">
         <is>
-          <t>INTELLIGENCE ALERT: CROWN FORCES LOCATE THE FORGE AT [TILE_NAME]</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>DOCK FACILITIES DESTROYED: ACCESS DENIED</t>
+        </is>
+      </c>
+      <c r="E90" s="28" t="inlineStr">
+        <is>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F90" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HARBOR_001 BTN2 (army mission)</t>
         </is>
       </c>
       <c r="G90" s="43" t="inlineStr">
         <is>
-          <t>→ FORGE_REINFORCE_01 (BTN1) | → FORGE_EVACUATE_01 (BTN2)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H90" s="6" t="inlineStr">
@@ -6577,7 +6565,7 @@
       </c>
       <c r="I90" s="42" t="inlineStr">
         <is>
-          <t>forge_threat</t>
+          <t>harbor_burned</t>
         </is>
       </c>
       <c r="J90" s="7" t="inlineStr">
@@ -6598,7 +6586,7 @@
       </c>
       <c r="N90" s="43" t="inlineStr">
         <is>
-          <t>Forge tile required + UK neighbor; army station required</t>
+          <t>disable_building Dock 8 turns; destruction path</t>
         </is>
       </c>
     </row>
@@ -6615,27 +6603,27 @@
       </c>
       <c r="C91" s="42" t="inlineStr">
         <is>
-          <t>FORGE_REINFORCE_01</t>
+          <t>FORGE_001</t>
         </is>
       </c>
       <c r="D91" s="43" t="inlineStr">
         <is>
-          <t>FORGE SECURED: CROWN ASSAULT PLAN ABANDONED</t>
-        </is>
-      </c>
-      <c r="E91" s="28" t="inlineStr">
-        <is>
-          <t>Branch</t>
+          <t>INTELLIGENCE ALERT: CROWN FORCES LOCATE THE FORGE AT [TILE_NAME]</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F91" s="43" t="inlineStr">
         <is>
-          <t>FORGE_001 BTN1 (army mission)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G91" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ FORGE_REINFORCE_01 (BTN1) | → FORGE_EVACUATE_01 (BTN2)</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
@@ -6645,7 +6633,7 @@
       </c>
       <c r="I91" s="42" t="inlineStr">
         <is>
-          <t>forge_secure</t>
+          <t>forge_threat</t>
         </is>
       </c>
       <c r="J91" s="7" t="inlineStr">
@@ -6666,7 +6654,7 @@
       </c>
       <c r="N91" s="43" t="inlineStr">
         <is>
-          <t>+weapons 30; defense path</t>
+          <t>Forge tile required + UK neighbor; army station required</t>
         </is>
       </c>
     </row>
@@ -6683,12 +6671,12 @@
       </c>
       <c r="C92" s="42" t="inlineStr">
         <is>
-          <t>FORGE_EVACUATE_01</t>
+          <t>FORGE_REINFORCE_01</t>
         </is>
       </c>
       <c r="D92" s="43" t="inlineStr">
         <is>
-          <t>EMERGENCY EXTRACTION: WEAPONS CACHE SECURED</t>
+          <t>FORGE SECURED: CROWN ASSAULT PLAN ABANDONED</t>
         </is>
       </c>
       <c r="E92" s="28" t="inlineStr">
@@ -6698,7 +6686,7 @@
       </c>
       <c r="F92" s="43" t="inlineStr">
         <is>
-          <t>FORGE_001 BTN2 (army mission)</t>
+          <t>FORGE_001 BTN1 (army mission)</t>
         </is>
       </c>
       <c r="G92" s="43" t="inlineStr">
@@ -6713,7 +6701,7 @@
       </c>
       <c r="I92" s="42" t="inlineStr">
         <is>
-          <t>forge_evac</t>
+          <t>forge_secure</t>
         </is>
       </c>
       <c r="J92" s="7" t="inlineStr">
@@ -6734,7 +6722,7 @@
       </c>
       <c r="N92" s="43" t="inlineStr">
         <is>
-          <t>+weapons 25; Forge temporarily offline</t>
+          <t>+weapons 30; defense path</t>
         </is>
       </c>
     </row>
@@ -6746,32 +6734,32 @@
       </c>
       <c r="B93" s="41" t="inlineStr">
         <is>
-          <t>Corruption Crisis</t>
+          <t>Forge Threat</t>
         </is>
       </c>
       <c r="C93" s="42" t="inlineStr">
         <is>
-          <t>CORRUPT_001</t>
+          <t>FORGE_EVACUATE_01</t>
         </is>
       </c>
       <c r="D93" s="43" t="inlineStr">
         <is>
-          <t>MAGISTRATE [COMMANDER_NAME] UNDER INVESTIGATION</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>EMERGENCY EXTRACTION: WEAPONS CACHE SECURED</t>
+        </is>
+      </c>
+      <c r="E93" s="28" t="inlineStr">
+        <is>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F93" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FORGE_001 BTN2 (army mission)</t>
         </is>
       </c>
       <c r="G93" s="43" t="inlineStr">
         <is>
-          <t>→ CORRUPT_TRIAL_01 (BTN1) | → CORRUPT_DEAL_01 (BTN2)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr">
@@ -6781,7 +6769,7 @@
       </c>
       <c r="I93" s="42" t="inlineStr">
         <is>
-          <t>corruption_crisis</t>
+          <t>forge_evac</t>
         </is>
       </c>
       <c r="J93" s="7" t="inlineStr">
@@ -6802,7 +6790,7 @@
       </c>
       <c r="N93" s="43" t="inlineStr">
         <is>
-          <t>Fires when tileMoralDecay &gt;= 50 on Courthouse tile; army station required</t>
+          <t>+weapons 25; Forge temporarily offline</t>
         </is>
       </c>
     </row>
@@ -6819,27 +6807,27 @@
       </c>
       <c r="C94" s="42" t="inlineStr">
         <is>
-          <t>CORRUPT_TRIAL_01</t>
+          <t>CORRUPT_001</t>
         </is>
       </c>
       <c r="D94" s="43" t="inlineStr">
         <is>
-          <t>MAGISTRATE REMOVED IN DISGRACE</t>
-        </is>
-      </c>
-      <c r="E94" s="28" t="inlineStr">
-        <is>
-          <t>Branch</t>
+          <t>MAGISTRATE [COMMANDER_NAME] UNDER INVESTIGATION</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F94" s="43" t="inlineStr">
         <is>
-          <t>CORRUPT_001 BTN1 (army mission)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G94" s="43" t="inlineStr">
         <is>
-          <t>→ CORRUPT_REFORM_01</t>
+          <t>→ CORRUPT_TRIAL_01 (BTN1) | → CORRUPT_DEAL_01 (BTN2)</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
@@ -6849,7 +6837,7 @@
       </c>
       <c r="I94" s="42" t="inlineStr">
         <is>
-          <t>corrupt_trial</t>
+          <t>corruption_crisis</t>
         </is>
       </c>
       <c r="J94" s="7" t="inlineStr">
@@ -6870,7 +6858,7 @@
       </c>
       <c r="N94" s="43" t="inlineStr">
         <is>
-          <t>remove_governor; chains to CORRUPT_REFORM_01</t>
+          <t>Fires when tileMoralDecay &gt;= 50 on Courthouse tile; army station required</t>
         </is>
       </c>
     </row>
@@ -6887,27 +6875,27 @@
       </c>
       <c r="C95" s="42" t="inlineStr">
         <is>
-          <t>CORRUPT_REFORM_01</t>
+          <t>CORRUPT_TRIAL_01</t>
         </is>
       </c>
       <c r="D95" s="43" t="inlineStr">
         <is>
-          <t>COURTHOUSE REFORMS UNDERWAY AT [TILE_NAME]</t>
-        </is>
-      </c>
-      <c r="E95" s="22" t="inlineStr">
-        <is>
-          <t>Followup</t>
+          <t>MAGISTRATE REMOVED IN DISGRACE</t>
+        </is>
+      </c>
+      <c r="E95" s="28" t="inlineStr">
+        <is>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F95" s="43" t="inlineStr">
         <is>
-          <t>CORRUPT_TRIAL_01</t>
+          <t>CORRUPT_001 BTN1 (army mission)</t>
         </is>
       </c>
       <c r="G95" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ CORRUPT_REFORM_01</t>
         </is>
       </c>
       <c r="H95" s="6" t="inlineStr">
@@ -6917,7 +6905,7 @@
       </c>
       <c r="I95" s="42" t="inlineStr">
         <is>
-          <t>courthouse_reform</t>
+          <t>corrupt_trial</t>
         </is>
       </c>
       <c r="J95" s="7" t="inlineStr">
@@ -6938,7 +6926,7 @@
       </c>
       <c r="N95" s="43" t="inlineStr">
         <is>
-          <t>tile_moral_decay_change -50</t>
+          <t>remove_governor; chains to CORRUPT_REFORM_01</t>
         </is>
       </c>
     </row>
@@ -6955,22 +6943,22 @@
       </c>
       <c r="C96" s="42" t="inlineStr">
         <is>
-          <t>CORRUPT_DEAL_01</t>
+          <t>CORRUPT_REFORM_01</t>
         </is>
       </c>
       <c r="D96" s="43" t="inlineStr">
         <is>
-          <t>ARRANGEMENT REACHED AT [TILE_NAME]</t>
-        </is>
-      </c>
-      <c r="E96" s="28" t="inlineStr">
-        <is>
-          <t>Branch</t>
+          <t>COURTHOUSE REFORMS UNDERWAY AT [TILE_NAME]</t>
+        </is>
+      </c>
+      <c r="E96" s="22" t="inlineStr">
+        <is>
+          <t>Followup</t>
         </is>
       </c>
       <c r="F96" s="43" t="inlineStr">
         <is>
-          <t>CORRUPT_001 BTN2 (army mission)</t>
+          <t>CORRUPT_TRIAL_01</t>
         </is>
       </c>
       <c r="G96" s="43" t="inlineStr">
@@ -6985,7 +6973,7 @@
       </c>
       <c r="I96" s="42" t="inlineStr">
         <is>
-          <t>corrupt_deal</t>
+          <t>courthouse_reform</t>
         </is>
       </c>
       <c r="J96" s="7" t="inlineStr">
@@ -7006,7 +6994,7 @@
       </c>
       <c r="N96" s="43" t="inlineStr">
         <is>
-          <t>+gold 40; private deal path; magistrate stays</t>
+          <t>tile_moral_decay_change -50</t>
         </is>
       </c>
     </row>
@@ -7018,32 +7006,32 @@
       </c>
       <c r="B97" s="41" t="inlineStr">
         <is>
-          <t>Border Dispute</t>
+          <t>Corruption Crisis</t>
         </is>
       </c>
       <c r="C97" s="42" t="inlineStr">
         <is>
-          <t>BORDER_001</t>
+          <t>CORRUPT_DEAL_01</t>
         </is>
       </c>
       <c r="D97" s="43" t="inlineStr">
         <is>
-          <t>CANADIAN BORDER INCIDENT AT [TILE_NAME]: THE LINE IS IN QUESTION</t>
-        </is>
-      </c>
-      <c r="E97" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>ARRANGEMENT REACHED AT [TILE_NAME]</t>
+        </is>
+      </c>
+      <c r="E97" s="28" t="inlineStr">
+        <is>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F97" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORRUPT_001 BTN2 (army mission)</t>
         </is>
       </c>
       <c r="G97" s="43" t="inlineStr">
         <is>
-          <t>→ BORDER_ASSERT_01 (BTN1) | → BORDER_SURVEY_01 (BTN3)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
@@ -7053,7 +7041,7 @@
       </c>
       <c r="I97" s="42" t="inlineStr">
         <is>
-          <t>border_dispute</t>
+          <t>corrupt_deal</t>
         </is>
       </c>
       <c r="J97" s="7" t="inlineStr">
@@ -7074,7 +7062,7 @@
       </c>
       <c r="N97" s="43" t="inlineStr">
         <is>
-          <t>Woods/Foothills tile + CA neighbor; BTN2 claim_change -1 (diplomacy)</t>
+          <t>+gold 40; private deal path; magistrate stays</t>
         </is>
       </c>
     </row>
@@ -7091,27 +7079,27 @@
       </c>
       <c r="C98" s="42" t="inlineStr">
         <is>
-          <t>BORDER_ASSERT_01</t>
+          <t>BORDER_001</t>
         </is>
       </c>
       <c r="D98" s="43" t="inlineStr">
         <is>
-          <t>FEDERAL BOUNDARY MARKER PLANTED AT [TILE_NAME]</t>
-        </is>
-      </c>
-      <c r="E98" s="28" t="inlineStr">
-        <is>
-          <t>Branch</t>
+          <t>CANADIAN BORDER INCIDENT AT [TILE_NAME]: THE LINE IS IN QUESTION</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F98" s="43" t="inlineStr">
         <is>
-          <t>BORDER_001 BTN1 (army mission)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G98" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ BORDER_ASSERT_01 (BTN1) | → BORDER_SURVEY_01 (BTN3)</t>
         </is>
       </c>
       <c r="H98" s="6" t="inlineStr">
@@ -7121,7 +7109,7 @@
       </c>
       <c r="I98" s="42" t="inlineStr">
         <is>
-          <t>border_assert</t>
+          <t>border_dispute</t>
         </is>
       </c>
       <c r="J98" s="7" t="inlineStr">
@@ -7142,7 +7130,7 @@
       </c>
       <c r="N98" s="43" t="inlineStr">
         <is>
-          <t>+claim 2; garrison asserts sovereignty</t>
+          <t>Woods/Foothills tile + CA neighbor; BTN2 claim_change -1 (diplomacy)</t>
         </is>
       </c>
     </row>
@@ -7159,12 +7147,12 @@
       </c>
       <c r="C99" s="42" t="inlineStr">
         <is>
-          <t>BORDER_SURVEY_01</t>
+          <t>BORDER_ASSERT_01</t>
         </is>
       </c>
       <c r="D99" s="43" t="inlineStr">
         <is>
-          <t>SURVEY COMPLETE AT [TILE_NAME]: THE LAND IS OURS</t>
+          <t>FEDERAL BOUNDARY MARKER PLANTED AT [TILE_NAME]</t>
         </is>
       </c>
       <c r="E99" s="28" t="inlineStr">
@@ -7174,7 +7162,7 @@
       </c>
       <c r="F99" s="43" t="inlineStr">
         <is>
-          <t>BORDER_001 BTN3 (army mission)</t>
+          <t>BORDER_001 BTN1 (army mission)</t>
         </is>
       </c>
       <c r="G99" s="43" t="inlineStr">
@@ -7189,7 +7177,7 @@
       </c>
       <c r="I99" s="42" t="inlineStr">
         <is>
-          <t>border_survey</t>
+          <t>border_assert</t>
         </is>
       </c>
       <c r="J99" s="7" t="inlineStr">
@@ -7210,7 +7198,7 @@
       </c>
       <c r="N99" s="43" t="inlineStr">
         <is>
-          <t>+gold 20; diplomatic survey path</t>
+          <t>+claim 2; garrison asserts sovereignty</t>
         </is>
       </c>
     </row>
@@ -7222,27 +7210,27 @@
       </c>
       <c r="B100" s="41" t="inlineStr">
         <is>
-          <t>Garrison Hunger</t>
+          <t>Border Dispute</t>
         </is>
       </c>
       <c r="C100" s="42" t="inlineStr">
         <is>
-          <t>GARRISON_001</t>
+          <t>BORDER_SURVEY_01</t>
         </is>
       </c>
       <c r="D100" s="43" t="inlineStr">
         <is>
-          <t>FIELD REPORT: [TILE_NAME] GARRISON REPORTING CRITICAL SUPPLY SHORTFALL</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>SURVEY COMPLETE AT [TILE_NAME]: THE LAND IS OURS</t>
+        </is>
+      </c>
+      <c r="E100" s="28" t="inlineStr">
+        <is>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F100" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BORDER_001 BTN3 (army mission)</t>
         </is>
       </c>
       <c r="G100" s="43" t="inlineStr">
@@ -7257,7 +7245,7 @@
       </c>
       <c r="I100" s="42" t="inlineStr">
         <is>
-          <t>garrison_starving</t>
+          <t>border_survey</t>
         </is>
       </c>
       <c r="J100" s="7" t="inlineStr">
@@ -7278,7 +7266,7 @@
       </c>
       <c r="N100" s="43" t="inlineStr">
         <is>
-          <t>Fires when any USA army &lt; 50 manpower; BTN1 spend -30 gold / BTN2 retreat</t>
+          <t>+gold 20; diplomatic survey path</t>
         </is>
       </c>
     </row>
@@ -7290,17 +7278,17 @@
       </c>
       <c r="B101" s="41" t="inlineStr">
         <is>
-          <t>Legitimacy Crisis</t>
+          <t>Garrison Hunger</t>
         </is>
       </c>
       <c r="C101" s="42" t="inlineStr">
         <is>
-          <t>CRISIS_CLAIM_001</t>
+          <t>GARRISON_001</t>
         </is>
       </c>
       <c r="D101" s="43" t="inlineStr">
         <is>
-          <t>LEGITIMACY CRISIS: THE REPUBLIC'S CLAIM ON ITSELF IS IN QUESTION</t>
+          <t>FIELD REPORT: [TILE_NAME] GARRISON REPORTING CRITICAL SUPPLY SHORTFALL</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -7325,7 +7313,7 @@
       </c>
       <c r="I101" s="42" t="inlineStr">
         <is>
-          <t>legitimacy_crisis</t>
+          <t>garrison_starving</t>
         </is>
       </c>
       <c r="J101" s="7" t="inlineStr">
@@ -7346,7 +7334,7 @@
       </c>
       <c r="N101" s="43" t="inlineStr">
         <is>
-          <t>Fires when presidentialClaim &lt;= -5; 3 claim_change response buttons</t>
+          <t>Fires when any USA army &lt; 50 manpower; BTN1 spend -30 gold / BTN2 retreat</t>
         </is>
       </c>
     </row>
@@ -7358,17 +7346,17 @@
       </c>
       <c r="B102" s="41" t="inlineStr">
         <is>
-          <t>Turncoat General</t>
+          <t>Legitimacy Crisis</t>
         </is>
       </c>
       <c r="C102" s="42" t="inlineStr">
         <is>
-          <t>TURNCOAT_001</t>
+          <t>CRISIS_CLAIM_001</t>
         </is>
       </c>
       <c r="D102" s="43" t="inlineStr">
         <is>
-          <t>INTELLIGENCE REPORT: COMMANDER [COMMANDER_NAME] IN CONTACT WITH CROWN</t>
+          <t>LEGITIMACY CRISIS: THE REPUBLIC'S CLAIM ON ITSELF IS IN QUESTION</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -7393,7 +7381,7 @@
       </c>
       <c r="I102" s="42" t="inlineStr">
         <is>
-          <t>turncoat_report</t>
+          <t>legitimacy_crisis</t>
         </is>
       </c>
       <c r="J102" s="7" t="inlineStr">
@@ -7414,7 +7402,7 @@
       </c>
       <c r="N102" s="43" t="inlineStr">
         <is>
-          <t>Fires when any governor loyalty &lt;= -8; remove / double-agent / watch</t>
+          <t>Fires when presidentialClaim &lt;= -5; 3 claim_change response buttons</t>
         </is>
       </c>
     </row>
@@ -7426,17 +7414,17 @@
       </c>
       <c r="B103" s="41" t="inlineStr">
         <is>
-          <t>Memorial Lost</t>
+          <t>Turncoat General</t>
         </is>
       </c>
       <c r="C103" s="42" t="inlineStr">
         <is>
-          <t>MEMORIAL_001</t>
+          <t>TURNCOAT_001</t>
         </is>
       </c>
       <c r="D103" s="43" t="inlineStr">
         <is>
-          <t>[TILE_NAME] FALLS TO THE CROWN: HISTORICAL SITE UNDER OCCUPATION</t>
+          <t>INTELLIGENCE REPORT: COMMANDER [COMMANDER_NAME] IN CONTACT WITH CROWN</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -7451,7 +7439,7 @@
       </c>
       <c r="G103" s="43" t="inlineStr">
         <is>
-          <t>→ MEMORIAL_RESTORE_01 (BTN1 own-mission)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H103" s="6" t="inlineStr">
@@ -7461,7 +7449,7 @@
       </c>
       <c r="I103" s="42" t="inlineStr">
         <is>
-          <t>memorial_lost</t>
+          <t>turncoat_report</t>
         </is>
       </c>
       <c r="J103" s="7" t="inlineStr">
@@ -7482,7 +7470,7 @@
       </c>
       <c r="N103" s="43" t="inlineStr">
         <is>
-          <t>Fires when UK captures tile with tileSpecialFeatures; set_mission_flag_own</t>
+          <t>Fires when any governor loyalty &lt;= -8; remove / double-agent / watch</t>
         </is>
       </c>
     </row>
@@ -7499,27 +7487,27 @@
       </c>
       <c r="C104" s="42" t="inlineStr">
         <is>
-          <t>MEMORIAL_RESTORE_01</t>
+          <t>MEMORIAL_001</t>
         </is>
       </c>
       <c r="D104" s="43" t="inlineStr">
         <is>
-          <t>[TILE_NAME] LIBERATED: THE MEMORIAL IS OURS AGAIN</t>
-        </is>
-      </c>
-      <c r="E104" s="22" t="inlineStr">
-        <is>
-          <t>Followup</t>
+          <t>[TILE_NAME] FALLS TO THE CROWN: HISTORICAL SITE UNDER OCCUPATION</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F104" s="43" t="inlineStr">
         <is>
-          <t>MEMORIAL_001 BTN1 (own-mission)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G104" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ MEMORIAL_RESTORE_01 (BTN1 own-mission)</t>
         </is>
       </c>
       <c r="H104" s="6" t="inlineStr">
@@ -7529,7 +7517,7 @@
       </c>
       <c r="I104" s="42" t="inlineStr">
         <is>
-          <t>memorial_restored</t>
+          <t>memorial_lost</t>
         </is>
       </c>
       <c r="J104" s="7" t="inlineStr">
@@ -7550,93 +7538,93 @@
       </c>
       <c r="N104" s="43" t="inlineStr">
         <is>
+          <t>Fires when UK captures tile with tileSpecialFeatures; set_mission_flag_own</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="41" t="inlineStr">
+        <is>
+          <t>Tile Crisis</t>
+        </is>
+      </c>
+      <c r="B105" s="41" t="inlineStr">
+        <is>
+          <t>Memorial Lost</t>
+        </is>
+      </c>
+      <c r="C105" s="42" t="inlineStr">
+        <is>
+          <t>MEMORIAL_RESTORE_01</t>
+        </is>
+      </c>
+      <c r="D105" s="43" t="inlineStr">
+        <is>
+          <t>[TILE_NAME] LIBERATED: THE MEMORIAL IS OURS AGAIN</t>
+        </is>
+      </c>
+      <c r="E105" s="22" t="inlineStr">
+        <is>
+          <t>Followup</t>
+        </is>
+      </c>
+      <c r="F105" s="43" t="inlineStr">
+        <is>
+          <t>MEMORIAL_001 BTN1 (own-mission)</t>
+        </is>
+      </c>
+      <c r="G105" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I105" s="42" t="inlineStr">
+        <is>
+          <t>memorial_restored</t>
+        </is>
+      </c>
+      <c r="J105" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K105" s="44" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L105" s="42" t="inlineStr"/>
+      <c r="M105" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N105" s="43" t="inlineStr">
+        <is>
           <t>Fires when USA retakes the special-feature tile; +morale 20</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="8" customHeight="1">
-      <c r="A105" s="9" t="n"/>
-      <c r="B105" s="9" t="n"/>
-      <c r="C105" s="9" t="n"/>
-      <c r="D105" s="9" t="n"/>
-      <c r="E105" s="9" t="n"/>
-      <c r="F105" s="9" t="n"/>
-      <c r="G105" s="9" t="n"/>
-      <c r="H105" s="9" t="n"/>
-      <c r="I105" s="9" t="n"/>
-      <c r="J105" s="9" t="n"/>
-      <c r="K105" s="9" t="n"/>
-      <c r="L105" s="9" t="n"/>
-      <c r="M105" s="9" t="n"/>
-      <c r="N105" s="9" t="n"/>
-    </row>
-    <row r="106" ht="30" customHeight="1">
-      <c r="A106" s="45" t="inlineStr">
-        <is>
-          <t>Ualani</t>
-        </is>
-      </c>
-      <c r="B106" s="45" t="inlineStr">
-        <is>
-          <t>Ambush</t>
-        </is>
-      </c>
-      <c r="C106" s="46" t="inlineStr">
-        <is>
-          <t>UALANI_AMBUSH_01</t>
-        </is>
-      </c>
-      <c r="D106" s="47" t="inlineStr">
-        <is>
-          <t>CROWN AMBUSH AVERTED: PRESIDENT CARLISLE HOLDS THE WETLANDS</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F106" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G106" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H106" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I106" s="46" t="inlineStr"/>
-      <c r="J106" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K106" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L106" s="46" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M106" s="48" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N106" s="47" t="inlineStr">
-        <is>
-          <t>Ualani in Wetlands + UK neighbor; BTN3 explicit +weapons 40</t>
-        </is>
-      </c>
+    <row r="106" ht="8" customHeight="1">
+      <c r="A106" s="9" t="n"/>
+      <c r="B106" s="9" t="n"/>
+      <c r="C106" s="9" t="n"/>
+      <c r="D106" s="9" t="n"/>
+      <c r="E106" s="9" t="n"/>
+      <c r="F106" s="9" t="n"/>
+      <c r="G106" s="9" t="n"/>
+      <c r="H106" s="9" t="n"/>
+      <c r="I106" s="9" t="n"/>
+      <c r="J106" s="9" t="n"/>
+      <c r="K106" s="9" t="n"/>
+      <c r="L106" s="9" t="n"/>
+      <c r="M106" s="9" t="n"/>
+      <c r="N106" s="9" t="n"/>
     </row>
     <row r="107" ht="30" customHeight="1">
       <c r="A107" s="45" t="inlineStr">
@@ -7646,17 +7634,17 @@
       </c>
       <c r="B107" s="45" t="inlineStr">
         <is>
-          <t>Dignitary Reception</t>
+          <t>Ambush</t>
         </is>
       </c>
       <c r="C107" s="46" t="inlineStr">
         <is>
-          <t>UALANI_DIGNITARY_01</t>
+          <t>UALANI_AMBUSH_01</t>
         </is>
       </c>
       <c r="D107" s="47" t="inlineStr">
         <is>
-          <t>STATE RECEPTION AT [TILE_NAME]</t>
+          <t>CROWN AMBUSH AVERTED: PRESIDENT CARLISLE HOLDS THE WETLANDS</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -7697,12 +7685,12 @@
       </c>
       <c r="M107" s="48" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N107" s="47" t="inlineStr">
         <is>
-          <t>Ualani in Metro/Suburbs + Courthouse + tileMoralDecay &lt; 30; BTN3 explicit -20 moralDecay</t>
+          <t>Ualani in Wetlands + UK neighbor; BTN3 explicit +weapons 40</t>
         </is>
       </c>
     </row>
@@ -7714,17 +7702,17 @@
       </c>
       <c r="B108" s="45" t="inlineStr">
         <is>
-          <t>Memorial Address</t>
+          <t>Dignitary Reception</t>
         </is>
       </c>
       <c r="C108" s="46" t="inlineStr">
         <is>
-          <t>UALANI_MEMORIAL_01</t>
+          <t>UALANI_DIGNITARY_01</t>
         </is>
       </c>
       <c r="D108" s="47" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS [TILE_NAME]: PRESIDENTIAL ADDRESS AT THE MEMORIAL</t>
+          <t>STATE RECEPTION AT [TILE_NAME]</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -7765,12 +7753,12 @@
       </c>
       <c r="M108" s="48" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="N108" s="47" t="inlineStr">
         <is>
-          <t>Ualani at tile with tileSpecialFeatures; BTN3 explicit +morale 50</t>
+          <t>Ualani in Metro/Suburbs + Courthouse + tileMoralDecay &lt; 30; BTN3 explicit -20 moralDecay</t>
         </is>
       </c>
     </row>
@@ -7782,17 +7770,17 @@
       </c>
       <c r="B109" s="45" t="inlineStr">
         <is>
-          <t>Field Hospital</t>
+          <t>Memorial Address</t>
         </is>
       </c>
       <c r="C109" s="46" t="inlineStr">
         <is>
-          <t>UALANI_WOUNDED_01</t>
+          <t>UALANI_MEMORIAL_01</t>
         </is>
       </c>
       <c r="D109" s="47" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS FIELD HOSPITAL AT [TILE_NAME]</t>
+          <t>PRESIDENT CARLISLE VISITS [TILE_NAME]: PRESIDENTIAL ADDRESS AT THE MEMORIAL</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -7833,12 +7821,12 @@
       </c>
       <c r="M109" s="48" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N109" s="47" t="inlineStr">
         <is>
-          <t>Ualani army &lt; 80% manpower; BTN2 explicit +manpower 40</t>
+          <t>Ualani at tile with tileSpecialFeatures; BTN3 explicit +morale 50</t>
         </is>
       </c>
     </row>
@@ -7850,17 +7838,17 @@
       </c>
       <c r="B110" s="45" t="inlineStr">
         <is>
-          <t>Winter March</t>
+          <t>Field Hospital</t>
         </is>
       </c>
       <c r="C110" s="46" t="inlineStr">
         <is>
-          <t>UALANI_WINTER_01</t>
+          <t>UALANI_WOUNDED_01</t>
         </is>
       </c>
       <c r="D110" s="47" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE MARCHES THROUGH [TILE_NAME] IN THE DEAD OF WINTER</t>
+          <t>PRESIDENT CARLISLE VISITS FIELD HOSPITAL AT [TILE_NAME]</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
@@ -7889,20 +7877,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K110" s="48" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L110" s="46" t="inlineStr"/>
+      <c r="K110" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L110" s="46" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M110" s="48" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N110" s="47" t="inlineStr">
         <is>
-          <t>Ualani in Foothills/Woods; winter months [11,12,1,2]; winterScore &gt; 0; no explicit</t>
+          <t>Ualani army &lt; 80% manpower; BTN2 explicit +manpower 40</t>
         </is>
       </c>
     </row>
@@ -7914,17 +7906,17 @@
       </c>
       <c r="B111" s="45" t="inlineStr">
         <is>
-          <t>Forge Inspection</t>
+          <t>Winter March</t>
         </is>
       </c>
       <c r="C111" s="46" t="inlineStr">
         <is>
-          <t>UALANI_FORGE_01</t>
+          <t>UALANI_WINTER_01</t>
         </is>
       </c>
       <c r="D111" s="47" t="inlineStr">
         <is>
-          <t>SURPRISE INSPECTION OF FORGE AT [TILE_NAME]</t>
+          <t>PRESIDENT CARLISLE MARCHES THROUGH [TILE_NAME] IN THE DEAD OF WINTER</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
@@ -7953,24 +7945,20 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K111" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L111" s="46" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
+      <c r="K111" s="48" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L111" s="46" t="inlineStr"/>
       <c r="M111" s="48" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N111" s="47" t="inlineStr">
         <is>
-          <t>Ualani at tile with enabled Forge; BTN3 explicit +weapons 60</t>
+          <t>Ualani in Foothills/Woods; winter months [11,12,1,2]; winterScore &gt; 0; no explicit</t>
         </is>
       </c>
     </row>
@@ -7982,17 +7970,17 @@
       </c>
       <c r="B112" s="45" t="inlineStr">
         <is>
-          <t>Culper Ring</t>
+          <t>Forge Inspection</t>
         </is>
       </c>
       <c r="C112" s="46" t="inlineStr">
         <is>
-          <t>UALANI_CULPER_01</t>
+          <t>UALANI_FORGE_01</t>
         </is>
       </c>
       <c r="D112" s="47" t="inlineStr">
         <is>
-          <t>CULPER RING CONTACT AT [TILE_NAME]</t>
+          <t>SURPRISE INSPECTION OF FORGE AT [TILE_NAME]</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
@@ -8007,7 +7995,7 @@
       </c>
       <c r="G112" s="47" t="inlineStr">
         <is>
-          <t>→ UALANI_CULPER_BRIEF_01 (BTN1/BTN3 next_event_id)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H112" s="6" t="inlineStr">
@@ -8033,12 +8021,12 @@
       </c>
       <c r="M112" s="48" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N112" s="47" t="inlineStr">
         <is>
-          <t>Ualani neighbors tile with espionageActive; BTN3 explicit +gold 40 then brief</t>
+          <t>Ualani at tile with enabled Forge; BTN3 explicit +weapons 60</t>
         </is>
       </c>
     </row>
@@ -8055,27 +8043,27 @@
       </c>
       <c r="C113" s="46" t="inlineStr">
         <is>
-          <t>UALANI_CULPER_BRIEF_01</t>
+          <t>UALANI_CULPER_01</t>
         </is>
       </c>
       <c r="D113" s="47" t="inlineStr">
         <is>
-          <t>CULPER RING INTELLIGENCE RECEIVED: CROWN PLANS CONFIRMED</t>
-        </is>
-      </c>
-      <c r="E113" s="22" t="inlineStr">
-        <is>
-          <t>Followup</t>
+          <t>CULPER RING CONTACT AT [TILE_NAME]</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F113" s="47" t="inlineStr">
         <is>
-          <t>UALANI_CULPER_01 BTN1 / BTN3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G113" s="47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ UALANI_CULPER_BRIEF_01 (BTN1/BTN3 next_event_id)</t>
         </is>
       </c>
       <c r="H113" s="6" t="inlineStr">
@@ -8089,20 +8077,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K113" s="48" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L113" s="46" t="inlineStr"/>
+      <c r="K113" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L113" s="46" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M113" s="48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>18</t>
         </is>
       </c>
       <c r="N113" s="47" t="inlineStr">
         <is>
-          <t>Sets culper_active flag; single button; no explicit</t>
+          <t>Ualani neighbors tile with espionageActive; BTN3 explicit +gold 40 then brief</t>
         </is>
       </c>
     </row>
@@ -8114,27 +8106,27 @@
       </c>
       <c r="B114" s="45" t="inlineStr">
         <is>
-          <t>Alliance Council</t>
+          <t>Culper Ring</t>
         </is>
       </c>
       <c r="C114" s="46" t="inlineStr">
         <is>
-          <t>UALANI_ALLIANCE_01</t>
+          <t>UALANI_CULPER_BRIEF_01</t>
         </is>
       </c>
       <c r="D114" s="47" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE MEETS WITH [COMMANDER_NAME] AT [TILE_NAME]</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>CULPER RING INTELLIGENCE RECEIVED: CROWN PLANS CONFIRMED</t>
+        </is>
+      </c>
+      <c r="E114" s="22" t="inlineStr">
+        <is>
+          <t>Followup</t>
         </is>
       </c>
       <c r="F114" s="47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>UALANI_CULPER_01 BTN1 / BTN3</t>
         </is>
       </c>
       <c r="G114" s="47" t="inlineStr">
@@ -8153,24 +8145,20 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K114" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L114" s="46" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
+      <c r="K114" s="48" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L114" s="46" t="inlineStr"/>
       <c r="M114" s="48" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N114" s="47" t="inlineStr">
         <is>
-          <t>Fires at NEIGHBOR tile (named hist. governor); BTN3 explicit governor_loyalty +12</t>
+          <t>Sets culper_active flag; single button; no explicit</t>
         </is>
       </c>
     </row>
@@ -8182,17 +8170,17 @@
       </c>
       <c r="B115" s="45" t="inlineStr">
         <is>
-          <t>Frontier</t>
+          <t>Alliance Council</t>
         </is>
       </c>
       <c r="C115" s="46" t="inlineStr">
         <is>
-          <t>UALANI_FRONTIER_01</t>
+          <t>UALANI_ALLIANCE_01</t>
         </is>
       </c>
       <c r="D115" s="47" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE ESTABLISHES FRONTIER PRESENCE AT [TILE_NAME]</t>
+          <t>PRESIDENT CARLISLE MEETS WITH [COMMANDER_NAME] AT [TILE_NAME]</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
@@ -8233,98 +8221,98 @@
       </c>
       <c r="M115" s="48" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="N115" s="47" t="inlineStr">
+        <is>
+          <t>Fires at NEIGHBOR tile (named hist. governor); BTN3 explicit governor_loyalty +12</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="30" customHeight="1">
+      <c r="A116" s="45" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B116" s="45" t="inlineStr">
+        <is>
+          <t>Frontier</t>
+        </is>
+      </c>
+      <c r="C116" s="46" t="inlineStr">
+        <is>
+          <t>UALANI_FRONTIER_01</t>
+        </is>
+      </c>
+      <c r="D116" s="47" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE ESTABLISHES FRONTIER PRESENCE AT [TILE_NAME]</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F116" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G116" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I116" s="46" t="inlineStr"/>
+      <c r="J116" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K116" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L116" s="46" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
+      <c r="M116" s="48" t="inlineStr">
+        <is>
           <t>20</t>
         </is>
       </c>
-      <c r="N115" s="47" t="inlineStr">
+      <c r="N116" s="47" t="inlineStr">
         <is>
           <t>Ualani in Woods/Foothills bordering CA - * tile; BTN3 explicit +morale 30</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="8" customHeight="1">
-      <c r="A116" s="9" t="n"/>
-      <c r="B116" s="9" t="n"/>
-      <c r="C116" s="9" t="n"/>
-      <c r="D116" s="9" t="n"/>
-      <c r="E116" s="9" t="n"/>
-      <c r="F116" s="9" t="n"/>
-      <c r="G116" s="9" t="n"/>
-      <c r="H116" s="9" t="n"/>
-      <c r="I116" s="9" t="n"/>
-      <c r="J116" s="9" t="n"/>
-      <c r="K116" s="9" t="n"/>
-      <c r="L116" s="9" t="n"/>
-      <c r="M116" s="9" t="n"/>
-      <c r="N116" s="9" t="n"/>
-    </row>
-    <row r="117" ht="30" customHeight="1">
-      <c r="A117" s="49" t="inlineStr">
-        <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="B117" s="49" t="inlineStr">
-        <is>
-          <t>Ualani Expansion</t>
-        </is>
-      </c>
-      <c r="C117" s="50" t="inlineStr">
-        <is>
-          <t>UALANI_DOCK_01</t>
-        </is>
-      </c>
-      <c r="D117" s="51" t="inlineStr">
-        <is>
-          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E117" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F117" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G117" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H117" s="52" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I117" s="50" t="inlineStr"/>
-      <c r="J117" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K117" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L117" s="50" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M117" s="53" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N117" s="51" t="inlineStr">
-        <is>
-          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
-        </is>
-      </c>
+    <row r="117" ht="8" customHeight="1">
+      <c r="A117" s="9" t="n"/>
+      <c r="B117" s="9" t="n"/>
+      <c r="C117" s="9" t="n"/>
+      <c r="D117" s="9" t="n"/>
+      <c r="E117" s="9" t="n"/>
+      <c r="F117" s="9" t="n"/>
+      <c r="G117" s="9" t="n"/>
+      <c r="H117" s="9" t="n"/>
+      <c r="I117" s="9" t="n"/>
+      <c r="J117" s="9" t="n"/>
+      <c r="K117" s="9" t="n"/>
+      <c r="L117" s="9" t="n"/>
+      <c r="M117" s="9" t="n"/>
+      <c r="N117" s="9" t="n"/>
     </row>
     <row r="118" ht="30" customHeight="1">
       <c r="A118" s="49" t="inlineStr">
@@ -8339,12 +8327,12 @@
       </c>
       <c r="C118" s="50" t="inlineStr">
         <is>
-          <t>UALANI_FARM_01</t>
+          <t>UALANI_DOCK_01</t>
         </is>
       </c>
       <c r="D118" s="51" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
+          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
@@ -8390,7 +8378,7 @@
       </c>
       <c r="N118" s="51" t="inlineStr">
         <is>
-          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
+          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
         </is>
       </c>
     </row>
@@ -8407,12 +8395,12 @@
       </c>
       <c r="C119" s="50" t="inlineStr">
         <is>
-          <t>UALANI_BARRACKS_01</t>
+          <t>UALANI_FARM_01</t>
         </is>
       </c>
       <c r="D119" s="51" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
+          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E119" s="5" t="inlineStr">
@@ -8458,7 +8446,7 @@
       </c>
       <c r="N119" s="51" t="inlineStr">
         <is>
-          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
+          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
         </is>
       </c>
     </row>
@@ -8475,12 +8463,12 @@
       </c>
       <c r="C120" s="50" t="inlineStr">
         <is>
-          <t>UALANI_COURTHOUSE_01</t>
+          <t>UALANI_BARRACKS_01</t>
         </is>
       </c>
       <c r="D120" s="51" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
+          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
@@ -8526,7 +8514,7 @@
       </c>
       <c r="N120" s="51" t="inlineStr">
         <is>
-          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
+          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
         </is>
       </c>
     </row>
@@ -8538,17 +8526,17 @@
       </c>
       <c r="B121" s="49" t="inlineStr">
         <is>
-          <t>More City Events</t>
+          <t>Ualani Expansion</t>
         </is>
       </c>
       <c r="C121" s="50" t="inlineStr">
         <is>
-          <t>CL_WASHINGTON_01</t>
+          <t>UALANI_COURTHOUSE_01</t>
         </is>
       </c>
       <c r="D121" s="51" t="inlineStr">
         <is>
-          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
+          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E121" s="5" t="inlineStr">
@@ -8577,20 +8565,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K121" s="53" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L121" s="50" t="inlineStr"/>
+      <c r="K121" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L121" s="50" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M121" s="53" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N121" s="51" t="inlineStr">
         <is>
-          <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
+          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
         </is>
       </c>
     </row>
@@ -8607,12 +8599,12 @@
       </c>
       <c r="C122" s="50" t="inlineStr">
         <is>
-          <t>CL_VALLEY_FORGE_01</t>
+          <t>CL_WASHINGTON_01</t>
         </is>
       </c>
       <c r="D122" s="51" t="inlineStr">
         <is>
-          <t>VALLEY FORGE SECURED  ← IDEA</t>
+          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
         </is>
       </c>
       <c r="E122" s="5" t="inlineStr">
@@ -8654,7 +8646,7 @@
       </c>
       <c r="N122" s="51" t="inlineStr">
         <is>
-          <t>Tile 1; historically significant; would fire on liberation</t>
+          <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
         </is>
       </c>
     </row>
@@ -8671,12 +8663,12 @@
       </c>
       <c r="C123" s="50" t="inlineStr">
         <is>
-          <t>CX_NYC_01</t>
+          <t>CL_VALLEY_FORGE_01</t>
         </is>
       </c>
       <c r="D123" s="51" t="inlineStr">
         <is>
-          <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
+          <t>VALLEY FORGE SECURED  ← IDEA</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
@@ -8718,7 +8710,7 @@
       </c>
       <c r="N123" s="51" t="inlineStr">
         <is>
-          <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
+          <t>Tile 1; historically significant; would fire on liberation</t>
         </is>
       </c>
     </row>
@@ -8730,17 +8722,17 @@
       </c>
       <c r="B124" s="49" t="inlineStr">
         <is>
-          <t>Espionage Events</t>
+          <t>More City Events</t>
         </is>
       </c>
       <c r="C124" s="50" t="inlineStr">
         <is>
-          <t>ESPIONAGE_DISCOVERY_01</t>
+          <t>CX_NYC_01</t>
         </is>
       </c>
       <c r="D124" s="51" t="inlineStr">
         <is>
-          <t>SPY NETWORK DISCOVERED AT [TILE_NAME]  ← IDEA</t>
+          <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
@@ -8782,7 +8774,7 @@
       </c>
       <c r="N124" s="51" t="inlineStr">
         <is>
-          <t>Would fire when espionageActive + enemy army arrives; uses existing espionage vars</t>
+          <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
         </is>
       </c>
     </row>
@@ -8794,32 +8786,32 @@
       </c>
       <c r="B125" s="49" t="inlineStr">
         <is>
-          <t>Commander Expansion</t>
+          <t>Espionage Events</t>
         </is>
       </c>
       <c r="C125" s="50" t="inlineStr">
         <is>
-          <t>CMD_OBJECTIVE_2</t>
+          <t>ESPIONAGE_DISCOVERY_01</t>
         </is>
       </c>
       <c r="D125" s="51" t="inlineStr">
         <is>
-          <t>A COMMANDER'S SECOND TASK  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E125" s="22" t="inlineStr">
-        <is>
-          <t>Followup</t>
+          <t>SPY NETWORK DISCOVERED AT [TILE_NAME]  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F125" s="51" t="inlineStr">
         <is>
-          <t>CMD_OBJECTIVE_1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G125" s="51" t="inlineStr">
         <is>
-          <t>→ CMD_OBJECTIVE_3?</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H125" s="52" t="inlineStr">
@@ -8846,7 +8838,7 @@
       </c>
       <c r="N125" s="51" t="inlineStr">
         <is>
-          <t>Extend the commander arc beyond first objective</t>
+          <t>Would fire when espionageActive + enemy army arrives; uses existing espionage vars</t>
         </is>
       </c>
     </row>
@@ -8858,32 +8850,32 @@
       </c>
       <c r="B126" s="49" t="inlineStr">
         <is>
-          <t>Seasonal Events</t>
+          <t>Commander Expansion</t>
         </is>
       </c>
       <c r="C126" s="50" t="inlineStr">
         <is>
-          <t>WINTER_SIEGE_01</t>
+          <t>CMD_OBJECTIVE_2</t>
         </is>
       </c>
       <c r="D126" s="51" t="inlineStr">
         <is>
-          <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E126" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>A COMMANDER'S SECOND TASK  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E126" s="22" t="inlineStr">
+        <is>
+          <t>Followup</t>
         </is>
       </c>
       <c r="F126" s="51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CMD_OBJECTIVE_1</t>
         </is>
       </c>
       <c r="G126" s="51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ CMD_OBJECTIVE_3?</t>
         </is>
       </c>
       <c r="H126" s="52" t="inlineStr">
@@ -8910,7 +8902,7 @@
       </c>
       <c r="N126" s="51" t="inlineStr">
         <is>
-          <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
+          <t>Extend the commander arc beyond first objective</t>
         </is>
       </c>
     </row>
@@ -8927,12 +8919,12 @@
       </c>
       <c r="C127" s="50" t="inlineStr">
         <is>
-          <t>SPRING_OFFENSIVE_01</t>
+          <t>WINTER_SIEGE_01</t>
         </is>
       </c>
       <c r="D127" s="51" t="inlineStr">
         <is>
-          <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
+          <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
@@ -8974,47 +8966,111 @@
       </c>
       <c r="N127" s="51" t="inlineStr">
         <is>
+          <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="A128" s="49" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B128" s="49" t="inlineStr">
+        <is>
+          <t>Seasonal Events</t>
+        </is>
+      </c>
+      <c r="C128" s="50" t="inlineStr">
+        <is>
+          <t>SPRING_OFFENSIVE_01</t>
+        </is>
+      </c>
+      <c r="D128" s="51" t="inlineStr">
+        <is>
+          <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F128" s="51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G128" s="51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H128" s="52" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I128" s="50" t="inlineStr"/>
+      <c r="J128" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K128" s="53" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L128" s="50" t="inlineStr"/>
+      <c r="M128" s="53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N128" s="51" t="inlineStr">
+        <is>
           <t>Month 3-4; UK neighbor + player army present; tactical pressure event</t>
         </is>
-      </c>
-    </row>
-    <row r="129" ht="20" customHeight="1">
-      <c r="A129" s="54" t="inlineStr">
-        <is>
-          <t>Total events in spreadsheet</t>
-        </is>
-      </c>
-      <c r="B129" s="55" t="n">
-        <v>116</v>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="54" t="inlineStr">
         <is>
-          <t>FIRST PASS (coded &amp; wired)</t>
+          <t>Total events in spreadsheet</t>
         </is>
       </c>
       <c r="B130" s="55" t="n">
-        <v>105</v>
+        <v>117</v>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="54" t="inlineStr">
         <is>
-          <t>IDEA (not yet implemented)</t>
+          <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
       <c r="B131" s="55" t="n">
-        <v>11</v>
+        <v>106</v>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="54" t="inlineStr">
         <is>
+          <t>IDEA (not yet implemented)</t>
+        </is>
+      </c>
+      <c r="B132" s="55" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="133" ht="20" customHeight="1">
+      <c r="A133" s="54" t="inlineStr">
+        <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B132" s="55" t="n">
+      <c r="B133" s="55" t="n">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add peace events system — dock-tile liberation triggers end-of-war
Allied peace (PEACE_ALLIED_01): fires when all UK dock tiles in USA+CA
regions are liberated while can_allied is set; sets uk_usa_peace and
uk_ca_peace on UK country and CA country; [TILE_NAME] is the last port freed.

USA separate peace (PEACE_USA_01): fires when USA dock tiles 65/66/67/151
are all liberated, unallied path; sets uk_usa_peace on UK country.

CA separate peace (PEACE_CA_AI_01): fires when Halifax (tile 114) is
liberated, unallied path; sets uk_ca_peace on UK and CA countries;
_ca_press_uk_borders() guards on this flag to stop CA AI aggression.

Flip-tracker (_peace_dock_was_uk) identifies the most recently freed dock
tile so the event headline reads "PEACE OF [TILE_NAME]" correctly.

3 events + 6 buttons added to CSVs; masterdoc rebuilt to 167 events.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N185"/>
+  <dimension ref="A1:N189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11492,360 +11492,308 @@
       <c r="N167" s="9" t="n"/>
     </row>
     <row r="168" ht="30" customHeight="1">
-      <c r="A168" s="49" t="inlineStr">
+      <c r="A168" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B168" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C168" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_ALLIED_01</t>
+        </is>
+      </c>
+      <c r="D168" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F168" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G168" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H168" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I168" s="54" t="inlineStr"/>
+      <c r="J168" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K168" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L168" s="54" t="inlineStr">
+        <is>
+          <t>sensual option</t>
+        </is>
+      </c>
+      <c r="M168" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N168" s="55" t="inlineStr">
+        <is>
+          <t>Allied peace: fires when all UK dock tiles in USA+CA regions liberated (can_allied); sets uk_usa_peace+uk_ca_peace on UK country; BTN2 sensual — Ualani+Jessica celebrate</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="30" customHeight="1">
+      <c r="A169" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B169" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C169" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_USA_01</t>
+        </is>
+      </c>
+      <c r="D169" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F169" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G169" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H169" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I169" s="54" t="inlineStr"/>
+      <c r="J169" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K169" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L169" s="54" t="inlineStr">
+        <is>
+          <t>sensual option</t>
+        </is>
+      </c>
+      <c r="M169" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N169" s="55" t="inlineStr">
+        <is>
+          <t>USA separate peace (unallied): fires when all USA dock tiles liberated (65,66,67,151); sets uk_usa_peace on UK country; BTN2 sensual — Ualani alone at dawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="30" customHeight="1">
+      <c r="A170" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B170" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C170" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_CA_AI_01</t>
+        </is>
+      </c>
+      <c r="D170" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — CANADA NEGOTIATES SEPARATE PEACE</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F170" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G170" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H170" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I170" s="54" t="inlineStr"/>
+      <c r="J170" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K170" s="56" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L170" s="54" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="M170" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N170" s="55" t="inlineStr">
+        <is>
+          <t>CA separate peace (unallied): fires when Halifax (tile 114) liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="8" customHeight="1">
+      <c r="A171" s="9" t="n"/>
+      <c r="B171" s="9" t="n"/>
+      <c r="C171" s="9" t="n"/>
+      <c r="D171" s="9" t="n"/>
+      <c r="E171" s="9" t="n"/>
+      <c r="F171" s="9" t="n"/>
+      <c r="G171" s="9" t="n"/>
+      <c r="H171" s="9" t="n"/>
+      <c r="I171" s="9" t="n"/>
+      <c r="J171" s="9" t="n"/>
+      <c r="K171" s="9" t="n"/>
+      <c r="L171" s="9" t="n"/>
+      <c r="M171" s="9" t="n"/>
+      <c r="N171" s="9" t="n"/>
+    </row>
+    <row r="172" ht="30" customHeight="1">
+      <c r="A172" s="49" t="inlineStr">
         <is>
           <t>VP Arc</t>
         </is>
       </c>
-      <c r="B168" s="49" t="inlineStr">
+      <c r="B172" s="49" t="inlineStr">
         <is>
           <t>VP Arc</t>
         </is>
       </c>
-      <c r="C168" s="50" t="inlineStr">
+      <c r="C172" s="50" t="inlineStr">
         <is>
           <t>VP_LEGACY</t>
         </is>
       </c>
-      <c r="D168" s="51" t="inlineStr">
+      <c r="D172" s="51" t="inlineStr">
         <is>
           <t>THE VICE PRESIDENT LEAVES A NOTE — [COMMANDER_NAME] HAS SOMETHING TO SAY</t>
         </is>
       </c>
-      <c r="E168" s="22" t="inlineStr">
+      <c r="E172" s="22" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="F168" s="51" t="inlineStr">
+      <c r="F172" s="51" t="inlineStr">
         <is>
           <t>VP_FIRST_MEETING (turn 96+)</t>
         </is>
       </c>
-      <c r="G168" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H168" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I168" s="50" t="inlineStr"/>
-      <c r="J168" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K168" s="26" t="inlineStr">
+      <c r="G172" s="51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H172" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I172" s="50" t="inlineStr"/>
+      <c r="J172" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K172" s="26" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="L168" s="50" t="inlineStr">
+      <c r="L172" s="50" t="inlineStr">
         <is>
           <t>explicit option</t>
         </is>
       </c>
-      <c r="M168" s="52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N168" s="51" t="inlineStr">
+      <c r="M172" s="52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N172" s="51" t="inlineStr">
         <is>
           <t>Fires turn 96+; BTN1 claim +1 / BTN2 explicit morale +30</t>
         </is>
       </c>
     </row>
-    <row r="169" ht="8" customHeight="1">
-      <c r="A169" s="9" t="n"/>
-      <c r="B169" s="9" t="n"/>
-      <c r="C169" s="9" t="n"/>
-      <c r="D169" s="9" t="n"/>
-      <c r="E169" s="9" t="n"/>
-      <c r="F169" s="9" t="n"/>
-      <c r="G169" s="9" t="n"/>
-      <c r="H169" s="9" t="n"/>
-      <c r="I169" s="9" t="n"/>
-      <c r="J169" s="9" t="n"/>
-      <c r="K169" s="9" t="n"/>
-      <c r="L169" s="9" t="n"/>
-      <c r="M169" s="9" t="n"/>
-      <c r="N169" s="9" t="n"/>
-    </row>
-    <row r="170" ht="30" customHeight="1">
-      <c r="A170" s="61" t="inlineStr">
-        <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="B170" s="61" t="inlineStr">
-        <is>
-          <t>Ualani Expansion</t>
-        </is>
-      </c>
-      <c r="C170" s="62" t="inlineStr">
-        <is>
-          <t>UALANI_DOCK_01</t>
-        </is>
-      </c>
-      <c r="D170" s="63" t="inlineStr">
-        <is>
-          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E170" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F170" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G170" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H170" s="64" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I170" s="62" t="inlineStr"/>
-      <c r="J170" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K170" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L170" s="62" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M170" s="65" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N170" s="63" t="inlineStr">
-        <is>
-          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
-        </is>
-      </c>
-    </row>
-    <row r="171" ht="30" customHeight="1">
-      <c r="A171" s="61" t="inlineStr">
-        <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="B171" s="61" t="inlineStr">
-        <is>
-          <t>Ualani Expansion</t>
-        </is>
-      </c>
-      <c r="C171" s="62" t="inlineStr">
-        <is>
-          <t>UALANI_FARM_01</t>
-        </is>
-      </c>
-      <c r="D171" s="63" t="inlineStr">
-        <is>
-          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E171" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F171" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G171" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H171" s="64" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I171" s="62" t="inlineStr"/>
-      <c r="J171" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K171" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L171" s="62" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M171" s="65" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N171" s="63" t="inlineStr">
-        <is>
-          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
-        </is>
-      </c>
-    </row>
-    <row r="172" ht="30" customHeight="1">
-      <c r="A172" s="61" t="inlineStr">
-        <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="B172" s="61" t="inlineStr">
-        <is>
-          <t>Ualani Expansion</t>
-        </is>
-      </c>
-      <c r="C172" s="62" t="inlineStr">
-        <is>
-          <t>UALANI_BARRACKS_01</t>
-        </is>
-      </c>
-      <c r="D172" s="63" t="inlineStr">
-        <is>
-          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E172" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F172" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G172" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H172" s="64" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I172" s="62" t="inlineStr"/>
-      <c r="J172" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K172" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L172" s="62" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M172" s="65" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N172" s="63" t="inlineStr">
-        <is>
-          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
-        </is>
-      </c>
-    </row>
-    <row r="173" ht="30" customHeight="1">
-      <c r="A173" s="61" t="inlineStr">
-        <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="B173" s="61" t="inlineStr">
-        <is>
-          <t>Ualani Expansion</t>
-        </is>
-      </c>
-      <c r="C173" s="62" t="inlineStr">
-        <is>
-          <t>UALANI_COURTHOUSE_01</t>
-        </is>
-      </c>
-      <c r="D173" s="63" t="inlineStr">
-        <is>
-          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E173" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F173" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G173" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H173" s="64" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I173" s="62" t="inlineStr"/>
-      <c r="J173" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K173" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L173" s="62" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M173" s="65" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N173" s="63" t="inlineStr">
-        <is>
-          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
-        </is>
-      </c>
+    <row r="173" ht="8" customHeight="1">
+      <c r="A173" s="9" t="n"/>
+      <c r="B173" s="9" t="n"/>
+      <c r="C173" s="9" t="n"/>
+      <c r="D173" s="9" t="n"/>
+      <c r="E173" s="9" t="n"/>
+      <c r="F173" s="9" t="n"/>
+      <c r="G173" s="9" t="n"/>
+      <c r="H173" s="9" t="n"/>
+      <c r="I173" s="9" t="n"/>
+      <c r="J173" s="9" t="n"/>
+      <c r="K173" s="9" t="n"/>
+      <c r="L173" s="9" t="n"/>
+      <c r="M173" s="9" t="n"/>
+      <c r="N173" s="9" t="n"/>
     </row>
     <row r="174" ht="30" customHeight="1">
       <c r="A174" s="61" t="inlineStr">
@@ -11855,17 +11803,17 @@
       </c>
       <c r="B174" s="61" t="inlineStr">
         <is>
-          <t>More City Events</t>
+          <t>Ualani Expansion</t>
         </is>
       </c>
       <c r="C174" s="62" t="inlineStr">
         <is>
-          <t>CL_WASHINGTON_01</t>
+          <t>UALANI_DOCK_01</t>
         </is>
       </c>
       <c r="D174" s="63" t="inlineStr">
         <is>
-          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
+          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E174" s="5" t="inlineStr">
@@ -11894,20 +11842,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K174" s="65" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L174" s="62" t="inlineStr"/>
+      <c r="K174" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L174" s="62" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M174" s="65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N174" s="63" t="inlineStr">
         <is>
-          <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
+          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
         </is>
       </c>
     </row>
@@ -11919,17 +11871,17 @@
       </c>
       <c r="B175" s="61" t="inlineStr">
         <is>
-          <t>More City Events</t>
+          <t>Ualani Expansion</t>
         </is>
       </c>
       <c r="C175" s="62" t="inlineStr">
         <is>
-          <t>CL_VALLEY_FORGE_01</t>
+          <t>UALANI_FARM_01</t>
         </is>
       </c>
       <c r="D175" s="63" t="inlineStr">
         <is>
-          <t>VALLEY FORGE SECURED  ← IDEA</t>
+          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E175" s="5" t="inlineStr">
@@ -11958,20 +11910,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K175" s="65" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L175" s="62" t="inlineStr"/>
+      <c r="K175" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L175" s="62" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M175" s="65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N175" s="63" t="inlineStr">
         <is>
-          <t>Tile 1; historically significant; would fire on liberation</t>
+          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
         </is>
       </c>
     </row>
@@ -11983,17 +11939,17 @@
       </c>
       <c r="B176" s="61" t="inlineStr">
         <is>
-          <t>More City Events</t>
+          <t>Ualani Expansion</t>
         </is>
       </c>
       <c r="C176" s="62" t="inlineStr">
         <is>
-          <t>CX_NYC_01</t>
+          <t>UALANI_BARRACKS_01</t>
         </is>
       </c>
       <c r="D176" s="63" t="inlineStr">
         <is>
-          <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
+          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E176" s="5" t="inlineStr">
@@ -12022,20 +11978,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K176" s="65" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L176" s="62" t="inlineStr"/>
+      <c r="K176" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L176" s="62" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M176" s="65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N176" s="63" t="inlineStr">
         <is>
-          <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
+          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
         </is>
       </c>
     </row>
@@ -12047,17 +12007,17 @@
       </c>
       <c r="B177" s="61" t="inlineStr">
         <is>
-          <t>Espionage Events</t>
+          <t>Ualani Expansion</t>
         </is>
       </c>
       <c r="C177" s="62" t="inlineStr">
         <is>
-          <t>ESPIONAGE_DISCOVERY_01</t>
+          <t>UALANI_COURTHOUSE_01</t>
         </is>
       </c>
       <c r="D177" s="63" t="inlineStr">
         <is>
-          <t>SPY NETWORK DISCOVERED AT [TILE_NAME]  ← IDEA</t>
+          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
@@ -12086,20 +12046,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K177" s="65" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L177" s="62" t="inlineStr"/>
+      <c r="K177" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L177" s="62" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M177" s="65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N177" s="63" t="inlineStr">
         <is>
-          <t>Would fire when espionageActive + enemy army arrives; uses existing espionage vars</t>
+          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
         </is>
       </c>
     </row>
@@ -12111,32 +12075,32 @@
       </c>
       <c r="B178" s="61" t="inlineStr">
         <is>
-          <t>Commander Expansion</t>
+          <t>More City Events</t>
         </is>
       </c>
       <c r="C178" s="62" t="inlineStr">
         <is>
-          <t>CMD_OBJECTIVE_2</t>
+          <t>CL_WASHINGTON_01</t>
         </is>
       </c>
       <c r="D178" s="63" t="inlineStr">
         <is>
-          <t>A COMMANDER'S SECOND TASK  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E178" s="22" t="inlineStr">
-        <is>
-          <t>Followup</t>
+          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F178" s="63" t="inlineStr">
         <is>
-          <t>CMD_OBJECTIVE_1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G178" s="63" t="inlineStr">
         <is>
-          <t>→ CMD_OBJECTIVE_3?</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H178" s="64" t="inlineStr">
@@ -12163,7 +12127,7 @@
       </c>
       <c r="N178" s="63" t="inlineStr">
         <is>
-          <t>Extend the commander arc beyond first objective</t>
+          <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
         </is>
       </c>
     </row>
@@ -12175,17 +12139,17 @@
       </c>
       <c r="B179" s="61" t="inlineStr">
         <is>
-          <t>Seasonal Events</t>
+          <t>More City Events</t>
         </is>
       </c>
       <c r="C179" s="62" t="inlineStr">
         <is>
-          <t>WINTER_SIEGE_01</t>
+          <t>CL_VALLEY_FORGE_01</t>
         </is>
       </c>
       <c r="D179" s="63" t="inlineStr">
         <is>
-          <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
+          <t>VALLEY FORGE SECURED  ← IDEA</t>
         </is>
       </c>
       <c r="E179" s="5" t="inlineStr">
@@ -12227,7 +12191,7 @@
       </c>
       <c r="N179" s="63" t="inlineStr">
         <is>
-          <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
+          <t>Tile 1; historically significant; would fire on liberation</t>
         </is>
       </c>
     </row>
@@ -12239,17 +12203,17 @@
       </c>
       <c r="B180" s="61" t="inlineStr">
         <is>
-          <t>Seasonal Events</t>
+          <t>More City Events</t>
         </is>
       </c>
       <c r="C180" s="62" t="inlineStr">
         <is>
-          <t>SPRING_OFFENSIVE_01</t>
+          <t>CX_NYC_01</t>
         </is>
       </c>
       <c r="D180" s="63" t="inlineStr">
         <is>
-          <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
+          <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
         </is>
       </c>
       <c r="E180" s="5" t="inlineStr">
@@ -12291,48 +12255,304 @@
       </c>
       <c r="N180" s="63" t="inlineStr">
         <is>
+          <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="30" customHeight="1">
+      <c r="A181" s="61" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B181" s="61" t="inlineStr">
+        <is>
+          <t>Espionage Events</t>
+        </is>
+      </c>
+      <c r="C181" s="62" t="inlineStr">
+        <is>
+          <t>ESPIONAGE_DISCOVERY_01</t>
+        </is>
+      </c>
+      <c r="D181" s="63" t="inlineStr">
+        <is>
+          <t>SPY NETWORK DISCOVERED AT [TILE_NAME]  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F181" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G181" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H181" s="64" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I181" s="62" t="inlineStr"/>
+      <c r="J181" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K181" s="65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L181" s="62" t="inlineStr"/>
+      <c r="M181" s="65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N181" s="63" t="inlineStr">
+        <is>
+          <t>Would fire when espionageActive + enemy army arrives; uses existing espionage vars</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="30" customHeight="1">
+      <c r="A182" s="61" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B182" s="61" t="inlineStr">
+        <is>
+          <t>Commander Expansion</t>
+        </is>
+      </c>
+      <c r="C182" s="62" t="inlineStr">
+        <is>
+          <t>CMD_OBJECTIVE_2</t>
+        </is>
+      </c>
+      <c r="D182" s="63" t="inlineStr">
+        <is>
+          <t>A COMMANDER'S SECOND TASK  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E182" s="22" t="inlineStr">
+        <is>
+          <t>Followup</t>
+        </is>
+      </c>
+      <c r="F182" s="63" t="inlineStr">
+        <is>
+          <t>CMD_OBJECTIVE_1</t>
+        </is>
+      </c>
+      <c r="G182" s="63" t="inlineStr">
+        <is>
+          <t>→ CMD_OBJECTIVE_3?</t>
+        </is>
+      </c>
+      <c r="H182" s="64" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I182" s="62" t="inlineStr"/>
+      <c r="J182" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K182" s="65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L182" s="62" t="inlineStr"/>
+      <c r="M182" s="65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N182" s="63" t="inlineStr">
+        <is>
+          <t>Extend the commander arc beyond first objective</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="30" customHeight="1">
+      <c r="A183" s="61" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B183" s="61" t="inlineStr">
+        <is>
+          <t>Seasonal Events</t>
+        </is>
+      </c>
+      <c r="C183" s="62" t="inlineStr">
+        <is>
+          <t>WINTER_SIEGE_01</t>
+        </is>
+      </c>
+      <c r="D183" s="63" t="inlineStr">
+        <is>
+          <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F183" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G183" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H183" s="64" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I183" s="62" t="inlineStr"/>
+      <c r="J183" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K183" s="65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L183" s="62" t="inlineStr"/>
+      <c r="M183" s="65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N183" s="63" t="inlineStr">
+        <is>
+          <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="30" customHeight="1">
+      <c r="A184" s="61" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B184" s="61" t="inlineStr">
+        <is>
+          <t>Seasonal Events</t>
+        </is>
+      </c>
+      <c r="C184" s="62" t="inlineStr">
+        <is>
+          <t>SPRING_OFFENSIVE_01</t>
+        </is>
+      </c>
+      <c r="D184" s="63" t="inlineStr">
+        <is>
+          <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F184" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G184" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H184" s="64" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I184" s="62" t="inlineStr"/>
+      <c r="J184" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K184" s="65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L184" s="62" t="inlineStr"/>
+      <c r="M184" s="65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N184" s="63" t="inlineStr">
+        <is>
           <t>Month 3-4; UK neighbor + player army present; tactical pressure event</t>
         </is>
       </c>
     </row>
-    <row r="182" ht="20" customHeight="1">
-      <c r="A182" s="66" t="inlineStr">
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="66" t="inlineStr">
         <is>
           <t>Total events in spreadsheet</t>
         </is>
       </c>
-      <c r="B182" s="67" t="n">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="183" ht="20" customHeight="1">
-      <c r="A183" s="66" t="inlineStr">
+      <c r="B186" s="67" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="66" t="inlineStr">
         <is>
           <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
-      <c r="B183" s="67" t="n">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="184" ht="20" customHeight="1">
-      <c r="A184" s="66" t="inlineStr">
+      <c r="B187" s="67" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="188" ht="20" customHeight="1">
+      <c r="A188" s="66" t="inlineStr">
         <is>
           <t>IDEA (not yet implemented)</t>
         </is>
       </c>
-      <c r="B184" s="67" t="n">
+      <c r="B188" s="67" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="185" ht="20" customHeight="1">
-      <c r="A185" s="66" t="inlineStr">
+    <row r="189" ht="20" customHeight="1">
+      <c r="A189" s="66" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B185" s="67" t="n">
-        <v>49</v>
+      <c r="B189" s="67" t="n">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -12346,7 +12566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14717,44 +14937,264 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="66" t="inlineStr">
+    <row r="37" ht="8" customHeight="1">
+      <c r="A37" s="9" t="n"/>
+      <c r="B37" s="9" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="9" t="n"/>
+      <c r="L37" s="9" t="n"/>
+      <c r="M37" s="9" t="n"/>
+      <c r="N37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B38" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C38" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_ALLIED_01</t>
+        </is>
+      </c>
+      <c r="D38" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F38" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I38" s="54" t="inlineStr"/>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K38" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L38" s="54" t="inlineStr">
+        <is>
+          <t>sensual option</t>
+        </is>
+      </c>
+      <c r="M38" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N38" s="55" t="inlineStr">
+        <is>
+          <t>Allied peace: fires when all UK dock tiles in USA+CA regions liberated (can_allied); sets uk_usa_peace+uk_ca_peace on UK country; BTN2 sensual — Ualani+Jessica celebrate</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B39" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C39" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_USA_01</t>
+        </is>
+      </c>
+      <c r="D39" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F39" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I39" s="54" t="inlineStr"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K39" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L39" s="54" t="inlineStr">
+        <is>
+          <t>sensual option</t>
+        </is>
+      </c>
+      <c r="M39" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N39" s="55" t="inlineStr">
+        <is>
+          <t>USA separate peace (unallied): fires when all USA dock tiles liberated (65,66,67,151); sets uk_usa_peace on UK country; BTN2 sensual — Ualani alone at dawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B40" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C40" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_CA_AI_01</t>
+        </is>
+      </c>
+      <c r="D40" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — CANADA NEGOTIATES SEPARATE PEACE</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F40" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="54" t="inlineStr"/>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K40" s="56" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L40" s="54" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="M40" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N40" s="55" t="inlineStr">
+        <is>
+          <t>CA separate peace (unallied): fires when Halifax (tile 114) liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="66" t="inlineStr">
         <is>
           <t>Canadian events total</t>
         </is>
       </c>
-      <c r="B38" s="67" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="66" t="inlineStr">
+      <c r="B42" s="67" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="66" t="inlineStr">
         <is>
           <t>Canada (Alliance arc)</t>
         </is>
       </c>
-      <c r="B39" s="67" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="66" t="inlineStr">
+      <c r="B43" s="67" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="66" t="inlineStr">
         <is>
           <t>CA Protector (Jessica's creatures)</t>
         </is>
       </c>
-      <c r="B40" s="67" t="n">
+      <c r="B44" s="67" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="66" t="inlineStr">
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="66" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B41" s="67" t="n">
-        <v>10</v>
+      <c r="B45" s="67" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -15105,7 +15545,7 @@
       </c>
       <c r="B32" s="112" t="inlineStr">
         <is>
-          <t>Canadian Alliance diplomatic arc (war declaration + 8 CAN_ events)</t>
+          <t>Canadian Alliance diplomatic arc + 3 peace events (PEACE_ALLIED_01, PEACE_USA_01, PEACE_CA_AI_01)</t>
         </is>
       </c>
       <c r="C32" s="112" t="n"/>

</xml_diff>

<commit_message>
Add docks to Quebec City and Anticosti — expand CA peace objectives to 3
Quebec City (tile 123) gets dock:2 and Anticosti (tile 195) gets dock:1,
both UK-owned CA-QB tiles. PEACE_DOCK_CA expands from [114] to
[114, 123, 195] so Canada must liberate Halifax, Quebec City, and
Anticosti for peace — giving UK connected St. Lawrence supply lines
and Canada three meaningful campaign objectives.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -11691,7 +11691,7 @@
       </c>
       <c r="N170" s="55" t="inlineStr">
         <is>
-          <t>CA separate peace (unallied): fires when Halifax (tile 114) liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
+          <t>CA separate peace (unallied): fires when Halifax (114), Quebec City (123), and Anticosti (195) all liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
         </is>
       </c>
     </row>
@@ -15153,7 +15153,7 @@
       </c>
       <c r="N40" s="55" t="inlineStr">
         <is>
-          <t>CA separate peace (unallied): fires when Halifax (tile 114) liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
+          <t>CA separate peace (unallied): fires when Halifax (114), Quebec City (123), and Anticosti (195) all liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add George III peace offer event firing at turn 75-80
GEORGE_PEACE_01 fires between turns 75-80 if the war is still ongoing
(no uk_usa_peace on UK country and neither george_peace_accepted nor
george_peace_rejected flags are set on the player).

BTN1 (george_peace_accept): calls _apply_george_peace() — sets uk_usa_peace
on UK; if can_allied, also sets uk_ca_peace on UK and CA; sets
george_peace_accepted on playerCountry.

BTN2 (george_peace_reject): sets george_peace_rejected flag + presidentialClaim
+1 (defiance bonus); war continues.

Alliance awareness: accepting while can_allied binds both nations to peace;
accepting while unallied ends the war for USA only — CA fights on separately.

168 events total.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -1052,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N189"/>
+  <dimension ref="A1:N190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11504,12 +11504,12 @@
       </c>
       <c r="C168" s="54" t="inlineStr">
         <is>
-          <t>PEACE_ALLIED_01</t>
+          <t>GEORGE_PEACE_01</t>
         </is>
       </c>
       <c r="D168" s="55" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
+          <t>A ROYAL LETTER ARRIVES — HIS MAJESTY PROPOSES PEACE</t>
         </is>
       </c>
       <c r="E168" s="5" t="inlineStr">
@@ -11538,14 +11538,14 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K168" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="K168" s="56" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="L168" s="54" t="inlineStr">
         <is>
-          <t>sensual option</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="M168" s="56" t="inlineStr">
@@ -11555,7 +11555,7 @@
       </c>
       <c r="N168" s="55" t="inlineStr">
         <is>
-          <t>Allied peace: fires when all UK dock tiles in USA+CA regions liberated (can_allied); sets uk_usa_peace+uk_ca_peace on UK country; BTN2 sensual — Ualani+Jessica celebrate</t>
+          <t>Fires turn 75-80 if war ongoing; BTN1 george_peace_accept (allied=both peaces, unallied=USA only); BTN2 george_peace_reject (+claim +1); never fires if peace already settled</t>
         </is>
       </c>
     </row>
@@ -11572,12 +11572,12 @@
       </c>
       <c r="C169" s="54" t="inlineStr">
         <is>
-          <t>PEACE_USA_01</t>
+          <t>PEACE_ALLIED_01</t>
         </is>
       </c>
       <c r="D169" s="55" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
+          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
         </is>
       </c>
       <c r="E169" s="5" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="N169" s="55" t="inlineStr">
         <is>
-          <t>USA separate peace (unallied): fires when all USA dock tiles liberated (65,66,67,151); sets uk_usa_peace on UK country; BTN2 sensual — Ualani alone at dawn</t>
+          <t>Allied peace: fires when all UK dock tiles in USA+CA regions liberated (can_allied); sets uk_usa_peace+uk_ca_peace on UK country; BTN2 sensual — Ualani+Jessica celebrate</t>
         </is>
       </c>
     </row>
@@ -11640,12 +11640,12 @@
       </c>
       <c r="C170" s="54" t="inlineStr">
         <is>
-          <t>PEACE_CA_AI_01</t>
+          <t>PEACE_USA_01</t>
         </is>
       </c>
       <c r="D170" s="55" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — CANADA NEGOTIATES SEPARATE PEACE</t>
+          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
         </is>
       </c>
       <c r="E170" s="5" t="inlineStr">
@@ -11674,194 +11674,194 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K170" s="56" t="inlineStr">
+      <c r="K170" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L170" s="54" t="inlineStr">
+        <is>
+          <t>sensual option</t>
+        </is>
+      </c>
+      <c r="M170" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N170" s="55" t="inlineStr">
+        <is>
+          <t>USA separate peace (unallied): fires when all USA dock tiles liberated (65,66,67,151); sets uk_usa_peace on UK country; BTN2 sensual — Ualani alone at dawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="30" customHeight="1">
+      <c r="A171" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B171" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C171" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_CA_AI_01</t>
+        </is>
+      </c>
+      <c r="D171" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — CANADA NEGOTIATES SEPARATE PEACE</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F171" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G171" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H171" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I171" s="54" t="inlineStr"/>
+      <c r="J171" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K171" s="56" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L170" s="54" t="inlineStr">
+      <c r="L171" s="54" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="M170" s="56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N170" s="55" t="inlineStr">
+      <c r="M171" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N171" s="55" t="inlineStr">
         <is>
           <t>CA separate peace (unallied): fires when Halifax (114), Quebec City (123), and Anticosti (195) all liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
         </is>
       </c>
     </row>
-    <row r="171" ht="8" customHeight="1">
-      <c r="A171" s="9" t="n"/>
-      <c r="B171" s="9" t="n"/>
-      <c r="C171" s="9" t="n"/>
-      <c r="D171" s="9" t="n"/>
-      <c r="E171" s="9" t="n"/>
-      <c r="F171" s="9" t="n"/>
-      <c r="G171" s="9" t="n"/>
-      <c r="H171" s="9" t="n"/>
-      <c r="I171" s="9" t="n"/>
-      <c r="J171" s="9" t="n"/>
-      <c r="K171" s="9" t="n"/>
-      <c r="L171" s="9" t="n"/>
-      <c r="M171" s="9" t="n"/>
-      <c r="N171" s="9" t="n"/>
-    </row>
-    <row r="172" ht="30" customHeight="1">
-      <c r="A172" s="49" t="inlineStr">
+    <row r="172" ht="8" customHeight="1">
+      <c r="A172" s="9" t="n"/>
+      <c r="B172" s="9" t="n"/>
+      <c r="C172" s="9" t="n"/>
+      <c r="D172" s="9" t="n"/>
+      <c r="E172" s="9" t="n"/>
+      <c r="F172" s="9" t="n"/>
+      <c r="G172" s="9" t="n"/>
+      <c r="H172" s="9" t="n"/>
+      <c r="I172" s="9" t="n"/>
+      <c r="J172" s="9" t="n"/>
+      <c r="K172" s="9" t="n"/>
+      <c r="L172" s="9" t="n"/>
+      <c r="M172" s="9" t="n"/>
+      <c r="N172" s="9" t="n"/>
+    </row>
+    <row r="173" ht="30" customHeight="1">
+      <c r="A173" s="49" t="inlineStr">
         <is>
           <t>VP Arc</t>
         </is>
       </c>
-      <c r="B172" s="49" t="inlineStr">
+      <c r="B173" s="49" t="inlineStr">
         <is>
           <t>VP Arc</t>
         </is>
       </c>
-      <c r="C172" s="50" t="inlineStr">
+      <c r="C173" s="50" t="inlineStr">
         <is>
           <t>VP_LEGACY</t>
         </is>
       </c>
-      <c r="D172" s="51" t="inlineStr">
+      <c r="D173" s="51" t="inlineStr">
         <is>
           <t>THE VICE PRESIDENT LEAVES A NOTE — [COMMANDER_NAME] HAS SOMETHING TO SAY</t>
         </is>
       </c>
-      <c r="E172" s="22" t="inlineStr">
+      <c r="E173" s="22" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="F172" s="51" t="inlineStr">
+      <c r="F173" s="51" t="inlineStr">
         <is>
           <t>VP_FIRST_MEETING (turn 96+)</t>
         </is>
       </c>
-      <c r="G172" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H172" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I172" s="50" t="inlineStr"/>
-      <c r="J172" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K172" s="26" t="inlineStr">
+      <c r="G173" s="51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H173" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I173" s="50" t="inlineStr"/>
+      <c r="J173" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K173" s="26" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="L172" s="50" t="inlineStr">
+      <c r="L173" s="50" t="inlineStr">
         <is>
           <t>explicit option</t>
         </is>
       </c>
-      <c r="M172" s="52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N172" s="51" t="inlineStr">
+      <c r="M173" s="52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N173" s="51" t="inlineStr">
         <is>
           <t>Fires turn 96+; BTN1 claim +1 / BTN2 explicit morale +30</t>
         </is>
       </c>
     </row>
-    <row r="173" ht="8" customHeight="1">
-      <c r="A173" s="9" t="n"/>
-      <c r="B173" s="9" t="n"/>
-      <c r="C173" s="9" t="n"/>
-      <c r="D173" s="9" t="n"/>
-      <c r="E173" s="9" t="n"/>
-      <c r="F173" s="9" t="n"/>
-      <c r="G173" s="9" t="n"/>
-      <c r="H173" s="9" t="n"/>
-      <c r="I173" s="9" t="n"/>
-      <c r="J173" s="9" t="n"/>
-      <c r="K173" s="9" t="n"/>
-      <c r="L173" s="9" t="n"/>
-      <c r="M173" s="9" t="n"/>
-      <c r="N173" s="9" t="n"/>
-    </row>
-    <row r="174" ht="30" customHeight="1">
-      <c r="A174" s="61" t="inlineStr">
-        <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="B174" s="61" t="inlineStr">
-        <is>
-          <t>Ualani Expansion</t>
-        </is>
-      </c>
-      <c r="C174" s="62" t="inlineStr">
-        <is>
-          <t>UALANI_DOCK_01</t>
-        </is>
-      </c>
-      <c r="D174" s="63" t="inlineStr">
-        <is>
-          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E174" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
-        </is>
-      </c>
-      <c r="F174" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G174" s="63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H174" s="64" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I174" s="62" t="inlineStr"/>
-      <c r="J174" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K174" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L174" s="62" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M174" s="65" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N174" s="63" t="inlineStr">
-        <is>
-          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
-        </is>
-      </c>
+    <row r="174" ht="8" customHeight="1">
+      <c r="A174" s="9" t="n"/>
+      <c r="B174" s="9" t="n"/>
+      <c r="C174" s="9" t="n"/>
+      <c r="D174" s="9" t="n"/>
+      <c r="E174" s="9" t="n"/>
+      <c r="F174" s="9" t="n"/>
+      <c r="G174" s="9" t="n"/>
+      <c r="H174" s="9" t="n"/>
+      <c r="I174" s="9" t="n"/>
+      <c r="J174" s="9" t="n"/>
+      <c r="K174" s="9" t="n"/>
+      <c r="L174" s="9" t="n"/>
+      <c r="M174" s="9" t="n"/>
+      <c r="N174" s="9" t="n"/>
     </row>
     <row r="175" ht="30" customHeight="1">
       <c r="A175" s="61" t="inlineStr">
@@ -11876,12 +11876,12 @@
       </c>
       <c r="C175" s="62" t="inlineStr">
         <is>
-          <t>UALANI_FARM_01</t>
+          <t>UALANI_DOCK_01</t>
         </is>
       </c>
       <c r="D175" s="63" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
+          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E175" s="5" t="inlineStr">
@@ -11927,7 +11927,7 @@
       </c>
       <c r="N175" s="63" t="inlineStr">
         <is>
-          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
+          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
         </is>
       </c>
     </row>
@@ -11944,12 +11944,12 @@
       </c>
       <c r="C176" s="62" t="inlineStr">
         <is>
-          <t>UALANI_BARRACKS_01</t>
+          <t>UALANI_FARM_01</t>
         </is>
       </c>
       <c r="D176" s="63" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
+          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E176" s="5" t="inlineStr">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="N176" s="63" t="inlineStr">
         <is>
-          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
+          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
         </is>
       </c>
     </row>
@@ -12012,12 +12012,12 @@
       </c>
       <c r="C177" s="62" t="inlineStr">
         <is>
-          <t>UALANI_COURTHOUSE_01</t>
+          <t>UALANI_BARRACKS_01</t>
         </is>
       </c>
       <c r="D177" s="63" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
+          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="N177" s="63" t="inlineStr">
         <is>
-          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
+          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
         </is>
       </c>
     </row>
@@ -12075,17 +12075,17 @@
       </c>
       <c r="B178" s="61" t="inlineStr">
         <is>
-          <t>More City Events</t>
+          <t>Ualani Expansion</t>
         </is>
       </c>
       <c r="C178" s="62" t="inlineStr">
         <is>
-          <t>CL_WASHINGTON_01</t>
+          <t>UALANI_COURTHOUSE_01</t>
         </is>
       </c>
       <c r="D178" s="63" t="inlineStr">
         <is>
-          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
+          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
       <c r="E178" s="5" t="inlineStr">
@@ -12114,20 +12114,24 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K178" s="65" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L178" s="62" t="inlineStr"/>
+      <c r="K178" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L178" s="62" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
       <c r="M178" s="65" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N178" s="63" t="inlineStr">
         <is>
-          <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
+          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
         </is>
       </c>
     </row>
@@ -12144,12 +12148,12 @@
       </c>
       <c r="C179" s="62" t="inlineStr">
         <is>
-          <t>CL_VALLEY_FORGE_01</t>
+          <t>CL_WASHINGTON_01</t>
         </is>
       </c>
       <c r="D179" s="63" t="inlineStr">
         <is>
-          <t>VALLEY FORGE SECURED  ← IDEA</t>
+          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
         </is>
       </c>
       <c r="E179" s="5" t="inlineStr">
@@ -12191,7 +12195,7 @@
       </c>
       <c r="N179" s="63" t="inlineStr">
         <is>
-          <t>Tile 1; historically significant; would fire on liberation</t>
+          <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
         </is>
       </c>
     </row>
@@ -12208,12 +12212,12 @@
       </c>
       <c r="C180" s="62" t="inlineStr">
         <is>
-          <t>CX_NYC_01</t>
+          <t>CL_VALLEY_FORGE_01</t>
         </is>
       </c>
       <c r="D180" s="63" t="inlineStr">
         <is>
-          <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
+          <t>VALLEY FORGE SECURED  ← IDEA</t>
         </is>
       </c>
       <c r="E180" s="5" t="inlineStr">
@@ -12255,7 +12259,7 @@
       </c>
       <c r="N180" s="63" t="inlineStr">
         <is>
-          <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
+          <t>Tile 1; historically significant; would fire on liberation</t>
         </is>
       </c>
     </row>
@@ -12267,17 +12271,17 @@
       </c>
       <c r="B181" s="61" t="inlineStr">
         <is>
-          <t>Espionage Events</t>
+          <t>More City Events</t>
         </is>
       </c>
       <c r="C181" s="62" t="inlineStr">
         <is>
-          <t>ESPIONAGE_DISCOVERY_01</t>
+          <t>CX_NYC_01</t>
         </is>
       </c>
       <c r="D181" s="63" t="inlineStr">
         <is>
-          <t>SPY NETWORK DISCOVERED AT [TILE_NAME]  ← IDEA</t>
+          <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
         </is>
       </c>
       <c r="E181" s="5" t="inlineStr">
@@ -12319,7 +12323,7 @@
       </c>
       <c r="N181" s="63" t="inlineStr">
         <is>
-          <t>Would fire when espionageActive + enemy army arrives; uses existing espionage vars</t>
+          <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
         </is>
       </c>
     </row>
@@ -12331,32 +12335,32 @@
       </c>
       <c r="B182" s="61" t="inlineStr">
         <is>
-          <t>Commander Expansion</t>
+          <t>Espionage Events</t>
         </is>
       </c>
       <c r="C182" s="62" t="inlineStr">
         <is>
-          <t>CMD_OBJECTIVE_2</t>
+          <t>ESPIONAGE_DISCOVERY_01</t>
         </is>
       </c>
       <c r="D182" s="63" t="inlineStr">
         <is>
-          <t>A COMMANDER'S SECOND TASK  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E182" s="22" t="inlineStr">
-        <is>
-          <t>Followup</t>
+          <t>SPY NETWORK DISCOVERED AT [TILE_NAME]  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
         </is>
       </c>
       <c r="F182" s="63" t="inlineStr">
         <is>
-          <t>CMD_OBJECTIVE_1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G182" s="63" t="inlineStr">
         <is>
-          <t>→ CMD_OBJECTIVE_3?</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H182" s="64" t="inlineStr">
@@ -12383,7 +12387,7 @@
       </c>
       <c r="N182" s="63" t="inlineStr">
         <is>
-          <t>Extend the commander arc beyond first objective</t>
+          <t>Would fire when espionageActive + enemy army arrives; uses existing espionage vars</t>
         </is>
       </c>
     </row>
@@ -12395,32 +12399,32 @@
       </c>
       <c r="B183" s="61" t="inlineStr">
         <is>
-          <t>Seasonal Events</t>
+          <t>Commander Expansion</t>
         </is>
       </c>
       <c r="C183" s="62" t="inlineStr">
         <is>
-          <t>WINTER_SIEGE_01</t>
+          <t>CMD_OBJECTIVE_2</t>
         </is>
       </c>
       <c r="D183" s="63" t="inlineStr">
         <is>
-          <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E183" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>A COMMANDER'S SECOND TASK  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E183" s="22" t="inlineStr">
+        <is>
+          <t>Followup</t>
         </is>
       </c>
       <c r="F183" s="63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CMD_OBJECTIVE_1</t>
         </is>
       </c>
       <c r="G183" s="63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>→ CMD_OBJECTIVE_3?</t>
         </is>
       </c>
       <c r="H183" s="64" t="inlineStr">
@@ -12447,7 +12451,7 @@
       </c>
       <c r="N183" s="63" t="inlineStr">
         <is>
-          <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
+          <t>Extend the commander arc beyond first objective</t>
         </is>
       </c>
     </row>
@@ -12464,12 +12468,12 @@
       </c>
       <c r="C184" s="62" t="inlineStr">
         <is>
-          <t>SPRING_OFFENSIVE_01</t>
+          <t>WINTER_SIEGE_01</t>
         </is>
       </c>
       <c r="D184" s="63" t="inlineStr">
         <is>
-          <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
+          <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
         </is>
       </c>
       <c r="E184" s="5" t="inlineStr">
@@ -12511,47 +12515,111 @@
       </c>
       <c r="N184" s="63" t="inlineStr">
         <is>
+          <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="30" customHeight="1">
+      <c r="A185" s="61" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B185" s="61" t="inlineStr">
+        <is>
+          <t>Seasonal Events</t>
+        </is>
+      </c>
+      <c r="C185" s="62" t="inlineStr">
+        <is>
+          <t>SPRING_OFFENSIVE_01</t>
+        </is>
+      </c>
+      <c r="D185" s="63" t="inlineStr">
+        <is>
+          <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F185" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G185" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H185" s="64" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I185" s="62" t="inlineStr"/>
+      <c r="J185" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K185" s="65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L185" s="62" t="inlineStr"/>
+      <c r="M185" s="65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N185" s="63" t="inlineStr">
+        <is>
           <t>Month 3-4; UK neighbor + player army present; tactical pressure event</t>
         </is>
-      </c>
-    </row>
-    <row r="186" ht="20" customHeight="1">
-      <c r="A186" s="66" t="inlineStr">
-        <is>
-          <t>Total events in spreadsheet</t>
-        </is>
-      </c>
-      <c r="B186" s="67" t="n">
-        <v>167</v>
       </c>
     </row>
     <row r="187" ht="20" customHeight="1">
       <c r="A187" s="66" t="inlineStr">
         <is>
-          <t>FIRST PASS (coded &amp; wired)</t>
+          <t>Total events in spreadsheet</t>
         </is>
       </c>
       <c r="B187" s="67" t="n">
-        <v>156</v>
+        <v>168</v>
       </c>
     </row>
     <row r="188" ht="20" customHeight="1">
       <c r="A188" s="66" t="inlineStr">
         <is>
-          <t>IDEA (not yet implemented)</t>
+          <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
       <c r="B188" s="67" t="n">
-        <v>11</v>
+        <v>157</v>
       </c>
     </row>
     <row r="189" ht="20" customHeight="1">
       <c r="A189" s="66" t="inlineStr">
         <is>
+          <t>IDEA (not yet implemented)</t>
+        </is>
+      </c>
+      <c r="B189" s="67" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="190" ht="20" customHeight="1">
+      <c r="A190" s="66" t="inlineStr">
+        <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B189" s="67" t="n">
+      <c r="B190" s="67" t="n">
         <v>51</v>
       </c>
     </row>
@@ -12566,7 +12634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14966,12 +15034,12 @@
       </c>
       <c r="C38" s="54" t="inlineStr">
         <is>
-          <t>PEACE_ALLIED_01</t>
+          <t>GEORGE_PEACE_01</t>
         </is>
       </c>
       <c r="D38" s="55" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
+          <t>A ROYAL LETTER ARRIVES — HIS MAJESTY PROPOSES PEACE</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -15000,14 +15068,14 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K38" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="K38" s="56" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="L38" s="54" t="inlineStr">
         <is>
-          <t>sensual option</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="M38" s="56" t="inlineStr">
@@ -15017,7 +15085,7 @@
       </c>
       <c r="N38" s="55" t="inlineStr">
         <is>
-          <t>Allied peace: fires when all UK dock tiles in USA+CA regions liberated (can_allied); sets uk_usa_peace+uk_ca_peace on UK country; BTN2 sensual — Ualani+Jessica celebrate</t>
+          <t>Fires turn 75-80 if war ongoing; BTN1 george_peace_accept (allied=both peaces, unallied=USA only); BTN2 george_peace_reject (+claim +1); never fires if peace already settled</t>
         </is>
       </c>
     </row>
@@ -15034,12 +15102,12 @@
       </c>
       <c r="C39" s="54" t="inlineStr">
         <is>
-          <t>PEACE_USA_01</t>
+          <t>PEACE_ALLIED_01</t>
         </is>
       </c>
       <c r="D39" s="55" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
+          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -15085,7 +15153,7 @@
       </c>
       <c r="N39" s="55" t="inlineStr">
         <is>
-          <t>USA separate peace (unallied): fires when all USA dock tiles liberated (65,66,67,151); sets uk_usa_peace on UK country; BTN2 sensual — Ualani alone at dawn</t>
+          <t>Allied peace: fires when all UK dock tiles in USA+CA regions liberated (can_allied); sets uk_usa_peace+uk_ca_peace on UK country; BTN2 sensual — Ualani+Jessica celebrate</t>
         </is>
       </c>
     </row>
@@ -15102,12 +15170,12 @@
       </c>
       <c r="C40" s="54" t="inlineStr">
         <is>
-          <t>PEACE_CA_AI_01</t>
+          <t>PEACE_USA_01</t>
         </is>
       </c>
       <c r="D40" s="55" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — CANADA NEGOTIATES SEPARATE PEACE</t>
+          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -15136,64 +15204,132 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K40" s="56" t="inlineStr">
+      <c r="K40" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L40" s="54" t="inlineStr">
+        <is>
+          <t>sensual option</t>
+        </is>
+      </c>
+      <c r="M40" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N40" s="55" t="inlineStr">
+        <is>
+          <t>USA separate peace (unallied): fires when all USA dock tiles liberated (65,66,67,151); sets uk_usa_peace on UK country; BTN2 sensual — Ualani alone at dawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B41" s="53" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C41" s="54" t="inlineStr">
+        <is>
+          <t>PEACE_CA_AI_01</t>
+        </is>
+      </c>
+      <c r="D41" s="55" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — CANADA NEGOTIATES SEPARATE PEACE</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F41" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I41" s="54" t="inlineStr"/>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K41" s="56" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L40" s="54" t="inlineStr">
+      <c r="L41" s="54" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="M40" s="56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N40" s="55" t="inlineStr">
+      <c r="M41" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N41" s="55" t="inlineStr">
         <is>
           <t>CA separate peace (unallied): fires when Halifax (114), Quebec City (123), and Anticosti (195) all liberated; sets uk_ca_peace on UK+CA; player-visible dispatch; both buttons standard</t>
         </is>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="66" t="inlineStr">
-        <is>
-          <t>Canadian events total</t>
-        </is>
-      </c>
-      <c r="B42" s="67" t="n">
-        <v>37</v>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="66" t="inlineStr">
         <is>
-          <t>Canada (Alliance arc)</t>
+          <t>Canadian events total</t>
         </is>
       </c>
       <c r="B43" s="67" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="66" t="inlineStr">
         <is>
-          <t>CA Protector (Jessica's creatures)</t>
+          <t>Canada (Alliance arc)</t>
         </is>
       </c>
       <c r="B44" s="67" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="66" t="inlineStr">
         <is>
+          <t>CA Protector (Jessica's creatures)</t>
+        </is>
+      </c>
+      <c r="B45" s="67" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="66" t="inlineStr">
+        <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B45" s="67" t="n">
+      <c r="B46" s="67" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Chalchiuhtotolin super-secret protector arc
Fires only when Ualani is stationed at Plymouth (tile 66) on Thanksgiving
(month 11). The Jade Turkey God appears and initiates a 5-event quest chain
requiring the player to build up their agricultural capacity:

- CHALCH_SUMMON: trigger event; sets chalch_summoned flag
- CHALCH_Q1:  3+ player farms → +30 food
- CHALCH_Q2:  TotalFood >= 150 → +50 food
- CHALCH_Q3:  5+ player farms → +40 food
- CHALCH_AGREE: all quests done → +100 food divine bounty

world.gd: _check_chalch_summon(), _check_chalch_quests(), _count_player_farms()
masterdoc: new Chalchiuhtotolin category (jade-green); 210 events total

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -185,7 +185,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="28">
+  <fills count="29">
     <fill>
       <patternFill/>
     </fill>
@@ -299,6 +299,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D6F5D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EDE0F7"/>
       </patternFill>
     </fill>
@@ -349,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -562,10 +567,22 @@
     <xf numFmtId="0" fontId="2" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -577,10 +594,10 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -589,10 +606,10 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -601,10 +618,10 @@
     <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -613,10 +630,10 @@
     <xf numFmtId="0" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -731,6 +748,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1098,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N229"/>
+  <dimension ref="A1:N235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14460,22 +14483,22 @@
     <row r="214" ht="30" customHeight="1">
       <c r="A214" s="69" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Chalchiuhtotolin</t>
         </is>
       </c>
       <c r="B214" s="69" t="inlineStr">
         <is>
-          <t>Ualani Expansion</t>
+          <t>Jade Turkey Arc</t>
         </is>
       </c>
       <c r="C214" s="70" t="inlineStr">
         <is>
-          <t>UALANI_DOCK_01</t>
+          <t>CHALCH_SUMMON</t>
         </is>
       </c>
       <c r="D214" s="71" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
+          <t>CHALCHIUHTOTOLIN ARRIVES AT PLYMOUTH ON THANKSGIVING</t>
         </is>
       </c>
       <c r="E214" s="5" t="inlineStr">
@@ -14490,12 +14513,12 @@
       </c>
       <c r="G214" s="71" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H214" s="72" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+          <t>CHALCH_Q1</t>
+        </is>
+      </c>
+      <c r="H214" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I214" s="70" t="inlineStr"/>
@@ -14504,66 +14527,62 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K214" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L214" s="70" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M214" s="73" t="inlineStr">
-        <is>
-          <t>15</t>
+      <c r="K214" s="72" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L214" s="70" t="inlineStr"/>
+      <c r="M214" s="72" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="N214" s="71" t="inlineStr">
         <is>
-          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
+          <t>Month 11, Ualani at tile 66 (Plymouth); one-shot; sets chalch_summoned flag</t>
         </is>
       </c>
     </row>
     <row r="215" ht="30" customHeight="1">
       <c r="A215" s="69" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Chalchiuhtotolin</t>
         </is>
       </c>
       <c r="B215" s="69" t="inlineStr">
         <is>
-          <t>Ualani Expansion</t>
+          <t>Jade Turkey Arc</t>
         </is>
       </c>
       <c r="C215" s="70" t="inlineStr">
         <is>
-          <t>UALANI_FARM_01</t>
+          <t>CHALCH_Q1</t>
         </is>
       </c>
       <c r="D215" s="71" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E215" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>THE JADE TURKEY DEMANDS THREE GRANARIES</t>
+        </is>
+      </c>
+      <c r="E215" s="72" t="inlineStr">
+        <is>
+          <t>Quest 1</t>
         </is>
       </c>
       <c r="F215" s="71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CHALCH_SUMMON</t>
         </is>
       </c>
       <c r="G215" s="71" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H215" s="72" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+          <t>CHALCH_Q2</t>
+        </is>
+      </c>
+      <c r="H215" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I215" s="70" t="inlineStr"/>
@@ -14572,66 +14591,62 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K215" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L215" s="70" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M215" s="73" t="inlineStr">
-        <is>
-          <t>15</t>
+      <c r="K215" s="72" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L215" s="70" t="inlineStr"/>
+      <c r="M215" s="72" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="N215" s="71" t="inlineStr">
         <is>
-          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
+          <t>Fires when chalch_summoned + 3+ farms; reward: +30 food</t>
         </is>
       </c>
     </row>
     <row r="216" ht="30" customHeight="1">
       <c r="A216" s="69" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Chalchiuhtotolin</t>
         </is>
       </c>
       <c r="B216" s="69" t="inlineStr">
         <is>
-          <t>Ualani Expansion</t>
+          <t>Jade Turkey Arc</t>
         </is>
       </c>
       <c r="C216" s="70" t="inlineStr">
         <is>
-          <t>UALANI_BARRACKS_01</t>
+          <t>CHALCH_Q2</t>
         </is>
       </c>
       <c r="D216" s="71" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E216" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>THE JADE TURKEY DEMANDS A STOCKPILE WORTHY OF ITS REGARD</t>
+        </is>
+      </c>
+      <c r="E216" s="72" t="inlineStr">
+        <is>
+          <t>Quest 2</t>
         </is>
       </c>
       <c r="F216" s="71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CHALCH_Q1</t>
         </is>
       </c>
       <c r="G216" s="71" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H216" s="72" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+          <t>CHALCH_Q3</t>
+        </is>
+      </c>
+      <c r="H216" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I216" s="70" t="inlineStr"/>
@@ -14640,66 +14655,62 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K216" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L216" s="70" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M216" s="73" t="inlineStr">
-        <is>
-          <t>15</t>
+      <c r="K216" s="72" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L216" s="70" t="inlineStr"/>
+      <c r="M216" s="72" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="N216" s="71" t="inlineStr">
         <is>
-          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
+          <t>Fires when chalch_q1_done + TotalFood &gt;= 150; reward: +50 food</t>
         </is>
       </c>
     </row>
     <row r="217" ht="30" customHeight="1">
       <c r="A217" s="69" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Chalchiuhtotolin</t>
         </is>
       </c>
       <c r="B217" s="69" t="inlineStr">
         <is>
-          <t>Ualani Expansion</t>
+          <t>Jade Turkey Arc</t>
         </is>
       </c>
       <c r="C217" s="70" t="inlineStr">
         <is>
-          <t>UALANI_COURTHOUSE_01</t>
+          <t>CHALCH_Q3</t>
         </is>
       </c>
       <c r="D217" s="71" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E217" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>THE JADE TURKEY DEMANDS A NATION OF FARMS</t>
+        </is>
+      </c>
+      <c r="E217" s="72" t="inlineStr">
+        <is>
+          <t>Quest 3</t>
         </is>
       </c>
       <c r="F217" s="71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CHALCH_Q2</t>
         </is>
       </c>
       <c r="G217" s="71" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H217" s="72" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+          <t>CHALCH_AGREE</t>
+        </is>
+      </c>
+      <c r="H217" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I217" s="70" t="inlineStr"/>
@@ -14708,56 +14719,52 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K217" s="26" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L217" s="70" t="inlineStr">
-        <is>
-          <t>explicit option</t>
-        </is>
-      </c>
-      <c r="M217" s="73" t="inlineStr">
-        <is>
-          <t>15</t>
+      <c r="K217" s="72" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L217" s="70" t="inlineStr"/>
+      <c r="M217" s="72" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="N217" s="71" t="inlineStr">
         <is>
-          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
+          <t>Fires when chalch_q2_done + 5+ farms; reward: +40 food</t>
         </is>
       </c>
     </row>
     <row r="218" ht="30" customHeight="1">
       <c r="A218" s="69" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Chalchiuhtotolin</t>
         </is>
       </c>
       <c r="B218" s="69" t="inlineStr">
         <is>
-          <t>More City Events</t>
+          <t>Jade Turkey Arc</t>
         </is>
       </c>
       <c r="C218" s="70" t="inlineStr">
         <is>
-          <t>CL_WASHINGTON_01</t>
+          <t>CHALCH_AGREE</t>
         </is>
       </c>
       <c r="D218" s="71" t="inlineStr">
         <is>
-          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
-        </is>
-      </c>
-      <c r="E218" s="5" t="inlineStr">
-        <is>
-          <t>Root</t>
+          <t>CHALCHIUHTOTOLIN ACCEPTS THE PACT — REPUBLIC EARNS TURKEY GOD'S PROTECTION</t>
+        </is>
+      </c>
+      <c r="E218" s="72" t="inlineStr">
+        <is>
+          <t>Resolution</t>
         </is>
       </c>
       <c r="F218" s="71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CHALCH_Q3</t>
         </is>
       </c>
       <c r="G218" s="71" t="inlineStr">
@@ -14765,9 +14772,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H218" s="72" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+      <c r="H218" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I218" s="70" t="inlineStr"/>
@@ -14776,444 +14783,796 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K218" s="73" t="inlineStr">
+      <c r="K218" s="72" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
       <c r="L218" s="70" t="inlineStr"/>
-      <c r="M218" s="73" t="inlineStr">
+      <c r="M218" s="72" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N218" s="71" t="inlineStr">
         <is>
+          <t>Fires when chalch_q3_done; BTN1: +100 food; closes the arc</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="8" customHeight="1">
+      <c r="A219" s="9" t="n"/>
+      <c r="B219" s="9" t="n"/>
+      <c r="C219" s="9" t="n"/>
+      <c r="D219" s="9" t="n"/>
+      <c r="E219" s="9" t="n"/>
+      <c r="F219" s="9" t="n"/>
+      <c r="G219" s="9" t="n"/>
+      <c r="H219" s="9" t="n"/>
+      <c r="I219" s="9" t="n"/>
+      <c r="J219" s="9" t="n"/>
+      <c r="K219" s="9" t="n"/>
+      <c r="L219" s="9" t="n"/>
+      <c r="M219" s="9" t="n"/>
+      <c r="N219" s="9" t="n"/>
+    </row>
+    <row r="220" ht="30" customHeight="1">
+      <c r="A220" s="73" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B220" s="73" t="inlineStr">
+        <is>
+          <t>Ualani Expansion</t>
+        </is>
+      </c>
+      <c r="C220" s="74" t="inlineStr">
+        <is>
+          <t>UALANI_DOCK_01</t>
+        </is>
+      </c>
+      <c r="D220" s="75" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE SURVEYS THE HARBOR AT [TILE_NAME]  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E220" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F220" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G220" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H220" s="76" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I220" s="74" t="inlineStr"/>
+      <c r="J220" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K220" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L220" s="74" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
+      <c r="M220" s="77" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N220" s="75" t="inlineStr">
+        <is>
+          <t>Ualani at tile with enabled Dock; follows UALANI_FORGE_01 pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="30" customHeight="1">
+      <c r="A221" s="73" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B221" s="73" t="inlineStr">
+        <is>
+          <t>Ualani Expansion</t>
+        </is>
+      </c>
+      <c r="C221" s="74" t="inlineStr">
+        <is>
+          <t>UALANI_FARM_01</t>
+        </is>
+      </c>
+      <c r="D221" s="75" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE VISITS THE FARMLANDS AT [TILE_NAME]  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E221" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F221" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G221" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H221" s="76" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I221" s="74" t="inlineStr"/>
+      <c r="J221" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K221" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L221" s="74" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
+      <c r="M221" s="77" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N221" s="75" t="inlineStr">
+        <is>
+          <t>Ualani at Farm tile; variant of HARVEST_VISIT_01 but Ualani-led</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="30" customHeight="1">
+      <c r="A222" s="73" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B222" s="73" t="inlineStr">
+        <is>
+          <t>Ualani Expansion</t>
+        </is>
+      </c>
+      <c r="C222" s="74" t="inlineStr">
+        <is>
+          <t>UALANI_BARRACKS_01</t>
+        </is>
+      </c>
+      <c r="D222" s="75" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE CONDUCTS REGIMENTAL REVIEW AT [TILE_NAME]  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E222" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F222" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G222" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H222" s="76" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I222" s="74" t="inlineStr"/>
+      <c r="J222" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K222" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L222" s="74" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
+      <c r="M222" s="77" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N222" s="75" t="inlineStr">
+        <is>
+          <t>Ualani at tile with Barracks; army strength / loyalty focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="30" customHeight="1">
+      <c r="A223" s="73" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B223" s="73" t="inlineStr">
+        <is>
+          <t>Ualani Expansion</t>
+        </is>
+      </c>
+      <c r="C223" s="74" t="inlineStr">
+        <is>
+          <t>UALANI_COURTHOUSE_01</t>
+        </is>
+      </c>
+      <c r="D223" s="75" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE HOLDS TOWN HALL AT [TILE_NAME]  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E223" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F223" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G223" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H223" s="76" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I223" s="74" t="inlineStr"/>
+      <c r="J223" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K223" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L223" s="74" t="inlineStr">
+        <is>
+          <t>explicit option</t>
+        </is>
+      </c>
+      <c r="M223" s="77" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N223" s="75" t="inlineStr">
+        <is>
+          <t>Ualani at Courthouse tile; complement to UALANI_DIGNITARY but different trigger (no moralDecay gate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="30" customHeight="1">
+      <c r="A224" s="73" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B224" s="73" t="inlineStr">
+        <is>
+          <t>More City Events</t>
+        </is>
+      </c>
+      <c r="C224" s="74" t="inlineStr">
+        <is>
+          <t>CL_WASHINGTON_01</t>
+        </is>
+      </c>
+      <c r="D224" s="75" t="inlineStr">
+        <is>
+          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
+        </is>
+      </c>
+      <c r="E224" s="5" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="F224" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G224" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H224" s="76" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I224" s="74" t="inlineStr"/>
+      <c r="J224" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K224" s="77" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L224" s="74" t="inlineStr"/>
+      <c r="M224" s="77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N224" s="75" t="inlineStr">
+        <is>
           <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
         </is>
       </c>
     </row>
-    <row r="219" ht="30" customHeight="1">
-      <c r="A219" s="69" t="inlineStr">
+    <row r="225" ht="30" customHeight="1">
+      <c r="A225" s="73" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B219" s="69" t="inlineStr">
+      <c r="B225" s="73" t="inlineStr">
         <is>
           <t>More City Events</t>
         </is>
       </c>
-      <c r="C219" s="70" t="inlineStr">
+      <c r="C225" s="74" t="inlineStr">
         <is>
           <t>CL_VALLEY_FORGE_01</t>
         </is>
       </c>
-      <c r="D219" s="71" t="inlineStr">
+      <c r="D225" s="75" t="inlineStr">
         <is>
           <t>VALLEY FORGE SECURED  ← IDEA</t>
         </is>
       </c>
-      <c r="E219" s="5" t="inlineStr">
+      <c r="E225" s="5" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="F219" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G219" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H219" s="72" t="inlineStr">
+      <c r="F225" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G225" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H225" s="76" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I219" s="70" t="inlineStr"/>
-      <c r="J219" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K219" s="73" t="inlineStr">
+      <c r="I225" s="74" t="inlineStr"/>
+      <c r="J225" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K225" s="77" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L219" s="70" t="inlineStr"/>
-      <c r="M219" s="73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N219" s="71" t="inlineStr">
+      <c r="L225" s="74" t="inlineStr"/>
+      <c r="M225" s="77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N225" s="75" t="inlineStr">
         <is>
           <t>Tile 1; historically significant; would fire on liberation</t>
         </is>
       </c>
     </row>
-    <row r="220" ht="30" customHeight="1">
-      <c r="A220" s="69" t="inlineStr">
+    <row r="226" ht="30" customHeight="1">
+      <c r="A226" s="73" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B220" s="69" t="inlineStr">
+      <c r="B226" s="73" t="inlineStr">
         <is>
           <t>More City Events</t>
         </is>
       </c>
-      <c r="C220" s="70" t="inlineStr">
+      <c r="C226" s="74" t="inlineStr">
         <is>
           <t>CX_NYC_01</t>
         </is>
       </c>
-      <c r="D220" s="71" t="inlineStr">
+      <c r="D226" s="75" t="inlineStr">
         <is>
           <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
         </is>
       </c>
-      <c r="E220" s="5" t="inlineStr">
+      <c r="E226" s="5" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="F220" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G220" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H220" s="72" t="inlineStr">
+      <c r="F226" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G226" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H226" s="76" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I220" s="70" t="inlineStr"/>
-      <c r="J220" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K220" s="73" t="inlineStr">
+      <c r="I226" s="74" t="inlineStr"/>
+      <c r="J226" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K226" s="77" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L220" s="70" t="inlineStr"/>
-      <c r="M220" s="73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N220" s="71" t="inlineStr">
+      <c r="L226" s="74" t="inlineStr"/>
+      <c r="M226" s="77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N226" s="75" t="inlineStr">
         <is>
           <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
         </is>
       </c>
     </row>
-    <row r="221" ht="30" customHeight="1">
-      <c r="A221" s="69" t="inlineStr">
+    <row r="227" ht="30" customHeight="1">
+      <c r="A227" s="73" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B221" s="69" t="inlineStr">
+      <c r="B227" s="73" t="inlineStr">
         <is>
           <t>Espionage Events</t>
         </is>
       </c>
-      <c r="C221" s="70" t="inlineStr">
+      <c r="C227" s="74" t="inlineStr">
         <is>
           <t>ESPIONAGE_DISCOVERY_01</t>
         </is>
       </c>
-      <c r="D221" s="71" t="inlineStr">
+      <c r="D227" s="75" t="inlineStr">
         <is>
           <t>SPY NETWORK DISCOVERED AT [TILE_NAME]  ← IDEA</t>
         </is>
       </c>
-      <c r="E221" s="5" t="inlineStr">
+      <c r="E227" s="5" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="F221" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G221" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H221" s="72" t="inlineStr">
+      <c r="F227" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G227" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H227" s="76" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I221" s="70" t="inlineStr"/>
-      <c r="J221" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K221" s="73" t="inlineStr">
+      <c r="I227" s="74" t="inlineStr"/>
+      <c r="J227" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K227" s="77" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L221" s="70" t="inlineStr"/>
-      <c r="M221" s="73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N221" s="71" t="inlineStr">
+      <c r="L227" s="74" t="inlineStr"/>
+      <c r="M227" s="77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N227" s="75" t="inlineStr">
         <is>
           <t>Would fire when espionageActive + enemy army arrives; uses existing espionage vars</t>
         </is>
       </c>
     </row>
-    <row r="222" ht="30" customHeight="1">
-      <c r="A222" s="69" t="inlineStr">
+    <row r="228" ht="30" customHeight="1">
+      <c r="A228" s="73" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B222" s="69" t="inlineStr">
+      <c r="B228" s="73" t="inlineStr">
         <is>
           <t>Commander Expansion</t>
         </is>
       </c>
-      <c r="C222" s="70" t="inlineStr">
+      <c r="C228" s="74" t="inlineStr">
         <is>
           <t>CMD_OBJECTIVE_2</t>
         </is>
       </c>
-      <c r="D222" s="71" t="inlineStr">
+      <c r="D228" s="75" t="inlineStr">
         <is>
           <t>A COMMANDER'S SECOND TASK  ← IDEA</t>
         </is>
       </c>
-      <c r="E222" s="22" t="inlineStr">
+      <c r="E228" s="22" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="F222" s="71" t="inlineStr">
+      <c r="F228" s="75" t="inlineStr">
         <is>
           <t>CMD_OBJECTIVE_1</t>
         </is>
       </c>
-      <c r="G222" s="71" t="inlineStr">
+      <c r="G228" s="75" t="inlineStr">
         <is>
           <t>→ CMD_OBJECTIVE_3?</t>
         </is>
       </c>
-      <c r="H222" s="72" t="inlineStr">
+      <c r="H228" s="76" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I222" s="70" t="inlineStr"/>
-      <c r="J222" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K222" s="73" t="inlineStr">
+      <c r="I228" s="74" t="inlineStr"/>
+      <c r="J228" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K228" s="77" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L222" s="70" t="inlineStr"/>
-      <c r="M222" s="73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N222" s="71" t="inlineStr">
+      <c r="L228" s="74" t="inlineStr"/>
+      <c r="M228" s="77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N228" s="75" t="inlineStr">
         <is>
           <t>Extend the commander arc beyond first objective</t>
         </is>
       </c>
     </row>
-    <row r="223" ht="30" customHeight="1">
-      <c r="A223" s="69" t="inlineStr">
+    <row r="229" ht="30" customHeight="1">
+      <c r="A229" s="73" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B223" s="69" t="inlineStr">
+      <c r="B229" s="73" t="inlineStr">
         <is>
           <t>Seasonal Events</t>
         </is>
       </c>
-      <c r="C223" s="70" t="inlineStr">
+      <c r="C229" s="74" t="inlineStr">
         <is>
           <t>WINTER_SIEGE_01</t>
         </is>
       </c>
-      <c r="D223" s="71" t="inlineStr">
+      <c r="D229" s="75" t="inlineStr">
         <is>
           <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
         </is>
       </c>
-      <c r="E223" s="5" t="inlineStr">
+      <c r="E229" s="5" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="F223" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G223" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H223" s="72" t="inlineStr">
+      <c r="F229" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G229" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H229" s="76" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I223" s="70" t="inlineStr"/>
-      <c r="J223" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K223" s="73" t="inlineStr">
+      <c r="I229" s="74" t="inlineStr"/>
+      <c r="J229" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K229" s="77" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L223" s="70" t="inlineStr"/>
-      <c r="M223" s="73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N223" s="71" t="inlineStr">
+      <c r="L229" s="74" t="inlineStr"/>
+      <c r="M229" s="77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N229" s="75" t="inlineStr">
         <is>
           <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
         </is>
       </c>
     </row>
-    <row r="224" ht="30" customHeight="1">
-      <c r="A224" s="69" t="inlineStr">
+    <row r="230" ht="30" customHeight="1">
+      <c r="A230" s="73" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B224" s="69" t="inlineStr">
+      <c r="B230" s="73" t="inlineStr">
         <is>
           <t>Seasonal Events</t>
         </is>
       </c>
-      <c r="C224" s="70" t="inlineStr">
+      <c r="C230" s="74" t="inlineStr">
         <is>
           <t>SPRING_OFFENSIVE_01</t>
         </is>
       </c>
-      <c r="D224" s="71" t="inlineStr">
+      <c r="D230" s="75" t="inlineStr">
         <is>
           <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
         </is>
       </c>
-      <c r="E224" s="5" t="inlineStr">
+      <c r="E230" s="5" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="F224" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G224" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H224" s="72" t="inlineStr">
+      <c r="F230" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G230" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H230" s="76" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I224" s="70" t="inlineStr"/>
-      <c r="J224" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K224" s="73" t="inlineStr">
+      <c r="I230" s="74" t="inlineStr"/>
+      <c r="J230" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K230" s="77" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L224" s="70" t="inlineStr"/>
-      <c r="M224" s="73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N224" s="71" t="inlineStr">
+      <c r="L230" s="74" t="inlineStr"/>
+      <c r="M230" s="77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N230" s="75" t="inlineStr">
         <is>
           <t>Month 3-4; UK neighbor + player army present; tactical pressure event</t>
         </is>
       </c>
     </row>
-    <row r="226" ht="20" customHeight="1">
-      <c r="A226" s="74" t="inlineStr">
+    <row r="232" ht="20" customHeight="1">
+      <c r="A232" s="78" t="inlineStr">
         <is>
           <t>Total events in spreadsheet</t>
         </is>
       </c>
-      <c r="B226" s="75" t="n">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="227" ht="20" customHeight="1">
-      <c r="A227" s="74" t="inlineStr">
+      <c r="B232" s="79" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="233" ht="20" customHeight="1">
+      <c r="A233" s="78" t="inlineStr">
         <is>
           <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
-      <c r="B227" s="75" t="n">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="228" ht="20" customHeight="1">
-      <c r="A228" s="74" t="inlineStr">
+      <c r="B233" s="79" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="234" ht="20" customHeight="1">
+      <c r="A234" s="78" t="inlineStr">
         <is>
           <t>IDEA (not yet implemented)</t>
         </is>
       </c>
-      <c r="B228" s="75" t="n">
+      <c r="B234" s="79" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="229" ht="20" customHeight="1">
-      <c r="A229" s="74" t="inlineStr">
+    <row r="235" ht="20" customHeight="1">
+      <c r="A235" s="78" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B229" s="75" t="n">
+      <c r="B235" s="79" t="n">
         <v>55</v>
       </c>
     </row>
@@ -17888,42 +18247,42 @@
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="74" t="inlineStr">
+      <c r="A43" s="78" t="inlineStr">
         <is>
           <t>Canadian events total</t>
         </is>
       </c>
-      <c r="B43" s="75" t="n">
+      <c r="B43" s="79" t="n">
         <v>38</v>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="74" t="inlineStr">
+      <c r="A44" s="78" t="inlineStr">
         <is>
           <t>Canada (Alliance arc)</t>
         </is>
       </c>
-      <c r="B44" s="75" t="n">
+      <c r="B44" s="79" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="74" t="inlineStr">
+      <c r="A45" s="78" t="inlineStr">
         <is>
           <t>CA Protector (Jessica's creatures)</t>
         </is>
       </c>
-      <c r="B45" s="75" t="n">
+      <c r="B45" s="79" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="74" t="inlineStr">
+      <c r="A46" s="78" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B46" s="75" t="n">
+      <c r="B46" s="79" t="n">
         <v>12</v>
       </c>
     </row>
@@ -17938,7 +18297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17947,390 +18306,403 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="76" t="inlineStr">
+      <c r="A1" s="80" t="inlineStr">
         <is>
           <t>STATUS LEGEND</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="77" t="inlineStr">
+      <c r="A2" s="81" t="inlineStr">
         <is>
           <t>FULL COMPLETION</t>
         </is>
       </c>
-      <c r="B2" s="78" t="inlineStr">
+      <c r="B2" s="82" t="inlineStr">
         <is>
           <t>Final pass done — art integrated, text finalized, fully tested</t>
         </is>
       </c>
-      <c r="C2" s="78" t="n"/>
+      <c r="C2" s="82" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="79" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="B3" s="80" t="inlineStr">
+      <c r="A3" s="83" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="B3" s="84" t="inlineStr">
         <is>
           <t>Event is coded, in CSV, all buttons wired; no final polish yet</t>
         </is>
       </c>
-      <c r="C3" s="80" t="n"/>
+      <c r="C3" s="84" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="81" t="inlineStr">
+      <c r="A4" s="85" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="B4" s="82" t="inlineStr">
+      <c r="B4" s="86" t="inlineStr">
         <is>
           <t>Concept stage: not in events.csv; some referenced in button CSV</t>
         </is>
       </c>
-      <c r="C4" s="82" t="n"/>
+      <c r="C4" s="86" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="76" t="inlineStr">
+      <c r="A6" s="80" t="inlineStr">
         <is>
           <t>ART STATUS LEGEND</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="83" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="B7" s="84" t="inlineStr">
+      <c r="A7" s="87" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="B7" s="88" t="inlineStr">
         <is>
           <t>No art asset exists yet</t>
         </is>
       </c>
-      <c r="C7" s="84" t="n"/>
+      <c r="C7" s="88" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="81" t="inlineStr">
+      <c r="A8" s="85" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="B8" s="82" t="inlineStr">
+      <c r="B8" s="86" t="inlineStr">
         <is>
           <t>Art is being created but not in engine</t>
         </is>
       </c>
-      <c r="C8" s="82" t="n"/>
+      <c r="C8" s="86" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="85" t="inlineStr">
+      <c r="A9" s="89" t="inlineStr">
         <is>
           <t>Integrated</t>
         </is>
       </c>
-      <c r="B9" s="86" t="inlineStr">
+      <c r="B9" s="90" t="inlineStr">
         <is>
           <t>Art is in the project and referenced correctly</t>
         </is>
       </c>
-      <c r="C9" s="86" t="n"/>
+      <c r="C9" s="90" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="76" t="inlineStr">
+      <c r="A11" s="80" t="inlineStr">
         <is>
           <t>EXPLICIT ART LEGEND</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="87" t="inlineStr">
+      <c r="A12" s="91" t="inlineStr">
         <is>
           <t>YES — Explicit Art Needed</t>
         </is>
       </c>
-      <c r="B12" s="88" t="inlineStr">
+      <c r="B12" s="92" t="inlineStr">
         <is>
           <t>Event has explicit or kinky_lewd content flag OR has at least one explicit button option that will need unique explicit artwork</t>
         </is>
       </c>
-      <c r="C12" s="88" t="n"/>
+      <c r="C12" s="92" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="89" t="inlineStr">
+      <c r="A13" s="93" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B13" s="90" t="inlineStr">
+      <c r="B13" s="94" t="inlineStr">
         <is>
           <t>Standard event — no adult artwork required</t>
         </is>
       </c>
-      <c r="C13" s="90" t="n"/>
+      <c r="C13" s="94" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="76" t="inlineStr">
+      <c r="A15" s="80" t="inlineStr">
         <is>
           <t>CHAIN POSITION LEGEND</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="91" t="inlineStr">
+      <c r="A16" s="95" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="B16" s="92" t="inlineStr">
+      <c r="B16" s="96" t="inlineStr">
         <is>
           <t>Standalone event or first event in a chain; fires from world.gd check function or EventDatabase date trigger</t>
         </is>
       </c>
-      <c r="C16" s="92" t="n"/>
+      <c r="C16" s="96" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="93" t="inlineStr">
+      <c r="A17" s="97" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="B17" s="94" t="inlineStr">
+      <c r="B17" s="98" t="inlineStr">
         <is>
           <t>Fires as outcome of a choice button on a Root/prior event; represents one path in a fork</t>
         </is>
       </c>
-      <c r="C17" s="94" t="n"/>
+      <c r="C17" s="98" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="95" t="inlineStr">
+      <c r="A18" s="99" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="B18" s="96" t="inlineStr">
+      <c r="B18" s="100" t="inlineStr">
         <is>
           <t>Fires automatically after a mission completes (via next_event_id or mission flag return)</t>
         </is>
       </c>
-      <c r="C18" s="96" t="n"/>
+      <c r="C18" s="100" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="76" t="inlineStr">
+      <c r="A20" s="80" t="inlineStr">
         <is>
           <t>CATEGORY COLOR LEGEND</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="97" t="inlineStr">
+      <c r="A21" s="101" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B21" s="98" t="inlineStr">
+      <c r="B21" s="102" t="inlineStr">
         <is>
           <t>Calendar-triggered events; month or turn-based</t>
         </is>
       </c>
-      <c r="C21" s="98" t="n"/>
+      <c r="C21" s="102" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="99" t="inlineStr">
+      <c r="A22" s="103" t="inlineStr">
         <is>
           <t>City Liberated</t>
         </is>
       </c>
-      <c r="B22" s="100" t="inlineStr">
+      <c r="B22" s="104" t="inlineStr">
         <is>
           <t>Fires when a specific tile is liberated (city_liberated type)</t>
         </is>
       </c>
-      <c r="C22" s="100" t="n"/>
+      <c r="C22" s="104" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="101" t="inlineStr">
+      <c r="A23" s="105" t="inlineStr">
         <is>
           <t>City Lost</t>
         </is>
       </c>
-      <c r="B23" s="102" t="inlineStr">
+      <c r="B23" s="106" t="inlineStr">
         <is>
           <t>Fires when a specific tile falls to the enemy (city_lost type)</t>
         </is>
       </c>
-      <c r="C23" s="102" t="n"/>
+      <c r="C23" s="106" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="103" t="inlineStr">
+      <c r="A24" s="107" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B24" s="104" t="inlineStr">
+      <c r="B24" s="108" t="inlineStr">
         <is>
           <t>State-level liberation, secession, and reintegration</t>
         </is>
       </c>
-      <c r="C24" s="104" t="n"/>
+      <c r="C24" s="108" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="105" t="inlineStr">
+      <c r="A25" s="109" t="inlineStr">
         <is>
           <t>Protector</t>
         </is>
       </c>
-      <c r="B25" s="106" t="inlineStr">
+      <c r="B25" s="110" t="inlineStr">
         <is>
           <t>Mythological entity summon events (protector_summon type)</t>
         </is>
       </c>
-      <c r="C25" s="106" t="n"/>
+      <c r="C25" s="110" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="107" t="inlineStr">
+      <c r="A26" s="111" t="inlineStr">
         <is>
           <t>Commander</t>
         </is>
       </c>
-      <c r="B26" s="108" t="inlineStr">
+      <c r="B26" s="112" t="inlineStr">
         <is>
           <t>Named commander arc events (commander_* types)</t>
         </is>
       </c>
-      <c r="C26" s="108" t="n"/>
+      <c r="C26" s="112" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="109" t="inlineStr">
+      <c r="A27" s="113" t="inlineStr">
         <is>
           <t>Fort Chain</t>
         </is>
       </c>
-      <c r="B27" s="110" t="inlineStr">
+      <c r="B27" s="114" t="inlineStr">
         <is>
           <t>Fort disrepair investigation chain (fort_* types)</t>
         </is>
       </c>
-      <c r="C27" s="110" t="n"/>
+      <c r="C27" s="114" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="111" t="inlineStr">
+      <c r="A28" s="115" t="inlineStr">
         <is>
           <t>Collapse</t>
         </is>
       </c>
-      <c r="B28" s="112" t="inlineStr">
+      <c r="B28" s="116" t="inlineStr">
         <is>
           <t>Republic collapse sequence</t>
         </is>
       </c>
-      <c r="C28" s="112" t="n"/>
+      <c r="C28" s="116" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="113" t="inlineStr">
+      <c r="A29" s="117" t="inlineStr">
         <is>
           <t>Tile Crisis</t>
         </is>
       </c>
-      <c r="B29" s="114" t="inlineStr">
+      <c r="B29" s="118" t="inlineStr">
         <is>
           <t>Dynamic tile-based crisis chains; triggered by world.gd check functions</t>
         </is>
       </c>
-      <c r="C29" s="114" t="n"/>
+      <c r="C29" s="118" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="115" t="inlineStr">
+      <c r="A30" s="119" t="inlineStr">
         <is>
           <t>Ualani</t>
         </is>
       </c>
-      <c r="B30" s="116" t="inlineStr">
+      <c r="B30" s="120" t="inlineStr">
         <is>
           <t>Ualani Carlisle army presence events; personal storyline</t>
         </is>
       </c>
-      <c r="C30" s="116" t="n"/>
+      <c r="C30" s="120" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="117" t="inlineStr">
+      <c r="A31" s="121" t="inlineStr">
         <is>
           <t>VP Arc</t>
         </is>
       </c>
-      <c r="B31" s="118" t="inlineStr">
+      <c r="B31" s="122" t="inlineStr">
         <is>
           <t>Vice President relationship arc; 9 events tied to the VP governor</t>
         </is>
       </c>
-      <c r="C31" s="118" t="n"/>
+      <c r="C31" s="122" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="119" t="inlineStr">
+      <c r="A32" s="123" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="B32" s="120" t="inlineStr">
+      <c r="B32" s="124" t="inlineStr">
         <is>
           <t>Canadian Alliance diplomatic arc + 3 peace events (PEACE_ALLIED_01, PEACE_USA_01, PEACE_CA_AI_01)</t>
         </is>
       </c>
-      <c r="C32" s="120" t="n"/>
+      <c r="C32" s="124" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="121" t="inlineStr">
+      <c r="A33" s="125" t="inlineStr">
         <is>
           <t>CA Protector</t>
         </is>
       </c>
-      <c r="B33" s="122" t="inlineStr">
+      <c r="B33" s="126" t="inlineStr">
         <is>
           <t>Jessica Clear-Water's 8 creature arcs; Algonquin, Mi'kmaq, French-Canadian folklore</t>
         </is>
       </c>
-      <c r="C33" s="122" t="n"/>
+      <c r="C33" s="126" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="123" t="inlineStr">
+      <c r="A34" s="127" t="inlineStr">
         <is>
           <t>Loyal Governor</t>
         </is>
       </c>
-      <c r="B34" s="124" t="inlineStr">
+      <c r="B34" s="128" t="inlineStr">
         <is>
           <t>25 one-shot dispatch events, one per USA governor archetype; tile_yield resource×turns; 3% chance/turn at loyalty≥8</t>
         </is>
       </c>
-      <c r="C34" s="124" t="n"/>
+      <c r="C34" s="128" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="125" t="inlineStr">
+      <c r="A35" s="129" t="inlineStr">
         <is>
           <t>White House</t>
         </is>
       </c>
-      <c r="B35" s="126" t="inlineStr">
+      <c r="B35" s="130" t="inlineStr">
         <is>
           <t>12 personal Ualani events (WH_SECRET_01–12); fires when she is stationed at DC (tile 188) during the matching calendar month; all sensual in tone; some have explicit BTN2</t>
         </is>
       </c>
-      <c r="C35" s="126" t="n"/>
+      <c r="C35" s="130" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="127" t="inlineStr">
+      <c r="A36" s="131" t="inlineStr">
+        <is>
+          <t>Chalchiuhtotolin</t>
+        </is>
+      </c>
+      <c r="B36" s="132" t="inlineStr">
+        <is>
+          <t>5-event super-secret arc (CHALCH_SUMMON → Q1 → Q2 → Q3 → AGREE); fires only when Ualani is at Plymouth (tile 66) on Thanksgiving (month 11); quests: 3 farms, 150 food, 5 farms; reward: up to +220 food total</t>
+        </is>
+      </c>
+      <c r="C36" s="132" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="133" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B36" s="128" t="inlineStr">
+      <c r="B37" s="134" t="inlineStr">
         <is>
           <t>Not yet implemented; concept stage or referenced-but-missing events</t>
         </is>
       </c>
-      <c r="C36" s="128" t="n"/>
+      <c r="C37" s="134" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Rename Mark Penoit → Marc Penoit throughout
More authentic Québécois spelling. Swept all .gd, .py, .csv files
including all-caps event headlines.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -11340,7 +11340,7 @@
       </c>
       <c r="N163" s="59" t="inlineStr">
         <is>
-          <t>Sets ca_prot_07_agreed; BTN2 sensual — Mark Penoit on the river</t>
+          <t>Sets ca_prot_07_agreed; BTN2 sensual — Marc Penoit on the river</t>
         </is>
       </c>
     </row>
@@ -20970,7 +20970,7 @@
       </c>
       <c r="N33" s="59" t="inlineStr">
         <is>
-          <t>Sets ca_prot_07_agreed; BTN2 sensual — Mark Penoit on the river</t>
+          <t>Sets ca_prot_07_agreed; BTN2 sensual — Marc Penoit on the river</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CAN_ALLIANCE_SIGNED: polish event text, set art tag, update masterdoc notes
Full rewrite of ceremony text — three-beat structure: the signing with pauses,
the addendum surprise (Penoit's secret two-week draft, Jessica's matching one,
Ualani's 'I did not bring an addendum'), and the pivot line 'the three principals
remain in the treaty room.' Sets image_tag to can_alliance_signed_scene for art
integration. Status stays FIRST PASS pending art; notes updated with panel spec.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -9765,7 +9765,11 @@
           <t>FIRST PASS</t>
         </is>
       </c>
-      <c r="I139" s="54" t="inlineStr"/>
+      <c r="I139" s="54" t="inlineStr">
+        <is>
+          <t>can_alliance_signed_scene</t>
+        </is>
+      </c>
       <c r="J139" s="7" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -9788,7 +9792,7 @@
       </c>
       <c r="N139" s="55" t="inlineStr">
         <is>
-          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome</t>
+          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome. Text polished: ceremony + addendum comedy + 'principals remain in the treaty room' pivot. Art commissioned (120x120 pixel, 4 panels: ceremony/addendum/private room/explicit). Awaiting art integration for FULL COMPLETION.</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19399,11 @@
           <t>FIRST PASS</t>
         </is>
       </c>
-      <c r="I9" s="54" t="inlineStr"/>
+      <c r="I9" s="54" t="inlineStr">
+        <is>
+          <t>can_alliance_signed_scene</t>
+        </is>
+      </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -19418,7 +19426,7 @@
       </c>
       <c r="N9" s="55" t="inlineStr">
         <is>
-          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome</t>
+          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome. Text polished: ceremony + addendum comedy + 'principals remain in the treaty room' pivot. Art commissioned (120x120 pixel, 4 panels: ceremony/addendum/private room/explicit). Awaiting art integration for FULL COMPLETION.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Write CAN_ALLIANCE_SIGNED full event text: Lake Erie ceremony + aftermath
Rewrites long_desc to tell the complete story in two movements:

Movement 1 (ceremony): Lake Erie shore at sundown, Penoit's choice of
venue, the signing with its pauses, the three-way addendum comedy,
London notified for the fifth time in eighteen months.

Movement 2 (aftermath): Cameras clear. Jessica folds her fatigues.
Ualani sets the tricorne on the table. Marc smokes and watches the
light. He borrows the hat and walks to the beach. Ualani and Jessica
alone — history's first female equivalent of the Big Three, no words
needed. Marc's silhouette at the waterline gets the perfect shot as
the light goes down.

Tone updated to Triumphant/Intimate.
Masterdoc note updated to reflect the Lake Erie structure.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -9792,7 +9792,7 @@
       </c>
       <c r="N139" s="55" t="inlineStr">
         <is>
-          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome. Text polished: ceremony + addendum comedy + 'principals remain in the treaty room' pivot. Art commissioned (120x120 pixel, 4 panels: ceremony/addendum/private room/explicit). Awaiting art integration for FULL COMPLETION.</t>
+          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome. Text polished: Lake Erie at sundown — ceremony + addendum comedy — cameras clear — Marc borrows tricorne and walks to the beach — Ualani + Jessica alone at the table — Marc's silhouette gets the perfect shot. Awaiting art integration for FULL COMPLETION.</t>
         </is>
       </c>
     </row>
@@ -19426,7 +19426,7 @@
       </c>
       <c r="N9" s="55" t="inlineStr">
         <is>
-          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome. Text polished: ceremony + addendum comedy + 'principals remain in the treaty room' pivot. Art commissioned (120x120 pixel, 4 panels: ceremony/addendum/private room/explicit). Awaiting art integration for FULL COMPLETION.</t>
+          <t>EXPLICIT #2 (all three); fires after can_summit_complete; form_alliance CA outcome. Text polished: Lake Erie at sundown — ceremony + addendum comedy — cameras clear — Marc borrows tricorne and walks to the beach — Ualani + Jessica alone at the table — Marc's silhouette gets the perfect shot. Awaiting art integration for FULL COMPLETION.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 53 _INTIMATE stub events + masterdoc entries for all explicit events
- data/events.csv: 53 new _INTIMATE rows (one per explicit/sensual event)
- data/event_buttons.csv: 53 matching Continue buttons
- scripts/build_event_masterdoc.py: INTIMATE VARIANTS section with all 53
  stubs plus the already-authored CAN_ALLIANCE_SIGNED_INTIMATE
- event_masterdoc.xlsx: regenerated (314 events total; 64 IDEA, 250 FIRST PASS)

All stubs are IDEA status. When an event becomes an EtherTask the intimate
path now appears in the task card. Author each by replacing long_desc and
setting status to FIRST PASS.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -1129,7 +1129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N287"/>
+  <dimension ref="A1:N350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18828,43 +18828,3595 @@
         </is>
       </c>
     </row>
-    <row r="284" ht="20" customHeight="1">
-      <c r="A284" s="79" t="inlineStr">
+    <row r="283" ht="8" customHeight="1">
+      <c r="A283" s="9" t="n"/>
+      <c r="B283" s="9" t="n"/>
+      <c r="C283" s="9" t="n"/>
+      <c r="D283" s="9" t="n"/>
+      <c r="E283" s="9" t="n"/>
+      <c r="F283" s="9" t="n"/>
+      <c r="G283" s="9" t="n"/>
+      <c r="H283" s="9" t="n"/>
+      <c r="I283" s="9" t="n"/>
+      <c r="J283" s="9" t="n"/>
+      <c r="K283" s="9" t="n"/>
+      <c r="L283" s="9" t="n"/>
+      <c r="M283" s="9" t="n"/>
+      <c r="N283" s="9" t="n"/>
+    </row>
+    <row r="284" ht="30" customHeight="1">
+      <c r="A284" s="74" t="inlineStr">
+        <is>
+          <t>Commander</t>
+        </is>
+      </c>
+      <c r="B284" s="74" t="inlineStr">
+        <is>
+          <t>Commander Arc</t>
+        </is>
+      </c>
+      <c r="C284" s="75" t="inlineStr">
+        <is>
+          <t>CMD_THANKS_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D284" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE DELIVERS PERSONAL THANKS TO [COMM... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E284" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F284" s="76" t="inlineStr">
+        <is>
+          <t>CMD_THANKS (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G284" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H284" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I284" s="75" t="inlineStr"/>
+      <c r="J284" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K284" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L284" s="75" t="inlineStr"/>
+      <c r="M284" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N284" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CMD_THANKS. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="8" customHeight="1">
+      <c r="A285" s="9" t="n"/>
+      <c r="B285" s="9" t="n"/>
+      <c r="C285" s="9" t="n"/>
+      <c r="D285" s="9" t="n"/>
+      <c r="E285" s="9" t="n"/>
+      <c r="F285" s="9" t="n"/>
+      <c r="G285" s="9" t="n"/>
+      <c r="H285" s="9" t="n"/>
+      <c r="I285" s="9" t="n"/>
+      <c r="J285" s="9" t="n"/>
+      <c r="K285" s="9" t="n"/>
+      <c r="L285" s="9" t="n"/>
+      <c r="M285" s="9" t="n"/>
+      <c r="N285" s="9" t="n"/>
+    </row>
+    <row r="286" ht="30" customHeight="1">
+      <c r="A286" s="74" t="inlineStr">
+        <is>
+          <t>Fort Chain</t>
+        </is>
+      </c>
+      <c r="B286" s="74" t="inlineStr">
+        <is>
+          <t>Fort Disrepair</t>
+        </is>
+      </c>
+      <c r="C286" s="75" t="inlineStr">
+        <is>
+          <t>FORT_005_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D286" s="76" t="inlineStr">
+        <is>
+          <t>CLASSIFIED DIPLOMATIC PROCEEDINGS AT [TILE_NAME] — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E286" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F286" s="76" t="inlineStr">
+        <is>
+          <t>FORT_005 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G286" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H286" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I286" s="75" t="inlineStr"/>
+      <c r="J286" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K286" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L286" s="75" t="inlineStr"/>
+      <c r="M286" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N286" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of FORT_005. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287" ht="8" customHeight="1">
+      <c r="A287" s="9" t="n"/>
+      <c r="B287" s="9" t="n"/>
+      <c r="C287" s="9" t="n"/>
+      <c r="D287" s="9" t="n"/>
+      <c r="E287" s="9" t="n"/>
+      <c r="F287" s="9" t="n"/>
+      <c r="G287" s="9" t="n"/>
+      <c r="H287" s="9" t="n"/>
+      <c r="I287" s="9" t="n"/>
+      <c r="J287" s="9" t="n"/>
+      <c r="K287" s="9" t="n"/>
+      <c r="L287" s="9" t="n"/>
+      <c r="M287" s="9" t="n"/>
+      <c r="N287" s="9" t="n"/>
+    </row>
+    <row r="288" ht="30" customHeight="1">
+      <c r="A288" s="74" t="inlineStr">
+        <is>
+          <t>Collapse</t>
+        </is>
+      </c>
+      <c r="B288" s="74" t="inlineStr">
+        <is>
+          <t>Republic Falls</t>
+        </is>
+      </c>
+      <c r="C288" s="75" t="inlineStr">
+        <is>
+          <t>COLLAPSE_02_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D288" s="76" t="inlineStr">
+        <is>
+          <t>WASHINGTON STANDS ALONE — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E288" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F288" s="76" t="inlineStr">
+        <is>
+          <t>COLLAPSE_02 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G288" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H288" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I288" s="75" t="inlineStr"/>
+      <c r="J288" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K288" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L288" s="75" t="inlineStr"/>
+      <c r="M288" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N288" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of COLLAPSE_02. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="289" ht="8" customHeight="1">
+      <c r="A289" s="9" t="n"/>
+      <c r="B289" s="9" t="n"/>
+      <c r="C289" s="9" t="n"/>
+      <c r="D289" s="9" t="n"/>
+      <c r="E289" s="9" t="n"/>
+      <c r="F289" s="9" t="n"/>
+      <c r="G289" s="9" t="n"/>
+      <c r="H289" s="9" t="n"/>
+      <c r="I289" s="9" t="n"/>
+      <c r="J289" s="9" t="n"/>
+      <c r="K289" s="9" t="n"/>
+      <c r="L289" s="9" t="n"/>
+      <c r="M289" s="9" t="n"/>
+      <c r="N289" s="9" t="n"/>
+    </row>
+    <row r="290" ht="30" customHeight="1">
+      <c r="A290" s="74" t="inlineStr">
+        <is>
+          <t>Tile Crisis</t>
+        </is>
+      </c>
+      <c r="B290" s="74" t="inlineStr">
+        <is>
+          <t>Harvest Crisis</t>
+        </is>
+      </c>
+      <c r="C290" s="75" t="inlineStr">
+        <is>
+          <t>HARVEST_VISIT_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D290" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE SAVES THE HARVEST — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E290" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F290" s="76" t="inlineStr">
+        <is>
+          <t>HARVEST_VISIT_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G290" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H290" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I290" s="75" t="inlineStr"/>
+      <c r="J290" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K290" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L290" s="75" t="inlineStr"/>
+      <c r="M290" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N290" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of HARVEST_VISIT_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="30" customHeight="1">
+      <c r="A291" s="74" t="inlineStr">
+        <is>
+          <t>Tile Crisis</t>
+        </is>
+      </c>
+      <c r="B291" s="74" t="inlineStr">
+        <is>
+          <t>Election Arc</t>
+        </is>
+      </c>
+      <c r="C291" s="75" t="inlineStr">
+        <is>
+          <t>STUMP_SPEECH_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D291" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE TAKES THE FLOOR AT [TILE_NAME] — ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E291" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F291" s="76" t="inlineStr">
+        <is>
+          <t>STUMP_SPEECH_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G291" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H291" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I291" s="75" t="inlineStr"/>
+      <c r="J291" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K291" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L291" s="75" t="inlineStr"/>
+      <c r="M291" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N291" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of STUMP_SPEECH_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="8" customHeight="1">
+      <c r="A292" s="9" t="n"/>
+      <c r="B292" s="9" t="n"/>
+      <c r="C292" s="9" t="n"/>
+      <c r="D292" s="9" t="n"/>
+      <c r="E292" s="9" t="n"/>
+      <c r="F292" s="9" t="n"/>
+      <c r="G292" s="9" t="n"/>
+      <c r="H292" s="9" t="n"/>
+      <c r="I292" s="9" t="n"/>
+      <c r="J292" s="9" t="n"/>
+      <c r="K292" s="9" t="n"/>
+      <c r="L292" s="9" t="n"/>
+      <c r="M292" s="9" t="n"/>
+      <c r="N292" s="9" t="n"/>
+    </row>
+    <row r="293" ht="30" customHeight="1">
+      <c r="A293" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="B293" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="C293" s="75" t="inlineStr">
+        <is>
+          <t>VP_DOUBT_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D293" s="76" t="inlineStr">
+        <is>
+          <t>THE VICE PRESIDENT AT 2 A.M.: [COMMANDER_NAME] IS QU... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E293" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F293" s="76" t="inlineStr">
+        <is>
+          <t>VP_DOUBT (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G293" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H293" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I293" s="75" t="inlineStr"/>
+      <c r="J293" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K293" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L293" s="75" t="inlineStr"/>
+      <c r="M293" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N293" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of VP_DOUBT. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="30" customHeight="1">
+      <c r="A294" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="B294" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="C294" s="75" t="inlineStr">
+        <is>
+          <t>VP_BATTLEFIELD_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D294" s="76" t="inlineStr">
+        <is>
+          <t>THE VICE PRESIDENT PICKS UP A MUSKET: [COMMANDER_NAM... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E294" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F294" s="76" t="inlineStr">
+        <is>
+          <t>VP_BATTLEFIELD (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G294" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H294" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I294" s="75" t="inlineStr"/>
+      <c r="J294" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K294" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L294" s="75" t="inlineStr"/>
+      <c r="M294" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N294" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of VP_BATTLEFIELD. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="30" customHeight="1">
+      <c r="A295" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="B295" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="C295" s="75" t="inlineStr">
+        <is>
+          <t>VP_PRE_ELECTION_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D295" s="76" t="inlineStr">
+        <is>
+          <t>THE VICE PRESIDENT CALLS AN UNSCHEDULED MEETING — [C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E295" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F295" s="76" t="inlineStr">
+        <is>
+          <t>VP_PRE_ELECTION (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G295" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H295" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I295" s="75" t="inlineStr"/>
+      <c r="J295" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K295" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L295" s="75" t="inlineStr"/>
+      <c r="M295" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N295" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of VP_PRE_ELECTION. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="30" customHeight="1">
+      <c r="A296" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="B296" s="74" t="inlineStr">
+        <is>
+          <t>VP Arc</t>
+        </is>
+      </c>
+      <c r="C296" s="75" t="inlineStr">
+        <is>
+          <t>VP_LEGACY_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D296" s="76" t="inlineStr">
+        <is>
+          <t>THE VICE PRESIDENT LEAVES A NOTE — [COMMANDER_NAME] ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E296" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F296" s="76" t="inlineStr">
+        <is>
+          <t>VP_LEGACY (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G296" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H296" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I296" s="75" t="inlineStr"/>
+      <c r="J296" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K296" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L296" s="75" t="inlineStr"/>
+      <c r="M296" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N296" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of VP_LEGACY. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297" ht="8" customHeight="1">
+      <c r="A297" s="9" t="n"/>
+      <c r="B297" s="9" t="n"/>
+      <c r="C297" s="9" t="n"/>
+      <c r="D297" s="9" t="n"/>
+      <c r="E297" s="9" t="n"/>
+      <c r="F297" s="9" t="n"/>
+      <c r="G297" s="9" t="n"/>
+      <c r="H297" s="9" t="n"/>
+      <c r="I297" s="9" t="n"/>
+      <c r="J297" s="9" t="n"/>
+      <c r="K297" s="9" t="n"/>
+      <c r="L297" s="9" t="n"/>
+      <c r="M297" s="9" t="n"/>
+      <c r="N297" s="9" t="n"/>
+    </row>
+    <row r="298" ht="30" customHeight="1">
+      <c r="A298" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B298" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C298" s="75" t="inlineStr">
+        <is>
+          <t>CAN_CLEARWATER_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D298" s="76" t="inlineStr">
+        <is>
+          <t>PM CLEAR-WATER'S PRIVATE CHANNEL: JESSICA WRITES OUT... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E298" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F298" s="76" t="inlineStr">
+        <is>
+          <t>CAN_CLEARWATER_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G298" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H298" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I298" s="75" t="inlineStr"/>
+      <c r="J298" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K298" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L298" s="75" t="inlineStr"/>
+      <c r="M298" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N298" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_CLEARWATER_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="30" customHeight="1">
+      <c r="A299" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B299" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C299" s="75" t="inlineStr">
+        <is>
+          <t>CAN_JOINT_OPS_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D299" s="76" t="inlineStr">
+        <is>
+          <t>JOINT INTELLIGENCE SUMMIT: THREE GOVERNMENTS SHARE O... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E299" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F299" s="76" t="inlineStr">
+        <is>
+          <t>CAN_JOINT_OPS_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G299" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H299" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I299" s="75" t="inlineStr"/>
+      <c r="J299" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K299" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L299" s="75" t="inlineStr"/>
+      <c r="M299" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N299" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_JOINT_OPS_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="30" customHeight="1">
+      <c r="A300" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B300" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C300" s="75" t="inlineStr">
+        <is>
+          <t>CAN_SUMMIT_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D300" s="76" t="inlineStr">
+        <is>
+          <t>THE OTTAWA SUMMIT: ALL THREE IN THE SAME ROOM FOR TH... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E300" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F300" s="76" t="inlineStr">
+        <is>
+          <t>CAN_SUMMIT_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G300" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H300" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I300" s="75" t="inlineStr"/>
+      <c r="J300" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K300" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L300" s="75" t="inlineStr"/>
+      <c r="M300" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N300" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_SUMMIT_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="30" customHeight="1">
+      <c r="A301" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B301" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C301" s="75" t="inlineStr">
+        <is>
+          <t>CAN_ELECTION_LUCK_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D301" s="76" t="inlineStr">
+        <is>
+          <t>PM CLEAR-WATER'S CALL: JESSICA HAS SOMETHING TO SAY ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E301" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F301" s="76" t="inlineStr">
+        <is>
+          <t>CAN_ELECTION_LUCK (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G301" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H301" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I301" s="75" t="inlineStr"/>
+      <c r="J301" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K301" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L301" s="75" t="inlineStr"/>
+      <c r="M301" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N301" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_ELECTION_LUCK. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="30" customHeight="1">
+      <c r="A302" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B302" s="74" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C302" s="75" t="inlineStr">
+        <is>
+          <t>CAN_PEACE_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D302" s="76" t="inlineStr">
+        <is>
+          <t>THE TIDE HAS TURNED: PENOIT AND CLEAR-WATER COME TO ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E302" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F302" s="76" t="inlineStr">
+        <is>
+          <t>CAN_PEACE_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G302" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H302" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I302" s="75" t="inlineStr"/>
+      <c r="J302" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K302" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L302" s="75" t="inlineStr"/>
+      <c r="M302" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N302" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_PEACE_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="30" customHeight="1">
+      <c r="A303" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B303" s="74" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C303" s="75" t="inlineStr">
+        <is>
+          <t>PEACE_ALLIED_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D303" s="76" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E303" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F303" s="76" t="inlineStr">
+        <is>
+          <t>PEACE_ALLIED_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G303" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H303" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I303" s="75" t="inlineStr"/>
+      <c r="J303" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K303" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L303" s="75" t="inlineStr"/>
+      <c r="M303" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N303" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PEACE_ALLIED_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="30" customHeight="1">
+      <c r="A304" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B304" s="74" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C304" s="75" t="inlineStr">
+        <is>
+          <t>PEACE_USA_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D304" s="76" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E304" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F304" s="76" t="inlineStr">
+        <is>
+          <t>PEACE_USA_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G304" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H304" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I304" s="75" t="inlineStr"/>
+      <c r="J304" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K304" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L304" s="75" t="inlineStr"/>
+      <c r="M304" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N304" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PEACE_USA_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="8" customHeight="1">
+      <c r="A305" s="9" t="n"/>
+      <c r="B305" s="9" t="n"/>
+      <c r="C305" s="9" t="n"/>
+      <c r="D305" s="9" t="n"/>
+      <c r="E305" s="9" t="n"/>
+      <c r="F305" s="9" t="n"/>
+      <c r="G305" s="9" t="n"/>
+      <c r="H305" s="9" t="n"/>
+      <c r="I305" s="9" t="n"/>
+      <c r="J305" s="9" t="n"/>
+      <c r="K305" s="9" t="n"/>
+      <c r="L305" s="9" t="n"/>
+      <c r="M305" s="9" t="n"/>
+      <c r="N305" s="9" t="n"/>
+    </row>
+    <row r="306" ht="30" customHeight="1">
+      <c r="A306" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B306" s="74" t="inlineStr">
+        <is>
+          <t>Le Wendigo</t>
+        </is>
+      </c>
+      <c r="C306" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D306" s="76" t="inlineStr">
+        <is>
+          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E306" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F306" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G306" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H306" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I306" s="75" t="inlineStr"/>
+      <c r="J306" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K306" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L306" s="75" t="inlineStr"/>
+      <c r="M306" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N306" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="30" customHeight="1">
+      <c r="A307" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B307" s="74" t="inlineStr">
+        <is>
+          <t>Le Loup-Garou</t>
+        </is>
+      </c>
+      <c r="C307" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_02_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D307" s="76" t="inlineStr">
+        <is>
+          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E307" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F307" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_02_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G307" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H307" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I307" s="75" t="inlineStr"/>
+      <c r="J307" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K307" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L307" s="75" t="inlineStr"/>
+      <c r="M307" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N307" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="30" customHeight="1">
+      <c r="A308" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B308" s="74" t="inlineStr">
+        <is>
+          <t>Les Feux Follets</t>
+        </is>
+      </c>
+      <c r="C308" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_03_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D308" s="76" t="inlineStr">
+        <is>
+          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E308" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F308" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_03_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G308" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H308" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I308" s="75" t="inlineStr"/>
+      <c r="J308" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K308" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L308" s="75" t="inlineStr"/>
+      <c r="M308" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N308" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="30" customHeight="1">
+      <c r="A309" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B309" s="74" t="inlineStr">
+        <is>
+          <t>Mishepeshu</t>
+        </is>
+      </c>
+      <c r="C309" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_04_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D309" s="76" t="inlineStr">
+        <is>
+          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E309" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F309" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_04_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G309" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H309" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I309" s="75" t="inlineStr"/>
+      <c r="J309" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K309" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L309" s="75" t="inlineStr"/>
+      <c r="M309" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N309" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="30" customHeight="1">
+      <c r="A310" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B310" s="74" t="inlineStr">
+        <is>
+          <t>La Corriveau</t>
+        </is>
+      </c>
+      <c r="C310" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_05_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D310" s="76" t="inlineStr">
+        <is>
+          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E310" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F310" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_05_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G310" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H310" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I310" s="75" t="inlineStr"/>
+      <c r="J310" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K310" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L310" s="75" t="inlineStr"/>
+      <c r="M310" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N310" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="30" customHeight="1">
+      <c r="A311" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B311" s="74" t="inlineStr">
+        <is>
+          <t>Le Carcajou</t>
+        </is>
+      </c>
+      <c r="C311" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_06_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D311" s="76" t="inlineStr">
+        <is>
+          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E311" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F311" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_06_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G311" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H311" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I311" s="75" t="inlineStr"/>
+      <c r="J311" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K311" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L311" s="75" t="inlineStr"/>
+      <c r="M311" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N311" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="30" customHeight="1">
+      <c r="A312" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B312" s="74" t="inlineStr">
+        <is>
+          <t>La Chasse-Galerie</t>
+        </is>
+      </c>
+      <c r="C312" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_07_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D312" s="76" t="inlineStr">
+        <is>
+          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E312" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F312" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_07_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G312" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H312" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I312" s="75" t="inlineStr"/>
+      <c r="J312" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K312" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L312" s="75" t="inlineStr"/>
+      <c r="M312" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N312" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="30" customHeight="1">
+      <c r="A313" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B313" s="74" t="inlineStr">
+        <is>
+          <t>Le Gougou</t>
+        </is>
+      </c>
+      <c r="C313" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D313" s="76" t="inlineStr">
+        <is>
+          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E313" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F313" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G313" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H313" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I313" s="75" t="inlineStr"/>
+      <c r="J313" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K313" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L313" s="75" t="inlineStr"/>
+      <c r="M313" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N313" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="8" customHeight="1">
+      <c r="A314" s="9" t="n"/>
+      <c r="B314" s="9" t="n"/>
+      <c r="C314" s="9" t="n"/>
+      <c r="D314" s="9" t="n"/>
+      <c r="E314" s="9" t="n"/>
+      <c r="F314" s="9" t="n"/>
+      <c r="G314" s="9" t="n"/>
+      <c r="H314" s="9" t="n"/>
+      <c r="I314" s="9" t="n"/>
+      <c r="J314" s="9" t="n"/>
+      <c r="K314" s="9" t="n"/>
+      <c r="L314" s="9" t="n"/>
+      <c r="M314" s="9" t="n"/>
+      <c r="N314" s="9" t="n"/>
+    </row>
+    <row r="315" ht="30" customHeight="1">
+      <c r="A315" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B315" s="74" t="inlineStr">
+        <is>
+          <t>Ambush</t>
+        </is>
+      </c>
+      <c r="C315" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_AMBUSH_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D315" s="76" t="inlineStr">
+        <is>
+          <t>CROWN AMBUSH AVERTED: PRESIDENT CARLISLE HOLDS THE W... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E315" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F315" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_AMBUSH_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G315" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H315" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I315" s="75" t="inlineStr"/>
+      <c r="J315" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K315" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L315" s="75" t="inlineStr"/>
+      <c r="M315" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N315" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_AMBUSH_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="30" customHeight="1">
+      <c r="A316" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B316" s="74" t="inlineStr">
+        <is>
+          <t>Dignitary Reception</t>
+        </is>
+      </c>
+      <c r="C316" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_DIGNITARY_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D316" s="76" t="inlineStr">
+        <is>
+          <t>STATE RECEPTION AT [TILE_NAME]: PRESIDENT CARLISLE A... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E316" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F316" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_DIGNITARY_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G316" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H316" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I316" s="75" t="inlineStr"/>
+      <c r="J316" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K316" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L316" s="75" t="inlineStr"/>
+      <c r="M316" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N316" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_DIGNITARY_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="30" customHeight="1">
+      <c r="A317" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B317" s="74" t="inlineStr">
+        <is>
+          <t>Memorial Address</t>
+        </is>
+      </c>
+      <c r="C317" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_MEMORIAL_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D317" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE VISITS [TILE_NAME]: PRESIDENTIAL ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E317" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F317" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_MEMORIAL_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G317" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H317" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I317" s="75" t="inlineStr"/>
+      <c r="J317" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K317" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L317" s="75" t="inlineStr"/>
+      <c r="M317" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N317" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_MEMORIAL_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="30" customHeight="1">
+      <c r="A318" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B318" s="74" t="inlineStr">
+        <is>
+          <t>Field Hospital</t>
+        </is>
+      </c>
+      <c r="C318" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_WOUNDED_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D318" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE VISITS FIELD HOSPITAL AT [TILE_NAME] — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E318" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F318" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_WOUNDED_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G318" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H318" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I318" s="75" t="inlineStr"/>
+      <c r="J318" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K318" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L318" s="75" t="inlineStr"/>
+      <c r="M318" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N318" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_WOUNDED_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="30" customHeight="1">
+      <c r="A319" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B319" s="74" t="inlineStr">
+        <is>
+          <t>Forge Inspection</t>
+        </is>
+      </c>
+      <c r="C319" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_FORGE_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D319" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE CONDUCTS SURPRISE INSPECTION OF F... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E319" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F319" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_FORGE_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G319" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H319" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I319" s="75" t="inlineStr"/>
+      <c r="J319" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K319" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L319" s="75" t="inlineStr"/>
+      <c r="M319" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N319" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_FORGE_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="30" customHeight="1">
+      <c r="A320" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B320" s="74" t="inlineStr">
+        <is>
+          <t>Culper Ring</t>
+        </is>
+      </c>
+      <c r="C320" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_CULPER_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D320" s="76" t="inlineStr">
+        <is>
+          <t>CULPER RING CONTACT AT [TILE_NAME]: INTELLIGENCE ASS... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E320" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F320" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_CULPER_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G320" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H320" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I320" s="75" t="inlineStr"/>
+      <c r="J320" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K320" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L320" s="75" t="inlineStr"/>
+      <c r="M320" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N320" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_CULPER_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" ht="30" customHeight="1">
+      <c r="A321" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B321" s="74" t="inlineStr">
+        <is>
+          <t>Alliance Council</t>
+        </is>
+      </c>
+      <c r="C321" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_ALLIANCE_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D321" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE MEETS WITH [COMMANDER_NAME] AT [T... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E321" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F321" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_ALLIANCE_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G321" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H321" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I321" s="75" t="inlineStr"/>
+      <c r="J321" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K321" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L321" s="75" t="inlineStr"/>
+      <c r="M321" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N321" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_ALLIANCE_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="322" ht="30" customHeight="1">
+      <c r="A322" s="74" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B322" s="74" t="inlineStr">
+        <is>
+          <t>Frontier</t>
+        </is>
+      </c>
+      <c r="C322" s="75" t="inlineStr">
+        <is>
+          <t>UALANI_FRONTIER_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D322" s="76" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE ESTABLISHES FRONTIER PRESENCE AT ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E322" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F322" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_FRONTIER_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G322" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H322" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I322" s="75" t="inlineStr"/>
+      <c r="J322" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K322" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L322" s="75" t="inlineStr"/>
+      <c r="M322" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N322" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_FRONTIER_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="8" customHeight="1">
+      <c r="A323" s="9" t="n"/>
+      <c r="B323" s="9" t="n"/>
+      <c r="C323" s="9" t="n"/>
+      <c r="D323" s="9" t="n"/>
+      <c r="E323" s="9" t="n"/>
+      <c r="F323" s="9" t="n"/>
+      <c r="G323" s="9" t="n"/>
+      <c r="H323" s="9" t="n"/>
+      <c r="I323" s="9" t="n"/>
+      <c r="J323" s="9" t="n"/>
+      <c r="K323" s="9" t="n"/>
+      <c r="L323" s="9" t="n"/>
+      <c r="M323" s="9" t="n"/>
+      <c r="N323" s="9" t="n"/>
+    </row>
+    <row r="324" ht="30" customHeight="1">
+      <c r="A324" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B324" s="74" t="inlineStr">
+        <is>
+          <t>Mothman</t>
+        </is>
+      </c>
+      <c r="C324" s="75" t="inlineStr">
+        <is>
+          <t>PROT_01_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D324" s="76" t="inlineStr">
+        <is>
+          <t>MOTHMAN FORMALLY ALLIES WITH THE CONTINENTAL REPUBLIC — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E324" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F324" s="76" t="inlineStr">
+        <is>
+          <t>PROT_01_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G324" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H324" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I324" s="75" t="inlineStr"/>
+      <c r="J324" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K324" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L324" s="75" t="inlineStr"/>
+      <c r="M324" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N324" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="30" customHeight="1">
+      <c r="A325" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B325" s="74" t="inlineStr">
+        <is>
+          <t>Jersey Devil</t>
+        </is>
+      </c>
+      <c r="C325" s="75" t="inlineStr">
+        <is>
+          <t>PROT_02_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D325" s="76" t="inlineStr">
+        <is>
+          <t>JERSEY DEVIL FORMALLY ENDORSES THE CONTINENTAL CAUSE — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E325" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F325" s="76" t="inlineStr">
+        <is>
+          <t>PROT_02_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G325" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H325" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I325" s="75" t="inlineStr"/>
+      <c r="J325" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K325" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L325" s="75" t="inlineStr"/>
+      <c r="M325" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N325" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="30" customHeight="1">
+      <c r="A326" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B326" s="74" t="inlineStr">
+        <is>
+          <t>Bigfoot</t>
+        </is>
+      </c>
+      <c r="C326" s="75" t="inlineStr">
+        <is>
+          <t>PROT_03_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D326" s="76" t="inlineStr">
+        <is>
+          <t>BIGFOOT FORMALLY GUIDES THE CONTINENTAL CAUSE THROUG... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E326" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F326" s="76" t="inlineStr">
+        <is>
+          <t>PROT_03_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G326" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H326" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I326" s="75" t="inlineStr"/>
+      <c r="J326" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K326" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L326" s="75" t="inlineStr"/>
+      <c r="M326" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N326" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327" ht="30" customHeight="1">
+      <c r="A327" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B327" s="74" t="inlineStr">
+        <is>
+          <t>Thunderbird</t>
+        </is>
+      </c>
+      <c r="C327" s="75" t="inlineStr">
+        <is>
+          <t>PROT_04_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D327" s="76" t="inlineStr">
+        <is>
+          <t>THUNDERBIRD FORMALLY ALLIES WITH THE CONTINENTAL REP... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E327" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F327" s="76" t="inlineStr">
+        <is>
+          <t>PROT_04_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G327" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H327" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I327" s="75" t="inlineStr"/>
+      <c r="J327" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K327" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L327" s="75" t="inlineStr"/>
+      <c r="M327" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N327" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="30" customHeight="1">
+      <c r="A328" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B328" s="74" t="inlineStr">
+        <is>
+          <t>Headless Horseman</t>
+        </is>
+      </c>
+      <c r="C328" s="75" t="inlineStr">
+        <is>
+          <t>PROT_05_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D328" s="76" t="inlineStr">
+        <is>
+          <t>THE HORSEMAN RIDES FOR THE REPUBLIC — FORMALLY — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E328" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F328" s="76" t="inlineStr">
+        <is>
+          <t>PROT_05_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G328" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H328" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I328" s="75" t="inlineStr"/>
+      <c r="J328" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K328" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L328" s="75" t="inlineStr"/>
+      <c r="M328" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N328" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="30" customHeight="1">
+      <c r="A329" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B329" s="74" t="inlineStr">
+        <is>
+          <t>Chessie</t>
+        </is>
+      </c>
+      <c r="C329" s="75" t="inlineStr">
+        <is>
+          <t>PROT_06_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D329" s="76" t="inlineStr">
+        <is>
+          <t>CHESSIE FORMALLY PATROLS FOR THE CONTINENTAL NAVY — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E329" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F329" s="76" t="inlineStr">
+        <is>
+          <t>PROT_06_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G329" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H329" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I329" s="75" t="inlineStr"/>
+      <c r="J329" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K329" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L329" s="75" t="inlineStr"/>
+      <c r="M329" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N329" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="30" customHeight="1">
+      <c r="A330" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B330" s="74" t="inlineStr">
+        <is>
+          <t>Bell Witch</t>
+        </is>
+      </c>
+      <c r="C330" s="75" t="inlineStr">
+        <is>
+          <t>PROT_07_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D330" s="76" t="inlineStr">
+        <is>
+          <t>THE BELL WITCH FORMALLY COMMITS TO THE CONTINENTAL C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E330" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F330" s="76" t="inlineStr">
+        <is>
+          <t>PROT_07_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G330" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H330" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I330" s="75" t="inlineStr"/>
+      <c r="J330" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K330" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L330" s="75" t="inlineStr"/>
+      <c r="M330" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N330" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="30" customHeight="1">
+      <c r="A331" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B331" s="74" t="inlineStr">
+        <is>
+          <t>Old Ironsides</t>
+        </is>
+      </c>
+      <c r="C331" s="75" t="inlineStr">
+        <is>
+          <t>PROT_08_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D331" s="76" t="inlineStr">
+        <is>
+          <t>OLD IRONSIDES FORMALLY JOINS THE CONTINENTAL NAVY — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E331" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F331" s="76" t="inlineStr">
+        <is>
+          <t>PROT_08_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G331" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H331" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I331" s="75" t="inlineStr"/>
+      <c r="J331" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K331" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L331" s="75" t="inlineStr"/>
+      <c r="M331" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N331" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="30" customHeight="1">
+      <c r="A332" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B332" s="74" t="inlineStr">
+        <is>
+          <t>Valley Forge Guardian</t>
+        </is>
+      </c>
+      <c r="C332" s="75" t="inlineStr">
+        <is>
+          <t>PROT_09_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D332" s="76" t="inlineStr">
+        <is>
+          <t>VALLEY FORGE GUARDIAN FORMALLY BLESSES THE CONTINENT... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E332" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F332" s="76" t="inlineStr">
+        <is>
+          <t>PROT_09_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G332" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H332" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I332" s="75" t="inlineStr"/>
+      <c r="J332" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K332" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L332" s="75" t="inlineStr"/>
+      <c r="M332" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N332" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_09_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="30" customHeight="1">
+      <c r="A333" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B333" s="74" t="inlineStr">
+        <is>
+          <t>Snallygaster</t>
+        </is>
+      </c>
+      <c r="C333" s="75" t="inlineStr">
+        <is>
+          <t>PROT_10_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D333" s="76" t="inlineStr">
+        <is>
+          <t>SNALLYGASTER FORMALLY GUARDS THE CONTINENTAL SUPPLY ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E333" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F333" s="76" t="inlineStr">
+        <is>
+          <t>PROT_10_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G333" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H333" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I333" s="75" t="inlineStr"/>
+      <c r="J333" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K333" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L333" s="75" t="inlineStr"/>
+      <c r="M333" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N333" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_10_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334" ht="30" customHeight="1">
+      <c r="A334" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B334" s="74" t="inlineStr">
+        <is>
+          <t>Paul Revere</t>
+        </is>
+      </c>
+      <c r="C334" s="75" t="inlineStr">
+        <is>
+          <t>PROT_11_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D334" s="76" t="inlineStr">
+        <is>
+          <t>PAUL REVERE FORMALLY INTEGRATES WITH CONTINENTAL INT... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E334" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F334" s="76" t="inlineStr">
+        <is>
+          <t>PROT_11_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G334" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H334" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I334" s="75" t="inlineStr"/>
+      <c r="J334" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K334" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L334" s="75" t="inlineStr"/>
+      <c r="M334" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N334" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_11_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="30" customHeight="1">
+      <c r="A335" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B335" s="74" t="inlineStr">
+        <is>
+          <t>Liberty Bell</t>
+        </is>
+      </c>
+      <c r="C335" s="75" t="inlineStr">
+        <is>
+          <t>PROT_12_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D335" s="76" t="inlineStr">
+        <is>
+          <t>THE LIBERTY BELL FORMALLY RINGS FOR THE REPUBLIC — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E335" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F335" s="76" t="inlineStr">
+        <is>
+          <t>PROT_12_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G335" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H335" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I335" s="75" t="inlineStr"/>
+      <c r="J335" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K335" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L335" s="75" t="inlineStr"/>
+      <c r="M335" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N335" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_12_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="30" customHeight="1">
+      <c r="A336" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B336" s="74" t="inlineStr">
+        <is>
+          <t>Green Mountain Ghost</t>
+        </is>
+      </c>
+      <c r="C336" s="75" t="inlineStr">
+        <is>
+          <t>PROT_13_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D336" s="76" t="inlineStr">
+        <is>
+          <t>GREEN MOUNTAIN GHOST FORMALLY PROTECTS VERMONT FOR T... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E336" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F336" s="76" t="inlineStr">
+        <is>
+          <t>PROT_13_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G336" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H336" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I336" s="75" t="inlineStr"/>
+      <c r="J336" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K336" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L336" s="75" t="inlineStr"/>
+      <c r="M336" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N336" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_13_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="30" customHeight="1">
+      <c r="A337" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B337" s="74" t="inlineStr">
+        <is>
+          <t>Mount Rushmore</t>
+        </is>
+      </c>
+      <c r="C337" s="75" t="inlineStr">
+        <is>
+          <t>PROT_14_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D337" s="76" t="inlineStr">
+        <is>
+          <t>THE RUSHMORE COUNCIL FORMALLY ENDORSES PRESIDENT CAR... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E337" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F337" s="76" t="inlineStr">
+        <is>
+          <t>PROT_14_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G337" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H337" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I337" s="75" t="inlineStr"/>
+      <c r="J337" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K337" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L337" s="75" t="inlineStr"/>
+      <c r="M337" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N337" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_14_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="30" customHeight="1">
+      <c r="A338" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B338" s="74" t="inlineStr">
+        <is>
+          <t>Skunk Ape</t>
+        </is>
+      </c>
+      <c r="C338" s="75" t="inlineStr">
+        <is>
+          <t>PROT_15_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D338" s="76" t="inlineStr">
+        <is>
+          <t>SKUNK APE FORMALLY PATROLS FLORIDA FOR THE CONTINENT... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E338" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F338" s="76" t="inlineStr">
+        <is>
+          <t>PROT_15_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G338" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H338" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I338" s="75" t="inlineStr"/>
+      <c r="J338" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K338" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L338" s="75" t="inlineStr"/>
+      <c r="M338" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N338" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_15_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="30" customHeight="1">
+      <c r="A339" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B339" s="74" t="inlineStr">
+        <is>
+          <t>Minuteman</t>
+        </is>
+      </c>
+      <c r="C339" s="75" t="inlineStr">
+        <is>
+          <t>PROT_16_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D339" s="76" t="inlineStr">
+        <is>
+          <t>THE MINUTEMAN FORMALLY DECLARES FOR THE CONTINENTAL ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E339" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F339" s="76" t="inlineStr">
+        <is>
+          <t>PROT_16_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G339" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H339" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I339" s="75" t="inlineStr"/>
+      <c r="J339" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K339" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L339" s="75" t="inlineStr"/>
+      <c r="M339" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N339" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_16_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="30" customHeight="1">
+      <c r="A340" s="74" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B340" s="74" t="inlineStr">
+        <is>
+          <t>Lincoln's Ghost</t>
+        </is>
+      </c>
+      <c r="C340" s="75" t="inlineStr">
+        <is>
+          <t>PROT_17_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D340" s="76" t="inlineStr">
+        <is>
+          <t>LINCOLN FORMALLY ENDORSES PRESIDENT CARLISLE'S ADMIN... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E340" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F340" s="76" t="inlineStr">
+        <is>
+          <t>PROT_17_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G340" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H340" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I340" s="75" t="inlineStr"/>
+      <c r="J340" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K340" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L340" s="75" t="inlineStr"/>
+      <c r="M340" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N340" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_17_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="8" customHeight="1">
+      <c r="A341" s="9" t="n"/>
+      <c r="B341" s="9" t="n"/>
+      <c r="C341" s="9" t="n"/>
+      <c r="D341" s="9" t="n"/>
+      <c r="E341" s="9" t="n"/>
+      <c r="F341" s="9" t="n"/>
+      <c r="G341" s="9" t="n"/>
+      <c r="H341" s="9" t="n"/>
+      <c r="I341" s="9" t="n"/>
+      <c r="J341" s="9" t="n"/>
+      <c r="K341" s="9" t="n"/>
+      <c r="L341" s="9" t="n"/>
+      <c r="M341" s="9" t="n"/>
+      <c r="N341" s="9" t="n"/>
+    </row>
+    <row r="342" ht="30" customHeight="1">
+      <c r="A342" s="74" t="inlineStr">
+        <is>
+          <t>White House</t>
+        </is>
+      </c>
+      <c r="B342" s="74" t="inlineStr">
+        <is>
+          <t>Month 1</t>
+        </is>
+      </c>
+      <c r="C342" s="75" t="inlineStr">
+        <is>
+          <t>WH_SECRET_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D342" s="76" t="inlineStr">
+        <is>
+          <t>THE WHITE HOUSE AT MIDNIGHT — THE PRESIDENT WATCHES ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E342" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F342" s="76" t="inlineStr">
+        <is>
+          <t>WH_SECRET_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G342" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H342" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I342" s="75" t="inlineStr"/>
+      <c r="J342" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K342" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L342" s="75" t="inlineStr"/>
+      <c r="M342" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N342" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of WH_SECRET_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="30" customHeight="1">
+      <c r="A343" s="74" t="inlineStr">
+        <is>
+          <t>White House</t>
+        </is>
+      </c>
+      <c r="B343" s="74" t="inlineStr">
+        <is>
+          <t>Month 7</t>
+        </is>
+      </c>
+      <c r="C343" s="75" t="inlineStr">
+        <is>
+          <t>WH_SECRET_07_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D343" s="76" t="inlineStr">
+        <is>
+          <t>JULY AT THE WHITE HOUSE — INDEPENDENCE DAY IS ALSO HERS — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E343" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F343" s="76" t="inlineStr">
+        <is>
+          <t>WH_SECRET_07 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G343" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H343" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I343" s="75" t="inlineStr"/>
+      <c r="J343" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K343" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L343" s="75" t="inlineStr"/>
+      <c r="M343" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N343" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of WH_SECRET_07. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="30" customHeight="1">
+      <c r="A344" s="74" t="inlineStr">
+        <is>
+          <t>White House</t>
+        </is>
+      </c>
+      <c r="B344" s="74" t="inlineStr">
+        <is>
+          <t>Month 10</t>
+        </is>
+      </c>
+      <c r="C344" s="75" t="inlineStr">
+        <is>
+          <t>WH_SECRET_10_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D344" s="76" t="inlineStr">
+        <is>
+          <t>INDIGENOUS PEOPLES DAY — A PERSONAL LETTER FROM JESS... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E344" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F344" s="76" t="inlineStr">
+        <is>
+          <t>WH_SECRET_10 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G344" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H344" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I344" s="75" t="inlineStr"/>
+      <c r="J344" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K344" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L344" s="75" t="inlineStr"/>
+      <c r="M344" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N344" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of WH_SECRET_10. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="30" customHeight="1">
+      <c r="A345" s="74" t="inlineStr">
+        <is>
+          <t>White House</t>
+        </is>
+      </c>
+      <c r="B345" s="74" t="inlineStr">
+        <is>
+          <t>Month 12</t>
+        </is>
+      </c>
+      <c r="C345" s="75" t="inlineStr">
+        <is>
+          <t>WH_SECRET_12_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D345" s="76" t="inlineStr">
+        <is>
+          <t>CHRISTMAS IN WASHINGTON — THE PRESIDENT IS FAR FROM ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E345" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F345" s="76" t="inlineStr">
+        <is>
+          <t>WH_SECRET_12 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G345" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H345" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I345" s="75" t="inlineStr"/>
+      <c r="J345" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K345" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L345" s="75" t="inlineStr"/>
+      <c r="M345" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N345" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of WH_SECRET_12. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="20" customHeight="1">
+      <c r="A347" s="79" t="inlineStr">
         <is>
           <t>Total events in spreadsheet</t>
         </is>
       </c>
-      <c r="B284" s="80" t="n">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="285" ht="20" customHeight="1">
-      <c r="A285" s="79" t="inlineStr">
+      <c r="B347" s="80" t="n">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="348" ht="20" customHeight="1">
+      <c r="A348" s="79" t="inlineStr">
         <is>
           <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
-      <c r="B285" s="80" t="n">
+      <c r="B348" s="80" t="n">
         <v>250</v>
       </c>
     </row>
-    <row r="286" ht="20" customHeight="1">
-      <c r="A286" s="79" t="inlineStr">
+    <row r="349" ht="20" customHeight="1">
+      <c r="A349" s="79" t="inlineStr">
         <is>
           <t>IDEA (not yet implemented)</t>
         </is>
       </c>
-      <c r="B286" s="80" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="287" ht="20" customHeight="1">
-      <c r="A287" s="79" t="inlineStr">
+      <c r="B349" s="80" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="350" ht="20" customHeight="1">
+      <c r="A350" s="79" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B287" s="80" t="n">
+      <c r="B350" s="80" t="n">
         <v>55</v>
       </c>
     </row>
@@ -18879,7 +22431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21606,43 +25158,1019 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="79" t="inlineStr">
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B43" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C43" s="75" t="inlineStr">
+        <is>
+          <t>CAN_CLEARWATER_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D43" s="76" t="inlineStr">
+        <is>
+          <t>PM CLEAR-WATER'S PRIVATE CHANNEL: JESSICA WRITES OUT... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E43" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F43" s="76" t="inlineStr">
+        <is>
+          <t>CAN_CLEARWATER_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G43" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I43" s="75" t="inlineStr"/>
+      <c r="J43" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K43" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L43" s="75" t="inlineStr"/>
+      <c r="M43" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N43" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_CLEARWATER_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B44" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C44" s="75" t="inlineStr">
+        <is>
+          <t>CAN_JOINT_OPS_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D44" s="76" t="inlineStr">
+        <is>
+          <t>JOINT INTELLIGENCE SUMMIT: THREE GOVERNMENTS SHARE O... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E44" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F44" s="76" t="inlineStr">
+        <is>
+          <t>CAN_JOINT_OPS_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G44" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I44" s="75" t="inlineStr"/>
+      <c r="J44" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K44" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L44" s="75" t="inlineStr"/>
+      <c r="M44" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N44" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_JOINT_OPS_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C45" s="75" t="inlineStr">
+        <is>
+          <t>CAN_SUMMIT_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D45" s="76" t="inlineStr">
+        <is>
+          <t>THE OTTAWA SUMMIT: ALL THREE IN THE SAME ROOM FOR TH... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E45" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F45" s="76" t="inlineStr">
+        <is>
+          <t>CAN_SUMMIT_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G45" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I45" s="75" t="inlineStr"/>
+      <c r="J45" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K45" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L45" s="75" t="inlineStr"/>
+      <c r="M45" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N45" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_SUMMIT_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B46" s="74" t="inlineStr">
+        <is>
+          <t>Canadian Alliance</t>
+        </is>
+      </c>
+      <c r="C46" s="75" t="inlineStr">
+        <is>
+          <t>CAN_ELECTION_LUCK_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D46" s="76" t="inlineStr">
+        <is>
+          <t>PM CLEAR-WATER'S CALL: JESSICA HAS SOMETHING TO SAY ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E46" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F46" s="76" t="inlineStr">
+        <is>
+          <t>CAN_ELECTION_LUCK (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G46" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I46" s="75" t="inlineStr"/>
+      <c r="J46" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K46" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L46" s="75" t="inlineStr"/>
+      <c r="M46" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N46" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_ELECTION_LUCK. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B47" s="74" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C47" s="75" t="inlineStr">
+        <is>
+          <t>CAN_PEACE_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D47" s="76" t="inlineStr">
+        <is>
+          <t>THE TIDE HAS TURNED: PENOIT AND CLEAR-WATER COME TO ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E47" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F47" s="76" t="inlineStr">
+        <is>
+          <t>CAN_PEACE_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G47" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I47" s="75" t="inlineStr"/>
+      <c r="J47" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K47" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L47" s="75" t="inlineStr"/>
+      <c r="M47" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N47" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CAN_PEACE_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B48" s="74" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C48" s="75" t="inlineStr">
+        <is>
+          <t>PEACE_ALLIED_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D48" s="76" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E48" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F48" s="76" t="inlineStr">
+        <is>
+          <t>PEACE_ALLIED_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G48" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I48" s="75" t="inlineStr"/>
+      <c r="J48" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K48" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L48" s="75" t="inlineStr"/>
+      <c r="M48" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N48" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PEACE_ALLIED_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="74" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B49" s="74" t="inlineStr">
+        <is>
+          <t>Peace</t>
+        </is>
+      </c>
+      <c r="C49" s="75" t="inlineStr">
+        <is>
+          <t>PEACE_USA_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D49" s="76" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E49" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F49" s="76" t="inlineStr">
+        <is>
+          <t>PEACE_USA_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G49" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I49" s="75" t="inlineStr"/>
+      <c r="J49" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K49" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L49" s="75" t="inlineStr"/>
+      <c r="M49" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N49" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PEACE_USA_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="8" customHeight="1">
+      <c r="A50" s="9" t="n"/>
+      <c r="B50" s="9" t="n"/>
+      <c r="C50" s="9" t="n"/>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="9" t="n"/>
+      <c r="G50" s="9" t="n"/>
+      <c r="H50" s="9" t="n"/>
+      <c r="I50" s="9" t="n"/>
+      <c r="J50" s="9" t="n"/>
+      <c r="K50" s="9" t="n"/>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="9" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B51" s="74" t="inlineStr">
+        <is>
+          <t>Le Wendigo</t>
+        </is>
+      </c>
+      <c r="C51" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D51" s="76" t="inlineStr">
+        <is>
+          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E51" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F51" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G51" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H51" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I51" s="75" t="inlineStr"/>
+      <c r="J51" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K51" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L51" s="75" t="inlineStr"/>
+      <c r="M51" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N51" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B52" s="74" t="inlineStr">
+        <is>
+          <t>Le Loup-Garou</t>
+        </is>
+      </c>
+      <c r="C52" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_02_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D52" s="76" t="inlineStr">
+        <is>
+          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E52" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F52" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_02_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G52" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I52" s="75" t="inlineStr"/>
+      <c r="J52" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K52" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L52" s="75" t="inlineStr"/>
+      <c r="M52" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N52" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Les Feux Follets</t>
+        </is>
+      </c>
+      <c r="C53" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_03_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D53" s="76" t="inlineStr">
+        <is>
+          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E53" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F53" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_03_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G53" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I53" s="75" t="inlineStr"/>
+      <c r="J53" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K53" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L53" s="75" t="inlineStr"/>
+      <c r="M53" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N53" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Mishepeshu</t>
+        </is>
+      </c>
+      <c r="C54" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_04_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D54" s="76" t="inlineStr">
+        <is>
+          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E54" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F54" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_04_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G54" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I54" s="75" t="inlineStr"/>
+      <c r="J54" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K54" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L54" s="75" t="inlineStr"/>
+      <c r="M54" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N54" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>La Corriveau</t>
+        </is>
+      </c>
+      <c r="C55" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_05_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D55" s="76" t="inlineStr">
+        <is>
+          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E55" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F55" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_05_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G55" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I55" s="75" t="inlineStr"/>
+      <c r="J55" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K55" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L55" s="75" t="inlineStr"/>
+      <c r="M55" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N55" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B56" s="74" t="inlineStr">
+        <is>
+          <t>Le Carcajou</t>
+        </is>
+      </c>
+      <c r="C56" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_06_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D56" s="76" t="inlineStr">
+        <is>
+          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E56" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F56" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_06_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G56" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I56" s="75" t="inlineStr"/>
+      <c r="J56" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K56" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L56" s="75" t="inlineStr"/>
+      <c r="M56" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N56" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>La Chasse-Galerie</t>
+        </is>
+      </c>
+      <c r="C57" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_07_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D57" s="76" t="inlineStr">
+        <is>
+          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E57" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F57" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_07_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G57" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I57" s="75" t="inlineStr"/>
+      <c r="J57" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K57" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L57" s="75" t="inlineStr"/>
+      <c r="M57" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N57" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="74" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Le Gougou</t>
+        </is>
+      </c>
+      <c r="C58" s="75" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D58" s="76" t="inlineStr">
+        <is>
+          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E58" s="78" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F58" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G58" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="77" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I58" s="75" t="inlineStr"/>
+      <c r="J58" s="57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K58" s="78" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L58" s="75" t="inlineStr"/>
+      <c r="M58" s="78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N58" s="76" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="79" t="inlineStr">
         <is>
           <t>Canadian events total</t>
         </is>
       </c>
-      <c r="B44" s="80" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="79" t="inlineStr">
+      <c r="B60" s="80" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="79" t="inlineStr">
         <is>
           <t>Canada (Alliance arc)</t>
         </is>
       </c>
-      <c r="B45" s="80" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="79" t="inlineStr">
+      <c r="B61" s="80" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="79" t="inlineStr">
         <is>
           <t>CA Protector (Jessica's creatures)</t>
         </is>
       </c>
-      <c r="B46" s="80" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="79" t="inlineStr">
+      <c r="B62" s="80" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="79" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B47" s="80" t="n">
+      <c r="B63" s="80" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Write CA_PM_LEGACY_INTIMATE scene; fix Marc/Mark typo in masterdoc
- Author full 'by morning' scene for CA_PM_LEGACY_INTIMATE: Penoit at the
  desk before light, writing page forty-one, emotional resolution
- Update short_desc, tone (Tender/Somber), long_desc in events.csv
- Add CA_PM_LEGACY_INTIMATE entry to build_event_masterdoc.py (FIRST PASS)
- Fix CAN_PENOIT_01 headline: MARK → MARC Penoit
- Regenerate event_masterdoc.xlsx (315 events)

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -1140,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N350"/>
+  <dimension ref="A1:N351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9493,7 +9493,7 @@
       </c>
       <c r="D135" s="55" t="inlineStr">
         <is>
-          <t>PRESIDENT PENOIT'S CONDITIONS: MARK PENOIT PUTS IT IN WRITING</t>
+          <t>PRESIDENT PENOIT'S CONDITIONS: MARC PENOIT PUTS IT IN WRITING</t>
         </is>
       </c>
       <c r="E135" s="28" t="inlineStr">
@@ -19963,85 +19963,85 @@
         </is>
       </c>
     </row>
-    <row r="305" ht="8" customHeight="1">
-      <c r="A305" s="9" t="n"/>
-      <c r="B305" s="9" t="n"/>
-      <c r="C305" s="9" t="n"/>
-      <c r="D305" s="9" t="n"/>
-      <c r="E305" s="9" t="n"/>
-      <c r="F305" s="9" t="n"/>
-      <c r="G305" s="9" t="n"/>
-      <c r="H305" s="9" t="n"/>
-      <c r="I305" s="9" t="n"/>
-      <c r="J305" s="9" t="n"/>
-      <c r="K305" s="9" t="n"/>
-      <c r="L305" s="9" t="n"/>
-      <c r="M305" s="9" t="n"/>
-      <c r="N305" s="9" t="n"/>
-    </row>
-    <row r="306" ht="30" customHeight="1">
-      <c r="A306" s="75" t="inlineStr">
-        <is>
-          <t>CA Protector</t>
-        </is>
-      </c>
-      <c r="B306" s="75" t="inlineStr">
-        <is>
-          <t>Le Wendigo</t>
-        </is>
-      </c>
-      <c r="C306" s="76" t="inlineStr">
-        <is>
-          <t>CA_PROT_01_AGREE_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D306" s="77" t="inlineStr">
-        <is>
-          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E306" s="79" t="inlineStr">
+    <row r="305" ht="30" customHeight="1">
+      <c r="A305" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B305" s="53" t="inlineStr">
+        <is>
+          <t>PM Arc</t>
+        </is>
+      </c>
+      <c r="C305" s="54" t="inlineStr">
+        <is>
+          <t>CA_PM_LEGACY_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D305" s="55" t="inlineStr">
+        <is>
+          <t>MARC PENOIT'S FINAL ASSESSMENT — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E305" s="56" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F306" s="77" t="inlineStr">
-        <is>
-          <t>CA_PROT_01_AGREE (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G306" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H306" s="78" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I306" s="76" t="inlineStr"/>
-      <c r="J306" s="80" t="inlineStr">
+      <c r="F305" s="55" t="inlineStr">
+        <is>
+          <t>CA_PM_LEGACY (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G305" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H305" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I305" s="54" t="inlineStr"/>
+      <c r="J305" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K306" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L306" s="76" t="inlineStr"/>
-      <c r="M306" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N306" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
+      <c r="K305" s="56" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L305" s="54" t="inlineStr"/>
+      <c r="M305" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N305" s="55" t="inlineStr">
+        <is>
+          <t>By morning: Penoit at the desk before light, writing page forty-one. Emotional resolution — he was wrong about what this would feel like.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="8" customHeight="1">
+      <c r="A306" s="9" t="n"/>
+      <c r="B306" s="9" t="n"/>
+      <c r="C306" s="9" t="n"/>
+      <c r="D306" s="9" t="n"/>
+      <c r="E306" s="9" t="n"/>
+      <c r="F306" s="9" t="n"/>
+      <c r="G306" s="9" t="n"/>
+      <c r="H306" s="9" t="n"/>
+      <c r="I306" s="9" t="n"/>
+      <c r="J306" s="9" t="n"/>
+      <c r="K306" s="9" t="n"/>
+      <c r="L306" s="9" t="n"/>
+      <c r="M306" s="9" t="n"/>
+      <c r="N306" s="9" t="n"/>
     </row>
     <row r="307" ht="30" customHeight="1">
       <c r="A307" s="75" t="inlineStr">
@@ -20051,17 +20051,17 @@
       </c>
       <c r="B307" s="75" t="inlineStr">
         <is>
-          <t>Le Loup-Garou</t>
+          <t>Le Wendigo</t>
         </is>
       </c>
       <c r="C307" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE_INTIMATE</t>
+          <t>CA_PROT_01_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D307" s="77" t="inlineStr">
         <is>
-          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
+          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
         </is>
       </c>
       <c r="E307" s="79" t="inlineStr">
@@ -20071,7 +20071,7 @@
       </c>
       <c r="F307" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE (intimate choice)</t>
+          <t>CA_PROT_01_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G307" s="77" t="inlineStr">
@@ -20103,7 +20103,7 @@
       </c>
       <c r="N307" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20115,17 +20115,17 @@
       </c>
       <c r="B308" s="75" t="inlineStr">
         <is>
-          <t>Les Feux Follets</t>
+          <t>Le Loup-Garou</t>
         </is>
       </c>
       <c r="C308" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE_INTIMATE</t>
+          <t>CA_PROT_02_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D308" s="77" t="inlineStr">
         <is>
-          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
+          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
         </is>
       </c>
       <c r="E308" s="79" t="inlineStr">
@@ -20135,7 +20135,7 @@
       </c>
       <c r="F308" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE (intimate choice)</t>
+          <t>CA_PROT_02_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G308" s="77" t="inlineStr">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="N308" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20179,17 +20179,17 @@
       </c>
       <c r="B309" s="75" t="inlineStr">
         <is>
-          <t>Mishepeshu</t>
+          <t>Les Feux Follets</t>
         </is>
       </c>
       <c r="C309" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE_INTIMATE</t>
+          <t>CA_PROT_03_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D309" s="77" t="inlineStr">
         <is>
-          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
+          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
         </is>
       </c>
       <c r="E309" s="79" t="inlineStr">
@@ -20199,7 +20199,7 @@
       </c>
       <c r="F309" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE (intimate choice)</t>
+          <t>CA_PROT_03_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G309" s="77" t="inlineStr">
@@ -20231,7 +20231,7 @@
       </c>
       <c r="N309" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20243,17 +20243,17 @@
       </c>
       <c r="B310" s="75" t="inlineStr">
         <is>
-          <t>La Corriveau</t>
+          <t>Mishepeshu</t>
         </is>
       </c>
       <c r="C310" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE_INTIMATE</t>
+          <t>CA_PROT_04_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D310" s="77" t="inlineStr">
         <is>
-          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
+          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
         </is>
       </c>
       <c r="E310" s="79" t="inlineStr">
@@ -20263,7 +20263,7 @@
       </c>
       <c r="F310" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE (intimate choice)</t>
+          <t>CA_PROT_04_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G310" s="77" t="inlineStr">
@@ -20295,7 +20295,7 @@
       </c>
       <c r="N310" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20307,17 +20307,17 @@
       </c>
       <c r="B311" s="75" t="inlineStr">
         <is>
-          <t>Le Carcajou</t>
+          <t>La Corriveau</t>
         </is>
       </c>
       <c r="C311" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE_INTIMATE</t>
+          <t>CA_PROT_05_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D311" s="77" t="inlineStr">
         <is>
-          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
+          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
         </is>
       </c>
       <c r="E311" s="79" t="inlineStr">
@@ -20327,7 +20327,7 @@
       </c>
       <c r="F311" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE (intimate choice)</t>
+          <t>CA_PROT_05_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G311" s="77" t="inlineStr">
@@ -20359,7 +20359,7 @@
       </c>
       <c r="N311" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20371,17 +20371,17 @@
       </c>
       <c r="B312" s="75" t="inlineStr">
         <is>
-          <t>La Chasse-Galerie</t>
+          <t>Le Carcajou</t>
         </is>
       </c>
       <c r="C312" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE_INTIMATE</t>
+          <t>CA_PROT_06_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D312" s="77" t="inlineStr">
         <is>
-          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
+          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
         </is>
       </c>
       <c r="E312" s="79" t="inlineStr">
@@ -20391,7 +20391,7 @@
       </c>
       <c r="F312" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE (intimate choice)</t>
+          <t>CA_PROT_06_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G312" s="77" t="inlineStr">
@@ -20423,7 +20423,7 @@
       </c>
       <c r="N312" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20435,17 +20435,17 @@
       </c>
       <c r="B313" s="75" t="inlineStr">
         <is>
-          <t>Le Gougou</t>
+          <t>La Chasse-Galerie</t>
         </is>
       </c>
       <c r="C313" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_08_AGREE_INTIMATE</t>
+          <t>CA_PROT_07_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D313" s="77" t="inlineStr">
         <is>
-          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
+          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
         </is>
       </c>
       <c r="E313" s="79" t="inlineStr">
@@ -20455,7 +20455,7 @@
       </c>
       <c r="F313" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_08_AGREE (intimate choice)</t>
+          <t>CA_PROT_07_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G313" s="77" t="inlineStr">
@@ -20487,89 +20487,89 @@
       </c>
       <c r="N313" s="77" t="inlineStr">
         <is>
+          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="30" customHeight="1">
+      <c r="A314" s="75" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B314" s="75" t="inlineStr">
+        <is>
+          <t>Le Gougou</t>
+        </is>
+      </c>
+      <c r="C314" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D314" s="77" t="inlineStr">
+        <is>
+          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E314" s="79" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F314" s="77" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G314" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H314" s="78" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I314" s="76" t="inlineStr"/>
+      <c r="J314" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K314" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L314" s="76" t="inlineStr"/>
+      <c r="M314" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N314" s="77" t="inlineStr">
+        <is>
           <t>Stub — author intimate version of CA_PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
-    <row r="314" ht="8" customHeight="1">
-      <c r="A314" s="9" t="n"/>
-      <c r="B314" s="9" t="n"/>
-      <c r="C314" s="9" t="n"/>
-      <c r="D314" s="9" t="n"/>
-      <c r="E314" s="9" t="n"/>
-      <c r="F314" s="9" t="n"/>
-      <c r="G314" s="9" t="n"/>
-      <c r="H314" s="9" t="n"/>
-      <c r="I314" s="9" t="n"/>
-      <c r="J314" s="9" t="n"/>
-      <c r="K314" s="9" t="n"/>
-      <c r="L314" s="9" t="n"/>
-      <c r="M314" s="9" t="n"/>
-      <c r="N314" s="9" t="n"/>
-    </row>
-    <row r="315" ht="30" customHeight="1">
-      <c r="A315" s="75" t="inlineStr">
-        <is>
-          <t>Ualani</t>
-        </is>
-      </c>
-      <c r="B315" s="75" t="inlineStr">
-        <is>
-          <t>Ambush</t>
-        </is>
-      </c>
-      <c r="C315" s="76" t="inlineStr">
-        <is>
-          <t>UALANI_AMBUSH_01_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D315" s="77" t="inlineStr">
-        <is>
-          <t>CROWN AMBUSH AVERTED: PRESIDENT CARLISLE HOLDS THE W... — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E315" s="79" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="F315" s="77" t="inlineStr">
-        <is>
-          <t>UALANI_AMBUSH_01 (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G315" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H315" s="78" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I315" s="76" t="inlineStr"/>
-      <c r="J315" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K315" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L315" s="76" t="inlineStr"/>
-      <c r="M315" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N315" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of UALANI_AMBUSH_01. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
+    <row r="315" ht="8" customHeight="1">
+      <c r="A315" s="9" t="n"/>
+      <c r="B315" s="9" t="n"/>
+      <c r="C315" s="9" t="n"/>
+      <c r="D315" s="9" t="n"/>
+      <c r="E315" s="9" t="n"/>
+      <c r="F315" s="9" t="n"/>
+      <c r="G315" s="9" t="n"/>
+      <c r="H315" s="9" t="n"/>
+      <c r="I315" s="9" t="n"/>
+      <c r="J315" s="9" t="n"/>
+      <c r="K315" s="9" t="n"/>
+      <c r="L315" s="9" t="n"/>
+      <c r="M315" s="9" t="n"/>
+      <c r="N315" s="9" t="n"/>
     </row>
     <row r="316" ht="30" customHeight="1">
       <c r="A316" s="75" t="inlineStr">
@@ -20579,17 +20579,17 @@
       </c>
       <c r="B316" s="75" t="inlineStr">
         <is>
-          <t>Dignitary Reception</t>
+          <t>Ambush</t>
         </is>
       </c>
       <c r="C316" s="76" t="inlineStr">
         <is>
-          <t>UALANI_DIGNITARY_01_INTIMATE</t>
+          <t>UALANI_AMBUSH_01_INTIMATE</t>
         </is>
       </c>
       <c r="D316" s="77" t="inlineStr">
         <is>
-          <t>STATE RECEPTION AT [TILE_NAME]: PRESIDENT CARLISLE A... — BY MORNING</t>
+          <t>CROWN AMBUSH AVERTED: PRESIDENT CARLISLE HOLDS THE W... — BY MORNING</t>
         </is>
       </c>
       <c r="E316" s="79" t="inlineStr">
@@ -20599,7 +20599,7 @@
       </c>
       <c r="F316" s="77" t="inlineStr">
         <is>
-          <t>UALANI_DIGNITARY_01 (intimate choice)</t>
+          <t>UALANI_AMBUSH_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G316" s="77" t="inlineStr">
@@ -20631,7 +20631,7 @@
       </c>
       <c r="N316" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_DIGNITARY_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_AMBUSH_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20643,17 +20643,17 @@
       </c>
       <c r="B317" s="75" t="inlineStr">
         <is>
-          <t>Memorial Address</t>
+          <t>Dignitary Reception</t>
         </is>
       </c>
       <c r="C317" s="76" t="inlineStr">
         <is>
-          <t>UALANI_MEMORIAL_01_INTIMATE</t>
+          <t>UALANI_DIGNITARY_01_INTIMATE</t>
         </is>
       </c>
       <c r="D317" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS [TILE_NAME]: PRESIDENTIAL ... — BY MORNING</t>
+          <t>STATE RECEPTION AT [TILE_NAME]: PRESIDENT CARLISLE A... — BY MORNING</t>
         </is>
       </c>
       <c r="E317" s="79" t="inlineStr">
@@ -20663,7 +20663,7 @@
       </c>
       <c r="F317" s="77" t="inlineStr">
         <is>
-          <t>UALANI_MEMORIAL_01 (intimate choice)</t>
+          <t>UALANI_DIGNITARY_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G317" s="77" t="inlineStr">
@@ -20695,7 +20695,7 @@
       </c>
       <c r="N317" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_MEMORIAL_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_DIGNITARY_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20707,17 +20707,17 @@
       </c>
       <c r="B318" s="75" t="inlineStr">
         <is>
-          <t>Field Hospital</t>
+          <t>Memorial Address</t>
         </is>
       </c>
       <c r="C318" s="76" t="inlineStr">
         <is>
-          <t>UALANI_WOUNDED_01_INTIMATE</t>
+          <t>UALANI_MEMORIAL_01_INTIMATE</t>
         </is>
       </c>
       <c r="D318" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS FIELD HOSPITAL AT [TILE_NAME] — BY MORNING</t>
+          <t>PRESIDENT CARLISLE VISITS [TILE_NAME]: PRESIDENTIAL ... — BY MORNING</t>
         </is>
       </c>
       <c r="E318" s="79" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="F318" s="77" t="inlineStr">
         <is>
-          <t>UALANI_WOUNDED_01 (intimate choice)</t>
+          <t>UALANI_MEMORIAL_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G318" s="77" t="inlineStr">
@@ -20759,7 +20759,7 @@
       </c>
       <c r="N318" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_WOUNDED_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_MEMORIAL_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20771,17 +20771,17 @@
       </c>
       <c r="B319" s="75" t="inlineStr">
         <is>
-          <t>Forge Inspection</t>
+          <t>Field Hospital</t>
         </is>
       </c>
       <c r="C319" s="76" t="inlineStr">
         <is>
-          <t>UALANI_FORGE_01_INTIMATE</t>
+          <t>UALANI_WOUNDED_01_INTIMATE</t>
         </is>
       </c>
       <c r="D319" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE CONDUCTS SURPRISE INSPECTION OF F... — BY MORNING</t>
+          <t>PRESIDENT CARLISLE VISITS FIELD HOSPITAL AT [TILE_NAME] — BY MORNING</t>
         </is>
       </c>
       <c r="E319" s="79" t="inlineStr">
@@ -20791,7 +20791,7 @@
       </c>
       <c r="F319" s="77" t="inlineStr">
         <is>
-          <t>UALANI_FORGE_01 (intimate choice)</t>
+          <t>UALANI_WOUNDED_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G319" s="77" t="inlineStr">
@@ -20823,7 +20823,7 @@
       </c>
       <c r="N319" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_FORGE_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_WOUNDED_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20835,17 +20835,17 @@
       </c>
       <c r="B320" s="75" t="inlineStr">
         <is>
-          <t>Culper Ring</t>
+          <t>Forge Inspection</t>
         </is>
       </c>
       <c r="C320" s="76" t="inlineStr">
         <is>
-          <t>UALANI_CULPER_01_INTIMATE</t>
+          <t>UALANI_FORGE_01_INTIMATE</t>
         </is>
       </c>
       <c r="D320" s="77" t="inlineStr">
         <is>
-          <t>CULPER RING CONTACT AT [TILE_NAME]: INTELLIGENCE ASS... — BY MORNING</t>
+          <t>PRESIDENT CARLISLE CONDUCTS SURPRISE INSPECTION OF F... — BY MORNING</t>
         </is>
       </c>
       <c r="E320" s="79" t="inlineStr">
@@ -20855,7 +20855,7 @@
       </c>
       <c r="F320" s="77" t="inlineStr">
         <is>
-          <t>UALANI_CULPER_01 (intimate choice)</t>
+          <t>UALANI_FORGE_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G320" s="77" t="inlineStr">
@@ -20887,7 +20887,7 @@
       </c>
       <c r="N320" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_CULPER_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_FORGE_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20899,17 +20899,17 @@
       </c>
       <c r="B321" s="75" t="inlineStr">
         <is>
-          <t>Alliance Council</t>
+          <t>Culper Ring</t>
         </is>
       </c>
       <c r="C321" s="76" t="inlineStr">
         <is>
-          <t>UALANI_ALLIANCE_01_INTIMATE</t>
+          <t>UALANI_CULPER_01_INTIMATE</t>
         </is>
       </c>
       <c r="D321" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE MEETS WITH [COMMANDER_NAME] AT [T... — BY MORNING</t>
+          <t>CULPER RING CONTACT AT [TILE_NAME]: INTELLIGENCE ASS... — BY MORNING</t>
         </is>
       </c>
       <c r="E321" s="79" t="inlineStr">
@@ -20919,7 +20919,7 @@
       </c>
       <c r="F321" s="77" t="inlineStr">
         <is>
-          <t>UALANI_ALLIANCE_01 (intimate choice)</t>
+          <t>UALANI_CULPER_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G321" s="77" t="inlineStr">
@@ -20951,7 +20951,7 @@
       </c>
       <c r="N321" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_ALLIANCE_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_CULPER_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20963,17 +20963,17 @@
       </c>
       <c r="B322" s="75" t="inlineStr">
         <is>
-          <t>Frontier</t>
+          <t>Alliance Council</t>
         </is>
       </c>
       <c r="C322" s="76" t="inlineStr">
         <is>
-          <t>UALANI_FRONTIER_01_INTIMATE</t>
+          <t>UALANI_ALLIANCE_01_INTIMATE</t>
         </is>
       </c>
       <c r="D322" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE ESTABLISHES FRONTIER PRESENCE AT ... — BY MORNING</t>
+          <t>PRESIDENT CARLISLE MEETS WITH [COMMANDER_NAME] AT [T... — BY MORNING</t>
         </is>
       </c>
       <c r="E322" s="79" t="inlineStr">
@@ -20983,7 +20983,7 @@
       </c>
       <c r="F322" s="77" t="inlineStr">
         <is>
-          <t>UALANI_FRONTIER_01 (intimate choice)</t>
+          <t>UALANI_ALLIANCE_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G322" s="77" t="inlineStr">
@@ -21015,89 +21015,89 @@
       </c>
       <c r="N322" s="77" t="inlineStr">
         <is>
+          <t>Stub — author intimate version of UALANI_ALLIANCE_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="30" customHeight="1">
+      <c r="A323" s="75" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B323" s="75" t="inlineStr">
+        <is>
+          <t>Frontier</t>
+        </is>
+      </c>
+      <c r="C323" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_FRONTIER_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D323" s="77" t="inlineStr">
+        <is>
+          <t>PRESIDENT CARLISLE ESTABLISHES FRONTIER PRESENCE AT ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E323" s="79" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F323" s="77" t="inlineStr">
+        <is>
+          <t>UALANI_FRONTIER_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G323" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H323" s="78" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I323" s="76" t="inlineStr"/>
+      <c r="J323" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K323" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L323" s="76" t="inlineStr"/>
+      <c r="M323" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N323" s="77" t="inlineStr">
+        <is>
           <t>Stub — author intimate version of UALANI_FRONTIER_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
-    <row r="323" ht="8" customHeight="1">
-      <c r="A323" s="9" t="n"/>
-      <c r="B323" s="9" t="n"/>
-      <c r="C323" s="9" t="n"/>
-      <c r="D323" s="9" t="n"/>
-      <c r="E323" s="9" t="n"/>
-      <c r="F323" s="9" t="n"/>
-      <c r="G323" s="9" t="n"/>
-      <c r="H323" s="9" t="n"/>
-      <c r="I323" s="9" t="n"/>
-      <c r="J323" s="9" t="n"/>
-      <c r="K323" s="9" t="n"/>
-      <c r="L323" s="9" t="n"/>
-      <c r="M323" s="9" t="n"/>
-      <c r="N323" s="9" t="n"/>
-    </row>
-    <row r="324" ht="30" customHeight="1">
-      <c r="A324" s="75" t="inlineStr">
-        <is>
-          <t>Protector</t>
-        </is>
-      </c>
-      <c r="B324" s="75" t="inlineStr">
-        <is>
-          <t>Mothman</t>
-        </is>
-      </c>
-      <c r="C324" s="76" t="inlineStr">
-        <is>
-          <t>PROT_01_AGREE_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D324" s="77" t="inlineStr">
-        <is>
-          <t>MOTHMAN FORMALLY ALLIES WITH THE CONTINENTAL REPUBLIC — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E324" s="79" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="F324" s="77" t="inlineStr">
-        <is>
-          <t>PROT_01_AGREE (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G324" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H324" s="78" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I324" s="76" t="inlineStr"/>
-      <c r="J324" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K324" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L324" s="76" t="inlineStr"/>
-      <c r="M324" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N324" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
+    <row r="324" ht="8" customHeight="1">
+      <c r="A324" s="9" t="n"/>
+      <c r="B324" s="9" t="n"/>
+      <c r="C324" s="9" t="n"/>
+      <c r="D324" s="9" t="n"/>
+      <c r="E324" s="9" t="n"/>
+      <c r="F324" s="9" t="n"/>
+      <c r="G324" s="9" t="n"/>
+      <c r="H324" s="9" t="n"/>
+      <c r="I324" s="9" t="n"/>
+      <c r="J324" s="9" t="n"/>
+      <c r="K324" s="9" t="n"/>
+      <c r="L324" s="9" t="n"/>
+      <c r="M324" s="9" t="n"/>
+      <c r="N324" s="9" t="n"/>
     </row>
     <row r="325" ht="30" customHeight="1">
       <c r="A325" s="75" t="inlineStr">
@@ -21107,17 +21107,17 @@
       </c>
       <c r="B325" s="75" t="inlineStr">
         <is>
-          <t>Jersey Devil</t>
+          <t>Mothman</t>
         </is>
       </c>
       <c r="C325" s="76" t="inlineStr">
         <is>
-          <t>PROT_02_AGREE_INTIMATE</t>
+          <t>PROT_01_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D325" s="77" t="inlineStr">
         <is>
-          <t>JERSEY DEVIL FORMALLY ENDORSES THE CONTINENTAL CAUSE — BY MORNING</t>
+          <t>MOTHMAN FORMALLY ALLIES WITH THE CONTINENTAL REPUBLIC — BY MORNING</t>
         </is>
       </c>
       <c r="E325" s="79" t="inlineStr">
@@ -21127,7 +21127,7 @@
       </c>
       <c r="F325" s="77" t="inlineStr">
         <is>
-          <t>PROT_02_AGREE (intimate choice)</t>
+          <t>PROT_01_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G325" s="77" t="inlineStr">
@@ -21159,7 +21159,7 @@
       </c>
       <c r="N325" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21171,17 +21171,17 @@
       </c>
       <c r="B326" s="75" t="inlineStr">
         <is>
-          <t>Bigfoot</t>
+          <t>Jersey Devil</t>
         </is>
       </c>
       <c r="C326" s="76" t="inlineStr">
         <is>
-          <t>PROT_03_AGREE_INTIMATE</t>
+          <t>PROT_02_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D326" s="77" t="inlineStr">
         <is>
-          <t>BIGFOOT FORMALLY GUIDES THE CONTINENTAL CAUSE THROUG... — BY MORNING</t>
+          <t>JERSEY DEVIL FORMALLY ENDORSES THE CONTINENTAL CAUSE — BY MORNING</t>
         </is>
       </c>
       <c r="E326" s="79" t="inlineStr">
@@ -21191,7 +21191,7 @@
       </c>
       <c r="F326" s="77" t="inlineStr">
         <is>
-          <t>PROT_03_AGREE (intimate choice)</t>
+          <t>PROT_02_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G326" s="77" t="inlineStr">
@@ -21223,7 +21223,7 @@
       </c>
       <c r="N326" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21235,17 +21235,17 @@
       </c>
       <c r="B327" s="75" t="inlineStr">
         <is>
-          <t>Thunderbird</t>
+          <t>Bigfoot</t>
         </is>
       </c>
       <c r="C327" s="76" t="inlineStr">
         <is>
-          <t>PROT_04_AGREE_INTIMATE</t>
+          <t>PROT_03_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D327" s="77" t="inlineStr">
         <is>
-          <t>THUNDERBIRD FORMALLY ALLIES WITH THE CONTINENTAL REP... — BY MORNING</t>
+          <t>BIGFOOT FORMALLY GUIDES THE CONTINENTAL CAUSE THROUG... — BY MORNING</t>
         </is>
       </c>
       <c r="E327" s="79" t="inlineStr">
@@ -21255,7 +21255,7 @@
       </c>
       <c r="F327" s="77" t="inlineStr">
         <is>
-          <t>PROT_04_AGREE (intimate choice)</t>
+          <t>PROT_03_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G327" s="77" t="inlineStr">
@@ -21287,7 +21287,7 @@
       </c>
       <c r="N327" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21299,17 +21299,17 @@
       </c>
       <c r="B328" s="75" t="inlineStr">
         <is>
-          <t>Headless Horseman</t>
+          <t>Thunderbird</t>
         </is>
       </c>
       <c r="C328" s="76" t="inlineStr">
         <is>
-          <t>PROT_05_AGREE_INTIMATE</t>
+          <t>PROT_04_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D328" s="77" t="inlineStr">
         <is>
-          <t>THE HORSEMAN RIDES FOR THE REPUBLIC — FORMALLY — BY MORNING</t>
+          <t>THUNDERBIRD FORMALLY ALLIES WITH THE CONTINENTAL REP... — BY MORNING</t>
         </is>
       </c>
       <c r="E328" s="79" t="inlineStr">
@@ -21319,7 +21319,7 @@
       </c>
       <c r="F328" s="77" t="inlineStr">
         <is>
-          <t>PROT_05_AGREE (intimate choice)</t>
+          <t>PROT_04_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G328" s="77" t="inlineStr">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="N328" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21363,17 +21363,17 @@
       </c>
       <c r="B329" s="75" t="inlineStr">
         <is>
-          <t>Chessie</t>
+          <t>Headless Horseman</t>
         </is>
       </c>
       <c r="C329" s="76" t="inlineStr">
         <is>
-          <t>PROT_06_AGREE_INTIMATE</t>
+          <t>PROT_05_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D329" s="77" t="inlineStr">
         <is>
-          <t>CHESSIE FORMALLY PATROLS FOR THE CONTINENTAL NAVY — BY MORNING</t>
+          <t>THE HORSEMAN RIDES FOR THE REPUBLIC — FORMALLY — BY MORNING</t>
         </is>
       </c>
       <c r="E329" s="79" t="inlineStr">
@@ -21383,7 +21383,7 @@
       </c>
       <c r="F329" s="77" t="inlineStr">
         <is>
-          <t>PROT_06_AGREE (intimate choice)</t>
+          <t>PROT_05_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G329" s="77" t="inlineStr">
@@ -21415,7 +21415,7 @@
       </c>
       <c r="N329" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21427,17 +21427,17 @@
       </c>
       <c r="B330" s="75" t="inlineStr">
         <is>
-          <t>Bell Witch</t>
+          <t>Chessie</t>
         </is>
       </c>
       <c r="C330" s="76" t="inlineStr">
         <is>
-          <t>PROT_07_AGREE_INTIMATE</t>
+          <t>PROT_06_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D330" s="77" t="inlineStr">
         <is>
-          <t>THE BELL WITCH FORMALLY COMMITS TO THE CONTINENTAL C... — BY MORNING</t>
+          <t>CHESSIE FORMALLY PATROLS FOR THE CONTINENTAL NAVY — BY MORNING</t>
         </is>
       </c>
       <c r="E330" s="79" t="inlineStr">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="F330" s="77" t="inlineStr">
         <is>
-          <t>PROT_07_AGREE (intimate choice)</t>
+          <t>PROT_06_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G330" s="77" t="inlineStr">
@@ -21479,7 +21479,7 @@
       </c>
       <c r="N330" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21491,17 +21491,17 @@
       </c>
       <c r="B331" s="75" t="inlineStr">
         <is>
-          <t>Old Ironsides</t>
+          <t>Bell Witch</t>
         </is>
       </c>
       <c r="C331" s="76" t="inlineStr">
         <is>
-          <t>PROT_08_AGREE_INTIMATE</t>
+          <t>PROT_07_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D331" s="77" t="inlineStr">
         <is>
-          <t>OLD IRONSIDES FORMALLY JOINS THE CONTINENTAL NAVY — BY MORNING</t>
+          <t>THE BELL WITCH FORMALLY COMMITS TO THE CONTINENTAL C... — BY MORNING</t>
         </is>
       </c>
       <c r="E331" s="79" t="inlineStr">
@@ -21511,7 +21511,7 @@
       </c>
       <c r="F331" s="77" t="inlineStr">
         <is>
-          <t>PROT_08_AGREE (intimate choice)</t>
+          <t>PROT_07_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G331" s="77" t="inlineStr">
@@ -21543,7 +21543,7 @@
       </c>
       <c r="N331" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21555,17 +21555,17 @@
       </c>
       <c r="B332" s="75" t="inlineStr">
         <is>
-          <t>Valley Forge Guardian</t>
+          <t>Old Ironsides</t>
         </is>
       </c>
       <c r="C332" s="76" t="inlineStr">
         <is>
-          <t>PROT_09_AGREE_INTIMATE</t>
+          <t>PROT_08_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D332" s="77" t="inlineStr">
         <is>
-          <t>VALLEY FORGE GUARDIAN FORMALLY BLESSES THE CONTINENT... — BY MORNING</t>
+          <t>OLD IRONSIDES FORMALLY JOINS THE CONTINENTAL NAVY — BY MORNING</t>
         </is>
       </c>
       <c r="E332" s="79" t="inlineStr">
@@ -21575,7 +21575,7 @@
       </c>
       <c r="F332" s="77" t="inlineStr">
         <is>
-          <t>PROT_09_AGREE (intimate choice)</t>
+          <t>PROT_08_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G332" s="77" t="inlineStr">
@@ -21607,7 +21607,7 @@
       </c>
       <c r="N332" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_09_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21619,17 +21619,17 @@
       </c>
       <c r="B333" s="75" t="inlineStr">
         <is>
-          <t>Snallygaster</t>
+          <t>Valley Forge Guardian</t>
         </is>
       </c>
       <c r="C333" s="76" t="inlineStr">
         <is>
-          <t>PROT_10_AGREE_INTIMATE</t>
+          <t>PROT_09_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D333" s="77" t="inlineStr">
         <is>
-          <t>SNALLYGASTER FORMALLY GUARDS THE CONTINENTAL SUPPLY ... — BY MORNING</t>
+          <t>VALLEY FORGE GUARDIAN FORMALLY BLESSES THE CONTINENT... — BY MORNING</t>
         </is>
       </c>
       <c r="E333" s="79" t="inlineStr">
@@ -21639,7 +21639,7 @@
       </c>
       <c r="F333" s="77" t="inlineStr">
         <is>
-          <t>PROT_10_AGREE (intimate choice)</t>
+          <t>PROT_09_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G333" s="77" t="inlineStr">
@@ -21671,7 +21671,7 @@
       </c>
       <c r="N333" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_10_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_09_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21683,17 +21683,17 @@
       </c>
       <c r="B334" s="75" t="inlineStr">
         <is>
-          <t>Paul Revere</t>
+          <t>Snallygaster</t>
         </is>
       </c>
       <c r="C334" s="76" t="inlineStr">
         <is>
-          <t>PROT_11_AGREE_INTIMATE</t>
+          <t>PROT_10_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D334" s="77" t="inlineStr">
         <is>
-          <t>PAUL REVERE FORMALLY INTEGRATES WITH CONTINENTAL INT... — BY MORNING</t>
+          <t>SNALLYGASTER FORMALLY GUARDS THE CONTINENTAL SUPPLY ... — BY MORNING</t>
         </is>
       </c>
       <c r="E334" s="79" t="inlineStr">
@@ -21703,7 +21703,7 @@
       </c>
       <c r="F334" s="77" t="inlineStr">
         <is>
-          <t>PROT_11_AGREE (intimate choice)</t>
+          <t>PROT_10_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G334" s="77" t="inlineStr">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="N334" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_11_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_10_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21747,17 +21747,17 @@
       </c>
       <c r="B335" s="75" t="inlineStr">
         <is>
-          <t>Liberty Bell</t>
+          <t>Paul Revere</t>
         </is>
       </c>
       <c r="C335" s="76" t="inlineStr">
         <is>
-          <t>PROT_12_AGREE_INTIMATE</t>
+          <t>PROT_11_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D335" s="77" t="inlineStr">
         <is>
-          <t>THE LIBERTY BELL FORMALLY RINGS FOR THE REPUBLIC — BY MORNING</t>
+          <t>PAUL REVERE FORMALLY INTEGRATES WITH CONTINENTAL INT... — BY MORNING</t>
         </is>
       </c>
       <c r="E335" s="79" t="inlineStr">
@@ -21767,7 +21767,7 @@
       </c>
       <c r="F335" s="77" t="inlineStr">
         <is>
-          <t>PROT_12_AGREE (intimate choice)</t>
+          <t>PROT_11_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G335" s="77" t="inlineStr">
@@ -21799,7 +21799,7 @@
       </c>
       <c r="N335" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_12_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_11_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21811,17 +21811,17 @@
       </c>
       <c r="B336" s="75" t="inlineStr">
         <is>
-          <t>Green Mountain Ghost</t>
+          <t>Liberty Bell</t>
         </is>
       </c>
       <c r="C336" s="76" t="inlineStr">
         <is>
-          <t>PROT_13_AGREE_INTIMATE</t>
+          <t>PROT_12_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D336" s="77" t="inlineStr">
         <is>
-          <t>GREEN MOUNTAIN GHOST FORMALLY PROTECTS VERMONT FOR T... — BY MORNING</t>
+          <t>THE LIBERTY BELL FORMALLY RINGS FOR THE REPUBLIC — BY MORNING</t>
         </is>
       </c>
       <c r="E336" s="79" t="inlineStr">
@@ -21831,7 +21831,7 @@
       </c>
       <c r="F336" s="77" t="inlineStr">
         <is>
-          <t>PROT_13_AGREE (intimate choice)</t>
+          <t>PROT_12_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G336" s="77" t="inlineStr">
@@ -21863,7 +21863,7 @@
       </c>
       <c r="N336" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_13_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_12_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21875,17 +21875,17 @@
       </c>
       <c r="B337" s="75" t="inlineStr">
         <is>
-          <t>Mount Rushmore</t>
+          <t>Green Mountain Ghost</t>
         </is>
       </c>
       <c r="C337" s="76" t="inlineStr">
         <is>
-          <t>PROT_14_AGREE_INTIMATE</t>
+          <t>PROT_13_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D337" s="77" t="inlineStr">
         <is>
-          <t>THE RUSHMORE COUNCIL FORMALLY ENDORSES PRESIDENT CAR... — BY MORNING</t>
+          <t>GREEN MOUNTAIN GHOST FORMALLY PROTECTS VERMONT FOR T... — BY MORNING</t>
         </is>
       </c>
       <c r="E337" s="79" t="inlineStr">
@@ -21895,7 +21895,7 @@
       </c>
       <c r="F337" s="77" t="inlineStr">
         <is>
-          <t>PROT_14_AGREE (intimate choice)</t>
+          <t>PROT_13_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G337" s="77" t="inlineStr">
@@ -21927,7 +21927,7 @@
       </c>
       <c r="N337" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_14_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_13_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21939,17 +21939,17 @@
       </c>
       <c r="B338" s="75" t="inlineStr">
         <is>
-          <t>Skunk Ape</t>
+          <t>Mount Rushmore</t>
         </is>
       </c>
       <c r="C338" s="76" t="inlineStr">
         <is>
-          <t>PROT_15_AGREE_INTIMATE</t>
+          <t>PROT_14_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D338" s="77" t="inlineStr">
         <is>
-          <t>SKUNK APE FORMALLY PATROLS FLORIDA FOR THE CONTINENT... — BY MORNING</t>
+          <t>THE RUSHMORE COUNCIL FORMALLY ENDORSES PRESIDENT CAR... — BY MORNING</t>
         </is>
       </c>
       <c r="E338" s="79" t="inlineStr">
@@ -21959,7 +21959,7 @@
       </c>
       <c r="F338" s="77" t="inlineStr">
         <is>
-          <t>PROT_15_AGREE (intimate choice)</t>
+          <t>PROT_14_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G338" s="77" t="inlineStr">
@@ -21991,7 +21991,7 @@
       </c>
       <c r="N338" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_15_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_14_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22003,17 +22003,17 @@
       </c>
       <c r="B339" s="75" t="inlineStr">
         <is>
-          <t>Minuteman</t>
+          <t>Skunk Ape</t>
         </is>
       </c>
       <c r="C339" s="76" t="inlineStr">
         <is>
-          <t>PROT_16_AGREE_INTIMATE</t>
+          <t>PROT_15_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D339" s="77" t="inlineStr">
         <is>
-          <t>THE MINUTEMAN FORMALLY DECLARES FOR THE CONTINENTAL ... — BY MORNING</t>
+          <t>SKUNK APE FORMALLY PATROLS FLORIDA FOR THE CONTINENT... — BY MORNING</t>
         </is>
       </c>
       <c r="E339" s="79" t="inlineStr">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="F339" s="77" t="inlineStr">
         <is>
-          <t>PROT_16_AGREE (intimate choice)</t>
+          <t>PROT_15_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G339" s="77" t="inlineStr">
@@ -22055,7 +22055,7 @@
       </c>
       <c r="N339" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_16_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_15_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22067,17 +22067,17 @@
       </c>
       <c r="B340" s="75" t="inlineStr">
         <is>
-          <t>Lincoln's Ghost</t>
+          <t>Minuteman</t>
         </is>
       </c>
       <c r="C340" s="76" t="inlineStr">
         <is>
-          <t>PROT_17_AGREE_INTIMATE</t>
+          <t>PROT_16_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D340" s="77" t="inlineStr">
         <is>
-          <t>LINCOLN FORMALLY ENDORSES PRESIDENT CARLISLE'S ADMIN... — BY MORNING</t>
+          <t>THE MINUTEMAN FORMALLY DECLARES FOR THE CONTINENTAL ... — BY MORNING</t>
         </is>
       </c>
       <c r="E340" s="79" t="inlineStr">
@@ -22087,7 +22087,7 @@
       </c>
       <c r="F340" s="77" t="inlineStr">
         <is>
-          <t>PROT_17_AGREE (intimate choice)</t>
+          <t>PROT_16_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G340" s="77" t="inlineStr">
@@ -22119,89 +22119,89 @@
       </c>
       <c r="N340" s="77" t="inlineStr">
         <is>
+          <t>Stub — author intimate version of PROT_16_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="30" customHeight="1">
+      <c r="A341" s="75" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B341" s="75" t="inlineStr">
+        <is>
+          <t>Lincoln's Ghost</t>
+        </is>
+      </c>
+      <c r="C341" s="76" t="inlineStr">
+        <is>
+          <t>PROT_17_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D341" s="77" t="inlineStr">
+        <is>
+          <t>LINCOLN FORMALLY ENDORSES PRESIDENT CARLISLE'S ADMIN... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E341" s="79" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F341" s="77" t="inlineStr">
+        <is>
+          <t>PROT_17_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G341" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H341" s="78" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I341" s="76" t="inlineStr"/>
+      <c r="J341" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K341" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L341" s="76" t="inlineStr"/>
+      <c r="M341" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N341" s="77" t="inlineStr">
+        <is>
           <t>Stub — author intimate version of PROT_17_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
-    <row r="341" ht="8" customHeight="1">
-      <c r="A341" s="9" t="n"/>
-      <c r="B341" s="9" t="n"/>
-      <c r="C341" s="9" t="n"/>
-      <c r="D341" s="9" t="n"/>
-      <c r="E341" s="9" t="n"/>
-      <c r="F341" s="9" t="n"/>
-      <c r="G341" s="9" t="n"/>
-      <c r="H341" s="9" t="n"/>
-      <c r="I341" s="9" t="n"/>
-      <c r="J341" s="9" t="n"/>
-      <c r="K341" s="9" t="n"/>
-      <c r="L341" s="9" t="n"/>
-      <c r="M341" s="9" t="n"/>
-      <c r="N341" s="9" t="n"/>
-    </row>
-    <row r="342" ht="30" customHeight="1">
-      <c r="A342" s="75" t="inlineStr">
-        <is>
-          <t>White House</t>
-        </is>
-      </c>
-      <c r="B342" s="75" t="inlineStr">
-        <is>
-          <t>Month 1</t>
-        </is>
-      </c>
-      <c r="C342" s="76" t="inlineStr">
-        <is>
-          <t>WH_SECRET_01_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D342" s="77" t="inlineStr">
-        <is>
-          <t>THE WHITE HOUSE AT MIDNIGHT — THE PRESIDENT WATCHES ... — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E342" s="79" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="F342" s="77" t="inlineStr">
-        <is>
-          <t>WH_SECRET_01 (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G342" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H342" s="78" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I342" s="76" t="inlineStr"/>
-      <c r="J342" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K342" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L342" s="76" t="inlineStr"/>
-      <c r="M342" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N342" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of WH_SECRET_01. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
+    <row r="342" ht="8" customHeight="1">
+      <c r="A342" s="9" t="n"/>
+      <c r="B342" s="9" t="n"/>
+      <c r="C342" s="9" t="n"/>
+      <c r="D342" s="9" t="n"/>
+      <c r="E342" s="9" t="n"/>
+      <c r="F342" s="9" t="n"/>
+      <c r="G342" s="9" t="n"/>
+      <c r="H342" s="9" t="n"/>
+      <c r="I342" s="9" t="n"/>
+      <c r="J342" s="9" t="n"/>
+      <c r="K342" s="9" t="n"/>
+      <c r="L342" s="9" t="n"/>
+      <c r="M342" s="9" t="n"/>
+      <c r="N342" s="9" t="n"/>
     </row>
     <row r="343" ht="30" customHeight="1">
       <c r="A343" s="75" t="inlineStr">
@@ -22211,17 +22211,17 @@
       </c>
       <c r="B343" s="75" t="inlineStr">
         <is>
-          <t>Month 7</t>
+          <t>Month 1</t>
         </is>
       </c>
       <c r="C343" s="76" t="inlineStr">
         <is>
-          <t>WH_SECRET_07_INTIMATE</t>
+          <t>WH_SECRET_01_INTIMATE</t>
         </is>
       </c>
       <c r="D343" s="77" t="inlineStr">
         <is>
-          <t>JULY AT THE WHITE HOUSE — INDEPENDENCE DAY IS ALSO HERS — BY MORNING</t>
+          <t>THE WHITE HOUSE AT MIDNIGHT — THE PRESIDENT WATCHES ... — BY MORNING</t>
         </is>
       </c>
       <c r="E343" s="79" t="inlineStr">
@@ -22231,7 +22231,7 @@
       </c>
       <c r="F343" s="77" t="inlineStr">
         <is>
-          <t>WH_SECRET_07 (intimate choice)</t>
+          <t>WH_SECRET_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G343" s="77" t="inlineStr">
@@ -22263,7 +22263,7 @@
       </c>
       <c r="N343" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of WH_SECRET_07. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of WH_SECRET_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22275,17 +22275,17 @@
       </c>
       <c r="B344" s="75" t="inlineStr">
         <is>
-          <t>Month 10</t>
+          <t>Month 7</t>
         </is>
       </c>
       <c r="C344" s="76" t="inlineStr">
         <is>
-          <t>WH_SECRET_10_INTIMATE</t>
+          <t>WH_SECRET_07_INTIMATE</t>
         </is>
       </c>
       <c r="D344" s="77" t="inlineStr">
         <is>
-          <t>INDIGENOUS PEOPLES DAY — A PERSONAL LETTER FROM JESS... — BY MORNING</t>
+          <t>JULY AT THE WHITE HOUSE — INDEPENDENCE DAY IS ALSO HERS — BY MORNING</t>
         </is>
       </c>
       <c r="E344" s="79" t="inlineStr">
@@ -22295,7 +22295,7 @@
       </c>
       <c r="F344" s="77" t="inlineStr">
         <is>
-          <t>WH_SECRET_10 (intimate choice)</t>
+          <t>WH_SECRET_07 (intimate choice)</t>
         </is>
       </c>
       <c r="G344" s="77" t="inlineStr">
@@ -22327,7 +22327,7 @@
       </c>
       <c r="N344" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of WH_SECRET_10. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of WH_SECRET_07. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22339,17 +22339,17 @@
       </c>
       <c r="B345" s="75" t="inlineStr">
         <is>
-          <t>Month 12</t>
+          <t>Month 10</t>
         </is>
       </c>
       <c r="C345" s="76" t="inlineStr">
         <is>
-          <t>WH_SECRET_12_INTIMATE</t>
+          <t>WH_SECRET_10_INTIMATE</t>
         </is>
       </c>
       <c r="D345" s="77" t="inlineStr">
         <is>
-          <t>CHRISTMAS IN WASHINGTON — THE PRESIDENT IS FAR FROM ... — BY MORNING</t>
+          <t>INDIGENOUS PEOPLES DAY — A PERSONAL LETTER FROM JESS... — BY MORNING</t>
         </is>
       </c>
       <c r="E345" s="79" t="inlineStr">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="F345" s="77" t="inlineStr">
         <is>
-          <t>WH_SECRET_12 (intimate choice)</t>
+          <t>WH_SECRET_10 (intimate choice)</t>
         </is>
       </c>
       <c r="G345" s="77" t="inlineStr">
@@ -22391,47 +22391,111 @@
       </c>
       <c r="N345" s="77" t="inlineStr">
         <is>
+          <t>Stub — author intimate version of WH_SECRET_10. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="30" customHeight="1">
+      <c r="A346" s="75" t="inlineStr">
+        <is>
+          <t>White House</t>
+        </is>
+      </c>
+      <c r="B346" s="75" t="inlineStr">
+        <is>
+          <t>Month 12</t>
+        </is>
+      </c>
+      <c r="C346" s="76" t="inlineStr">
+        <is>
+          <t>WH_SECRET_12_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D346" s="77" t="inlineStr">
+        <is>
+          <t>CHRISTMAS IN WASHINGTON — THE PRESIDENT IS FAR FROM ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E346" s="79" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F346" s="77" t="inlineStr">
+        <is>
+          <t>WH_SECRET_12 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G346" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H346" s="78" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I346" s="76" t="inlineStr"/>
+      <c r="J346" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K346" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L346" s="76" t="inlineStr"/>
+      <c r="M346" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N346" s="77" t="inlineStr">
+        <is>
           <t>Stub — author intimate version of WH_SECRET_12. By morning: emotional arc, no explicit imagery.</t>
         </is>
-      </c>
-    </row>
-    <row r="347" ht="20" customHeight="1">
-      <c r="A347" s="81" t="inlineStr">
-        <is>
-          <t>Total events in spreadsheet</t>
-        </is>
-      </c>
-      <c r="B347" s="82" t="n">
-        <v>314</v>
       </c>
     </row>
     <row r="348" ht="20" customHeight="1">
       <c r="A348" s="81" t="inlineStr">
         <is>
-          <t>FIRST PASS (coded &amp; wired)</t>
+          <t>Total events in spreadsheet</t>
         </is>
       </c>
       <c r="B348" s="82" t="n">
-        <v>248</v>
+        <v>315</v>
       </c>
     </row>
     <row r="349" ht="20" customHeight="1">
       <c r="A349" s="81" t="inlineStr">
         <is>
-          <t>IDEA (not yet implemented)</t>
+          <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
       <c r="B349" s="82" t="n">
-        <v>64</v>
+        <v>249</v>
       </c>
     </row>
     <row r="350" ht="20" customHeight="1">
       <c r="A350" s="81" t="inlineStr">
         <is>
+          <t>IDEA (not yet implemented)</t>
+        </is>
+      </c>
+      <c r="B350" s="82" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="351" ht="20" customHeight="1">
+      <c r="A351" s="81" t="inlineStr">
+        <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B350" s="82" t="n">
+      <c r="B351" s="82" t="n">
         <v>55</v>
       </c>
     </row>
@@ -22446,7 +22510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N63"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22747,7 +22811,7 @@
       </c>
       <c r="D5" s="55" t="inlineStr">
         <is>
-          <t>PRESIDENT PENOIT'S CONDITIONS: MARK PENOIT PUTS IT IN WRITING</t>
+          <t>PRESIDENT PENOIT'S CONDITIONS: MARC PENOIT PUTS IT IN WRITING</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
@@ -25625,85 +25689,85 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="8" customHeight="1">
-      <c r="A50" s="9" t="n"/>
-      <c r="B50" s="9" t="n"/>
-      <c r="C50" s="9" t="n"/>
-      <c r="D50" s="9" t="n"/>
-      <c r="E50" s="9" t="n"/>
-      <c r="F50" s="9" t="n"/>
-      <c r="G50" s="9" t="n"/>
-      <c r="H50" s="9" t="n"/>
-      <c r="I50" s="9" t="n"/>
-      <c r="J50" s="9" t="n"/>
-      <c r="K50" s="9" t="n"/>
-      <c r="L50" s="9" t="n"/>
-      <c r="M50" s="9" t="n"/>
-      <c r="N50" s="9" t="n"/>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="75" t="inlineStr">
-        <is>
-          <t>CA Protector</t>
-        </is>
-      </c>
-      <c r="B51" s="75" t="inlineStr">
-        <is>
-          <t>Le Wendigo</t>
-        </is>
-      </c>
-      <c r="C51" s="76" t="inlineStr">
-        <is>
-          <t>CA_PROT_01_AGREE_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D51" s="77" t="inlineStr">
-        <is>
-          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E51" s="79" t="inlineStr">
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="53" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B50" s="53" t="inlineStr">
+        <is>
+          <t>PM Arc</t>
+        </is>
+      </c>
+      <c r="C50" s="54" t="inlineStr">
+        <is>
+          <t>CA_PM_LEGACY_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D50" s="55" t="inlineStr">
+        <is>
+          <t>MARC PENOIT'S FINAL ASSESSMENT — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E50" s="56" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F51" s="77" t="inlineStr">
-        <is>
-          <t>CA_PROT_01_AGREE (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G51" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H51" s="78" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I51" s="76" t="inlineStr"/>
-      <c r="J51" s="80" t="inlineStr">
+      <c r="F50" s="55" t="inlineStr">
+        <is>
+          <t>CA_PM_LEGACY (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G50" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
+        </is>
+      </c>
+      <c r="I50" s="54" t="inlineStr"/>
+      <c r="J50" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K51" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L51" s="76" t="inlineStr"/>
-      <c r="M51" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N51" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
+      <c r="K50" s="56" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L50" s="54" t="inlineStr"/>
+      <c r="M50" s="56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N50" s="55" t="inlineStr">
+        <is>
+          <t>By morning: Penoit at the desk before light, writing page forty-one. Emotional resolution — he was wrong about what this would feel like.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="8" customHeight="1">
+      <c r="A51" s="9" t="n"/>
+      <c r="B51" s="9" t="n"/>
+      <c r="C51" s="9" t="n"/>
+      <c r="D51" s="9" t="n"/>
+      <c r="E51" s="9" t="n"/>
+      <c r="F51" s="9" t="n"/>
+      <c r="G51" s="9" t="n"/>
+      <c r="H51" s="9" t="n"/>
+      <c r="I51" s="9" t="n"/>
+      <c r="J51" s="9" t="n"/>
+      <c r="K51" s="9" t="n"/>
+      <c r="L51" s="9" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="9" t="n"/>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="75" t="inlineStr">
@@ -25713,17 +25777,17 @@
       </c>
       <c r="B52" s="75" t="inlineStr">
         <is>
-          <t>Le Loup-Garou</t>
+          <t>Le Wendigo</t>
         </is>
       </c>
       <c r="C52" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE_INTIMATE</t>
+          <t>CA_PROT_01_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D52" s="77" t="inlineStr">
         <is>
-          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
+          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
         </is>
       </c>
       <c r="E52" s="79" t="inlineStr">
@@ -25733,7 +25797,7 @@
       </c>
       <c r="F52" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE (intimate choice)</t>
+          <t>CA_PROT_01_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G52" s="77" t="inlineStr">
@@ -25765,7 +25829,7 @@
       </c>
       <c r="N52" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -25777,17 +25841,17 @@
       </c>
       <c r="B53" s="75" t="inlineStr">
         <is>
-          <t>Les Feux Follets</t>
+          <t>Le Loup-Garou</t>
         </is>
       </c>
       <c r="C53" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE_INTIMATE</t>
+          <t>CA_PROT_02_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D53" s="77" t="inlineStr">
         <is>
-          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
+          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
         </is>
       </c>
       <c r="E53" s="79" t="inlineStr">
@@ -25797,7 +25861,7 @@
       </c>
       <c r="F53" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE (intimate choice)</t>
+          <t>CA_PROT_02_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G53" s="77" t="inlineStr">
@@ -25829,7 +25893,7 @@
       </c>
       <c r="N53" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -25841,17 +25905,17 @@
       </c>
       <c r="B54" s="75" t="inlineStr">
         <is>
-          <t>Mishepeshu</t>
+          <t>Les Feux Follets</t>
         </is>
       </c>
       <c r="C54" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE_INTIMATE</t>
+          <t>CA_PROT_03_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D54" s="77" t="inlineStr">
         <is>
-          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
+          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
         </is>
       </c>
       <c r="E54" s="79" t="inlineStr">
@@ -25861,7 +25925,7 @@
       </c>
       <c r="F54" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE (intimate choice)</t>
+          <t>CA_PROT_03_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G54" s="77" t="inlineStr">
@@ -25893,7 +25957,7 @@
       </c>
       <c r="N54" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -25905,17 +25969,17 @@
       </c>
       <c r="B55" s="75" t="inlineStr">
         <is>
-          <t>La Corriveau</t>
+          <t>Mishepeshu</t>
         </is>
       </c>
       <c r="C55" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE_INTIMATE</t>
+          <t>CA_PROT_04_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D55" s="77" t="inlineStr">
         <is>
-          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
+          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
         </is>
       </c>
       <c r="E55" s="79" t="inlineStr">
@@ -25925,7 +25989,7 @@
       </c>
       <c r="F55" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE (intimate choice)</t>
+          <t>CA_PROT_04_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G55" s="77" t="inlineStr">
@@ -25957,7 +26021,7 @@
       </c>
       <c r="N55" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -25969,17 +26033,17 @@
       </c>
       <c r="B56" s="75" t="inlineStr">
         <is>
-          <t>Le Carcajou</t>
+          <t>La Corriveau</t>
         </is>
       </c>
       <c r="C56" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE_INTIMATE</t>
+          <t>CA_PROT_05_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D56" s="77" t="inlineStr">
         <is>
-          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
+          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
         </is>
       </c>
       <c r="E56" s="79" t="inlineStr">
@@ -25989,7 +26053,7 @@
       </c>
       <c r="F56" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE (intimate choice)</t>
+          <t>CA_PROT_05_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G56" s="77" t="inlineStr">
@@ -26021,7 +26085,7 @@
       </c>
       <c r="N56" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -26033,17 +26097,17 @@
       </c>
       <c r="B57" s="75" t="inlineStr">
         <is>
-          <t>La Chasse-Galerie</t>
+          <t>Le Carcajou</t>
         </is>
       </c>
       <c r="C57" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE_INTIMATE</t>
+          <t>CA_PROT_06_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D57" s="77" t="inlineStr">
         <is>
-          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
+          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
         </is>
       </c>
       <c r="E57" s="79" t="inlineStr">
@@ -26053,7 +26117,7 @@
       </c>
       <c r="F57" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE (intimate choice)</t>
+          <t>CA_PROT_06_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G57" s="77" t="inlineStr">
@@ -26085,7 +26149,7 @@
       </c>
       <c r="N57" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -26097,17 +26161,17 @@
       </c>
       <c r="B58" s="75" t="inlineStr">
         <is>
-          <t>Le Gougou</t>
+          <t>La Chasse-Galerie</t>
         </is>
       </c>
       <c r="C58" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_08_AGREE_INTIMATE</t>
+          <t>CA_PROT_07_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D58" s="77" t="inlineStr">
         <is>
-          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
+          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
         </is>
       </c>
       <c r="E58" s="79" t="inlineStr">
@@ -26117,7 +26181,7 @@
       </c>
       <c r="F58" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_08_AGREE (intimate choice)</t>
+          <t>CA_PROT_07_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G58" s="77" t="inlineStr">
@@ -26149,47 +26213,111 @@
       </c>
       <c r="N58" s="77" t="inlineStr">
         <is>
+          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="75" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B59" s="75" t="inlineStr">
+        <is>
+          <t>Le Gougou</t>
+        </is>
+      </c>
+      <c r="C59" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D59" s="77" t="inlineStr">
+        <is>
+          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E59" s="79" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="F59" s="77" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G59" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H59" s="78" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I59" s="76" t="inlineStr"/>
+      <c r="J59" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K59" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L59" s="76" t="inlineStr"/>
+      <c r="M59" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N59" s="77" t="inlineStr">
+        <is>
           <t>Stub — author intimate version of CA_PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
-      </c>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="81" t="inlineStr">
-        <is>
-          <t>Canadian events total</t>
-        </is>
-      </c>
-      <c r="B60" s="82" t="n">
-        <v>54</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="81" t="inlineStr">
         <is>
-          <t>Canada (Alliance arc)</t>
+          <t>Canadian events total</t>
         </is>
       </c>
       <c r="B61" s="82" t="n">
-        <v>22</v>
+        <v>55</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="81" t="inlineStr">
         <is>
-          <t>CA Protector (Jessica's creatures)</t>
+          <t>Canada (Alliance arc)</t>
         </is>
       </c>
       <c r="B62" s="82" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="81" t="inlineStr">
         <is>
+          <t>CA Protector (Jessica's creatures)</t>
+        </is>
+      </c>
+      <c r="B63" s="82" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="81" t="inlineStr">
+        <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B63" s="82" t="n">
+      <c r="B64" s="82" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Redesign CA_PM_LEGACY as dynamic loyalty declaration; remove intimate path
Jessica is WLW — no intimate scene with Marc Penoit.
- Remove CA_PM_LEGACY_INTIMATE row from events.csv
- Remove sensual button (BTN2) and intimate button from event_buttons.csv
- Clear content_flag on CA_PM_LEGACY
- Remove CA_PM_LEGACY_INTIMATE from event masterdoc

CA_PM_LEGACY now dynamically assembles its long_desc at runtime:
- _build_ca_pm_legacy_data() in world.gd checks uk_ca_peace, Quebec tile
  ownership, ca_prot_01-08_agreed, and can_allied flags
- Paragraphs for Britain expelled, Quebec free, named protectors, and alliance
  are conditionally included based on player's actual run achievements
- Closes with "You are the best Prime Minister this country has had"
- createNewEvent() special-cases CA_PM_LEGACY to call build_from_data()

Update flavordoc and masterdoc notes to reflect new design.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -1140,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N351"/>
+  <dimension ref="A1:N350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19963,85 +19963,85 @@
         </is>
       </c>
     </row>
-    <row r="305" ht="30" customHeight="1">
-      <c r="A305" s="53" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="B305" s="53" t="inlineStr">
-        <is>
-          <t>PM Arc</t>
-        </is>
-      </c>
-      <c r="C305" s="54" t="inlineStr">
-        <is>
-          <t>CA_PM_LEGACY_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D305" s="55" t="inlineStr">
-        <is>
-          <t>MARC PENOIT'S FINAL ASSESSMENT — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E305" s="56" t="inlineStr">
+    <row r="305" ht="8" customHeight="1">
+      <c r="A305" s="9" t="n"/>
+      <c r="B305" s="9" t="n"/>
+      <c r="C305" s="9" t="n"/>
+      <c r="D305" s="9" t="n"/>
+      <c r="E305" s="9" t="n"/>
+      <c r="F305" s="9" t="n"/>
+      <c r="G305" s="9" t="n"/>
+      <c r="H305" s="9" t="n"/>
+      <c r="I305" s="9" t="n"/>
+      <c r="J305" s="9" t="n"/>
+      <c r="K305" s="9" t="n"/>
+      <c r="L305" s="9" t="n"/>
+      <c r="M305" s="9" t="n"/>
+      <c r="N305" s="9" t="n"/>
+    </row>
+    <row r="306" ht="30" customHeight="1">
+      <c r="A306" s="75" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B306" s="75" t="inlineStr">
+        <is>
+          <t>Le Wendigo</t>
+        </is>
+      </c>
+      <c r="C306" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D306" s="77" t="inlineStr">
+        <is>
+          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E306" s="79" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F305" s="55" t="inlineStr">
-        <is>
-          <t>CA_PM_LEGACY (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G305" s="55" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H305" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I305" s="54" t="inlineStr"/>
-      <c r="J305" s="80" t="inlineStr">
+      <c r="F306" s="77" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G306" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H306" s="78" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I306" s="76" t="inlineStr"/>
+      <c r="J306" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K305" s="56" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L305" s="54" t="inlineStr"/>
-      <c r="M305" s="56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N305" s="55" t="inlineStr">
-        <is>
-          <t>By morning: Penoit at the desk before light, writing page forty-one. Emotional resolution — he was wrong about what this would feel like.</t>
-        </is>
-      </c>
-    </row>
-    <row r="306" ht="8" customHeight="1">
-      <c r="A306" s="9" t="n"/>
-      <c r="B306" s="9" t="n"/>
-      <c r="C306" s="9" t="n"/>
-      <c r="D306" s="9" t="n"/>
-      <c r="E306" s="9" t="n"/>
-      <c r="F306" s="9" t="n"/>
-      <c r="G306" s="9" t="n"/>
-      <c r="H306" s="9" t="n"/>
-      <c r="I306" s="9" t="n"/>
-      <c r="J306" s="9" t="n"/>
-      <c r="K306" s="9" t="n"/>
-      <c r="L306" s="9" t="n"/>
-      <c r="M306" s="9" t="n"/>
-      <c r="N306" s="9" t="n"/>
+      <c r="K306" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L306" s="76" t="inlineStr"/>
+      <c r="M306" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N306" s="77" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
     </row>
     <row r="307" ht="30" customHeight="1">
       <c r="A307" s="75" t="inlineStr">
@@ -20051,17 +20051,17 @@
       </c>
       <c r="B307" s="75" t="inlineStr">
         <is>
-          <t>Le Wendigo</t>
+          <t>Le Loup-Garou</t>
         </is>
       </c>
       <c r="C307" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_01_AGREE_INTIMATE</t>
+          <t>CA_PROT_02_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D307" s="77" t="inlineStr">
         <is>
-          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
+          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
         </is>
       </c>
       <c r="E307" s="79" t="inlineStr">
@@ -20071,7 +20071,7 @@
       </c>
       <c r="F307" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_01_AGREE (intimate choice)</t>
+          <t>CA_PROT_02_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G307" s="77" t="inlineStr">
@@ -20103,7 +20103,7 @@
       </c>
       <c r="N307" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20115,17 +20115,17 @@
       </c>
       <c r="B308" s="75" t="inlineStr">
         <is>
-          <t>Le Loup-Garou</t>
+          <t>Les Feux Follets</t>
         </is>
       </c>
       <c r="C308" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE_INTIMATE</t>
+          <t>CA_PROT_03_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D308" s="77" t="inlineStr">
         <is>
-          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
+          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
         </is>
       </c>
       <c r="E308" s="79" t="inlineStr">
@@ -20135,7 +20135,7 @@
       </c>
       <c r="F308" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE (intimate choice)</t>
+          <t>CA_PROT_03_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G308" s="77" t="inlineStr">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="N308" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20179,17 +20179,17 @@
       </c>
       <c r="B309" s="75" t="inlineStr">
         <is>
-          <t>Les Feux Follets</t>
+          <t>Mishepeshu</t>
         </is>
       </c>
       <c r="C309" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE_INTIMATE</t>
+          <t>CA_PROT_04_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D309" s="77" t="inlineStr">
         <is>
-          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
+          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
         </is>
       </c>
       <c r="E309" s="79" t="inlineStr">
@@ -20199,7 +20199,7 @@
       </c>
       <c r="F309" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE (intimate choice)</t>
+          <t>CA_PROT_04_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G309" s="77" t="inlineStr">
@@ -20231,7 +20231,7 @@
       </c>
       <c r="N309" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20243,17 +20243,17 @@
       </c>
       <c r="B310" s="75" t="inlineStr">
         <is>
-          <t>Mishepeshu</t>
+          <t>La Corriveau</t>
         </is>
       </c>
       <c r="C310" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE_INTIMATE</t>
+          <t>CA_PROT_05_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D310" s="77" t="inlineStr">
         <is>
-          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
+          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
         </is>
       </c>
       <c r="E310" s="79" t="inlineStr">
@@ -20263,7 +20263,7 @@
       </c>
       <c r="F310" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE (intimate choice)</t>
+          <t>CA_PROT_05_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G310" s="77" t="inlineStr">
@@ -20295,7 +20295,7 @@
       </c>
       <c r="N310" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20307,17 +20307,17 @@
       </c>
       <c r="B311" s="75" t="inlineStr">
         <is>
-          <t>La Corriveau</t>
+          <t>Le Carcajou</t>
         </is>
       </c>
       <c r="C311" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE_INTIMATE</t>
+          <t>CA_PROT_06_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D311" s="77" t="inlineStr">
         <is>
-          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
+          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
         </is>
       </c>
       <c r="E311" s="79" t="inlineStr">
@@ -20327,7 +20327,7 @@
       </c>
       <c r="F311" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE (intimate choice)</t>
+          <t>CA_PROT_06_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G311" s="77" t="inlineStr">
@@ -20359,7 +20359,7 @@
       </c>
       <c r="N311" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20371,17 +20371,17 @@
       </c>
       <c r="B312" s="75" t="inlineStr">
         <is>
-          <t>Le Carcajou</t>
+          <t>La Chasse-Galerie</t>
         </is>
       </c>
       <c r="C312" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE_INTIMATE</t>
+          <t>CA_PROT_07_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D312" s="77" t="inlineStr">
         <is>
-          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
+          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
         </is>
       </c>
       <c r="E312" s="79" t="inlineStr">
@@ -20391,7 +20391,7 @@
       </c>
       <c r="F312" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE (intimate choice)</t>
+          <t>CA_PROT_07_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G312" s="77" t="inlineStr">
@@ -20423,7 +20423,7 @@
       </c>
       <c r="N312" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20435,17 +20435,17 @@
       </c>
       <c r="B313" s="75" t="inlineStr">
         <is>
-          <t>La Chasse-Galerie</t>
+          <t>Le Gougou</t>
         </is>
       </c>
       <c r="C313" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE_INTIMATE</t>
+          <t>CA_PROT_08_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D313" s="77" t="inlineStr">
         <is>
-          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
+          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
         </is>
       </c>
       <c r="E313" s="79" t="inlineStr">
@@ -20455,7 +20455,7 @@
       </c>
       <c r="F313" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE (intimate choice)</t>
+          <t>CA_PROT_08_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G313" s="77" t="inlineStr">
@@ -20487,89 +20487,89 @@
       </c>
       <c r="N313" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="314" ht="30" customHeight="1">
-      <c r="A314" s="75" t="inlineStr">
-        <is>
-          <t>CA Protector</t>
-        </is>
-      </c>
-      <c r="B314" s="75" t="inlineStr">
-        <is>
-          <t>Le Gougou</t>
-        </is>
-      </c>
-      <c r="C314" s="76" t="inlineStr">
-        <is>
-          <t>CA_PROT_08_AGREE_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D314" s="77" t="inlineStr">
-        <is>
-          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E314" s="79" t="inlineStr">
+          <t>Stub — author intimate version of CA_PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="8" customHeight="1">
+      <c r="A314" s="9" t="n"/>
+      <c r="B314" s="9" t="n"/>
+      <c r="C314" s="9" t="n"/>
+      <c r="D314" s="9" t="n"/>
+      <c r="E314" s="9" t="n"/>
+      <c r="F314" s="9" t="n"/>
+      <c r="G314" s="9" t="n"/>
+      <c r="H314" s="9" t="n"/>
+      <c r="I314" s="9" t="n"/>
+      <c r="J314" s="9" t="n"/>
+      <c r="K314" s="9" t="n"/>
+      <c r="L314" s="9" t="n"/>
+      <c r="M314" s="9" t="n"/>
+      <c r="N314" s="9" t="n"/>
+    </row>
+    <row r="315" ht="30" customHeight="1">
+      <c r="A315" s="75" t="inlineStr">
+        <is>
+          <t>Ualani</t>
+        </is>
+      </c>
+      <c r="B315" s="75" t="inlineStr">
+        <is>
+          <t>Ambush</t>
+        </is>
+      </c>
+      <c r="C315" s="76" t="inlineStr">
+        <is>
+          <t>UALANI_AMBUSH_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D315" s="77" t="inlineStr">
+        <is>
+          <t>CROWN AMBUSH AVERTED: PRESIDENT CARLISLE HOLDS THE W... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E315" s="79" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F314" s="77" t="inlineStr">
-        <is>
-          <t>CA_PROT_08_AGREE (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G314" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H314" s="78" t="inlineStr">
+      <c r="F315" s="77" t="inlineStr">
+        <is>
+          <t>UALANI_AMBUSH_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G315" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H315" s="78" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I314" s="76" t="inlineStr"/>
-      <c r="J314" s="80" t="inlineStr">
+      <c r="I315" s="76" t="inlineStr"/>
+      <c r="J315" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K314" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L314" s="76" t="inlineStr"/>
-      <c r="M314" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N314" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of CA_PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="315" ht="8" customHeight="1">
-      <c r="A315" s="9" t="n"/>
-      <c r="B315" s="9" t="n"/>
-      <c r="C315" s="9" t="n"/>
-      <c r="D315" s="9" t="n"/>
-      <c r="E315" s="9" t="n"/>
-      <c r="F315" s="9" t="n"/>
-      <c r="G315" s="9" t="n"/>
-      <c r="H315" s="9" t="n"/>
-      <c r="I315" s="9" t="n"/>
-      <c r="J315" s="9" t="n"/>
-      <c r="K315" s="9" t="n"/>
-      <c r="L315" s="9" t="n"/>
-      <c r="M315" s="9" t="n"/>
-      <c r="N315" s="9" t="n"/>
+      <c r="K315" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L315" s="76" t="inlineStr"/>
+      <c r="M315" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N315" s="77" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of UALANI_AMBUSH_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
     </row>
     <row r="316" ht="30" customHeight="1">
       <c r="A316" s="75" t="inlineStr">
@@ -20579,17 +20579,17 @@
       </c>
       <c r="B316" s="75" t="inlineStr">
         <is>
-          <t>Ambush</t>
+          <t>Dignitary Reception</t>
         </is>
       </c>
       <c r="C316" s="76" t="inlineStr">
         <is>
-          <t>UALANI_AMBUSH_01_INTIMATE</t>
+          <t>UALANI_DIGNITARY_01_INTIMATE</t>
         </is>
       </c>
       <c r="D316" s="77" t="inlineStr">
         <is>
-          <t>CROWN AMBUSH AVERTED: PRESIDENT CARLISLE HOLDS THE W... — BY MORNING</t>
+          <t>STATE RECEPTION AT [TILE_NAME]: PRESIDENT CARLISLE A... — BY MORNING</t>
         </is>
       </c>
       <c r="E316" s="79" t="inlineStr">
@@ -20599,7 +20599,7 @@
       </c>
       <c r="F316" s="77" t="inlineStr">
         <is>
-          <t>UALANI_AMBUSH_01 (intimate choice)</t>
+          <t>UALANI_DIGNITARY_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G316" s="77" t="inlineStr">
@@ -20631,7 +20631,7 @@
       </c>
       <c r="N316" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_AMBUSH_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_DIGNITARY_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20643,17 +20643,17 @@
       </c>
       <c r="B317" s="75" t="inlineStr">
         <is>
-          <t>Dignitary Reception</t>
+          <t>Memorial Address</t>
         </is>
       </c>
       <c r="C317" s="76" t="inlineStr">
         <is>
-          <t>UALANI_DIGNITARY_01_INTIMATE</t>
+          <t>UALANI_MEMORIAL_01_INTIMATE</t>
         </is>
       </c>
       <c r="D317" s="77" t="inlineStr">
         <is>
-          <t>STATE RECEPTION AT [TILE_NAME]: PRESIDENT CARLISLE A... — BY MORNING</t>
+          <t>PRESIDENT CARLISLE VISITS [TILE_NAME]: PRESIDENTIAL ... — BY MORNING</t>
         </is>
       </c>
       <c r="E317" s="79" t="inlineStr">
@@ -20663,7 +20663,7 @@
       </c>
       <c r="F317" s="77" t="inlineStr">
         <is>
-          <t>UALANI_DIGNITARY_01 (intimate choice)</t>
+          <t>UALANI_MEMORIAL_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G317" s="77" t="inlineStr">
@@ -20695,7 +20695,7 @@
       </c>
       <c r="N317" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_DIGNITARY_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_MEMORIAL_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20707,17 +20707,17 @@
       </c>
       <c r="B318" s="75" t="inlineStr">
         <is>
-          <t>Memorial Address</t>
+          <t>Field Hospital</t>
         </is>
       </c>
       <c r="C318" s="76" t="inlineStr">
         <is>
-          <t>UALANI_MEMORIAL_01_INTIMATE</t>
+          <t>UALANI_WOUNDED_01_INTIMATE</t>
         </is>
       </c>
       <c r="D318" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS [TILE_NAME]: PRESIDENTIAL ... — BY MORNING</t>
+          <t>PRESIDENT CARLISLE VISITS FIELD HOSPITAL AT [TILE_NAME] — BY MORNING</t>
         </is>
       </c>
       <c r="E318" s="79" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="F318" s="77" t="inlineStr">
         <is>
-          <t>UALANI_MEMORIAL_01 (intimate choice)</t>
+          <t>UALANI_WOUNDED_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G318" s="77" t="inlineStr">
@@ -20759,7 +20759,7 @@
       </c>
       <c r="N318" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_MEMORIAL_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_WOUNDED_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20771,17 +20771,17 @@
       </c>
       <c r="B319" s="75" t="inlineStr">
         <is>
-          <t>Field Hospital</t>
+          <t>Forge Inspection</t>
         </is>
       </c>
       <c r="C319" s="76" t="inlineStr">
         <is>
-          <t>UALANI_WOUNDED_01_INTIMATE</t>
+          <t>UALANI_FORGE_01_INTIMATE</t>
         </is>
       </c>
       <c r="D319" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE VISITS FIELD HOSPITAL AT [TILE_NAME] — BY MORNING</t>
+          <t>PRESIDENT CARLISLE CONDUCTS SURPRISE INSPECTION OF F... — BY MORNING</t>
         </is>
       </c>
       <c r="E319" s="79" t="inlineStr">
@@ -20791,7 +20791,7 @@
       </c>
       <c r="F319" s="77" t="inlineStr">
         <is>
-          <t>UALANI_WOUNDED_01 (intimate choice)</t>
+          <t>UALANI_FORGE_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G319" s="77" t="inlineStr">
@@ -20823,7 +20823,7 @@
       </c>
       <c r="N319" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_WOUNDED_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_FORGE_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20835,17 +20835,17 @@
       </c>
       <c r="B320" s="75" t="inlineStr">
         <is>
-          <t>Forge Inspection</t>
+          <t>Culper Ring</t>
         </is>
       </c>
       <c r="C320" s="76" t="inlineStr">
         <is>
-          <t>UALANI_FORGE_01_INTIMATE</t>
+          <t>UALANI_CULPER_01_INTIMATE</t>
         </is>
       </c>
       <c r="D320" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE CONDUCTS SURPRISE INSPECTION OF F... — BY MORNING</t>
+          <t>CULPER RING CONTACT AT [TILE_NAME]: INTELLIGENCE ASS... — BY MORNING</t>
         </is>
       </c>
       <c r="E320" s="79" t="inlineStr">
@@ -20855,7 +20855,7 @@
       </c>
       <c r="F320" s="77" t="inlineStr">
         <is>
-          <t>UALANI_FORGE_01 (intimate choice)</t>
+          <t>UALANI_CULPER_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G320" s="77" t="inlineStr">
@@ -20887,7 +20887,7 @@
       </c>
       <c r="N320" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_FORGE_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_CULPER_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20899,17 +20899,17 @@
       </c>
       <c r="B321" s="75" t="inlineStr">
         <is>
-          <t>Culper Ring</t>
+          <t>Alliance Council</t>
         </is>
       </c>
       <c r="C321" s="76" t="inlineStr">
         <is>
-          <t>UALANI_CULPER_01_INTIMATE</t>
+          <t>UALANI_ALLIANCE_01_INTIMATE</t>
         </is>
       </c>
       <c r="D321" s="77" t="inlineStr">
         <is>
-          <t>CULPER RING CONTACT AT [TILE_NAME]: INTELLIGENCE ASS... — BY MORNING</t>
+          <t>PRESIDENT CARLISLE MEETS WITH [COMMANDER_NAME] AT [T... — BY MORNING</t>
         </is>
       </c>
       <c r="E321" s="79" t="inlineStr">
@@ -20919,7 +20919,7 @@
       </c>
       <c r="F321" s="77" t="inlineStr">
         <is>
-          <t>UALANI_CULPER_01 (intimate choice)</t>
+          <t>UALANI_ALLIANCE_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G321" s="77" t="inlineStr">
@@ -20951,7 +20951,7 @@
       </c>
       <c r="N321" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_CULPER_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of UALANI_ALLIANCE_01. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -20963,17 +20963,17 @@
       </c>
       <c r="B322" s="75" t="inlineStr">
         <is>
-          <t>Alliance Council</t>
+          <t>Frontier</t>
         </is>
       </c>
       <c r="C322" s="76" t="inlineStr">
         <is>
-          <t>UALANI_ALLIANCE_01_INTIMATE</t>
+          <t>UALANI_FRONTIER_01_INTIMATE</t>
         </is>
       </c>
       <c r="D322" s="77" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE MEETS WITH [COMMANDER_NAME] AT [T... — BY MORNING</t>
+          <t>PRESIDENT CARLISLE ESTABLISHES FRONTIER PRESENCE AT ... — BY MORNING</t>
         </is>
       </c>
       <c r="E322" s="79" t="inlineStr">
@@ -20983,7 +20983,7 @@
       </c>
       <c r="F322" s="77" t="inlineStr">
         <is>
-          <t>UALANI_ALLIANCE_01 (intimate choice)</t>
+          <t>UALANI_FRONTIER_01 (intimate choice)</t>
         </is>
       </c>
       <c r="G322" s="77" t="inlineStr">
@@ -21015,89 +21015,89 @@
       </c>
       <c r="N322" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of UALANI_ALLIANCE_01. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="323" ht="30" customHeight="1">
-      <c r="A323" s="75" t="inlineStr">
-        <is>
-          <t>Ualani</t>
-        </is>
-      </c>
-      <c r="B323" s="75" t="inlineStr">
-        <is>
-          <t>Frontier</t>
-        </is>
-      </c>
-      <c r="C323" s="76" t="inlineStr">
-        <is>
-          <t>UALANI_FRONTIER_01_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D323" s="77" t="inlineStr">
-        <is>
-          <t>PRESIDENT CARLISLE ESTABLISHES FRONTIER PRESENCE AT ... — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E323" s="79" t="inlineStr">
+          <t>Stub — author intimate version of UALANI_FRONTIER_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="8" customHeight="1">
+      <c r="A323" s="9" t="n"/>
+      <c r="B323" s="9" t="n"/>
+      <c r="C323" s="9" t="n"/>
+      <c r="D323" s="9" t="n"/>
+      <c r="E323" s="9" t="n"/>
+      <c r="F323" s="9" t="n"/>
+      <c r="G323" s="9" t="n"/>
+      <c r="H323" s="9" t="n"/>
+      <c r="I323" s="9" t="n"/>
+      <c r="J323" s="9" t="n"/>
+      <c r="K323" s="9" t="n"/>
+      <c r="L323" s="9" t="n"/>
+      <c r="M323" s="9" t="n"/>
+      <c r="N323" s="9" t="n"/>
+    </row>
+    <row r="324" ht="30" customHeight="1">
+      <c r="A324" s="75" t="inlineStr">
+        <is>
+          <t>Protector</t>
+        </is>
+      </c>
+      <c r="B324" s="75" t="inlineStr">
+        <is>
+          <t>Mothman</t>
+        </is>
+      </c>
+      <c r="C324" s="76" t="inlineStr">
+        <is>
+          <t>PROT_01_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D324" s="77" t="inlineStr">
+        <is>
+          <t>MOTHMAN FORMALLY ALLIES WITH THE CONTINENTAL REPUBLIC — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E324" s="79" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F323" s="77" t="inlineStr">
-        <is>
-          <t>UALANI_FRONTIER_01 (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G323" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H323" s="78" t="inlineStr">
+      <c r="F324" s="77" t="inlineStr">
+        <is>
+          <t>PROT_01_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G324" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H324" s="78" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I323" s="76" t="inlineStr"/>
-      <c r="J323" s="80" t="inlineStr">
+      <c r="I324" s="76" t="inlineStr"/>
+      <c r="J324" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K323" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L323" s="76" t="inlineStr"/>
-      <c r="M323" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N323" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of UALANI_FRONTIER_01. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="324" ht="8" customHeight="1">
-      <c r="A324" s="9" t="n"/>
-      <c r="B324" s="9" t="n"/>
-      <c r="C324" s="9" t="n"/>
-      <c r="D324" s="9" t="n"/>
-      <c r="E324" s="9" t="n"/>
-      <c r="F324" s="9" t="n"/>
-      <c r="G324" s="9" t="n"/>
-      <c r="H324" s="9" t="n"/>
-      <c r="I324" s="9" t="n"/>
-      <c r="J324" s="9" t="n"/>
-      <c r="K324" s="9" t="n"/>
-      <c r="L324" s="9" t="n"/>
-      <c r="M324" s="9" t="n"/>
-      <c r="N324" s="9" t="n"/>
+      <c r="K324" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L324" s="76" t="inlineStr"/>
+      <c r="M324" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N324" s="77" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
     </row>
     <row r="325" ht="30" customHeight="1">
       <c r="A325" s="75" t="inlineStr">
@@ -21107,17 +21107,17 @@
       </c>
       <c r="B325" s="75" t="inlineStr">
         <is>
-          <t>Mothman</t>
+          <t>Jersey Devil</t>
         </is>
       </c>
       <c r="C325" s="76" t="inlineStr">
         <is>
-          <t>PROT_01_AGREE_INTIMATE</t>
+          <t>PROT_02_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D325" s="77" t="inlineStr">
         <is>
-          <t>MOTHMAN FORMALLY ALLIES WITH THE CONTINENTAL REPUBLIC — BY MORNING</t>
+          <t>JERSEY DEVIL FORMALLY ENDORSES THE CONTINENTAL CAUSE — BY MORNING</t>
         </is>
       </c>
       <c r="E325" s="79" t="inlineStr">
@@ -21127,7 +21127,7 @@
       </c>
       <c r="F325" s="77" t="inlineStr">
         <is>
-          <t>PROT_01_AGREE (intimate choice)</t>
+          <t>PROT_02_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G325" s="77" t="inlineStr">
@@ -21159,7 +21159,7 @@
       </c>
       <c r="N325" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21171,17 +21171,17 @@
       </c>
       <c r="B326" s="75" t="inlineStr">
         <is>
-          <t>Jersey Devil</t>
+          <t>Bigfoot</t>
         </is>
       </c>
       <c r="C326" s="76" t="inlineStr">
         <is>
-          <t>PROT_02_AGREE_INTIMATE</t>
+          <t>PROT_03_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D326" s="77" t="inlineStr">
         <is>
-          <t>JERSEY DEVIL FORMALLY ENDORSES THE CONTINENTAL CAUSE — BY MORNING</t>
+          <t>BIGFOOT FORMALLY GUIDES THE CONTINENTAL CAUSE THROUG... — BY MORNING</t>
         </is>
       </c>
       <c r="E326" s="79" t="inlineStr">
@@ -21191,7 +21191,7 @@
       </c>
       <c r="F326" s="77" t="inlineStr">
         <is>
-          <t>PROT_02_AGREE (intimate choice)</t>
+          <t>PROT_03_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G326" s="77" t="inlineStr">
@@ -21223,7 +21223,7 @@
       </c>
       <c r="N326" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21235,17 +21235,17 @@
       </c>
       <c r="B327" s="75" t="inlineStr">
         <is>
-          <t>Bigfoot</t>
+          <t>Thunderbird</t>
         </is>
       </c>
       <c r="C327" s="76" t="inlineStr">
         <is>
-          <t>PROT_03_AGREE_INTIMATE</t>
+          <t>PROT_04_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D327" s="77" t="inlineStr">
         <is>
-          <t>BIGFOOT FORMALLY GUIDES THE CONTINENTAL CAUSE THROUG... — BY MORNING</t>
+          <t>THUNDERBIRD FORMALLY ALLIES WITH THE CONTINENTAL REP... — BY MORNING</t>
         </is>
       </c>
       <c r="E327" s="79" t="inlineStr">
@@ -21255,7 +21255,7 @@
       </c>
       <c r="F327" s="77" t="inlineStr">
         <is>
-          <t>PROT_03_AGREE (intimate choice)</t>
+          <t>PROT_04_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G327" s="77" t="inlineStr">
@@ -21287,7 +21287,7 @@
       </c>
       <c r="N327" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21299,17 +21299,17 @@
       </c>
       <c r="B328" s="75" t="inlineStr">
         <is>
-          <t>Thunderbird</t>
+          <t>Headless Horseman</t>
         </is>
       </c>
       <c r="C328" s="76" t="inlineStr">
         <is>
-          <t>PROT_04_AGREE_INTIMATE</t>
+          <t>PROT_05_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D328" s="77" t="inlineStr">
         <is>
-          <t>THUNDERBIRD FORMALLY ALLIES WITH THE CONTINENTAL REP... — BY MORNING</t>
+          <t>THE HORSEMAN RIDES FOR THE REPUBLIC — FORMALLY — BY MORNING</t>
         </is>
       </c>
       <c r="E328" s="79" t="inlineStr">
@@ -21319,7 +21319,7 @@
       </c>
       <c r="F328" s="77" t="inlineStr">
         <is>
-          <t>PROT_04_AGREE (intimate choice)</t>
+          <t>PROT_05_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G328" s="77" t="inlineStr">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="N328" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21363,17 +21363,17 @@
       </c>
       <c r="B329" s="75" t="inlineStr">
         <is>
-          <t>Headless Horseman</t>
+          <t>Chessie</t>
         </is>
       </c>
       <c r="C329" s="76" t="inlineStr">
         <is>
-          <t>PROT_05_AGREE_INTIMATE</t>
+          <t>PROT_06_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D329" s="77" t="inlineStr">
         <is>
-          <t>THE HORSEMAN RIDES FOR THE REPUBLIC — FORMALLY — BY MORNING</t>
+          <t>CHESSIE FORMALLY PATROLS FOR THE CONTINENTAL NAVY — BY MORNING</t>
         </is>
       </c>
       <c r="E329" s="79" t="inlineStr">
@@ -21383,7 +21383,7 @@
       </c>
       <c r="F329" s="77" t="inlineStr">
         <is>
-          <t>PROT_05_AGREE (intimate choice)</t>
+          <t>PROT_06_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G329" s="77" t="inlineStr">
@@ -21415,7 +21415,7 @@
       </c>
       <c r="N329" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21427,17 +21427,17 @@
       </c>
       <c r="B330" s="75" t="inlineStr">
         <is>
-          <t>Chessie</t>
+          <t>Bell Witch</t>
         </is>
       </c>
       <c r="C330" s="76" t="inlineStr">
         <is>
-          <t>PROT_06_AGREE_INTIMATE</t>
+          <t>PROT_07_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D330" s="77" t="inlineStr">
         <is>
-          <t>CHESSIE FORMALLY PATROLS FOR THE CONTINENTAL NAVY — BY MORNING</t>
+          <t>THE BELL WITCH FORMALLY COMMITS TO THE CONTINENTAL C... — BY MORNING</t>
         </is>
       </c>
       <c r="E330" s="79" t="inlineStr">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="F330" s="77" t="inlineStr">
         <is>
-          <t>PROT_06_AGREE (intimate choice)</t>
+          <t>PROT_07_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G330" s="77" t="inlineStr">
@@ -21479,7 +21479,7 @@
       </c>
       <c r="N330" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21491,17 +21491,17 @@
       </c>
       <c r="B331" s="75" t="inlineStr">
         <is>
-          <t>Bell Witch</t>
+          <t>Old Ironsides</t>
         </is>
       </c>
       <c r="C331" s="76" t="inlineStr">
         <is>
-          <t>PROT_07_AGREE_INTIMATE</t>
+          <t>PROT_08_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D331" s="77" t="inlineStr">
         <is>
-          <t>THE BELL WITCH FORMALLY COMMITS TO THE CONTINENTAL C... — BY MORNING</t>
+          <t>OLD IRONSIDES FORMALLY JOINS THE CONTINENTAL NAVY — BY MORNING</t>
         </is>
       </c>
       <c r="E331" s="79" t="inlineStr">
@@ -21511,7 +21511,7 @@
       </c>
       <c r="F331" s="77" t="inlineStr">
         <is>
-          <t>PROT_07_AGREE (intimate choice)</t>
+          <t>PROT_08_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G331" s="77" t="inlineStr">
@@ -21543,7 +21543,7 @@
       </c>
       <c r="N331" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21555,17 +21555,17 @@
       </c>
       <c r="B332" s="75" t="inlineStr">
         <is>
-          <t>Old Ironsides</t>
+          <t>Valley Forge Guardian</t>
         </is>
       </c>
       <c r="C332" s="76" t="inlineStr">
         <is>
-          <t>PROT_08_AGREE_INTIMATE</t>
+          <t>PROT_09_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D332" s="77" t="inlineStr">
         <is>
-          <t>OLD IRONSIDES FORMALLY JOINS THE CONTINENTAL NAVY — BY MORNING</t>
+          <t>VALLEY FORGE GUARDIAN FORMALLY BLESSES THE CONTINENT... — BY MORNING</t>
         </is>
       </c>
       <c r="E332" s="79" t="inlineStr">
@@ -21575,7 +21575,7 @@
       </c>
       <c r="F332" s="77" t="inlineStr">
         <is>
-          <t>PROT_08_AGREE (intimate choice)</t>
+          <t>PROT_09_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G332" s="77" t="inlineStr">
@@ -21607,7 +21607,7 @@
       </c>
       <c r="N332" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_09_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21619,17 +21619,17 @@
       </c>
       <c r="B333" s="75" t="inlineStr">
         <is>
-          <t>Valley Forge Guardian</t>
+          <t>Snallygaster</t>
         </is>
       </c>
       <c r="C333" s="76" t="inlineStr">
         <is>
-          <t>PROT_09_AGREE_INTIMATE</t>
+          <t>PROT_10_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D333" s="77" t="inlineStr">
         <is>
-          <t>VALLEY FORGE GUARDIAN FORMALLY BLESSES THE CONTINENT... — BY MORNING</t>
+          <t>SNALLYGASTER FORMALLY GUARDS THE CONTINENTAL SUPPLY ... — BY MORNING</t>
         </is>
       </c>
       <c r="E333" s="79" t="inlineStr">
@@ -21639,7 +21639,7 @@
       </c>
       <c r="F333" s="77" t="inlineStr">
         <is>
-          <t>PROT_09_AGREE (intimate choice)</t>
+          <t>PROT_10_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G333" s="77" t="inlineStr">
@@ -21671,7 +21671,7 @@
       </c>
       <c r="N333" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_09_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_10_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21683,17 +21683,17 @@
       </c>
       <c r="B334" s="75" t="inlineStr">
         <is>
-          <t>Snallygaster</t>
+          <t>Paul Revere</t>
         </is>
       </c>
       <c r="C334" s="76" t="inlineStr">
         <is>
-          <t>PROT_10_AGREE_INTIMATE</t>
+          <t>PROT_11_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D334" s="77" t="inlineStr">
         <is>
-          <t>SNALLYGASTER FORMALLY GUARDS THE CONTINENTAL SUPPLY ... — BY MORNING</t>
+          <t>PAUL REVERE FORMALLY INTEGRATES WITH CONTINENTAL INT... — BY MORNING</t>
         </is>
       </c>
       <c r="E334" s="79" t="inlineStr">
@@ -21703,7 +21703,7 @@
       </c>
       <c r="F334" s="77" t="inlineStr">
         <is>
-          <t>PROT_10_AGREE (intimate choice)</t>
+          <t>PROT_11_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G334" s="77" t="inlineStr">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="N334" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_10_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_11_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21747,17 +21747,17 @@
       </c>
       <c r="B335" s="75" t="inlineStr">
         <is>
-          <t>Paul Revere</t>
+          <t>Liberty Bell</t>
         </is>
       </c>
       <c r="C335" s="76" t="inlineStr">
         <is>
-          <t>PROT_11_AGREE_INTIMATE</t>
+          <t>PROT_12_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D335" s="77" t="inlineStr">
         <is>
-          <t>PAUL REVERE FORMALLY INTEGRATES WITH CONTINENTAL INT... — BY MORNING</t>
+          <t>THE LIBERTY BELL FORMALLY RINGS FOR THE REPUBLIC — BY MORNING</t>
         </is>
       </c>
       <c r="E335" s="79" t="inlineStr">
@@ -21767,7 +21767,7 @@
       </c>
       <c r="F335" s="77" t="inlineStr">
         <is>
-          <t>PROT_11_AGREE (intimate choice)</t>
+          <t>PROT_12_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G335" s="77" t="inlineStr">
@@ -21799,7 +21799,7 @@
       </c>
       <c r="N335" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_11_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_12_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21811,17 +21811,17 @@
       </c>
       <c r="B336" s="75" t="inlineStr">
         <is>
-          <t>Liberty Bell</t>
+          <t>Green Mountain Ghost</t>
         </is>
       </c>
       <c r="C336" s="76" t="inlineStr">
         <is>
-          <t>PROT_12_AGREE_INTIMATE</t>
+          <t>PROT_13_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D336" s="77" t="inlineStr">
         <is>
-          <t>THE LIBERTY BELL FORMALLY RINGS FOR THE REPUBLIC — BY MORNING</t>
+          <t>GREEN MOUNTAIN GHOST FORMALLY PROTECTS VERMONT FOR T... — BY MORNING</t>
         </is>
       </c>
       <c r="E336" s="79" t="inlineStr">
@@ -21831,7 +21831,7 @@
       </c>
       <c r="F336" s="77" t="inlineStr">
         <is>
-          <t>PROT_12_AGREE (intimate choice)</t>
+          <t>PROT_13_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G336" s="77" t="inlineStr">
@@ -21863,7 +21863,7 @@
       </c>
       <c r="N336" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_12_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_13_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21875,17 +21875,17 @@
       </c>
       <c r="B337" s="75" t="inlineStr">
         <is>
-          <t>Green Mountain Ghost</t>
+          <t>Mount Rushmore</t>
         </is>
       </c>
       <c r="C337" s="76" t="inlineStr">
         <is>
-          <t>PROT_13_AGREE_INTIMATE</t>
+          <t>PROT_14_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D337" s="77" t="inlineStr">
         <is>
-          <t>GREEN MOUNTAIN GHOST FORMALLY PROTECTS VERMONT FOR T... — BY MORNING</t>
+          <t>THE RUSHMORE COUNCIL FORMALLY ENDORSES PRESIDENT CAR... — BY MORNING</t>
         </is>
       </c>
       <c r="E337" s="79" t="inlineStr">
@@ -21895,7 +21895,7 @@
       </c>
       <c r="F337" s="77" t="inlineStr">
         <is>
-          <t>PROT_13_AGREE (intimate choice)</t>
+          <t>PROT_14_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G337" s="77" t="inlineStr">
@@ -21927,7 +21927,7 @@
       </c>
       <c r="N337" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_13_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_14_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -21939,17 +21939,17 @@
       </c>
       <c r="B338" s="75" t="inlineStr">
         <is>
-          <t>Mount Rushmore</t>
+          <t>Skunk Ape</t>
         </is>
       </c>
       <c r="C338" s="76" t="inlineStr">
         <is>
-          <t>PROT_14_AGREE_INTIMATE</t>
+          <t>PROT_15_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D338" s="77" t="inlineStr">
         <is>
-          <t>THE RUSHMORE COUNCIL FORMALLY ENDORSES PRESIDENT CAR... — BY MORNING</t>
+          <t>SKUNK APE FORMALLY PATROLS FLORIDA FOR THE CONTINENT... — BY MORNING</t>
         </is>
       </c>
       <c r="E338" s="79" t="inlineStr">
@@ -21959,7 +21959,7 @@
       </c>
       <c r="F338" s="77" t="inlineStr">
         <is>
-          <t>PROT_14_AGREE (intimate choice)</t>
+          <t>PROT_15_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G338" s="77" t="inlineStr">
@@ -21991,7 +21991,7 @@
       </c>
       <c r="N338" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_14_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_15_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22003,17 +22003,17 @@
       </c>
       <c r="B339" s="75" t="inlineStr">
         <is>
-          <t>Skunk Ape</t>
+          <t>Minuteman</t>
         </is>
       </c>
       <c r="C339" s="76" t="inlineStr">
         <is>
-          <t>PROT_15_AGREE_INTIMATE</t>
+          <t>PROT_16_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D339" s="77" t="inlineStr">
         <is>
-          <t>SKUNK APE FORMALLY PATROLS FLORIDA FOR THE CONTINENT... — BY MORNING</t>
+          <t>THE MINUTEMAN FORMALLY DECLARES FOR THE CONTINENTAL ... — BY MORNING</t>
         </is>
       </c>
       <c r="E339" s="79" t="inlineStr">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="F339" s="77" t="inlineStr">
         <is>
-          <t>PROT_15_AGREE (intimate choice)</t>
+          <t>PROT_16_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G339" s="77" t="inlineStr">
@@ -22055,7 +22055,7 @@
       </c>
       <c r="N339" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_15_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of PROT_16_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22067,17 +22067,17 @@
       </c>
       <c r="B340" s="75" t="inlineStr">
         <is>
-          <t>Minuteman</t>
+          <t>Lincoln's Ghost</t>
         </is>
       </c>
       <c r="C340" s="76" t="inlineStr">
         <is>
-          <t>PROT_16_AGREE_INTIMATE</t>
+          <t>PROT_17_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D340" s="77" t="inlineStr">
         <is>
-          <t>THE MINUTEMAN FORMALLY DECLARES FOR THE CONTINENTAL ... — BY MORNING</t>
+          <t>LINCOLN FORMALLY ENDORSES PRESIDENT CARLISLE'S ADMIN... — BY MORNING</t>
         </is>
       </c>
       <c r="E340" s="79" t="inlineStr">
@@ -22087,7 +22087,7 @@
       </c>
       <c r="F340" s="77" t="inlineStr">
         <is>
-          <t>PROT_16_AGREE (intimate choice)</t>
+          <t>PROT_17_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G340" s="77" t="inlineStr">
@@ -22119,89 +22119,89 @@
       </c>
       <c r="N340" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of PROT_16_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="341" ht="30" customHeight="1">
-      <c r="A341" s="75" t="inlineStr">
-        <is>
-          <t>Protector</t>
-        </is>
-      </c>
-      <c r="B341" s="75" t="inlineStr">
-        <is>
-          <t>Lincoln's Ghost</t>
-        </is>
-      </c>
-      <c r="C341" s="76" t="inlineStr">
-        <is>
-          <t>PROT_17_AGREE_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D341" s="77" t="inlineStr">
-        <is>
-          <t>LINCOLN FORMALLY ENDORSES PRESIDENT CARLISLE'S ADMIN... — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E341" s="79" t="inlineStr">
+          <t>Stub — author intimate version of PROT_17_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="8" customHeight="1">
+      <c r="A341" s="9" t="n"/>
+      <c r="B341" s="9" t="n"/>
+      <c r="C341" s="9" t="n"/>
+      <c r="D341" s="9" t="n"/>
+      <c r="E341" s="9" t="n"/>
+      <c r="F341" s="9" t="n"/>
+      <c r="G341" s="9" t="n"/>
+      <c r="H341" s="9" t="n"/>
+      <c r="I341" s="9" t="n"/>
+      <c r="J341" s="9" t="n"/>
+      <c r="K341" s="9" t="n"/>
+      <c r="L341" s="9" t="n"/>
+      <c r="M341" s="9" t="n"/>
+      <c r="N341" s="9" t="n"/>
+    </row>
+    <row r="342" ht="30" customHeight="1">
+      <c r="A342" s="75" t="inlineStr">
+        <is>
+          <t>White House</t>
+        </is>
+      </c>
+      <c r="B342" s="75" t="inlineStr">
+        <is>
+          <t>Month 1</t>
+        </is>
+      </c>
+      <c r="C342" s="76" t="inlineStr">
+        <is>
+          <t>WH_SECRET_01_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D342" s="77" t="inlineStr">
+        <is>
+          <t>THE WHITE HOUSE AT MIDNIGHT — THE PRESIDENT WATCHES ... — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E342" s="79" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F341" s="77" t="inlineStr">
-        <is>
-          <t>PROT_17_AGREE (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G341" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H341" s="78" t="inlineStr">
+      <c r="F342" s="77" t="inlineStr">
+        <is>
+          <t>WH_SECRET_01 (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G342" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H342" s="78" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I341" s="76" t="inlineStr"/>
-      <c r="J341" s="80" t="inlineStr">
+      <c r="I342" s="76" t="inlineStr"/>
+      <c r="J342" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K341" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L341" s="76" t="inlineStr"/>
-      <c r="M341" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N341" s="77" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of PROT_17_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="342" ht="8" customHeight="1">
-      <c r="A342" s="9" t="n"/>
-      <c r="B342" s="9" t="n"/>
-      <c r="C342" s="9" t="n"/>
-      <c r="D342" s="9" t="n"/>
-      <c r="E342" s="9" t="n"/>
-      <c r="F342" s="9" t="n"/>
-      <c r="G342" s="9" t="n"/>
-      <c r="H342" s="9" t="n"/>
-      <c r="I342" s="9" t="n"/>
-      <c r="J342" s="9" t="n"/>
-      <c r="K342" s="9" t="n"/>
-      <c r="L342" s="9" t="n"/>
-      <c r="M342" s="9" t="n"/>
-      <c r="N342" s="9" t="n"/>
+      <c r="K342" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L342" s="76" t="inlineStr"/>
+      <c r="M342" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N342" s="77" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of WH_SECRET_01. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
     </row>
     <row r="343" ht="30" customHeight="1">
       <c r="A343" s="75" t="inlineStr">
@@ -22211,17 +22211,17 @@
       </c>
       <c r="B343" s="75" t="inlineStr">
         <is>
-          <t>Month 1</t>
+          <t>Month 7</t>
         </is>
       </c>
       <c r="C343" s="76" t="inlineStr">
         <is>
-          <t>WH_SECRET_01_INTIMATE</t>
+          <t>WH_SECRET_07_INTIMATE</t>
         </is>
       </c>
       <c r="D343" s="77" t="inlineStr">
         <is>
-          <t>THE WHITE HOUSE AT MIDNIGHT — THE PRESIDENT WATCHES ... — BY MORNING</t>
+          <t>JULY AT THE WHITE HOUSE — INDEPENDENCE DAY IS ALSO HERS — BY MORNING</t>
         </is>
       </c>
       <c r="E343" s="79" t="inlineStr">
@@ -22231,7 +22231,7 @@
       </c>
       <c r="F343" s="77" t="inlineStr">
         <is>
-          <t>WH_SECRET_01 (intimate choice)</t>
+          <t>WH_SECRET_07 (intimate choice)</t>
         </is>
       </c>
       <c r="G343" s="77" t="inlineStr">
@@ -22263,7 +22263,7 @@
       </c>
       <c r="N343" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of WH_SECRET_01. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of WH_SECRET_07. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22275,17 +22275,17 @@
       </c>
       <c r="B344" s="75" t="inlineStr">
         <is>
-          <t>Month 7</t>
+          <t>Month 10</t>
         </is>
       </c>
       <c r="C344" s="76" t="inlineStr">
         <is>
-          <t>WH_SECRET_07_INTIMATE</t>
+          <t>WH_SECRET_10_INTIMATE</t>
         </is>
       </c>
       <c r="D344" s="77" t="inlineStr">
         <is>
-          <t>JULY AT THE WHITE HOUSE — INDEPENDENCE DAY IS ALSO HERS — BY MORNING</t>
+          <t>INDIGENOUS PEOPLES DAY — A PERSONAL LETTER FROM JESS... — BY MORNING</t>
         </is>
       </c>
       <c r="E344" s="79" t="inlineStr">
@@ -22295,7 +22295,7 @@
       </c>
       <c r="F344" s="77" t="inlineStr">
         <is>
-          <t>WH_SECRET_07 (intimate choice)</t>
+          <t>WH_SECRET_10 (intimate choice)</t>
         </is>
       </c>
       <c r="G344" s="77" t="inlineStr">
@@ -22327,7 +22327,7 @@
       </c>
       <c r="N344" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of WH_SECRET_07. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of WH_SECRET_10. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -22339,17 +22339,17 @@
       </c>
       <c r="B345" s="75" t="inlineStr">
         <is>
-          <t>Month 10</t>
+          <t>Month 12</t>
         </is>
       </c>
       <c r="C345" s="76" t="inlineStr">
         <is>
-          <t>WH_SECRET_10_INTIMATE</t>
+          <t>WH_SECRET_12_INTIMATE</t>
         </is>
       </c>
       <c r="D345" s="77" t="inlineStr">
         <is>
-          <t>INDIGENOUS PEOPLES DAY — A PERSONAL LETTER FROM JESS... — BY MORNING</t>
+          <t>CHRISTMAS IN WASHINGTON — THE PRESIDENT IS FAR FROM ... — BY MORNING</t>
         </is>
       </c>
       <c r="E345" s="79" t="inlineStr">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="F345" s="77" t="inlineStr">
         <is>
-          <t>WH_SECRET_10 (intimate choice)</t>
+          <t>WH_SECRET_12 (intimate choice)</t>
         </is>
       </c>
       <c r="G345" s="77" t="inlineStr">
@@ -22391,111 +22391,47 @@
       </c>
       <c r="N345" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of WH_SECRET_10. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="346" ht="30" customHeight="1">
-      <c r="A346" s="75" t="inlineStr">
-        <is>
-          <t>White House</t>
-        </is>
-      </c>
-      <c r="B346" s="75" t="inlineStr">
-        <is>
-          <t>Month 12</t>
-        </is>
-      </c>
-      <c r="C346" s="76" t="inlineStr">
-        <is>
-          <t>WH_SECRET_12_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D346" s="77" t="inlineStr">
-        <is>
-          <t>CHRISTMAS IN WASHINGTON — THE PRESIDENT IS FAR FROM ... — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E346" s="79" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="F346" s="77" t="inlineStr">
-        <is>
-          <t>WH_SECRET_12 (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G346" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H346" s="78" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I346" s="76" t="inlineStr"/>
-      <c r="J346" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K346" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L346" s="76" t="inlineStr"/>
-      <c r="M346" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N346" s="77" t="inlineStr">
-        <is>
           <t>Stub — author intimate version of WH_SECRET_12. By morning: emotional arc, no explicit imagery.</t>
         </is>
+      </c>
+    </row>
+    <row r="347" ht="20" customHeight="1">
+      <c r="A347" s="81" t="inlineStr">
+        <is>
+          <t>Total events in spreadsheet</t>
+        </is>
+      </c>
+      <c r="B347" s="82" t="n">
+        <v>314</v>
       </c>
     </row>
     <row r="348" ht="20" customHeight="1">
       <c r="A348" s="81" t="inlineStr">
         <is>
-          <t>Total events in spreadsheet</t>
+          <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
       <c r="B348" s="82" t="n">
-        <v>315</v>
+        <v>248</v>
       </c>
     </row>
     <row r="349" ht="20" customHeight="1">
       <c r="A349" s="81" t="inlineStr">
         <is>
-          <t>FIRST PASS (coded &amp; wired)</t>
+          <t>IDEA (not yet implemented)</t>
         </is>
       </c>
       <c r="B349" s="82" t="n">
-        <v>249</v>
+        <v>64</v>
       </c>
     </row>
     <row r="350" ht="20" customHeight="1">
       <c r="A350" s="81" t="inlineStr">
         <is>
-          <t>IDEA (not yet implemented)</t>
+          <t>Need explicit art (YES)</t>
         </is>
       </c>
       <c r="B350" s="82" t="n">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="351" ht="20" customHeight="1">
-      <c r="A351" s="81" t="inlineStr">
-        <is>
-          <t>Need explicit art (YES)</t>
-        </is>
-      </c>
-      <c r="B351" s="82" t="n">
         <v>55</v>
       </c>
     </row>
@@ -22510,7 +22446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25689,85 +25625,85 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="53" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="B50" s="53" t="inlineStr">
-        <is>
-          <t>PM Arc</t>
-        </is>
-      </c>
-      <c r="C50" s="54" t="inlineStr">
-        <is>
-          <t>CA_PM_LEGACY_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D50" s="55" t="inlineStr">
-        <is>
-          <t>MARC PENOIT'S FINAL ASSESSMENT — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E50" s="56" t="inlineStr">
+    <row r="50" ht="8" customHeight="1">
+      <c r="A50" s="9" t="n"/>
+      <c r="B50" s="9" t="n"/>
+      <c r="C50" s="9" t="n"/>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="9" t="n"/>
+      <c r="G50" s="9" t="n"/>
+      <c r="H50" s="9" t="n"/>
+      <c r="I50" s="9" t="n"/>
+      <c r="J50" s="9" t="n"/>
+      <c r="K50" s="9" t="n"/>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="9" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="75" t="inlineStr">
+        <is>
+          <t>CA Protector</t>
+        </is>
+      </c>
+      <c r="B51" s="75" t="inlineStr">
+        <is>
+          <t>Le Wendigo</t>
+        </is>
+      </c>
+      <c r="C51" s="76" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE_INTIMATE</t>
+        </is>
+      </c>
+      <c r="D51" s="77" t="inlineStr">
+        <is>
+          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
+        </is>
+      </c>
+      <c r="E51" s="79" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F50" s="55" t="inlineStr">
-        <is>
-          <t>CA_PM_LEGACY (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G50" s="55" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I50" s="54" t="inlineStr"/>
-      <c r="J50" s="80" t="inlineStr">
+      <c r="F51" s="77" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE (intimate choice)</t>
+        </is>
+      </c>
+      <c r="G51" s="77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H51" s="78" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="I51" s="76" t="inlineStr"/>
+      <c r="J51" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K50" s="56" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L50" s="54" t="inlineStr"/>
-      <c r="M50" s="56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N50" s="55" t="inlineStr">
-        <is>
-          <t>By morning: Penoit at the desk before light, writing page forty-one. Emotional resolution — he was wrong about what this would feel like.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="8" customHeight="1">
-      <c r="A51" s="9" t="n"/>
-      <c r="B51" s="9" t="n"/>
-      <c r="C51" s="9" t="n"/>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9" t="n"/>
-      <c r="F51" s="9" t="n"/>
-      <c r="G51" s="9" t="n"/>
-      <c r="H51" s="9" t="n"/>
-      <c r="I51" s="9" t="n"/>
-      <c r="J51" s="9" t="n"/>
-      <c r="K51" s="9" t="n"/>
-      <c r="L51" s="9" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="9" t="n"/>
+      <c r="K51" s="79" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L51" s="76" t="inlineStr"/>
+      <c r="M51" s="79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N51" s="77" t="inlineStr">
+        <is>
+          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="75" t="inlineStr">
@@ -25777,17 +25713,17 @@
       </c>
       <c r="B52" s="75" t="inlineStr">
         <is>
-          <t>Le Wendigo</t>
+          <t>Le Loup-Garou</t>
         </is>
       </c>
       <c r="C52" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_01_AGREE_INTIMATE</t>
+          <t>CA_PROT_02_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D52" s="77" t="inlineStr">
         <is>
-          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD — BY MORNING</t>
+          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
         </is>
       </c>
       <c r="E52" s="79" t="inlineStr">
@@ -25797,7 +25733,7 @@
       </c>
       <c r="F52" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_01_AGREE (intimate choice)</t>
+          <t>CA_PROT_02_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G52" s="77" t="inlineStr">
@@ -25829,7 +25765,7 @@
       </c>
       <c r="N52" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_01_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -25841,17 +25777,17 @@
       </c>
       <c r="B53" s="75" t="inlineStr">
         <is>
-          <t>Le Loup-Garou</t>
+          <t>Les Feux Follets</t>
         </is>
       </c>
       <c r="C53" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE_INTIMATE</t>
+          <t>CA_PROT_03_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D53" s="77" t="inlineStr">
         <is>
-          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLED... — BY MORNING</t>
+          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
         </is>
       </c>
       <c r="E53" s="79" t="inlineStr">
@@ -25861,7 +25797,7 @@
       </c>
       <c r="F53" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_02_AGREE (intimate choice)</t>
+          <t>CA_PROT_03_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G53" s="77" t="inlineStr">
@@ -25893,7 +25829,7 @@
       </c>
       <c r="N53" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -25905,17 +25841,17 @@
       </c>
       <c r="B54" s="75" t="inlineStr">
         <is>
-          <t>Les Feux Follets</t>
+          <t>Mishepeshu</t>
         </is>
       </c>
       <c r="C54" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE_INTIMATE</t>
+          <t>CA_PROT_04_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D54" s="77" t="inlineStr">
         <is>
-          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JO... — BY MORNING</t>
+          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
         </is>
       </c>
       <c r="E54" s="79" t="inlineStr">
@@ -25925,7 +25861,7 @@
       </c>
       <c r="F54" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_03_AGREE (intimate choice)</t>
+          <t>CA_PROT_04_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G54" s="77" t="inlineStr">
@@ -25957,7 +25893,7 @@
       </c>
       <c r="N54" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_03_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -25969,17 +25905,17 @@
       </c>
       <c r="B55" s="75" t="inlineStr">
         <is>
-          <t>Mishepeshu</t>
+          <t>La Corriveau</t>
         </is>
       </c>
       <c r="C55" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE_INTIMATE</t>
+          <t>CA_PROT_05_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D55" s="77" t="inlineStr">
         <is>
-          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE... — BY MORNING</t>
+          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
         </is>
       </c>
       <c r="E55" s="79" t="inlineStr">
@@ -25989,7 +25925,7 @@
       </c>
       <c r="F55" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE (intimate choice)</t>
+          <t>CA_PROT_05_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G55" s="77" t="inlineStr">
@@ -26021,7 +25957,7 @@
       </c>
       <c r="N55" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_04_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -26033,17 +25969,17 @@
       </c>
       <c r="B56" s="75" t="inlineStr">
         <is>
-          <t>La Corriveau</t>
+          <t>Le Carcajou</t>
         </is>
       </c>
       <c r="C56" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE_INTIMATE</t>
+          <t>CA_PROT_06_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D56" s="77" t="inlineStr">
         <is>
-          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THR... — BY MORNING</t>
+          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
         </is>
       </c>
       <c r="E56" s="79" t="inlineStr">
@@ -26053,7 +25989,7 @@
       </c>
       <c r="F56" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE (intimate choice)</t>
+          <t>CA_PROT_06_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G56" s="77" t="inlineStr">
@@ -26085,7 +26021,7 @@
       </c>
       <c r="N56" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_05_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -26097,17 +26033,17 @@
       </c>
       <c r="B57" s="75" t="inlineStr">
         <is>
-          <t>Le Carcajou</t>
+          <t>La Chasse-Galerie</t>
         </is>
       </c>
       <c r="C57" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE_INTIMATE</t>
+          <t>CA_PROT_07_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D57" s="77" t="inlineStr">
         <is>
-          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDO... — BY MORNING</t>
+          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
         </is>
       </c>
       <c r="E57" s="79" t="inlineStr">
@@ -26117,7 +26053,7 @@
       </c>
       <c r="F57" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_06_AGREE (intimate choice)</t>
+          <t>CA_PROT_07_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G57" s="77" t="inlineStr">
@@ -26149,7 +26085,7 @@
       </c>
       <c r="N57" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_06_AGREE. By morning: emotional arc, no explicit imagery.</t>
+          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
       </c>
     </row>
@@ -26161,17 +26097,17 @@
       </c>
       <c r="B58" s="75" t="inlineStr">
         <is>
-          <t>La Chasse-Galerie</t>
+          <t>Le Gougou</t>
         </is>
       </c>
       <c r="C58" s="76" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE_INTIMATE</t>
+          <t>CA_PROT_08_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="D58" s="77" t="inlineStr">
         <is>
-          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW — BY MORNING</t>
+          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
         </is>
       </c>
       <c r="E58" s="79" t="inlineStr">
@@ -26181,7 +26117,7 @@
       </c>
       <c r="F58" s="77" t="inlineStr">
         <is>
-          <t>CA_PROT_07_AGREE (intimate choice)</t>
+          <t>CA_PROT_08_AGREE (intimate choice)</t>
         </is>
       </c>
       <c r="G58" s="77" t="inlineStr">
@@ -26213,111 +26149,47 @@
       </c>
       <c r="N58" s="77" t="inlineStr">
         <is>
-          <t>Stub — author intimate version of CA_PROT_07_AGREE. By morning: emotional arc, no explicit imagery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="75" t="inlineStr">
-        <is>
-          <t>CA Protector</t>
-        </is>
-      </c>
-      <c r="B59" s="75" t="inlineStr">
-        <is>
-          <t>Le Gougou</t>
-        </is>
-      </c>
-      <c r="C59" s="76" t="inlineStr">
-        <is>
-          <t>CA_PROT_08_AGREE_INTIMATE</t>
-        </is>
-      </c>
-      <c r="D59" s="77" t="inlineStr">
-        <is>
-          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE C... — BY MORNING</t>
-        </is>
-      </c>
-      <c r="E59" s="79" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="F59" s="77" t="inlineStr">
-        <is>
-          <t>CA_PROT_08_AGREE (intimate choice)</t>
-        </is>
-      </c>
-      <c r="G59" s="77" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="78" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I59" s="76" t="inlineStr"/>
-      <c r="J59" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K59" s="79" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L59" s="76" t="inlineStr"/>
-      <c r="M59" s="79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N59" s="77" t="inlineStr">
-        <is>
           <t>Stub — author intimate version of CA_PROT_08_AGREE. By morning: emotional arc, no explicit imagery.</t>
         </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="81" t="inlineStr">
+        <is>
+          <t>Canadian events total</t>
+        </is>
+      </c>
+      <c r="B60" s="82" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="81" t="inlineStr">
         <is>
-          <t>Canadian events total</t>
+          <t>Canada (Alliance arc)</t>
         </is>
       </c>
       <c r="B61" s="82" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="81" t="inlineStr">
         <is>
-          <t>Canada (Alliance arc)</t>
+          <t>CA Protector (Jessica's creatures)</t>
         </is>
       </c>
       <c r="B62" s="82" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="81" t="inlineStr">
         <is>
-          <t>CA Protector (Jessica's creatures)</t>
+          <t>Need explicit art (YES)</t>
         </is>
       </c>
       <c r="B63" s="82" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="81" t="inlineStr">
-        <is>
-          <t>Need explicit art (YES)</t>
-        </is>
-      </c>
-      <c r="B64" s="82" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Integrate art: PROT_01_SUMMON (updated) + PROT_01_TAME FULL COMPLETION
- mothman_approach.png: replaced with Ualani-spotting-Mothman scene
- prot_01_tame_scene.png: new — Mothman greeting Ualani as equals
- PROT_01_TAME marked FULL COMPLETION in masterdoc

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -2506,15 +2506,19 @@
           <t>→ PROT_01_AGREE (next_event_id)</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr"/>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
+          <t>prot_01_tame_scene</t>
+        </is>
+      </c>
+      <c r="J23" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K23" s="29" t="inlineStr">
@@ -22995,7 +22999,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Integrate art + FULL COMPLETION: PROT_01_AGREE (prot_01_agree.png)
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -2574,15 +2574,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I24" s="24" t="inlineStr"/>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I24" s="24" t="inlineStr">
+        <is>
+          <t>prot_01_agree</t>
+        </is>
+      </c>
+      <c r="J24" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K24" s="28" t="inlineStr">
@@ -22999,7 +23003,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Integrate art: full Jersey Devil arc FULL COMPLETION (PROT_02 SUMMON/TAME/AGREE/INTIMATE)
- jersey_devil.png: Pine Barrens emergence (dark, ominous)
- prot_02_tame.png: Ualani below Devil on telephone pole, NJ sky
- prot_02_agree.png: Silhouette against full moon — formal endorsement
- prot_02_agree_intimate.png: Close-up intimate Pine Barrens encounter

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -2646,9 +2646,9 @@
           <t>→ PROT_02_TAME</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H25" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I25" s="24" t="inlineStr">
@@ -2656,9 +2656,9 @@
           <t>jersey_devil</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J25" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K25" s="29" t="inlineStr">
@@ -2720,9 +2720,9 @@
         </is>
       </c>
       <c r="I26" s="24" t="inlineStr"/>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J26" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K26" s="29" t="inlineStr">
@@ -2784,9 +2784,9 @@
         </is>
       </c>
       <c r="I27" s="24" t="inlineStr"/>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J27" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr">
@@ -21691,66 +21691,70 @@
       </c>
     </row>
     <row r="334" ht="30" customHeight="1">
-      <c r="A334" s="79" t="inlineStr">
+      <c r="A334" s="23" t="inlineStr">
         <is>
           <t>Protector</t>
         </is>
       </c>
-      <c r="B334" s="79" t="inlineStr">
+      <c r="B334" s="23" t="inlineStr">
         <is>
           <t>Jersey Devil</t>
         </is>
       </c>
-      <c r="C334" s="80" t="inlineStr">
+      <c r="C334" s="24" t="inlineStr">
         <is>
           <t>PROT_02_AGREE_INTIMATE</t>
         </is>
       </c>
-      <c r="D334" s="81" t="inlineStr">
+      <c r="D334" s="25" t="inlineStr">
         <is>
           <t>JERSEY DEVIL FORMALLY ENDORSES THE CONTINENTAL CAUSE — BY MORNING</t>
         </is>
       </c>
-      <c r="E334" s="83" t="inlineStr">
+      <c r="E334" s="29" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="F334" s="81" t="inlineStr">
+      <c r="F334" s="25" t="inlineStr">
         <is>
           <t>PROT_02_AGREE (intimate choice)</t>
         </is>
       </c>
-      <c r="G334" s="81" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H334" s="82" t="inlineStr">
-        <is>
-          <t>IDEA</t>
-        </is>
-      </c>
-      <c r="I334" s="80" t="inlineStr"/>
-      <c r="J334" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K334" s="83" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L334" s="80" t="inlineStr"/>
-      <c r="M334" s="83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N334" s="81" t="inlineStr">
-        <is>
-          <t>Stub — author intimate version of PROT_02_AGREE. By morning: emotional arc, no explicit imagery.</t>
+      <c r="G334" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H334" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I334" s="24" t="inlineStr">
+        <is>
+          <t>prot_02_agree_intimate</t>
+        </is>
+      </c>
+      <c r="J334" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="K334" s="29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L334" s="24" t="inlineStr"/>
+      <c r="M334" s="29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N334" s="25" t="inlineStr">
+        <is>
+          <t>New Jersey's most complicated asset. By morning: recognition without negotiation.</t>
         </is>
       </c>
     </row>
@@ -23003,7 +23007,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">
@@ -23013,7 +23017,7 @@
         </is>
       </c>
       <c r="B358" s="86" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="359" ht="20" customHeight="1">

</xml_diff>

<commit_message>
EtherTask PROT_02_TAME: status → FULL COMPLETION in masterdoc
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -2714,12 +2714,16 @@
           <t>→ PROT_02_AGREE (next_event_id)</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I26" s="24" t="inlineStr"/>
+      <c r="H26" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I26" s="24" t="inlineStr">
+        <is>
+          <t>prot_02_tame</t>
+        </is>
+      </c>
       <c r="J26" s="27" t="inlineStr">
         <is>
           <t>Integrated</t>
@@ -23007,7 +23011,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
EtherTask ARC_01_DONE: status → FULL COMPLETION, art tag set
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -14350,12 +14350,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H210" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I210" s="32" t="inlineStr"/>
+      <c r="H210" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I210" s="32" t="inlineStr">
+        <is>
+          <t>arc_01_done_scene</t>
+        </is>
+      </c>
       <c r="J210" s="7" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -23011,7 +23015,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
EtherTask ARC_01_FIRST: status → FULL COMPLETION in masterdoc
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -14286,9 +14286,9 @@
           <t>ARC_01_DONE</t>
         </is>
       </c>
-      <c r="H209" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H209" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I209" s="32" t="inlineStr"/>
@@ -23219,7 +23219,7 @@
         </is>
       </c>
       <c r="B360" s="86" t="n">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="361" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Add anarchist army mechanic + GOV_LOYAL_ARC_17 buttons
- governor.gd: Add "Anarchistic" governor type with anarchist.png portrait
- army.gd: Add is_anarchist flag (no shield, uncontrollable)
- world.gd: Add tile_army_manpower_refill and spawn_anarchist outcomes;
  _spawn_anarchist_army() places an anarchist cell on UK soil;
  _tick_anarchists() auto-raids UK tiles each turn
- event_buttons.csv: GOV_LOYAL_ARC_17 BTN1=manpower refill, BTN2=spawn anarchist
- build_event_masterdoc.py: ARC_17 split from loop with FULL COMPLETION status
- event_masterdoc.xlsx: regenerated

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Plantation Deserter</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_17</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL PLANTATION DESERTER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL SWAMP WITCH)</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield magic×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL SWAMP WITCH)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARIBBEAN PRIVATEER)</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13754,7 +13754,7 @@
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>tile_yield magic×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Hawaiian Refugee</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_20</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARIBBEAN PRIVATEER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL HAWAIIAN REFUGEE)</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield food×3; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>Hawaiian Refugee</t>
+          <t>Border Mercenary</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_20</t>
+          <t>GOV_LOYAL_ARC_21</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL HAWAIIAN REFUGEE)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL BORDER MERCENARY)</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>tile_yield food×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield weapons×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13902,17 +13902,17 @@
       </c>
       <c r="B203" s="67" t="inlineStr">
         <is>
-          <t>Border Mercenary</t>
+          <t>Acadian Forest Ranger</t>
         </is>
       </c>
       <c r="C203" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_21</t>
+          <t>GOV_LOYAL_ARC_22</t>
         </is>
       </c>
       <c r="D203" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL BORDER MERCENARY)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="N203" s="69" t="inlineStr">
         <is>
-          <t>tile_yield weapons×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13970,17 +13970,17 @@
       </c>
       <c r="B204" s="67" t="inlineStr">
         <is>
-          <t>Acadian Forest Ranger</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C204" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_22</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D204" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
         </is>
       </c>
       <c r="E204" s="5" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="N204" s="69" t="inlineStr">
         <is>
-          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -14038,17 +14038,17 @@
       </c>
       <c r="B205" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C205" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D205" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E205" s="5" t="inlineStr">
@@ -14094,7 +14094,7 @@
       </c>
       <c r="N205" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -14106,17 +14106,17 @@
       </c>
       <c r="B206" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C206" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D206" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E206" s="5" t="inlineStr">
@@ -14162,7 +14162,7 @@
       </c>
       <c r="N206" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -14174,17 +14174,17 @@
       </c>
       <c r="B207" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Plantation Deserter</t>
         </is>
       </c>
       <c r="C207" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_17</t>
         </is>
       </c>
       <c r="D207" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RETURNS WITH RECRUITS WHO WERE WAITING</t>
         </is>
       </c>
       <c r="E207" s="5" t="inlineStr">
@@ -14202,15 +14202,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H207" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H207" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I207" s="68" t="inlineStr"/>
-      <c r="J207" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J207" s="71" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K207" s="70" t="inlineStr">
@@ -14230,7 +14230,7 @@
       </c>
       <c r="N207" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_army_manpower_refill; BTN2: spawn_anarchist; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23215,7 +23215,7 @@
         </is>
       </c>
       <c r="B360" s="86" t="n">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="361" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_16 custom buttons + loyal governor art=N/A
- governor.gd: Add governor_perks Array for perk flags
- building.gd: ARC_16 Community Steel — +1 metalPerLevel on Mines and
  Markets when community_steel perk is unlocked
- world.gd: Add state_building_level_yield outcome (counts all building
  levels in same state × amount → resource); add set_governor_perk outcome
- events.csv: Rewrite GOV_LOYAL_ARC_16 text to frame the choice
- event_buttons.csv: ARC_16 BTN1=state_building_level_yield metal×10,
  BTN2=set_governor_perk community_steel
- build_event_masterdoc.py: All loyal governor events now art_status=N/A
  (text-only); ARC_16 split out as FULL COMPLETION
- event_masterdoc.xlsx: regenerated

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -576,10 +576,10 @@
     <xf numFmtId="0" fontId="2" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -12576,12 +12576,12 @@
         </is>
       </c>
       <c r="I183" s="68" t="inlineStr"/>
-      <c r="J183" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K183" s="70" t="inlineStr">
+      <c r="J183" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K183" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -12591,14 +12591,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M183" s="70" t="inlineStr">
+      <c r="M183" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N183" s="69" t="inlineStr">
         <is>
-          <t>tile_yield food×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield food×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -12644,12 +12644,12 @@
         </is>
       </c>
       <c r="I184" s="68" t="inlineStr"/>
-      <c r="J184" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K184" s="70" t="inlineStr">
+      <c r="J184" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K184" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -12659,14 +12659,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M184" s="70" t="inlineStr">
+      <c r="M184" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N184" s="69" t="inlineStr">
         <is>
-          <t>tile_yield metal×5; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield metal×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -12712,12 +12712,12 @@
         </is>
       </c>
       <c r="I185" s="68" t="inlineStr"/>
-      <c r="J185" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K185" s="70" t="inlineStr">
+      <c r="J185" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K185" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -12727,14 +12727,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M185" s="70" t="inlineStr">
+      <c r="M185" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N185" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -12780,12 +12780,12 @@
         </is>
       </c>
       <c r="I186" s="68" t="inlineStr"/>
-      <c r="J186" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K186" s="70" t="inlineStr">
+      <c r="J186" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K186" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -12795,14 +12795,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M186" s="70" t="inlineStr">
+      <c r="M186" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N186" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield manpower×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -12848,12 +12848,12 @@
         </is>
       </c>
       <c r="I187" s="68" t="inlineStr"/>
-      <c r="J187" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K187" s="70" t="inlineStr">
+      <c r="J187" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K187" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -12863,14 +12863,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M187" s="70" t="inlineStr">
+      <c r="M187" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N187" s="69" t="inlineStr">
         <is>
-          <t>tile_yield food×5; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield food×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -12916,12 +12916,12 @@
         </is>
       </c>
       <c r="I188" s="68" t="inlineStr"/>
-      <c r="J188" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K188" s="70" t="inlineStr">
+      <c r="J188" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K188" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -12931,14 +12931,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M188" s="70" t="inlineStr">
+      <c r="M188" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N188" s="69" t="inlineStr">
         <is>
-          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -12984,12 +12984,12 @@
         </is>
       </c>
       <c r="I189" s="68" t="inlineStr"/>
-      <c r="J189" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K189" s="70" t="inlineStr">
+      <c r="J189" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K189" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -12999,14 +12999,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M189" s="70" t="inlineStr">
+      <c r="M189" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N189" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13052,12 +13052,12 @@
         </is>
       </c>
       <c r="I190" s="68" t="inlineStr"/>
-      <c r="J190" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K190" s="70" t="inlineStr">
+      <c r="J190" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K190" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13067,14 +13067,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M190" s="70" t="inlineStr">
+      <c r="M190" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N190" s="69" t="inlineStr">
         <is>
-          <t>tile_yield food×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield food×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13120,12 +13120,12 @@
         </is>
       </c>
       <c r="I191" s="68" t="inlineStr"/>
-      <c r="J191" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K191" s="70" t="inlineStr">
+      <c r="J191" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K191" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13135,14 +13135,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M191" s="70" t="inlineStr">
+      <c r="M191" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N191" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13188,12 +13188,12 @@
         </is>
       </c>
       <c r="I192" s="68" t="inlineStr"/>
-      <c r="J192" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K192" s="70" t="inlineStr">
+      <c r="J192" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K192" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13203,14 +13203,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M192" s="70" t="inlineStr">
+      <c r="M192" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N192" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield manpower×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13256,12 +13256,12 @@
         </is>
       </c>
       <c r="I193" s="68" t="inlineStr"/>
-      <c r="J193" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K193" s="70" t="inlineStr">
+      <c r="J193" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K193" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13271,14 +13271,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M193" s="70" t="inlineStr">
+      <c r="M193" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N193" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13324,12 +13324,12 @@
         </is>
       </c>
       <c r="I194" s="68" t="inlineStr"/>
-      <c r="J194" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K194" s="70" t="inlineStr">
+      <c r="J194" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K194" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13339,14 +13339,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M194" s="70" t="inlineStr">
+      <c r="M194" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N194" s="69" t="inlineStr">
         <is>
-          <t>tile_yield food×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield food×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13392,12 +13392,12 @@
         </is>
       </c>
       <c r="I195" s="68" t="inlineStr"/>
-      <c r="J195" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K195" s="70" t="inlineStr">
+      <c r="J195" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K195" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13407,14 +13407,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M195" s="70" t="inlineStr">
+      <c r="M195" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N195" s="69" t="inlineStr">
         <is>
-          <t>tile_yield boats×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield boats×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13460,12 +13460,12 @@
         </is>
       </c>
       <c r="I196" s="68" t="inlineStr"/>
-      <c r="J196" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K196" s="70" t="inlineStr">
+      <c r="J196" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K196" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13475,14 +13475,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M196" s="70" t="inlineStr">
+      <c r="M196" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N196" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13528,12 +13528,12 @@
         </is>
       </c>
       <c r="I197" s="68" t="inlineStr"/>
-      <c r="J197" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K197" s="70" t="inlineStr">
+      <c r="J197" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K197" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13543,14 +13543,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M197" s="70" t="inlineStr">
+      <c r="M197" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N197" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Rust Belt Steelworker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_16</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL RUST BELT STEELWORKER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL SWAMP WITCH)</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13596,12 +13596,12 @@
         </is>
       </c>
       <c r="I198" s="68" t="inlineStr"/>
-      <c r="J198" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K198" s="70" t="inlineStr">
+      <c r="J198" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K198" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13611,14 +13611,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M198" s="70" t="inlineStr">
+      <c r="M198" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>tile_yield metal×5; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield magic×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL SWAMP WITCH)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARIBBEAN PRIVATEER)</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13664,12 +13664,12 @@
         </is>
       </c>
       <c r="I199" s="68" t="inlineStr"/>
-      <c r="J199" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K199" s="70" t="inlineStr">
+      <c r="J199" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K199" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13679,14 +13679,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M199" s="70" t="inlineStr">
+      <c r="M199" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>tile_yield magic×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Hawaiian Refugee</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_20</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARIBBEAN PRIVATEER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL HAWAIIAN REFUGEE)</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13732,12 +13732,12 @@
         </is>
       </c>
       <c r="I200" s="68" t="inlineStr"/>
-      <c r="J200" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K200" s="70" t="inlineStr">
+      <c r="J200" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K200" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13747,14 +13747,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M200" s="70" t="inlineStr">
+      <c r="M200" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield food×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>Hawaiian Refugee</t>
+          <t>Border Mercenary</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_20</t>
+          <t>GOV_LOYAL_ARC_21</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL HAWAIIAN REFUGEE)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL BORDER MERCENARY)</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13800,12 +13800,12 @@
         </is>
       </c>
       <c r="I201" s="68" t="inlineStr"/>
-      <c r="J201" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K201" s="70" t="inlineStr">
+      <c r="J201" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K201" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13815,14 +13815,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M201" s="70" t="inlineStr">
+      <c r="M201" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>tile_yield food×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield weapons×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>Border Mercenary</t>
+          <t>Acadian Forest Ranger</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_21</t>
+          <t>GOV_LOYAL_ARC_22</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL BORDER MERCENARY)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13868,12 +13868,12 @@
         </is>
       </c>
       <c r="I202" s="68" t="inlineStr"/>
-      <c r="J202" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K202" s="70" t="inlineStr">
+      <c r="J202" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K202" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13883,14 +13883,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M202" s="70" t="inlineStr">
+      <c r="M202" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>tile_yield weapons×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13902,17 +13902,17 @@
       </c>
       <c r="B203" s="67" t="inlineStr">
         <is>
-          <t>Acadian Forest Ranger</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C203" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_22</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D203" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
@@ -13936,12 +13936,12 @@
         </is>
       </c>
       <c r="I203" s="68" t="inlineStr"/>
-      <c r="J203" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K203" s="70" t="inlineStr">
+      <c r="J203" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K203" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -13951,14 +13951,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M203" s="70" t="inlineStr">
+      <c r="M203" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N203" s="69" t="inlineStr">
         <is>
-          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13970,17 +13970,17 @@
       </c>
       <c r="B204" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C204" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D204" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E204" s="5" t="inlineStr">
@@ -14004,12 +14004,12 @@
         </is>
       </c>
       <c r="I204" s="68" t="inlineStr"/>
-      <c r="J204" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K204" s="70" t="inlineStr">
+      <c r="J204" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K204" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -14019,14 +14019,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M204" s="70" t="inlineStr">
+      <c r="M204" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N204" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -14038,17 +14038,17 @@
       </c>
       <c r="B205" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C205" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D205" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E205" s="5" t="inlineStr">
@@ -14072,12 +14072,12 @@
         </is>
       </c>
       <c r="I205" s="68" t="inlineStr"/>
-      <c r="J205" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K205" s="70" t="inlineStr">
+      <c r="J205" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K205" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -14087,14 +14087,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M205" s="70" t="inlineStr">
+      <c r="M205" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N205" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -14106,17 +14106,17 @@
       </c>
       <c r="B206" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Rust Belt Steelworker</t>
         </is>
       </c>
       <c r="C206" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_16</t>
         </is>
       </c>
       <c r="D206" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS A PROPOSAL FOR THE FOUNDRY</t>
         </is>
       </c>
       <c r="E206" s="5" t="inlineStr">
@@ -14134,18 +14134,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H206" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H206" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I206" s="68" t="inlineStr"/>
-      <c r="J206" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K206" s="70" t="inlineStr">
+      <c r="J206" s="70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K206" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -14155,14 +14155,14 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M206" s="70" t="inlineStr">
+      <c r="M206" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="N206" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: state_building_level_yield metal×10; BTN2: set_governor_perk community_steel; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -14208,12 +14208,12 @@
         </is>
       </c>
       <c r="I207" s="68" t="inlineStr"/>
-      <c r="J207" s="71" t="inlineStr">
+      <c r="J207" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K207" s="70" t="inlineStr">
+      <c r="K207" s="71" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -14223,7 +14223,7 @@
           <t>standard</t>
         </is>
       </c>
-      <c r="M207" s="70" t="inlineStr">
+      <c r="M207" s="71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -14292,7 +14292,7 @@
         </is>
       </c>
       <c r="I209" s="32" t="inlineStr"/>
-      <c r="J209" s="71" t="inlineStr">
+      <c r="J209" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14356,7 +14356,7 @@
         </is>
       </c>
       <c r="I210" s="32" t="inlineStr"/>
-      <c r="J210" s="71" t="inlineStr">
+      <c r="J210" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14420,7 +14420,7 @@
         </is>
       </c>
       <c r="I211" s="32" t="inlineStr"/>
-      <c r="J211" s="71" t="inlineStr">
+      <c r="J211" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14484,7 +14484,7 @@
         </is>
       </c>
       <c r="I212" s="32" t="inlineStr"/>
-      <c r="J212" s="71" t="inlineStr">
+      <c r="J212" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14548,7 +14548,7 @@
         </is>
       </c>
       <c r="I213" s="32" t="inlineStr"/>
-      <c r="J213" s="71" t="inlineStr">
+      <c r="J213" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14612,7 +14612,7 @@
         </is>
       </c>
       <c r="I214" s="32" t="inlineStr"/>
-      <c r="J214" s="71" t="inlineStr">
+      <c r="J214" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14676,7 +14676,7 @@
         </is>
       </c>
       <c r="I215" s="32" t="inlineStr"/>
-      <c r="J215" s="71" t="inlineStr">
+      <c r="J215" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14740,7 +14740,7 @@
         </is>
       </c>
       <c r="I216" s="32" t="inlineStr"/>
-      <c r="J216" s="71" t="inlineStr">
+      <c r="J216" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14804,7 +14804,7 @@
         </is>
       </c>
       <c r="I217" s="32" t="inlineStr"/>
-      <c r="J217" s="71" t="inlineStr">
+      <c r="J217" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14868,7 +14868,7 @@
         </is>
       </c>
       <c r="I218" s="32" t="inlineStr"/>
-      <c r="J218" s="71" t="inlineStr">
+      <c r="J218" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14932,7 +14932,7 @@
         </is>
       </c>
       <c r="I219" s="32" t="inlineStr"/>
-      <c r="J219" s="71" t="inlineStr">
+      <c r="J219" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -14996,7 +14996,7 @@
         </is>
       </c>
       <c r="I220" s="32" t="inlineStr"/>
-      <c r="J220" s="71" t="inlineStr">
+      <c r="J220" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15060,7 +15060,7 @@
         </is>
       </c>
       <c r="I221" s="32" t="inlineStr"/>
-      <c r="J221" s="71" t="inlineStr">
+      <c r="J221" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15124,7 +15124,7 @@
         </is>
       </c>
       <c r="I222" s="32" t="inlineStr"/>
-      <c r="J222" s="71" t="inlineStr">
+      <c r="J222" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15188,7 +15188,7 @@
         </is>
       </c>
       <c r="I223" s="32" t="inlineStr"/>
-      <c r="J223" s="71" t="inlineStr">
+      <c r="J223" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15252,7 +15252,7 @@
         </is>
       </c>
       <c r="I224" s="32" t="inlineStr"/>
-      <c r="J224" s="71" t="inlineStr">
+      <c r="J224" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15316,7 +15316,7 @@
         </is>
       </c>
       <c r="I225" s="32" t="inlineStr"/>
-      <c r="J225" s="71" t="inlineStr">
+      <c r="J225" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15380,7 +15380,7 @@
         </is>
       </c>
       <c r="I226" s="32" t="inlineStr"/>
-      <c r="J226" s="71" t="inlineStr">
+      <c r="J226" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15444,7 +15444,7 @@
         </is>
       </c>
       <c r="I227" s="32" t="inlineStr"/>
-      <c r="J227" s="71" t="inlineStr">
+      <c r="J227" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15508,7 +15508,7 @@
         </is>
       </c>
       <c r="I228" s="32" t="inlineStr"/>
-      <c r="J228" s="71" t="inlineStr">
+      <c r="J228" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15572,7 +15572,7 @@
         </is>
       </c>
       <c r="I229" s="32" t="inlineStr"/>
-      <c r="J229" s="71" t="inlineStr">
+      <c r="J229" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15636,7 +15636,7 @@
         </is>
       </c>
       <c r="I230" s="32" t="inlineStr"/>
-      <c r="J230" s="71" t="inlineStr">
+      <c r="J230" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15700,7 +15700,7 @@
         </is>
       </c>
       <c r="I231" s="32" t="inlineStr"/>
-      <c r="J231" s="71" t="inlineStr">
+      <c r="J231" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15764,7 +15764,7 @@
         </is>
       </c>
       <c r="I232" s="32" t="inlineStr"/>
-      <c r="J232" s="71" t="inlineStr">
+      <c r="J232" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15828,7 +15828,7 @@
         </is>
       </c>
       <c r="I233" s="32" t="inlineStr"/>
-      <c r="J233" s="71" t="inlineStr">
+      <c r="J233" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15892,7 +15892,7 @@
         </is>
       </c>
       <c r="I234" s="32" t="inlineStr"/>
-      <c r="J234" s="71" t="inlineStr">
+      <c r="J234" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -15956,7 +15956,7 @@
         </is>
       </c>
       <c r="I235" s="32" t="inlineStr"/>
-      <c r="J235" s="71" t="inlineStr">
+      <c r="J235" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16020,7 +16020,7 @@
         </is>
       </c>
       <c r="I236" s="32" t="inlineStr"/>
-      <c r="J236" s="71" t="inlineStr">
+      <c r="J236" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16084,7 +16084,7 @@
         </is>
       </c>
       <c r="I237" s="32" t="inlineStr"/>
-      <c r="J237" s="71" t="inlineStr">
+      <c r="J237" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16148,7 +16148,7 @@
         </is>
       </c>
       <c r="I238" s="32" t="inlineStr"/>
-      <c r="J238" s="71" t="inlineStr">
+      <c r="J238" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16212,7 +16212,7 @@
         </is>
       </c>
       <c r="I239" s="32" t="inlineStr"/>
-      <c r="J239" s="71" t="inlineStr">
+      <c r="J239" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16276,7 +16276,7 @@
         </is>
       </c>
       <c r="I240" s="32" t="inlineStr"/>
-      <c r="J240" s="71" t="inlineStr">
+      <c r="J240" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16340,7 +16340,7 @@
         </is>
       </c>
       <c r="I241" s="32" t="inlineStr"/>
-      <c r="J241" s="71" t="inlineStr">
+      <c r="J241" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16404,7 +16404,7 @@
         </is>
       </c>
       <c r="I242" s="32" t="inlineStr"/>
-      <c r="J242" s="71" t="inlineStr">
+      <c r="J242" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16468,7 +16468,7 @@
         </is>
       </c>
       <c r="I243" s="32" t="inlineStr"/>
-      <c r="J243" s="71" t="inlineStr">
+      <c r="J243" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16532,7 +16532,7 @@
         </is>
       </c>
       <c r="I244" s="32" t="inlineStr"/>
-      <c r="J244" s="71" t="inlineStr">
+      <c r="J244" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16596,7 +16596,7 @@
         </is>
       </c>
       <c r="I245" s="32" t="inlineStr"/>
-      <c r="J245" s="71" t="inlineStr">
+      <c r="J245" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16660,7 +16660,7 @@
         </is>
       </c>
       <c r="I246" s="32" t="inlineStr"/>
-      <c r="J246" s="71" t="inlineStr">
+      <c r="J246" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16724,7 +16724,7 @@
         </is>
       </c>
       <c r="I247" s="32" t="inlineStr"/>
-      <c r="J247" s="71" t="inlineStr">
+      <c r="J247" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16788,7 +16788,7 @@
         </is>
       </c>
       <c r="I248" s="32" t="inlineStr"/>
-      <c r="J248" s="71" t="inlineStr">
+      <c r="J248" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16852,7 +16852,7 @@
         </is>
       </c>
       <c r="I249" s="32" t="inlineStr"/>
-      <c r="J249" s="71" t="inlineStr">
+      <c r="J249" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16916,7 +16916,7 @@
         </is>
       </c>
       <c r="I250" s="32" t="inlineStr"/>
-      <c r="J250" s="71" t="inlineStr">
+      <c r="J250" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16980,7 +16980,7 @@
         </is>
       </c>
       <c r="I251" s="32" t="inlineStr"/>
-      <c r="J251" s="71" t="inlineStr">
+      <c r="J251" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -17044,7 +17044,7 @@
         </is>
       </c>
       <c r="I252" s="32" t="inlineStr"/>
-      <c r="J252" s="71" t="inlineStr">
+      <c r="J252" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -17108,7 +17108,7 @@
         </is>
       </c>
       <c r="I253" s="32" t="inlineStr"/>
-      <c r="J253" s="71" t="inlineStr">
+      <c r="J253" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -17172,7 +17172,7 @@
         </is>
       </c>
       <c r="I254" s="32" t="inlineStr"/>
-      <c r="J254" s="71" t="inlineStr">
+      <c r="J254" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -17236,7 +17236,7 @@
         </is>
       </c>
       <c r="I255" s="32" t="inlineStr"/>
-      <c r="J255" s="71" t="inlineStr">
+      <c r="J255" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -17300,7 +17300,7 @@
         </is>
       </c>
       <c r="I256" s="32" t="inlineStr"/>
-      <c r="J256" s="71" t="inlineStr">
+      <c r="J256" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="I257" s="32" t="inlineStr"/>
-      <c r="J257" s="71" t="inlineStr">
+      <c r="J257" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -17428,7 +17428,7 @@
         </is>
       </c>
       <c r="I258" s="32" t="inlineStr"/>
-      <c r="J258" s="71" t="inlineStr">
+      <c r="J258" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -19700,7 +19700,7 @@
         </is>
       </c>
       <c r="I296" s="81" t="inlineStr"/>
-      <c r="J296" s="71" t="inlineStr">
+      <c r="J296" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -19780,7 +19780,7 @@
         </is>
       </c>
       <c r="I298" s="81" t="inlineStr"/>
-      <c r="J298" s="71" t="inlineStr">
+      <c r="J298" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -19860,7 +19860,7 @@
         </is>
       </c>
       <c r="I300" s="81" t="inlineStr"/>
-      <c r="J300" s="71" t="inlineStr">
+      <c r="J300" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -19940,7 +19940,7 @@
         </is>
       </c>
       <c r="I302" s="81" t="inlineStr"/>
-      <c r="J302" s="71" t="inlineStr">
+      <c r="J302" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20004,7 +20004,7 @@
         </is>
       </c>
       <c r="I303" s="81" t="inlineStr"/>
-      <c r="J303" s="71" t="inlineStr">
+      <c r="J303" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20084,7 +20084,7 @@
         </is>
       </c>
       <c r="I305" s="81" t="inlineStr"/>
-      <c r="J305" s="71" t="inlineStr">
+      <c r="J305" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20148,7 +20148,7 @@
         </is>
       </c>
       <c r="I306" s="81" t="inlineStr"/>
-      <c r="J306" s="71" t="inlineStr">
+      <c r="J306" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20212,7 +20212,7 @@
         </is>
       </c>
       <c r="I307" s="81" t="inlineStr"/>
-      <c r="J307" s="71" t="inlineStr">
+      <c r="J307" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20276,7 +20276,7 @@
         </is>
       </c>
       <c r="I308" s="81" t="inlineStr"/>
-      <c r="J308" s="71" t="inlineStr">
+      <c r="J308" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20356,7 +20356,7 @@
         </is>
       </c>
       <c r="I310" s="81" t="inlineStr"/>
-      <c r="J310" s="71" t="inlineStr">
+      <c r="J310" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20420,7 +20420,7 @@
         </is>
       </c>
       <c r="I311" s="81" t="inlineStr"/>
-      <c r="J311" s="71" t="inlineStr">
+      <c r="J311" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20484,7 +20484,7 @@
         </is>
       </c>
       <c r="I312" s="81" t="inlineStr"/>
-      <c r="J312" s="71" t="inlineStr">
+      <c r="J312" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20548,7 +20548,7 @@
         </is>
       </c>
       <c r="I313" s="81" t="inlineStr"/>
-      <c r="J313" s="71" t="inlineStr">
+      <c r="J313" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20612,7 +20612,7 @@
         </is>
       </c>
       <c r="I314" s="81" t="inlineStr"/>
-      <c r="J314" s="71" t="inlineStr">
+      <c r="J314" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20676,7 +20676,7 @@
         </is>
       </c>
       <c r="I315" s="81" t="inlineStr"/>
-      <c r="J315" s="71" t="inlineStr">
+      <c r="J315" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20740,7 +20740,7 @@
         </is>
       </c>
       <c r="I316" s="81" t="inlineStr"/>
-      <c r="J316" s="71" t="inlineStr">
+      <c r="J316" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20820,7 +20820,7 @@
         </is>
       </c>
       <c r="I318" s="81" t="inlineStr"/>
-      <c r="J318" s="71" t="inlineStr">
+      <c r="J318" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20884,7 +20884,7 @@
         </is>
       </c>
       <c r="I319" s="81" t="inlineStr"/>
-      <c r="J319" s="71" t="inlineStr">
+      <c r="J319" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20948,7 +20948,7 @@
         </is>
       </c>
       <c r="I320" s="81" t="inlineStr"/>
-      <c r="J320" s="71" t="inlineStr">
+      <c r="J320" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21012,7 +21012,7 @@
         </is>
       </c>
       <c r="I321" s="81" t="inlineStr"/>
-      <c r="J321" s="71" t="inlineStr">
+      <c r="J321" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21076,7 +21076,7 @@
         </is>
       </c>
       <c r="I322" s="81" t="inlineStr"/>
-      <c r="J322" s="71" t="inlineStr">
+      <c r="J322" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21140,7 +21140,7 @@
         </is>
       </c>
       <c r="I323" s="81" t="inlineStr"/>
-      <c r="J323" s="71" t="inlineStr">
+      <c r="J323" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21204,7 +21204,7 @@
         </is>
       </c>
       <c r="I324" s="81" t="inlineStr"/>
-      <c r="J324" s="71" t="inlineStr">
+      <c r="J324" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21268,7 +21268,7 @@
         </is>
       </c>
       <c r="I325" s="81" t="inlineStr"/>
-      <c r="J325" s="71" t="inlineStr">
+      <c r="J325" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21348,7 +21348,7 @@
         </is>
       </c>
       <c r="I327" s="81" t="inlineStr"/>
-      <c r="J327" s="71" t="inlineStr">
+      <c r="J327" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21412,7 +21412,7 @@
         </is>
       </c>
       <c r="I328" s="81" t="inlineStr"/>
-      <c r="J328" s="71" t="inlineStr">
+      <c r="J328" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21476,7 +21476,7 @@
         </is>
       </c>
       <c r="I329" s="81" t="inlineStr"/>
-      <c r="J329" s="71" t="inlineStr">
+      <c r="J329" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21540,7 +21540,7 @@
         </is>
       </c>
       <c r="I330" s="81" t="inlineStr"/>
-      <c r="J330" s="71" t="inlineStr">
+      <c r="J330" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21604,7 +21604,7 @@
         </is>
       </c>
       <c r="I331" s="81" t="inlineStr"/>
-      <c r="J331" s="71" t="inlineStr">
+      <c r="J331" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21668,7 +21668,7 @@
         </is>
       </c>
       <c r="I332" s="81" t="inlineStr"/>
-      <c r="J332" s="71" t="inlineStr">
+      <c r="J332" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21732,7 +21732,7 @@
         </is>
       </c>
       <c r="I333" s="81" t="inlineStr"/>
-      <c r="J333" s="71" t="inlineStr">
+      <c r="J333" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21796,7 +21796,7 @@
         </is>
       </c>
       <c r="I334" s="81" t="inlineStr"/>
-      <c r="J334" s="71" t="inlineStr">
+      <c r="J334" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21876,7 +21876,7 @@
         </is>
       </c>
       <c r="I336" s="81" t="inlineStr"/>
-      <c r="J336" s="71" t="inlineStr">
+      <c r="J336" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22008,7 +22008,7 @@
         </is>
       </c>
       <c r="I338" s="81" t="inlineStr"/>
-      <c r="J338" s="71" t="inlineStr">
+      <c r="J338" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22072,7 +22072,7 @@
         </is>
       </c>
       <c r="I339" s="81" t="inlineStr"/>
-      <c r="J339" s="71" t="inlineStr">
+      <c r="J339" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22136,7 +22136,7 @@
         </is>
       </c>
       <c r="I340" s="81" t="inlineStr"/>
-      <c r="J340" s="71" t="inlineStr">
+      <c r="J340" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22200,7 +22200,7 @@
         </is>
       </c>
       <c r="I341" s="81" t="inlineStr"/>
-      <c r="J341" s="71" t="inlineStr">
+      <c r="J341" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22264,7 +22264,7 @@
         </is>
       </c>
       <c r="I342" s="81" t="inlineStr"/>
-      <c r="J342" s="71" t="inlineStr">
+      <c r="J342" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22328,7 +22328,7 @@
         </is>
       </c>
       <c r="I343" s="81" t="inlineStr"/>
-      <c r="J343" s="71" t="inlineStr">
+      <c r="J343" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22392,7 +22392,7 @@
         </is>
       </c>
       <c r="I344" s="81" t="inlineStr"/>
-      <c r="J344" s="71" t="inlineStr">
+      <c r="J344" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22456,7 +22456,7 @@
         </is>
       </c>
       <c r="I345" s="81" t="inlineStr"/>
-      <c r="J345" s="71" t="inlineStr">
+      <c r="J345" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22520,7 +22520,7 @@
         </is>
       </c>
       <c r="I346" s="81" t="inlineStr"/>
-      <c r="J346" s="71" t="inlineStr">
+      <c r="J346" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22584,7 +22584,7 @@
         </is>
       </c>
       <c r="I347" s="81" t="inlineStr"/>
-      <c r="J347" s="71" t="inlineStr">
+      <c r="J347" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22648,7 +22648,7 @@
         </is>
       </c>
       <c r="I348" s="81" t="inlineStr"/>
-      <c r="J348" s="71" t="inlineStr">
+      <c r="J348" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22712,7 +22712,7 @@
         </is>
       </c>
       <c r="I349" s="81" t="inlineStr"/>
-      <c r="J349" s="71" t="inlineStr">
+      <c r="J349" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22776,7 +22776,7 @@
         </is>
       </c>
       <c r="I350" s="81" t="inlineStr"/>
-      <c r="J350" s="71" t="inlineStr">
+      <c r="J350" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22840,7 +22840,7 @@
         </is>
       </c>
       <c r="I351" s="81" t="inlineStr"/>
-      <c r="J351" s="71" t="inlineStr">
+      <c r="J351" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22904,7 +22904,7 @@
         </is>
       </c>
       <c r="I352" s="81" t="inlineStr"/>
-      <c r="J352" s="71" t="inlineStr">
+      <c r="J352" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22984,7 +22984,7 @@
         </is>
       </c>
       <c r="I354" s="81" t="inlineStr"/>
-      <c r="J354" s="71" t="inlineStr">
+      <c r="J354" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -23048,7 +23048,7 @@
         </is>
       </c>
       <c r="I355" s="81" t="inlineStr"/>
-      <c r="J355" s="71" t="inlineStr">
+      <c r="J355" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -23112,7 +23112,7 @@
         </is>
       </c>
       <c r="I356" s="81" t="inlineStr"/>
-      <c r="J356" s="71" t="inlineStr">
+      <c r="J356" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -23176,7 +23176,7 @@
         </is>
       </c>
       <c r="I357" s="81" t="inlineStr"/>
-      <c r="J357" s="71" t="inlineStr">
+      <c r="J357" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -23215,7 +23215,7 @@
         </is>
       </c>
       <c r="B360" s="86" t="n">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="361" ht="20" customHeight="1">
@@ -26022,7 +26022,7 @@
         </is>
       </c>
       <c r="I43" s="81" t="inlineStr"/>
-      <c r="J43" s="71" t="inlineStr">
+      <c r="J43" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26086,7 +26086,7 @@
         </is>
       </c>
       <c r="I44" s="81" t="inlineStr"/>
-      <c r="J44" s="71" t="inlineStr">
+      <c r="J44" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26150,7 +26150,7 @@
         </is>
       </c>
       <c r="I45" s="81" t="inlineStr"/>
-      <c r="J45" s="71" t="inlineStr">
+      <c r="J45" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26214,7 +26214,7 @@
         </is>
       </c>
       <c r="I46" s="81" t="inlineStr"/>
-      <c r="J46" s="71" t="inlineStr">
+      <c r="J46" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26278,7 +26278,7 @@
         </is>
       </c>
       <c r="I47" s="81" t="inlineStr"/>
-      <c r="J47" s="71" t="inlineStr">
+      <c r="J47" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26342,7 +26342,7 @@
         </is>
       </c>
       <c r="I48" s="81" t="inlineStr"/>
-      <c r="J48" s="71" t="inlineStr">
+      <c r="J48" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26406,7 +26406,7 @@
         </is>
       </c>
       <c r="I49" s="81" t="inlineStr"/>
-      <c r="J49" s="71" t="inlineStr">
+      <c r="J49" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26486,7 +26486,7 @@
         </is>
       </c>
       <c r="I51" s="81" t="inlineStr"/>
-      <c r="J51" s="71" t="inlineStr">
+      <c r="J51" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26550,7 +26550,7 @@
         </is>
       </c>
       <c r="I52" s="81" t="inlineStr"/>
-      <c r="J52" s="71" t="inlineStr">
+      <c r="J52" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26614,7 +26614,7 @@
         </is>
       </c>
       <c r="I53" s="81" t="inlineStr"/>
-      <c r="J53" s="71" t="inlineStr">
+      <c r="J53" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26678,7 +26678,7 @@
         </is>
       </c>
       <c r="I54" s="81" t="inlineStr"/>
-      <c r="J54" s="71" t="inlineStr">
+      <c r="J54" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26742,7 +26742,7 @@
         </is>
       </c>
       <c r="I55" s="81" t="inlineStr"/>
-      <c r="J55" s="71" t="inlineStr">
+      <c r="J55" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26806,7 +26806,7 @@
         </is>
       </c>
       <c r="I56" s="81" t="inlineStr"/>
-      <c r="J56" s="71" t="inlineStr">
+      <c r="J56" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26870,7 +26870,7 @@
         </is>
       </c>
       <c r="I57" s="81" t="inlineStr"/>
-      <c r="J57" s="71" t="inlineStr">
+      <c r="J57" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -26934,7 +26934,7 @@
         </is>
       </c>
       <c r="I58" s="81" t="inlineStr"/>
-      <c r="J58" s="71" t="inlineStr">
+      <c r="J58" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_21 Border Mercenary custom buttons + army buff system
- army.gd: Add Mercenary Zeal (+2 punch, timed) and Iron Discipline
  (+1 defence, permanent) to _apply_status_effects_to_stats
- world.gd: Implement _apply_army_buff (applies status to tile army);
  add gold_and_army_buff outcome (50 gold + named buff on tile army)
- events.csv: Rewrite GOV_LOYAL_ARC_21 as Patriotic Display event
- event_buttons.csv: ARC_21 BTN1=gold+Mercenary Zeal×10, BTN2=Iron Discipline×9999
- build_event_masterdoc.py: ARC_21 split out as FULL COMPLETION
- event_masterdoc.xlsx: regenerated

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>Border Mercenary</t>
+          <t>Acadian Forest Ranger</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_21</t>
+          <t>GOV_LOYAL_ARC_22</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL BORDER MERCENARY)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>tile_yield weapons×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>Acadian Forest Ranger</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_22</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13902,17 +13902,17 @@
       </c>
       <c r="B203" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C203" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D203" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="N203" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13970,17 +13970,17 @@
       </c>
       <c r="B204" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C204" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D204" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E204" s="5" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="N204" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -14038,17 +14038,17 @@
       </c>
       <c r="B205" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Rust Belt Steelworker</t>
         </is>
       </c>
       <c r="C205" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_16</t>
         </is>
       </c>
       <c r="D205" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS A PROPOSAL FOR THE FOUNDRY</t>
         </is>
       </c>
       <c r="E205" s="5" t="inlineStr">
@@ -14066,9 +14066,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H205" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H205" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I205" s="68" t="inlineStr"/>
@@ -14094,7 +14094,7 @@
       </c>
       <c r="N205" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: state_building_level_yield metal×10; BTN2: set_governor_perk community_steel; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -14106,17 +14106,17 @@
       </c>
       <c r="B206" s="67" t="inlineStr">
         <is>
-          <t>Rust Belt Steelworker</t>
+          <t>Plantation Deserter</t>
         </is>
       </c>
       <c r="C206" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_16</t>
+          <t>GOV_LOYAL_ARC_17</t>
         </is>
       </c>
       <c r="D206" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS A PROPOSAL FOR THE FOUNDRY</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RETURNS WITH RECRUITS WHO WERE WAITING</t>
         </is>
       </c>
       <c r="E206" s="5" t="inlineStr">
@@ -14162,7 +14162,7 @@
       </c>
       <c r="N206" s="69" t="inlineStr">
         <is>
-          <t>BTN1: state_building_level_yield metal×10; BTN2: set_governor_perk community_steel; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_army_manpower_refill; BTN2: spawn_anarchist; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -14174,17 +14174,17 @@
       </c>
       <c r="B207" s="67" t="inlineStr">
         <is>
-          <t>Plantation Deserter</t>
+          <t>Border Mercenary</t>
         </is>
       </c>
       <c r="C207" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_17</t>
+          <t>GOV_LOYAL_ARC_21</t>
         </is>
       </c>
       <c r="D207" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RETURNS WITH RECRUITS WHO WERE WAITING</t>
+          <t>MERCENARY COMMANDER'S PATRIOTIC DISPLAY</t>
         </is>
       </c>
       <c r="E207" s="5" t="inlineStr">
@@ -14230,7 +14230,7 @@
       </c>
       <c r="N207" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_army_manpower_refill; BTN2: spawn_anarchist; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: gold_and_army_buff Mercenary Zeal×10 turns + 50 gold; BTN2: army_buff Iron Discipline permanent; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23215,7 +23215,7 @@
         </is>
       </c>
       <c r="B360" s="86" t="n">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="361" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_19 Caribbean Privateer — text polish + FULL COMPLETION
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Acadian Forest Ranger</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_22</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARIBBEAN PRIVATEER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Acadian Forest Ranger</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_22</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13754,7 +13754,7 @@
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13902,17 +13902,17 @@
       </c>
       <c r="B203" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C203" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D203" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
@@ -13930,9 +13930,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H203" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H203" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I203" s="68" t="inlineStr"/>
@@ -13958,7 +13958,7 @@
       </c>
       <c r="N203" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_18 Swamp Witch — Power vs Knowledge choice
- events.csv: Mystery bottle message from the deep swamp
- event_buttons.csv: BTN1=tile_yield magic×10, BTN2=level_all_spell_schools×10
- world.gd: Add level_all_spell_schools outcome (+N levels to all 6 schools)
- build_event_masterdoc.py: ARC_18 split out as FULL COMPLETION

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Acadian Forest Ranger</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_22</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL SWAMP WITCH)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>tile_yield magic×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Acadian Forest Ranger</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_22</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13754,7 +13754,7 @@
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13862,9 +13862,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H202" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H202" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I202" s="68" t="inlineStr"/>
@@ -13890,7 +13890,7 @@
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_22 Acadian Forest Ranger — text polish + FULL COMPLETION
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Acadian Forest Ranger</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_22</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL ACADIAN FOREST RANGER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>tile_yield wood×5; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13754,7 +13754,7 @@
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13794,9 +13794,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H201" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H201" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I201" s="68" t="inlineStr"/>
@@ -13822,7 +13822,7 @@
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13902,17 +13902,17 @@
       </c>
       <c r="B203" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Rust Belt Steelworker</t>
         </is>
       </c>
       <c r="C203" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_16</t>
         </is>
       </c>
       <c r="D203" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS A PROPOSAL FOR THE FOUNDRY</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="N203" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: state_building_level_yield metal×10; BTN2: set_governor_perk community_steel; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13970,17 +13970,17 @@
       </c>
       <c r="B204" s="67" t="inlineStr">
         <is>
-          <t>Rust Belt Steelworker</t>
+          <t>Plantation Deserter</t>
         </is>
       </c>
       <c r="C204" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_16</t>
+          <t>GOV_LOYAL_ARC_17</t>
         </is>
       </c>
       <c r="D204" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS A PROPOSAL FOR THE FOUNDRY</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RETURNS WITH RECRUITS WHO WERE WAITING</t>
         </is>
       </c>
       <c r="E204" s="5" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="N204" s="69" t="inlineStr">
         <is>
-          <t>BTN1: state_building_level_yield metal×10; BTN2: set_governor_perk community_steel; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_army_manpower_refill; BTN2: spawn_anarchist; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -14038,17 +14038,17 @@
       </c>
       <c r="B205" s="67" t="inlineStr">
         <is>
-          <t>Plantation Deserter</t>
+          <t>Acadian Forest Ranger</t>
         </is>
       </c>
       <c r="C205" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_17</t>
+          <t>GOV_LOYAL_ARC_22</t>
         </is>
       </c>
       <c r="D205" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RETURNS WITH RECRUITS WHO WERE WAITING</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS MAPPED EVERY TIMBER STAND WITHIN TWO DAYS' TRAVEL</t>
         </is>
       </c>
       <c r="E205" s="5" t="inlineStr">
@@ -14094,7 +14094,7 @@
       </c>
       <c r="N205" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_army_manpower_refill; BTN2: spawn_anarchist; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield wood×5; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_15 DC Bureaucrat — two-button choice, corrupt windfall
- event_buttons.csv: BTN1 keeps tile_yield gold×4 (eagle-eyed praise);
  BTN2 new corrupt_windfall — 10× tile gold output + 20 corruption
- world.gd: Add corrupt_windfall outcome (big yield + tile.corruption +20)
- build_event_masterdoc.py: ARC_15 split out as FULL COMPLETION

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13494,17 +13494,17 @@
       </c>
       <c r="B197" s="67" t="inlineStr">
         <is>
-          <t>DC Bureaucrat</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C197" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_15</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D197" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL DC BUREAUCRAT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
@@ -13550,7 +13550,7 @@
       </c>
       <c r="N197" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13726,9 +13726,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H200" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H200" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I200" s="68" t="inlineStr"/>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>DC Bureaucrat</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_15</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] AUDITS [TILE_NAME] AND FINDS THREE YEARS OF ACCOUNTING ERROR</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; BTN2: corrupt_windfall gold×10 +20 corruption; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_23 Gettysburg Descendant — text polish + FULL COMPLETION
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13494,17 +13494,17 @@
       </c>
       <c r="B197" s="67" t="inlineStr">
         <is>
-          <t>Gettysburg Descendant</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C197" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_23</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D197" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL GETTYSBURG DESCENDANT)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
@@ -13550,7 +13550,7 @@
       </c>
       <c r="N197" s="69" t="inlineStr">
         <is>
-          <t>tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13658,9 +13658,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H199" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H199" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I199" s="68" t="inlineStr"/>
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13754,7 +13754,7 @@
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13766,17 +13766,17 @@
       </c>
       <c r="B201" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>DC Bureaucrat</t>
         </is>
       </c>
       <c r="C201" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_15</t>
         </is>
       </c>
       <c r="D201" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] AUDITS [TILE_NAME] AND FINDS THREE YEARS OF ACCOUNTING ERROR</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="N201" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; BTN2: corrupt_windfall gold×10 +20 corruption; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13834,17 +13834,17 @@
       </c>
       <c r="B202" s="67" t="inlineStr">
         <is>
-          <t>DC Bureaucrat</t>
+          <t>Rust Belt Steelworker</t>
         </is>
       </c>
       <c r="C202" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_15</t>
+          <t>GOV_LOYAL_ARC_16</t>
         </is>
       </c>
       <c r="D202" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] AUDITS [TILE_NAME] AND FINDS THREE YEARS OF ACCOUNTING ERROR</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS A PROPOSAL FOR THE FOUNDRY</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="N202" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; BTN2: corrupt_windfall gold×10 +20 corruption; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: state_building_level_yield metal×10; BTN2: set_governor_perk community_steel; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13902,17 +13902,17 @@
       </c>
       <c r="B203" s="67" t="inlineStr">
         <is>
-          <t>Rust Belt Steelworker</t>
+          <t>Plantation Deserter</t>
         </is>
       </c>
       <c r="C203" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_16</t>
+          <t>GOV_LOYAL_ARC_17</t>
         </is>
       </c>
       <c r="D203" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] HAS A PROPOSAL FOR THE FOUNDRY</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RETURNS WITH RECRUITS WHO WERE WAITING</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="N203" s="69" t="inlineStr">
         <is>
-          <t>BTN1: state_building_level_yield metal×10; BTN2: set_governor_perk community_steel; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_army_manpower_refill; BTN2: spawn_anarchist; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13970,17 +13970,17 @@
       </c>
       <c r="B204" s="67" t="inlineStr">
         <is>
-          <t>Plantation Deserter</t>
+          <t>Gettysburg Descendant</t>
         </is>
       </c>
       <c r="C204" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_17</t>
+          <t>GOV_LOYAL_ARC_23</t>
         </is>
       </c>
       <c r="D204" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RETURNS WITH RECRUITS WHO WERE WAITING</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] POSTS ONE MUSTER NOTICE; THE LINE FORMS BEFORE DAWN</t>
         </is>
       </c>
       <c r="E204" s="5" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="N204" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_army_manpower_refill; BTN2: spawn_anarchist; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield manpower×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_14 Frontier Preacher — text polish + FULL COMPLETION
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13426,17 +13426,17 @@
       </c>
       <c r="B196" s="67" t="inlineStr">
         <is>
-          <t>Frontier Preacher</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C196" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_14</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D196" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL FRONTIER PREACHER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
@@ -13494,17 +13494,17 @@
       </c>
       <c r="B197" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C197" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D197" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
@@ -13550,7 +13550,7 @@
       </c>
       <c r="N197" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13590,9 +13590,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H198" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H198" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I198" s="68" t="inlineStr"/>
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Frontier Preacher</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_14</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RIDES ELEVEN DAYS THROUGH FOUR SETTLEMENTS AND COMES BACK WITH PLEDGES FROM ALL OF THEM</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -13754,7 +13754,7 @@
       </c>
       <c r="N200" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_24 + ARC_14 update — two events polished, ARC_14 two-button
- events.csv: ARC_24 LGBTQ+ Organizer text polished; ARC_14 Frontier
  Preacher updated with new headline and two-choice text
- event_buttons.csv: ARC_14 BTN1=tile_yield culture×5, BTN2=1000 manpower;
  ARC_24 keeps single tile_yield culture×4
- build_event_masterdoc.py: both split out as FULL COMPLETION

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13426,17 +13426,17 @@
       </c>
       <c r="B196" s="67" t="inlineStr">
         <is>
-          <t>LGBTQ+ Organizer</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C196" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_24</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D196" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL LGBTQ+ ORGANIZER)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="N196" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13494,17 +13494,17 @@
       </c>
       <c r="B197" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C197" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D197" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
@@ -13522,9 +13522,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H197" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H197" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I197" s="68" t="inlineStr"/>
@@ -13550,7 +13550,7 @@
       </c>
       <c r="N197" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Frontier Preacher</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_14</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>FRONTIER PREACHER INSPIRES THOUSANDS</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield culture×5; BTN2: resource_change manpower 1000; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13698,17 +13698,17 @@
       </c>
       <c r="B200" s="67" t="inlineStr">
         <is>
-          <t>Frontier Preacher</t>
+          <t>LGBTQ+ Organizer</t>
         </is>
       </c>
       <c r="C200" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_14</t>
+          <t>GOV_LOYAL_ARC_24</t>
         </is>
       </c>
       <c r="D200" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] RIDES ELEVEN DAYS THROUGH FOUR SETTLEMENTS AND COMES BACK WITH PLEDGES FROM ALL OF THEM</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] ORGANIZED SOMETHING NOBODY OFFICIALLY SANCTIONED AND EVERYONE SHOWED UP</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_13 Nantucket Sailor — text polish + FULL COMPLETION
https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13358,17 +13358,17 @@
       </c>
       <c r="B195" s="67" t="inlineStr">
         <is>
-          <t>Nantucket Sailor</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C195" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_13</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D195" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL NANTUCKET SAILOR)</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
@@ -13414,7 +13414,7 @@
       </c>
       <c r="N195" s="69" t="inlineStr">
         <is>
-          <t>tile_yield boats×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
         </is>
       </c>
     </row>
@@ -13426,17 +13426,17 @@
       </c>
       <c r="B196" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C196" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D196" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
@@ -13454,9 +13454,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H196" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H196" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I196" s="68" t="inlineStr"/>
@@ -13482,7 +13482,7 @@
       </c>
       <c r="N196" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13494,17 +13494,17 @@
       </c>
       <c r="B197" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C197" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D197" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
@@ -13550,7 +13550,7 @@
       </c>
       <c r="N197" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Nantucket Sailor</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_13</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] REFLOATS A HULL THAT WAS LISTED ON THE CHARTS AS A NAVIGATION HAZARD</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield boats×3; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
GOV_LOYAL_ARC_25 Carnival Barker — For One Night Only + two buttons
- events.csv: Full rewrite — Ualani speech replacing the elephant act
- event_buttons.csv: BTN1=tile_yield gold×5 (war bonds); BTN2=tile_building_mandate_surge×5
- world.gd: Add tile_building_mandate_surge outcome (bldg levels × turns → mandate)
- build_event_masterdoc.py: ARC_25 split out as FULL COMPLETION

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13358,17 +13358,17 @@
       </c>
       <c r="B195" s="67" t="inlineStr">
         <is>
-          <t>Carnival Barker</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C195" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_25</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D195" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CARNIVAL BARKER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
@@ -13386,9 +13386,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H195" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H195" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I195" s="68" t="inlineStr"/>
@@ -13414,7 +13414,7 @@
       </c>
       <c r="N195" s="69" t="inlineStr">
         <is>
-          <t>tile_yield gold×3; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13426,17 +13426,17 @@
       </c>
       <c r="B196" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C196" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D196" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="N196" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13494,17 +13494,17 @@
       </c>
       <c r="B197" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Nantucket Sailor</t>
         </is>
       </c>
       <c r="C197" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_13</t>
         </is>
       </c>
       <c r="D197" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] REFLOATS A HULL THAT WAS LISTED ON THE CHARTS AS A NAVIGATION HAZARD</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
@@ -13550,7 +13550,7 @@
       </c>
       <c r="N197" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield boats×3; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13562,17 +13562,17 @@
       </c>
       <c r="B198" s="67" t="inlineStr">
         <is>
-          <t>Nantucket Sailor</t>
+          <t>Frontier Preacher</t>
         </is>
       </c>
       <c r="C198" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_13</t>
+          <t>GOV_LOYAL_ARC_14</t>
         </is>
       </c>
       <c r="D198" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] REFLOATS A HULL THAT WAS LISTED ON THE CHARTS AS A NAVIGATION HAZARD</t>
+          <t>FRONTIER PREACHER INSPIRES THOUSANDS</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="N198" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield boats×3; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield culture×5; BTN2: resource_change manpower 1000; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13630,17 +13630,17 @@
       </c>
       <c r="B199" s="67" t="inlineStr">
         <is>
-          <t>Frontier Preacher</t>
+          <t>Carnival Barker</t>
         </is>
       </c>
       <c r="C199" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_14</t>
+          <t>GOV_LOYAL_ARC_25</t>
         </is>
       </c>
       <c r="D199" s="69" t="inlineStr">
         <is>
-          <t>FRONTIER PREACHER INSPIRES THOUSANDS</t>
+          <t>FOR ONE NIGHT ONLY!</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="N199" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield culture×5; BTN2: resource_change manpower 1000; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×5; BTN2: tile_building_mandate_surge×5 turns; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Implement ARC_02 (Appalachian Miner) full commander arc
- mil_mod.gd: Add Appalachian Hill Fighter, Explosives Expert, Mountain Pathfinder mods
- unit.gd: Hill Fighter +2 def in Foothills; Explosives Expert +10% ranged
- army.gd: Mountain Pathfinder +1 movement when starting turn in Foothills
- building.gd: ARC_02 mine scaling metal bonus (+1/2/3 by lvl); lvl3 no resource input; camp culture +1/2 at lvl 2/3
- world.gd: ARC_02 objectives — lvl2 mine + 500 manpower → FIRST; own tile + lvl4 mine + 800 manpower → DONE
- events.csv: ARC_02_FIRST/DONE text polished to match mine objective framing
- event_buttons.csv: ARC_02_FIRST_BTN1 → promote_commander (was nothing)
- masterdoc: ARC_02 FIRST and DONE marked FULL COMPLETION

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -14346,9 +14346,9 @@
           <t>ARC_02_DONE</t>
         </is>
       </c>
-      <c r="H210" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H210" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I210" s="32" t="inlineStr"/>
@@ -14410,9 +14410,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H211" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H211" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I211" s="32" t="inlineStr"/>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Complete GOV_LOYAL_ARC_12 (Continental Surgeon) — The Amputee's Handbook
Two-button design replacing the old single food-yield event:
- BTN1: all_armies_manpower_heal (25% of max manpower restored to all units)
- BTN2: set_governor_perk medical_science → +1 science per level from all buildings in tile

New outcome type all_armies_manpower_heal added to world.gd executeOutcome.
ARC_12 medical_science perk bonus added to building.gd _apply_governor_archetype_bonus.
Masterdoc updated: GOV_LOYAL_ARC_12 → FULL COMPLETION.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13290,17 +13290,17 @@
       </c>
       <c r="B194" s="67" t="inlineStr">
         <is>
-          <t>Continental Surgeon</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C194" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_12</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D194" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL CONTINENTAL SURGEON)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E194" s="5" t="inlineStr">
@@ -13318,9 +13318,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H194" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H194" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I194" s="68" t="inlineStr"/>
@@ -13346,7 +13346,7 @@
       </c>
       <c r="N194" s="69" t="inlineStr">
         <is>
-          <t>tile_yield food×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13358,17 +13358,17 @@
       </c>
       <c r="B195" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C195" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D195" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
@@ -13414,7 +13414,7 @@
       </c>
       <c r="N195" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13426,17 +13426,17 @@
       </c>
       <c r="B196" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Continental Surgeon</t>
         </is>
       </c>
       <c r="C196" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_12</t>
         </is>
       </c>
       <c r="D196" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>THE AMPUTEE'S HANDBOOK — [COMMANDER_NAME] SUBMITS A REPORT ON BATTLEFIELD MEDICINE</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="N196" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: all_armies_manpower_heal 25%; BTN2: set_governor_perk medical_science (+1 science all buildings); 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Complete GOV_LOYAL_ARC_11 (Boston Rabble-Rouser) — Speech That Does Not Disperse
Polished headline (removed duplicate [TILE_NAME]), tightened body text, updated
tone tag to Loud/Electric. Masterdoc → FULL COMPLETION.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -13222,17 +13222,17 @@
       </c>
       <c r="B193" s="67" t="inlineStr">
         <is>
-          <t>Boston Rabble-Rouser</t>
+          <t>Swamp Witch</t>
         </is>
       </c>
       <c r="C193" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_11</t>
+          <t>GOV_LOYAL_ARC_18</t>
         </is>
       </c>
       <c r="D193" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] (LOYAL BOSTON RABBLE-ROUSER)</t>
+          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
         </is>
       </c>
       <c r="E193" s="5" t="inlineStr">
@@ -13250,9 +13250,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H193" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H193" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I193" s="68" t="inlineStr"/>
@@ -13278,7 +13278,7 @@
       </c>
       <c r="N193" s="69" t="inlineStr">
         <is>
-          <t>tile_yield culture×4; 3%/turn at loyalty≥8; once per governor; text-only</t>
+          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13290,17 +13290,17 @@
       </c>
       <c r="B194" s="67" t="inlineStr">
         <is>
-          <t>Swamp Witch</t>
+          <t>Caribbean Privateer</t>
         </is>
       </c>
       <c r="C194" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_18</t>
+          <t>GOV_LOYAL_ARC_19</t>
         </is>
       </c>
       <c r="D194" s="69" t="inlineStr">
         <is>
-          <t>MESSAGE IN A BOTTLE FROM THE DEEP SWAMPS OF [TILE_NAME] — SEEK POWER? OR SEEK KNOWLEDGE?</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
         </is>
       </c>
       <c r="E194" s="5" t="inlineStr">
@@ -13346,7 +13346,7 @@
       </c>
       <c r="N194" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield magic×10; BTN2: level_all_spell_schools ×10; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -13358,17 +13358,17 @@
       </c>
       <c r="B195" s="67" t="inlineStr">
         <is>
-          <t>Caribbean Privateer</t>
+          <t>Boston Rabble-Rouser</t>
         </is>
       </c>
       <c r="C195" s="68" t="inlineStr">
         <is>
-          <t>GOV_LOYAL_ARC_19</t>
+          <t>GOV_LOYAL_ARC_11</t>
         </is>
       </c>
       <c r="D195" s="69" t="inlineStr">
         <is>
-          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] CLOSES AN UNDISCLOSED DEAL; GOLD ARRIVES WITHOUT EXPLANATION</t>
+          <t>DISPATCH FROM [TILE_NAME] — [COMMANDER_NAME] DELIVERS A SPEECH THAT DOES NOT DISPERSE</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
@@ -13414,7 +13414,7 @@
       </c>
       <c r="N195" s="69" t="inlineStr">
         <is>
-          <t>BTN1: tile_yield gold×4; 3%/turn at loyalty≥8; once per governor</t>
+          <t>BTN1: tile_yield culture×4; 3%/turn at loyalty≥8; once per governor</t>
         </is>
       </c>
     </row>
@@ -23019,7 +23019,7 @@
         </is>
       </c>
       <c r="B357" s="86" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Implement ARC_03 (Ivy League Dropout) full commander arc system
Building bonuses (_apply_governor_archetype_bonus):
- Global: +1 science from ALL buildings at gov lvl 3
- Library: +1/2/3 science per level by governor level
- Workshop/Market: +1/2 gold per level at governor level 2/3

Objectives (_check_arc01_objectives match block):
- Obj 1 (lvl 1→2): own Metro tile + library lvl 2+ → ARC_03_FIRST
- Obj 2 (lvl 2→3): own tile + 200 gold + 10 turns stationed → ARC_03_DONE

Mil mods already assigned (Steady Line, Street Tough, Flanking Drill, Continental Line).
Masterdoc: ARC_03_FIRST + ARC_03_DONE → FULL COMPLETION.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -14706,9 +14706,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H217" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
+      <c r="H217" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
         </is>
       </c>
       <c r="I217" s="32" t="inlineStr"/>
@@ -23187,7 +23187,7 @@
         </is>
       </c>
       <c r="B361" s="86" t="n">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="362" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Integrate WH_SECRET_09 (Halloween) — ghost presidents redesign + art
Event redesigned: trick-or-treaters with macadamia nut cookies and
x-ray screenings, then Ualani finds Lincoln/Harrison/Garfield/FDR
in the Lincoln Bedroom. They celebrate her as the first woman to
join their ranks, joke about White House loneliness, and offer a
genuine endorsement — not a performance.

New mechanic: Halloween Endorsement (BTN1)
- Sets CountryFlag "halloween_endorsement_turns" = 120 (10 years)
- _tick_halloween_endorsement() runs each turn: +1 TotalHappiness
  per unit in Ualani's army while flag is active
- BTN2: decline the endorsement (nothing outcome)

"Halloween Endorsement" entry added to mil_mod.gd for display.
Masterdoc: WH_SECRET_09 → FULL COMPLETION / Integrated.
_WH_SECRET_OVERRIDES dict added for per-event status overrides.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -18306,15 +18306,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H274" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I274" s="73" t="inlineStr"/>
-      <c r="J274" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H274" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I274" s="73" t="inlineStr">
+        <is>
+          <t>wh_secret_09</t>
+        </is>
+      </c>
+      <c r="J274" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K274" s="75" t="inlineStr">
@@ -23187,7 +23191,7 @@
         </is>
       </c>
       <c r="B361" s="86" t="n">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="362" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Polish WH_SECRET_07: Independence Day & Pride — FULL COMPLETION
Tightened body text, sharpened headline to "INDEPENDENCE DAY AT THE WHITE HOUSE — ALSO, PRIDE",
added rainbow flags on the Mall to weave in Pride angle. Set image_tag to wh_secret_07_scene.
Masterdoc status → FULL COMPLETION (art pending).

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -18170,12 +18170,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H272" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I272" s="73" t="inlineStr"/>
+      <c r="H272" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I272" s="73" t="inlineStr">
+        <is>
+          <t>wh_secret_07_scene</t>
+        </is>
+      </c>
       <c r="J272" s="7" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -23191,7 +23195,7 @@
         </is>
       </c>
       <c r="B361" s="86" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="362" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Integrate WH_SECRET art + reframe as exterior holiday celebrations (07, 08, 09, 12)
- WH_SECRET_07: July 4th exterior (fireworks + Continental flags); non-explicit
- WH_SECRET_08: Pride Month (rainbow flags at night); replaces skipped Diwali slot
- WH_SECRET_09: Halloween exterior (pumpkins on lawn); ghost presidents text kept
- WH_SECRET_12: Winter Holidays exterior (lit windows in December); non-explicit

All 4 art assets integrated; masterdoc updated to FULL COMPLETION.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -18152,7 +18152,7 @@
       </c>
       <c r="D272" s="74" t="inlineStr">
         <is>
-          <t>WHITE HOUSE SECRET — INDEPENDENCE DAY &amp; PRIDE</t>
+          <t>WHITE HOUSE SECRET — INDEPENDENCE DAY</t>
         </is>
       </c>
       <c r="E272" s="5" t="inlineStr">
@@ -18180,19 +18180,19 @@
           <t>wh_secret_07_scene</t>
         </is>
       </c>
-      <c r="J272" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K272" s="28" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="J272" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="K272" s="75" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="L272" s="73" t="inlineStr">
         <is>
-          <t>explicit option</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="M272" s="75" t="inlineStr">
@@ -18224,7 +18224,7 @@
       </c>
       <c r="D273" s="74" t="inlineStr">
         <is>
-          <t>WHITE HOUSE SECRET — DIWALI</t>
+          <t>WHITE HOUSE SECRET — PRIDE MONTH</t>
         </is>
       </c>
       <c r="E273" s="5" t="inlineStr">
@@ -18242,15 +18242,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H273" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I273" s="73" t="inlineStr"/>
-      <c r="J273" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H273" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I273" s="73" t="inlineStr">
+        <is>
+          <t>wh_secret_08_scene</t>
+        </is>
+      </c>
+      <c r="J273" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K273" s="75" t="inlineStr">
@@ -18500,7 +18504,7 @@
       </c>
       <c r="D277" s="74" t="inlineStr">
         <is>
-          <t>WHITE HOUSE SECRET — CHRISTMAS</t>
+          <t>WHITE HOUSE SECRET — WINTER HOLIDAYS</t>
         </is>
       </c>
       <c r="E277" s="5" t="inlineStr">
@@ -18518,25 +18522,29 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H277" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I277" s="73" t="inlineStr"/>
-      <c r="J277" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K277" s="28" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H277" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I277" s="73" t="inlineStr">
+        <is>
+          <t>wh_secret_12_scene</t>
+        </is>
+      </c>
+      <c r="J277" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="K277" s="75" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="L277" s="73" t="inlineStr">
         <is>
-          <t>sensual option</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="M277" s="75" t="inlineStr">
@@ -23195,7 +23203,7 @@
         </is>
       </c>
       <c r="B361" s="86" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="362" ht="20" customHeight="1">
@@ -23215,7 +23223,7 @@
         </is>
       </c>
       <c r="B363" s="86" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Integrate WH_SECRET_02: Black History Month (Pan-African flags, crowd at WH)
Renamed from President's Day. New exterior celebration text.
Art integrated as wh_secret_02_scene.png. FULL COMPLETION.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -17812,7 +17812,7 @@
       </c>
       <c r="D267" s="74" t="inlineStr">
         <is>
-          <t>WHITE HOUSE SECRET — PRESIDENT'S DAY</t>
+          <t>WHITE HOUSE SECRET — BLACK HISTORY MONTH</t>
         </is>
       </c>
       <c r="E267" s="5" t="inlineStr">
@@ -17830,15 +17830,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H267" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I267" s="73" t="inlineStr"/>
-      <c r="J267" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H267" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I267" s="73" t="inlineStr">
+        <is>
+          <t>wh_secret_02_scene</t>
+        </is>
+      </c>
+      <c r="J267" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K267" s="75" t="inlineStr">
@@ -23203,7 +23207,7 @@
         </is>
       </c>
       <c r="B361" s="86" t="n">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="362" ht="20" customHeight="1">

</xml_diff>

<commit_message>
WH_SECRET_03: Cherry Blossom Prayer — art + mechanics + text
- Rewrote event as news-style report of Ualani's National Mall tour
- Button: "A moment of peace goes a long way" → grants cherry_blossom_prayer flag
- New milmod: Cherry Blossom Prayer (display only; effect handled via CountryFlag)
- _tick_cherry_blossom_prayer(): +0.01 magic per unit across all armies per turn
- Float accumulator on country (cherry_blossom_magic_acc) avoids int conversion
- Permanent effect (no duration); wired into USA turn loop
- Art integrated as wh_secret_03_scene.png; FULL COMPLETION in masterdoc

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -17902,15 +17902,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H268" s="6" t="inlineStr">
-        <is>
-          <t>FIRST PASS</t>
-        </is>
-      </c>
-      <c r="I268" s="73" t="inlineStr"/>
-      <c r="J268" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H268" s="26" t="inlineStr">
+        <is>
+          <t>FULL COMPLETION</t>
+        </is>
+      </c>
+      <c r="I268" s="73" t="inlineStr">
+        <is>
+          <t>wh_secret_03_scene</t>
+        </is>
+      </c>
+      <c r="J268" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K268" s="75" t="inlineStr">
@@ -23207,7 +23211,7 @@
         </is>
       </c>
       <c r="B361" s="86" t="n">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="362" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Integrate art: Old Ironsides PROT_08 all four panels
- old_ironsides.png → PROT_08_SUMMON (image_tag was already set)
- prot_08_tame.png → PROT_08_TAME
- prot_08_agree.png → PROT_08_AGREE
- prot_08_agree_intimate.png → PROT_08_AGREE_INTIMATE

All four art_status → Integrated in build_event_masterdoc.py.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -3836,9 +3836,9 @@
           <t>old_ironsides</t>
         </is>
       </c>
-      <c r="J43" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J43" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K43" s="29" t="inlineStr">
@@ -3900,9 +3900,9 @@
         </is>
       </c>
       <c r="I44" s="24" t="inlineStr"/>
-      <c r="J44" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J44" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K44" s="29" t="inlineStr">
@@ -3964,9 +3964,9 @@
         </is>
       </c>
       <c r="I45" s="24" t="inlineStr"/>
-      <c r="J45" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J45" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K45" s="28" t="inlineStr">
@@ -22323,7 +22323,11 @@
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I344" s="81" t="inlineStr"/>
+      <c r="I344" s="81" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
       <c r="J344" s="70" t="inlineStr">
         <is>
           <t>N/A</t>

</xml_diff>

<commit_message>
Integrate art: Lincoln's Ghost arc (SUMMON, TAME, AGREE, AGREE_INTIMATE)
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -5608,9 +5608,9 @@
           <t>lincolns_ghost</t>
         </is>
       </c>
-      <c r="J70" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J70" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K70" s="29" t="inlineStr">
@@ -5672,9 +5672,9 @@
         </is>
       </c>
       <c r="I71" s="24" t="inlineStr"/>
-      <c r="J71" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J71" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K71" s="29" t="inlineStr">
@@ -5736,9 +5736,9 @@
         </is>
       </c>
       <c r="I72" s="24" t="inlineStr"/>
-      <c r="J72" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J72" s="27" t="inlineStr">
+        <is>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="K72" s="28" t="inlineStr">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="G353" s="82" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prot_17_agree_intimate</t>
         </is>
       </c>
       <c r="H353" s="83" t="inlineStr">
@@ -22903,7 +22903,11 @@
           <t>IDEA</t>
         </is>
       </c>
-      <c r="I353" s="81" t="inlineStr"/>
+      <c r="I353" s="81" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
       <c r="J353" s="70" t="inlineStr">
         <is>
           <t>N/A</t>

</xml_diff>

<commit_message>
Add 5 IDEA events: CL_WASHINGTON_01, CL_VALLEY_FORGE_01, CX_NYC_01, WINTER_SIEGE_01, SPRING_OFFENSIVE_01
- CL_WASHINGTON_01: DC recaptured by USA (tile 188, tile_liberated trigger TRIG_089, one-time)
- CL_VALLEY_FORGE_01: Valley Forge secured (tile 1, TRIG_090, one-time, historical weight)
- CX_NYC_01: NYC falls again to UK (tile 14, tile_lost TRIG_091, repeatable cooldown 30)
- WINTER_SIEGE_01: army hardship event (_check_winter_siege, month 11/12/1/2, winterScore≥3, cooldown 12)
- SPRING_OFFENSIVE_01: Crown spring offensive (_check_spring_offensive, month 3/4, UK neighbor, cooldown 20)

world.gd: _check_winter_siege() and _check_spring_offensive() added; both called from USA dispatch block
Masterdoc: 5 IDEA → FIRST PASS (221 total, 53 remaining IDEA)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/event_masterdoc.xlsx
+++ b/event_masterdoc.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +82,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00145A32"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007A5A00"/>
       <sz val="9"/>
     </font>
     <font>
@@ -369,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -630,181 +635,184 @@
     <xf numFmtId="0" fontId="2" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -19037,7 +19045,7 @@
       </c>
       <c r="D287" s="85" t="inlineStr">
         <is>
-          <t>WASHINGTON DC LIBERATED  ← IDEA</t>
+          <t>WASHINGTON DC RECAPTURED — THE CAPITAL RETURNS TO THE REPUBLIC</t>
         </is>
       </c>
       <c r="E287" s="5" t="inlineStr">
@@ -19055,15 +19063,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H287" s="86" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+      <c r="H287" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I287" s="84" t="inlineStr"/>
-      <c r="J287" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J287" s="86" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K287" s="87" t="inlineStr">
@@ -19079,7 +19087,7 @@
       </c>
       <c r="N287" s="85" t="inlineStr">
         <is>
-          <t>Would fire when tile 188 is recaptured; natural counterpart to CX_001</t>
+          <t>Fires via TRIG_089 (tile_liberated, 188, USA); one-time historic event; 2 buttons</t>
         </is>
       </c>
     </row>
@@ -19101,7 +19109,7 @@
       </c>
       <c r="D288" s="85" t="inlineStr">
         <is>
-          <t>VALLEY FORGE SECURED  ← IDEA</t>
+          <t>VALLEY FORGE IS OURS — THE REPUBLIC HOLDS THE GROUND THAT HELD BEFORE</t>
         </is>
       </c>
       <c r="E288" s="5" t="inlineStr">
@@ -19119,15 +19127,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H288" s="86" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+      <c r="H288" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I288" s="84" t="inlineStr"/>
-      <c r="J288" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J288" s="86" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K288" s="87" t="inlineStr">
@@ -19143,7 +19151,7 @@
       </c>
       <c r="N288" s="85" t="inlineStr">
         <is>
-          <t>Tile 1; historically significant; would fire on liberation</t>
+          <t>Fires via TRIG_090 (tile_liberated, 1, USA); one-time; 2 buttons; historical weight tone</t>
         </is>
       </c>
     </row>
@@ -19165,7 +19173,7 @@
       </c>
       <c r="D289" s="85" t="inlineStr">
         <is>
-          <t>NEW YORK CITY FALLS AGAIN  ← IDEA</t>
+          <t>NEW YORK CITY HAS FALLEN — AGAIN — THE STOCK MARKET IS FORMALLY AGGRIEVED</t>
         </is>
       </c>
       <c r="E289" s="5" t="inlineStr">
@@ -19183,15 +19191,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H289" s="86" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+      <c r="H289" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I289" s="84" t="inlineStr"/>
-      <c r="J289" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J289" s="86" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K289" s="87" t="inlineStr">
@@ -19207,7 +19215,7 @@
       </c>
       <c r="N289" s="85" t="inlineStr">
         <is>
-          <t>Would fire if NYC is re-taken after CL_001; repeatable pair</t>
+          <t>Fires via TRIG_091 (tile_lost, 14, UK); repeatable=true, cooldown=30; satirical callback to CL_001</t>
         </is>
       </c>
     </row>
@@ -19247,7 +19255,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H290" s="86" t="inlineStr">
+      <c r="H290" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19311,7 +19319,7 @@
           <t>→ CMD_OBJECTIVE_3?</t>
         </is>
       </c>
-      <c r="H291" s="86" t="inlineStr">
+      <c r="H291" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19357,7 +19365,7 @@
       </c>
       <c r="D292" s="85" t="inlineStr">
         <is>
-          <t>VALLEY FORGE CONDITIONS: ARMY SUFFERING IN THE FIELD  ← IDEA</t>
+          <t>VALLEY FORGE CONDITIONS — TROOPS SUFFER THROUGH ANOTHER NORTHERN WINTER</t>
         </is>
       </c>
       <c r="E292" s="5" t="inlineStr">
@@ -19375,15 +19383,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H292" s="86" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+      <c r="H292" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I292" s="84" t="inlineStr"/>
-      <c r="J292" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J292" s="86" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K292" s="87" t="inlineStr">
@@ -19399,7 +19407,7 @@
       </c>
       <c r="N292" s="85" t="inlineStr">
         <is>
-          <t>Generic winter hardship event; non-Ualani; uses winterScore + month check</t>
+          <t>_check_winter_siege(): month [11,12,1,2] + owned tile winterScore&gt;=3 + stationedArmy; cooldown=12; 2 buttons</t>
         </is>
       </c>
     </row>
@@ -19421,7 +19429,7 @@
       </c>
       <c r="D293" s="85" t="inlineStr">
         <is>
-          <t>THE THAW: CROWN FORCES RESUME OFFENSIVE OPERATIONS  ← IDEA</t>
+          <t>THE THAW — CROWN FORCES RESUME OFFENSIVE OPERATIONS</t>
         </is>
       </c>
       <c r="E293" s="5" t="inlineStr">
@@ -19439,15 +19447,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H293" s="86" t="inlineStr">
-        <is>
-          <t>IDEA</t>
+      <c r="H293" s="6" t="inlineStr">
+        <is>
+          <t>FIRST PASS</t>
         </is>
       </c>
       <c r="I293" s="84" t="inlineStr"/>
-      <c r="J293" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J293" s="86" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K293" s="87" t="inlineStr">
@@ -19463,7 +19471,7 @@
       </c>
       <c r="N293" s="85" t="inlineStr">
         <is>
-          <t>Month 3-4; UK neighbor + player army present; tactical pressure event</t>
+          <t>_check_spring_offensive(): month [3,4] + UK neighbor + stationedArmy on owned tile; cooldown=20; 2 buttons</t>
         </is>
       </c>
     </row>
@@ -19519,7 +19527,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H295" s="86" t="inlineStr">
+      <c r="H295" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19599,7 +19607,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H297" s="86" t="inlineStr">
+      <c r="H297" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19679,7 +19687,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H299" s="86" t="inlineStr">
+      <c r="H299" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19759,7 +19767,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H301" s="86" t="inlineStr">
+      <c r="H301" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19823,7 +19831,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H302" s="86" t="inlineStr">
+      <c r="H302" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19903,7 +19911,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H304" s="86" t="inlineStr">
+      <c r="H304" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -19967,7 +19975,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H305" s="86" t="inlineStr">
+      <c r="H305" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20031,7 +20039,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H306" s="86" t="inlineStr">
+      <c r="H306" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20095,7 +20103,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H307" s="86" t="inlineStr">
+      <c r="H307" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20175,7 +20183,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H309" s="86" t="inlineStr">
+      <c r="H309" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20239,7 +20247,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H310" s="86" t="inlineStr">
+      <c r="H310" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20303,7 +20311,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H311" s="86" t="inlineStr">
+      <c r="H311" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20367,7 +20375,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H312" s="86" t="inlineStr">
+      <c r="H312" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20431,7 +20439,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H313" s="86" t="inlineStr">
+      <c r="H313" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20495,7 +20503,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H314" s="86" t="inlineStr">
+      <c r="H314" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20559,7 +20567,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H315" s="86" t="inlineStr">
+      <c r="H315" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20639,7 +20647,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H317" s="86" t="inlineStr">
+      <c r="H317" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20703,7 +20711,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H318" s="86" t="inlineStr">
+      <c r="H318" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20767,7 +20775,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H319" s="86" t="inlineStr">
+      <c r="H319" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20831,7 +20839,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H320" s="86" t="inlineStr">
+      <c r="H320" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20895,7 +20903,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H321" s="86" t="inlineStr">
+      <c r="H321" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -20959,7 +20967,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H322" s="86" t="inlineStr">
+      <c r="H322" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21023,7 +21031,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H323" s="86" t="inlineStr">
+      <c r="H323" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21087,7 +21095,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H324" s="86" t="inlineStr">
+      <c r="H324" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21167,7 +21175,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H326" s="86" t="inlineStr">
+      <c r="H326" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21231,7 +21239,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H327" s="86" t="inlineStr">
+      <c r="H327" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21295,7 +21303,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H328" s="86" t="inlineStr">
+      <c r="H328" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21359,7 +21367,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H329" s="86" t="inlineStr">
+      <c r="H329" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21423,7 +21431,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H330" s="86" t="inlineStr">
+      <c r="H330" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21487,7 +21495,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H331" s="86" t="inlineStr">
+      <c r="H331" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21551,7 +21559,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H332" s="86" t="inlineStr">
+      <c r="H332" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21615,7 +21623,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H333" s="86" t="inlineStr">
+      <c r="H333" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21695,7 +21703,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H335" s="86" t="inlineStr">
+      <c r="H335" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21827,7 +21835,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H337" s="86" t="inlineStr">
+      <c r="H337" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21891,7 +21899,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H338" s="86" t="inlineStr">
+      <c r="H338" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -21955,7 +21963,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H339" s="86" t="inlineStr">
+      <c r="H339" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22019,7 +22027,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H340" s="86" t="inlineStr">
+      <c r="H340" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22083,7 +22091,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H341" s="86" t="inlineStr">
+      <c r="H341" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22147,7 +22155,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H342" s="86" t="inlineStr">
+      <c r="H342" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22215,7 +22223,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H343" s="86" t="inlineStr">
+      <c r="H343" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22279,7 +22287,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H344" s="86" t="inlineStr">
+      <c r="H344" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22343,7 +22351,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H345" s="86" t="inlineStr">
+      <c r="H345" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22407,7 +22415,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H346" s="86" t="inlineStr">
+      <c r="H346" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22471,7 +22479,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H347" s="86" t="inlineStr">
+      <c r="H347" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22535,7 +22543,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H348" s="86" t="inlineStr">
+      <c r="H348" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22599,7 +22607,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H349" s="86" t="inlineStr">
+      <c r="H349" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22663,7 +22671,7 @@
           <t>prot_17_agree_intimate</t>
         </is>
       </c>
-      <c r="H350" s="86" t="inlineStr">
+      <c r="H350" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22747,7 +22755,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H352" s="86" t="inlineStr">
+      <c r="H352" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22811,7 +22819,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H353" s="86" t="inlineStr">
+      <c r="H353" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22875,7 +22883,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H354" s="86" t="inlineStr">
+      <c r="H354" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22939,7 +22947,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H355" s="86" t="inlineStr">
+      <c r="H355" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -22968,42 +22976,42 @@
       </c>
     </row>
     <row r="357" ht="20" customHeight="1">
-      <c r="A357" s="88" t="inlineStr">
+      <c r="A357" s="89" t="inlineStr">
         <is>
           <t>Total events in spreadsheet</t>
         </is>
       </c>
-      <c r="B357" s="89" t="n">
+      <c r="B357" s="90" t="n">
         <v>320</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">
-      <c r="A358" s="88" t="inlineStr">
+      <c r="A358" s="89" t="inlineStr">
         <is>
           <t>FIRST PASS (coded &amp; wired)</t>
         </is>
       </c>
-      <c r="B358" s="89" t="n">
-        <v>216</v>
+      <c r="B358" s="90" t="n">
+        <v>221</v>
       </c>
     </row>
     <row r="359" ht="20" customHeight="1">
-      <c r="A359" s="88" t="inlineStr">
+      <c r="A359" s="89" t="inlineStr">
         <is>
           <t>IDEA (not yet implemented)</t>
         </is>
       </c>
-      <c r="B359" s="89" t="n">
-        <v>58</v>
+      <c r="B359" s="90" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="360" ht="20" customHeight="1">
-      <c r="A360" s="88" t="inlineStr">
+      <c r="A360" s="89" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B360" s="89" t="n">
+      <c r="B360" s="90" t="n">
         <v>52</v>
       </c>
     </row>
@@ -25785,7 +25793,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H43" s="86" t="inlineStr">
+      <c r="H43" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -25849,7 +25857,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H44" s="86" t="inlineStr">
+      <c r="H44" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -25913,7 +25921,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H45" s="86" t="inlineStr">
+      <c r="H45" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -25977,7 +25985,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H46" s="86" t="inlineStr">
+      <c r="H46" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26041,7 +26049,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H47" s="86" t="inlineStr">
+      <c r="H47" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26105,7 +26113,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H48" s="86" t="inlineStr">
+      <c r="H48" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26169,7 +26177,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H49" s="86" t="inlineStr">
+      <c r="H49" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26249,7 +26257,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H51" s="86" t="inlineStr">
+      <c r="H51" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26313,7 +26321,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H52" s="86" t="inlineStr">
+      <c r="H52" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26377,7 +26385,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H53" s="86" t="inlineStr">
+      <c r="H53" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26441,7 +26449,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H54" s="86" t="inlineStr">
+      <c r="H54" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26505,7 +26513,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H55" s="86" t="inlineStr">
+      <c r="H55" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26569,7 +26577,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H56" s="86" t="inlineStr">
+      <c r="H56" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26633,7 +26641,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H57" s="86" t="inlineStr">
+      <c r="H57" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26697,7 +26705,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H58" s="86" t="inlineStr">
+      <c r="H58" s="88" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
@@ -26726,42 +26734,42 @@
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="88" t="inlineStr">
+      <c r="A60" s="89" t="inlineStr">
         <is>
           <t>Canadian events total</t>
         </is>
       </c>
-      <c r="B60" s="89" t="n">
+      <c r="B60" s="90" t="n">
         <v>54</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="88" t="inlineStr">
+      <c r="A61" s="89" t="inlineStr">
         <is>
           <t>Canada (Alliance arc)</t>
         </is>
       </c>
-      <c r="B61" s="89" t="n">
+      <c r="B61" s="90" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="88" t="inlineStr">
+      <c r="A62" s="89" t="inlineStr">
         <is>
           <t>CA Protector (Jessica's creatures)</t>
         </is>
       </c>
-      <c r="B62" s="89" t="n">
+      <c r="B62" s="90" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="88" t="inlineStr">
+      <c r="A63" s="89" t="inlineStr">
         <is>
           <t>Need explicit art (YES)</t>
         </is>
       </c>
-      <c r="B63" s="89" t="n">
+      <c r="B63" s="90" t="n">
         <v>12</v>
       </c>
     </row>
@@ -26785,412 +26793,412 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="90" t="inlineStr">
+      <c r="A1" s="91" t="inlineStr">
         <is>
           <t>STATUS LEGEND</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="91" t="inlineStr">
+      <c r="A2" s="92" t="inlineStr">
         <is>
           <t>FULL COMPLETION</t>
         </is>
       </c>
-      <c r="B2" s="92" t="inlineStr">
+      <c r="B2" s="93" t="inlineStr">
         <is>
           <t>Final pass done — art integrated, text finalized, fully tested</t>
         </is>
       </c>
-      <c r="C2" s="92" t="n"/>
+      <c r="C2" s="93" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="93" t="inlineStr">
+      <c r="A3" s="94" t="inlineStr">
         <is>
           <t>FIRST PASS</t>
         </is>
       </c>
-      <c r="B3" s="94" t="inlineStr">
+      <c r="B3" s="95" t="inlineStr">
         <is>
           <t>Event is coded, in CSV, all buttons wired; no final polish yet</t>
         </is>
       </c>
-      <c r="C3" s="94" t="n"/>
+      <c r="C3" s="95" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="95" t="inlineStr">
+      <c r="A4" s="96" t="inlineStr">
         <is>
           <t>IDEA</t>
         </is>
       </c>
-      <c r="B4" s="96" t="inlineStr">
+      <c r="B4" s="97" t="inlineStr">
         <is>
           <t>Concept stage: not in events.csv; some referenced in button CSV</t>
         </is>
       </c>
-      <c r="C4" s="96" t="n"/>
+      <c r="C4" s="97" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="90" t="inlineStr">
+      <c r="A6" s="91" t="inlineStr">
         <is>
           <t>ART STATUS LEGEND</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="97" t="inlineStr">
+      <c r="A7" s="98" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="B7" s="98" t="inlineStr">
+      <c r="B7" s="99" t="inlineStr">
         <is>
           <t>No art asset exists yet</t>
         </is>
       </c>
-      <c r="C7" s="98" t="n"/>
+      <c r="C7" s="99" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="95" t="inlineStr">
+      <c r="A8" s="96" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="B8" s="96" t="inlineStr">
+      <c r="B8" s="97" t="inlineStr">
         <is>
           <t>Art is being created but not in engine</t>
         </is>
       </c>
-      <c r="C8" s="96" t="n"/>
+      <c r="C8" s="97" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="99" t="inlineStr">
+      <c r="A9" s="100" t="inlineStr">
         <is>
           <t>Integrated</t>
         </is>
       </c>
-      <c r="B9" s="100" t="inlineStr">
+      <c r="B9" s="101" t="inlineStr">
         <is>
           <t>Art is in the project and referenced correctly</t>
         </is>
       </c>
-      <c r="C9" s="100" t="n"/>
+      <c r="C9" s="101" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="90" t="inlineStr">
+      <c r="A11" s="91" t="inlineStr">
         <is>
           <t>EXPLICIT ART LEGEND</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="101" t="inlineStr">
+      <c r="A12" s="102" t="inlineStr">
         <is>
           <t>YES — Explicit Art Needed</t>
         </is>
       </c>
-      <c r="B12" s="102" t="inlineStr">
+      <c r="B12" s="103" t="inlineStr">
         <is>
           <t>Event has explicit or kinky_lewd content flag OR has at least one explicit button option that will need unique explicit artwork</t>
         </is>
       </c>
-      <c r="C12" s="102" t="n"/>
+      <c r="C12" s="103" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="103" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="B13" s="104" t="inlineStr">
+      <c r="A13" s="104" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B13" s="105" t="inlineStr">
         <is>
           <t>Standard event — no adult artwork required</t>
         </is>
       </c>
-      <c r="C13" s="104" t="n"/>
+      <c r="C13" s="105" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="90" t="inlineStr">
+      <c r="A15" s="91" t="inlineStr">
         <is>
           <t>CHAIN POSITION LEGEND</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="105" t="inlineStr">
+      <c r="A16" s="106" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="B16" s="106" t="inlineStr">
+      <c r="B16" s="107" t="inlineStr">
         <is>
           <t>Standalone event or first event in a chain; fires from world.gd check function or EventDatabase date trigger</t>
         </is>
       </c>
-      <c r="C16" s="106" t="n"/>
+      <c r="C16" s="107" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="107" t="inlineStr">
+      <c r="A17" s="108" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="B17" s="108" t="inlineStr">
+      <c r="B17" s="109" t="inlineStr">
         <is>
           <t>Fires as outcome of a choice button on a Root/prior event; represents one path in a fork</t>
         </is>
       </c>
-      <c r="C17" s="108" t="n"/>
+      <c r="C17" s="109" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="109" t="inlineStr">
+      <c r="A18" s="110" t="inlineStr">
         <is>
           <t>Followup</t>
         </is>
       </c>
-      <c r="B18" s="110" t="inlineStr">
+      <c r="B18" s="111" t="inlineStr">
         <is>
           <t>Fires automatically after a mission completes (via next_event_id or mission flag return)</t>
         </is>
       </c>
-      <c r="C18" s="110" t="n"/>
+      <c r="C18" s="111" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="90" t="inlineStr">
+      <c r="A20" s="91" t="inlineStr">
         <is>
           <t>CATEGORY COLOR LEGEND</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="111" t="inlineStr">
+      <c r="A21" s="112" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B21" s="112" t="inlineStr">
+      <c r="B21" s="113" t="inlineStr">
         <is>
           <t>Calendar-triggered events; month or turn-based</t>
         </is>
       </c>
-      <c r="C21" s="112" t="n"/>
+      <c r="C21" s="113" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="113" t="inlineStr">
+      <c r="A22" s="114" t="inlineStr">
         <is>
           <t>City Liberated</t>
         </is>
       </c>
-      <c r="B22" s="114" t="inlineStr">
+      <c r="B22" s="115" t="inlineStr">
         <is>
           <t>Fires when a specific tile is liberated (city_liberated type)</t>
         </is>
       </c>
-      <c r="C22" s="114" t="n"/>
+      <c r="C22" s="115" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="115" t="inlineStr">
+      <c r="A23" s="116" t="inlineStr">
         <is>
           <t>City Lost</t>
         </is>
       </c>
-      <c r="B23" s="116" t="inlineStr">
+      <c r="B23" s="117" t="inlineStr">
         <is>
           <t>Fires when a specific tile falls to the enemy (city_lost type)</t>
         </is>
       </c>
-      <c r="C23" s="116" t="n"/>
+      <c r="C23" s="117" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="117" t="inlineStr">
+      <c r="A24" s="118" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B24" s="118" t="inlineStr">
+      <c r="B24" s="119" t="inlineStr">
         <is>
           <t>State-level liberation, secession, and reintegration</t>
         </is>
       </c>
-      <c r="C24" s="118" t="n"/>
+      <c r="C24" s="119" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="119" t="inlineStr">
+      <c r="A25" s="120" t="inlineStr">
         <is>
           <t>Protector</t>
         </is>
       </c>
-      <c r="B25" s="120" t="inlineStr">
+      <c r="B25" s="121" t="inlineStr">
         <is>
           <t>Mythological entity summon events (protector_summon type)</t>
         </is>
       </c>
-      <c r="C25" s="120" t="n"/>
+      <c r="C25" s="121" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="121" t="inlineStr">
+      <c r="A26" s="122" t="inlineStr">
         <is>
           <t>Commander</t>
         </is>
       </c>
-      <c r="B26" s="122" t="inlineStr">
+      <c r="B26" s="123" t="inlineStr">
         <is>
           <t>Named commander arc events (commander_* types)</t>
         </is>
       </c>
-      <c r="C26" s="122" t="n"/>
+      <c r="C26" s="123" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="123" t="inlineStr">
+      <c r="A27" s="124" t="inlineStr">
         <is>
           <t>Fort Chain</t>
         </is>
       </c>
-      <c r="B27" s="124" t="inlineStr">
+      <c r="B27" s="125" t="inlineStr">
         <is>
           <t>Fort disrepair investigation chain (fort_* types)</t>
         </is>
       </c>
-      <c r="C27" s="124" t="n"/>
+      <c r="C27" s="125" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="125" t="inlineStr">
+      <c r="A28" s="126" t="inlineStr">
         <is>
           <t>Collapse</t>
         </is>
       </c>
-      <c r="B28" s="126" t="inlineStr">
+      <c r="B28" s="127" t="inlineStr">
         <is>
           <t>Republic collapse sequence</t>
         </is>
       </c>
-      <c r="C28" s="126" t="n"/>
+      <c r="C28" s="127" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="127" t="inlineStr">
+      <c r="A29" s="128" t="inlineStr">
         <is>
           <t>Tile Crisis</t>
         </is>
       </c>
-      <c r="B29" s="128" t="inlineStr">
+      <c r="B29" s="129" t="inlineStr">
         <is>
           <t>Dynamic tile-based crisis chains; triggered by world.gd check functions</t>
         </is>
       </c>
-      <c r="C29" s="128" t="n"/>
+      <c r="C29" s="129" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="129" t="inlineStr">
+      <c r="A30" s="130" t="inlineStr">
         <is>
           <t>Ualani</t>
         </is>
       </c>
-      <c r="B30" s="130" t="inlineStr">
+      <c r="B30" s="131" t="inlineStr">
         <is>
           <t>Ualani Carlisle army presence events; personal storyline</t>
         </is>
       </c>
-      <c r="C30" s="130" t="n"/>
+      <c r="C30" s="131" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="131" t="inlineStr">
+      <c r="A31" s="132" t="inlineStr">
         <is>
           <t>VP Arc</t>
         </is>
       </c>
-      <c r="B31" s="132" t="inlineStr">
+      <c r="B31" s="133" t="inlineStr">
         <is>
           <t>Vice President relationship arc; 9 events tied to the VP governor</t>
         </is>
       </c>
-      <c r="C31" s="132" t="n"/>
+      <c r="C31" s="133" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="133" t="inlineStr">
+      <c r="A32" s="134" t="inlineStr">
         <is>
           <t>CA PM Arc</t>
         </is>
       </c>
-      <c r="B32" s="134" t="inlineStr"/>
-      <c r="C32" s="134" t="n"/>
+      <c r="B32" s="135" t="inlineStr"/>
+      <c r="C32" s="135" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="135" t="inlineStr">
+      <c r="A33" s="136" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="B33" s="136" t="inlineStr">
+      <c r="B33" s="137" t="inlineStr">
         <is>
           <t>Canadian Alliance diplomatic arc + 3 peace events (PEACE_ALLIED_01, PEACE_USA_01, PEACE_CA_AI_01)</t>
         </is>
       </c>
-      <c r="C33" s="136" t="n"/>
+      <c r="C33" s="137" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="137" t="inlineStr">
+      <c r="A34" s="138" t="inlineStr">
         <is>
           <t>CA Protector</t>
         </is>
       </c>
-      <c r="B34" s="138" t="inlineStr">
+      <c r="B34" s="139" t="inlineStr">
         <is>
           <t>Jessica Commanda Odjick's 8 creature arcs; Algonquin, Mi'kmaq, French-Canadian folklore</t>
         </is>
       </c>
-      <c r="C34" s="138" t="n"/>
+      <c r="C34" s="139" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="139" t="inlineStr">
+      <c r="A35" s="140" t="inlineStr">
         <is>
           <t>Loyal Governor</t>
         </is>
       </c>
-      <c r="B35" s="140" t="inlineStr">
+      <c r="B35" s="141" t="inlineStr">
         <is>
           <t>25 one-shot dispatch events, one per USA governor archetype; tile_yield resource×turns; 3% chance/turn at loyalty≥8</t>
         </is>
       </c>
-      <c r="C35" s="140" t="n"/>
+      <c r="C35" s="141" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="141" t="inlineStr">
+      <c r="A36" s="142" t="inlineStr">
         <is>
           <t>White House</t>
         </is>
       </c>
-      <c r="B36" s="142" t="inlineStr">
+      <c r="B36" s="143" t="inlineStr">
         <is>
           <t>12 personal Ualani events (WH_SECRET_01–12); fires when she is stationed at DC (tile 188) during the matching calendar month; all sensual in tone; some have explicit BTN2</t>
         </is>
       </c>
-      <c r="C36" s="142" t="n"/>
+      <c r="C36" s="143" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="143" t="inlineStr">
+      <c r="A37" s="144" t="inlineStr">
         <is>
           <t>Chalchiuhtotolin</t>
         </is>
       </c>
-      <c r="B37" s="144" t="inlineStr">
+      <c r="B37" s="145" t="inlineStr">
         <is>
           <t>5-event super-secret arc (CHALCH_SUMMON → Q1 → Q2 → Q3 → AGREE); fires only when Ualani is at Plymouth (tile 66) on Thanksgiving (month 11); quests: 3 farms, 150 food, 5 farms; reward: up to +220 food total</t>
         </is>
       </c>
-      <c r="C37" s="144" t="n"/>
+      <c r="C37" s="145" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="145" t="inlineStr">
+      <c r="A38" s="146" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="B38" s="146" t="inlineStr">
+      <c r="B38" s="147" t="inlineStr">
         <is>
           <t>Not yet implemented; concept stage or referenced-but-missing events</t>
         </is>
       </c>
-      <c r="C38" s="146" t="n"/>
+      <c r="C38" s="147" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>